<commit_message>
docs: baseline do RAG atual no benchmark da fase 3
25 perguntas rodadas (gpt-oss-20b/120b via roteamento): 20/25
responderam "Não encontrado no corpus" e as 5 restantes citam só
LGPD/LAI genéricas, sem Lei 6.015 nem o Código de Normas do CE.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fase3/benchmark/planilha_benchmark.xlsx
+++ b/docs/fase3/benchmark/planilha_benchmark.xlsx
@@ -4522,13 +4522,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A77,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E77" s="8" t="n"/>
-      <c r="F77" s="8" t="n"/>
-      <c r="G77" s="8" t="n"/>
-      <c r="H77" s="8" t="n"/>
-      <c r="I77" s="8" t="n"/>
-      <c r="J77" s="8" t="n"/>
-      <c r="K77" s="8" t="n"/>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F77" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G77" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H77" s="8" t="inlineStr">
+        <is>
+          <t>manual_praticas_cartorarias_1_grau.pdf:p5; curso-159994-aula-10-aeca-completo.pdf:p13; Lei_licitacoes_contratos_administrativos_4ed.pdf:p13; curso-159994-aula-06-bonus-799b-completo.pdf:p23; curso-160250-aula-00-480f-completo.pdf:p4</t>
+        </is>
+      </c>
+      <c r="I77" s="8" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="J77" s="8" t="n">
+        <v>1956</v>
+      </c>
+      <c r="K77" s="8" t="n">
+        <v>122</v>
+      </c>
       <c r="L77" s="10">
         <f>IF(COUNT(J77:K77)=2,(J77*Parametros!$B$3+K77*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -4561,13 +4583,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A78,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E78" s="8" t="n"/>
-      <c r="F78" s="8" t="n"/>
-      <c r="G78" s="8" t="n"/>
-      <c r="H78" s="8" t="n"/>
-      <c r="I78" s="8" t="n"/>
-      <c r="J78" s="8" t="n"/>
-      <c r="K78" s="8" t="n"/>
+      <c r="E78" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F78" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G78" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H78" s="8" t="inlineStr">
+        <is>
+          <t>curso-160250-aula-01-b2c9-completo.pdf:p115; Lei_licitacoes_contratos_administrativos_4ed.pdf:p51; curso-159994-aula-06-43dd-completo.pdf:p59; curso-159994-aula-02-daa4-completo.pdf:p84; Lei_licitacoes_contratos_administrativos_4ed.pdf:p23</t>
+        </is>
+      </c>
+      <c r="I78" s="8" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="J78" s="8" t="n">
+        <v>2045</v>
+      </c>
+      <c r="K78" s="8" t="n">
+        <v>231</v>
+      </c>
       <c r="L78" s="10">
         <f>IF(COUNT(J78:K78)=2,(J78*Parametros!$B$3+K78*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -4600,13 +4644,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A79,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E79" s="8" t="n"/>
-      <c r="F79" s="8" t="n"/>
-      <c r="G79" s="8" t="n"/>
-      <c r="H79" s="8" t="n"/>
-      <c r="I79" s="8" t="n"/>
-      <c r="J79" s="8" t="n"/>
-      <c r="K79" s="8" t="n"/>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F79" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G79" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus</t>
+        </is>
+      </c>
+      <c r="H79" s="8" t="inlineStr">
+        <is>
+          <t>LGPD-2023-ANPD.pdf:p9; curso-159994-aula-02-daa4-completo.pdf:p65; Lei_licitacoes_contratos_administrativos_4ed.pdf:p75; curso-159994-aula-11-d0d4-completo.pdf:p51; curso-159994-aula-02-daa4-completo.pdf:p58</t>
+        </is>
+      </c>
+      <c r="I79" s="8" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="J79" s="8" t="n">
+        <v>1971</v>
+      </c>
+      <c r="K79" s="8" t="n">
+        <v>171</v>
+      </c>
       <c r="L79" s="10">
         <f>IF(COUNT(J79:K79)=2,(J79*Parametros!$B$3+K79*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -4639,13 +4705,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A80,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E80" s="8" t="n"/>
-      <c r="F80" s="8" t="n"/>
-      <c r="G80" s="8" t="n"/>
-      <c r="H80" s="8" t="n"/>
-      <c r="I80" s="8" t="n"/>
-      <c r="J80" s="8" t="n"/>
-      <c r="K80" s="8" t="n"/>
+      <c r="E80" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F80" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G80" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H80" s="8" t="inlineStr">
+        <is>
+          <t>GTA_executivo_federal_7ed.pdf:p8; gta_executivo_federal_7ed.pdf:p8; cartilha_inss_digital_oabsp.pdf:p34; GTA_executivo_federal_7ed.pdf:p34; gta_executivo_federal_7ed.pdf:p34</t>
+        </is>
+      </c>
+      <c r="I80" s="8" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="J80" s="8" t="n">
+        <v>1862</v>
+      </c>
+      <c r="K80" s="8" t="n">
+        <v>148</v>
+      </c>
       <c r="L80" s="10">
         <f>IF(COUNT(J80:K80)=2,(J80*Parametros!$B$3+K80*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -4678,13 +4766,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A81,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E81" s="8" t="n"/>
-      <c r="F81" s="8" t="n"/>
-      <c r="G81" s="8" t="n"/>
-      <c r="H81" s="8" t="n"/>
-      <c r="I81" s="8" t="n"/>
-      <c r="J81" s="8" t="n"/>
-      <c r="K81" s="8" t="n"/>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F81" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G81" s="8" t="inlineStr">
+        <is>
+          <t>**Não encontrado no corpus**</t>
+        </is>
+      </c>
+      <c r="H81" s="8" t="inlineStr">
+        <is>
+          <t>manual_praticas_cartorarias_1_grau.pdf:p27; GTA_executivo_federal_7ed.pdf:p28; gta_executivo_federal_7ed.pdf:p28; LGPD-2023-ANPD.pdf:p9; GTA_executivo_federal_7ed.pdf:p29</t>
+        </is>
+      </c>
+      <c r="I81" s="8" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="J81" s="8" t="n">
+        <v>1882</v>
+      </c>
+      <c r="K81" s="8" t="n">
+        <v>104</v>
+      </c>
       <c r="L81" s="10">
         <f>IF(COUNT(J81:K81)=2,(J81*Parametros!$B$3+K81*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -4717,13 +4827,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A82,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E82" s="8" t="n"/>
-      <c r="F82" s="8" t="n"/>
-      <c r="G82" s="8" t="n"/>
-      <c r="H82" s="8" t="n"/>
-      <c r="I82" s="8" t="n"/>
-      <c r="J82" s="8" t="n"/>
-      <c r="K82" s="8" t="n"/>
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F82" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G82" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H82" s="8" t="inlineStr">
+        <is>
+          <t>inss_beneficios.pdf:p1; cartilha_inss_digital_oabsp.pdf:p18; cartilha_inss_digital_oabsp.pdf:p42; GTA_executivo_federal_7ed.pdf:p40; gta_executivo_federal_7ed.pdf:p40</t>
+        </is>
+      </c>
+      <c r="I82" s="8" t="n">
+        <v>8.210000000000001</v>
+      </c>
+      <c r="J82" s="8" t="n">
+        <v>1592</v>
+      </c>
+      <c r="K82" s="8" t="n">
+        <v>363</v>
+      </c>
       <c r="L82" s="10">
         <f>IF(COUNT(J82:K82)=2,(J82*Parametros!$B$3+K82*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -4756,13 +4888,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A83,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E83" s="8" t="n"/>
-      <c r="F83" s="8" t="n"/>
-      <c r="G83" s="8" t="n"/>
-      <c r="H83" s="8" t="n"/>
-      <c r="I83" s="8" t="n"/>
-      <c r="J83" s="8" t="n"/>
-      <c r="K83" s="8" t="n"/>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F83" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G83" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H83" s="8" t="inlineStr">
+        <is>
+          <t>manual_praticas_cartorarias_1_grau.pdf:p40; curso-159994-aula-23-d320-completo.pdf:p8; curso-159994-aula-23-d320-completo.pdf:p36; curso-159994-aula-07-292a-completo.pdf:p102; curso-159994-aula-07-292a-completo.pdf:p76</t>
+        </is>
+      </c>
+      <c r="I83" s="8" t="n">
+        <v>13.87</v>
+      </c>
+      <c r="J83" s="8" t="n">
+        <v>1792</v>
+      </c>
+      <c r="K83" s="8" t="n">
+        <v>163</v>
+      </c>
       <c r="L83" s="10">
         <f>IF(COUNT(J83:K83)=2,(J83*Parametros!$B$3+K83*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -4795,13 +4949,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A84,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E84" s="8" t="n"/>
-      <c r="F84" s="8" t="n"/>
-      <c r="G84" s="8" t="n"/>
-      <c r="H84" s="8" t="n"/>
-      <c r="I84" s="8" t="n"/>
-      <c r="J84" s="8" t="n"/>
-      <c r="K84" s="8" t="n"/>
+      <c r="E84" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F84" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G84" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus</t>
+        </is>
+      </c>
+      <c r="H84" s="8" t="inlineStr">
+        <is>
+          <t>Lei_licitacoes_contratos_administrativos_4ed.pdf:p141; LGPD-2023-ANPD.pdf:p48; curso-159994-aula-24-bf9f-completo.pdf:p63; GTA_executivo_federal_7ed.pdf:p31; gta_executivo_federal_7ed.pdf:p31</t>
+        </is>
+      </c>
+      <c r="I84" s="8" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="J84" s="8" t="n">
+        <v>1938</v>
+      </c>
+      <c r="K84" s="8" t="n">
+        <v>242</v>
+      </c>
       <c r="L84" s="10">
         <f>IF(COUNT(J84:K84)=2,(J84*Parametros!$B$3+K84*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -4834,13 +5010,56 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A85,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E85" s="8" t="n"/>
-      <c r="F85" s="8" t="n"/>
-      <c r="G85" s="8" t="n"/>
-      <c r="H85" s="8" t="n"/>
-      <c r="I85" s="8" t="n"/>
-      <c r="J85" s="8" t="n"/>
-      <c r="K85" s="8" t="n"/>
+      <c r="E85" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F85" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G85" s="8" t="inlineStr">
+        <is>
+          <t>**Resposta**
+Para que a polícia possa obter dados de um proprietário por ofício, é necessário observar as disposições legais que regulam o acesso a dados pessoais e a atuação policial.  
+**1. Princípio da Necessidade e da Finalidade**  
+- **LGPD**: o tratamento de dados pessoais só pode ocorrer quando houver uma base legal (art. 5º).  
+- **Polícia**: a coleta de dados deve estar vinculada a uma finalidade legítima, como investigação de infração de trânsito ou de crime.
+**2. Necessidade de Ordem Judicial ou Autorização Legal**  
+- **CPC**: a citação e a obtenção de documentos de terceiros normalmente requerem **ordem judicial** (art. 225).  
+- **CTB**: não há previsão específica que autorize a polícia a solicitar dados de proprietários sem ordem judicial; a lei exige que a informação seja obtida por meio de procedimento legalmente previsto.  
+**3. Procedimento a Seguir**  
+- **Rejeitar** o ofício se não houver ordem judicial ou base legal clara.  
+- **Solicitar** à autoridade policial que apresente a **ordem judicial** ou outro documento que comprove a base legal (por exemplo, autorização de investigação criminal).  
+- **Verificar** se existe alguma norma específica que autorize a polícia a acessar dados sem ordem judicial (ex.: Lei de Execução Penal, Lei de Segurança Pública). Se existir, seguir o procedimento previsto.  
+**4. Caso a Ordem Judicial Não Esteja Disponível**  
+- **Encaminhar** o pedido ao juiz competente para que seja emitida a ordem de acesso aos dados.  
+- **Manter** o sigilo e a confidencialidade dos dados, conforme exigido pela LGPD.  
+**Resumo em Lista**  
+- **LGPD**: exigir base legal (consentimento, obrigação legal, etc.).  
+- **CPC**: requer ordem judicial para obtenção de dados de terceiros.  
+- **CTB**: não autoriza acesso sem ordem judicial.  
+- **Procedimento**: rejeitar ofício sem ordem, solicitar ordem judicial ou verificar norma específica que autorize.  
+---  
+Se houver alguma dúvida adicional sobre a base legal específica ou sobre a necessidade de autorização judicial, consulte o órgão jurídico competente.</t>
+        </is>
+      </c>
+      <c r="H85" s="8" t="inlineStr">
+        <is>
+          <t>curso-159994-aula-04-b323-completo.pdf:p36; curso-159994-aula-04-b323-completo.pdf:p45; LGPD-2023-ANPD.pdf:p13; manual_praticas_cartorarias_1_grau.pdf:p32; curso-159994-aula-04-b323-completo.pdf:p35</t>
+        </is>
+      </c>
+      <c r="I85" s="8" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="J85" s="8" t="n">
+        <v>1882</v>
+      </c>
+      <c r="K85" s="8" t="n">
+        <v>905</v>
+      </c>
       <c r="L85" s="10">
         <f>IF(COUNT(J85:K85)=2,(J85*Parametros!$B$3+K85*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -4873,13 +5092,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A86,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E86" s="8" t="n"/>
-      <c r="F86" s="8" t="n"/>
-      <c r="G86" s="8" t="n"/>
-      <c r="H86" s="8" t="n"/>
-      <c r="I86" s="8" t="n"/>
-      <c r="J86" s="8" t="n"/>
-      <c r="K86" s="8" t="n"/>
+      <c r="E86" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F86" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G86" s="8" t="inlineStr">
+        <is>
+          <t>**Não encontrado no corpus**</t>
+        </is>
+      </c>
+      <c r="H86" s="8" t="inlineStr">
+        <is>
+          <t>GTA_executivo_federal_7ed.pdf:p49; gta_executivo_federal_7ed.pdf:p49; curso-159994-aula-21-f255-completo.pdf:p10; LGPD-2023-ANPD.pdf:p25; Lei_licitacoes_contratos_administrativos_4ed.pdf:p78</t>
+        </is>
+      </c>
+      <c r="I86" s="8" t="n">
+        <v>18.06</v>
+      </c>
+      <c r="J86" s="8" t="n">
+        <v>1682</v>
+      </c>
+      <c r="K86" s="8" t="n">
+        <v>97</v>
+      </c>
       <c r="L86" s="10">
         <f>IF(COUNT(J86:K86)=2,(J86*Parametros!$B$3+K86*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -4912,13 +5153,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A87,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E87" s="8" t="n"/>
-      <c r="F87" s="8" t="n"/>
-      <c r="G87" s="8" t="n"/>
-      <c r="H87" s="8" t="n"/>
-      <c r="I87" s="8" t="n"/>
-      <c r="J87" s="8" t="n"/>
-      <c r="K87" s="8" t="n"/>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F87" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G87" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus</t>
+        </is>
+      </c>
+      <c r="H87" s="8" t="inlineStr">
+        <is>
+          <t>GTA_executivo_federal_7ed.pdf:p62; gta_executivo_federal_7ed.pdf:p62; GTA_executivo_federal_7ed.pdf:p52; gta_executivo_federal_7ed.pdf:p52; GTA_executivo_federal_7ed.pdf:p38</t>
+        </is>
+      </c>
+      <c r="I87" s="8" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="J87" s="8" t="n">
+        <v>1789</v>
+      </c>
+      <c r="K87" s="8" t="n">
+        <v>147</v>
+      </c>
       <c r="L87" s="10">
         <f>IF(COUNT(J87:K87)=2,(J87*Parametros!$B$3+K87*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -4951,13 +5214,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A88,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E88" s="8" t="n"/>
-      <c r="F88" s="8" t="n"/>
-      <c r="G88" s="8" t="n"/>
-      <c r="H88" s="8" t="n"/>
-      <c r="I88" s="8" t="n"/>
-      <c r="J88" s="8" t="n"/>
-      <c r="K88" s="8" t="n"/>
+      <c r="E88" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F88" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G88" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus</t>
+        </is>
+      </c>
+      <c r="H88" s="8" t="inlineStr">
+        <is>
+          <t>GTA_executivo_federal_7ed.pdf:p17; gta_executivo_federal_7ed.pdf:p17; Lei_licitacoes_contratos_administrativos_4ed.pdf:p23; curso-159994-aula-06-43dd-completo.pdf:p56; inss_beneficios.pdf:p1</t>
+        </is>
+      </c>
+      <c r="I88" s="8" t="n">
+        <v>7.22</v>
+      </c>
+      <c r="J88" s="8" t="n">
+        <v>1560</v>
+      </c>
+      <c r="K88" s="8" t="n">
+        <v>201</v>
+      </c>
       <c r="L88" s="10">
         <f>IF(COUNT(J88:K88)=2,(J88*Parametros!$B$3+K88*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -4990,13 +5275,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A89,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E89" s="8" t="n"/>
-      <c r="F89" s="8" t="n"/>
-      <c r="G89" s="8" t="n"/>
-      <c r="H89" s="8" t="n"/>
-      <c r="I89" s="8" t="n"/>
-      <c r="J89" s="8" t="n"/>
-      <c r="K89" s="8" t="n"/>
+      <c r="E89" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F89" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G89" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H89" s="8" t="inlineStr">
+        <is>
+          <t>Lei_licitacoes_contratos_administrativos_4ed.pdf:p119; manual_praticas_cartorarias_1_grau.pdf:p21; Lei_licitacoes_contratos_administrativos_4ed.pdf:p73; curso-159994-aula-02-daa4-completo.pdf:p65; Lei_licitacoes_contratos_administrativos_4ed.pdf:p24</t>
+        </is>
+      </c>
+      <c r="I89" s="8" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="J89" s="8" t="n">
+        <v>1628</v>
+      </c>
+      <c r="K89" s="8" t="n">
+        <v>254</v>
+      </c>
       <c r="L89" s="10">
         <f>IF(COUNT(J89:K89)=2,(J89*Parametros!$B$3+K89*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -5029,13 +5336,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A90,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E90" s="8" t="n"/>
-      <c r="F90" s="8" t="n"/>
-      <c r="G90" s="8" t="n"/>
-      <c r="H90" s="8" t="n"/>
-      <c r="I90" s="8" t="n"/>
-      <c r="J90" s="8" t="n"/>
-      <c r="K90" s="8" t="n"/>
+      <c r="E90" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F90" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G90" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus</t>
+        </is>
+      </c>
+      <c r="H90" s="8" t="inlineStr">
+        <is>
+          <t>GTA_executivo_federal_7ed.pdf:p61; gta_executivo_federal_7ed.pdf:p61; curso-159994-aula-06-43dd-completo.pdf:p15; curso-159994-aula-14-478b-completo.pdf:p7; curso-159994-aula-02-daa4-completo.pdf:p13</t>
+        </is>
+      </c>
+      <c r="I90" s="8" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="J90" s="8" t="n">
+        <v>1915</v>
+      </c>
+      <c r="K90" s="8" t="n">
+        <v>312</v>
+      </c>
       <c r="L90" s="10">
         <f>IF(COUNT(J90:K90)=2,(J90*Parametros!$B$3+K90*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -5068,13 +5397,44 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A91,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E91" s="8" t="n"/>
-      <c r="F91" s="8" t="n"/>
-      <c r="G91" s="8" t="n"/>
-      <c r="H91" s="8" t="n"/>
-      <c r="I91" s="8" t="n"/>
-      <c r="J91" s="8" t="n"/>
-      <c r="K91" s="8" t="n"/>
+      <c r="E91" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F91" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G91" s="8" t="inlineStr">
+        <is>
+          <t>**Não.**  
+A cópia do documento contém **dados de saúde**, que são dados pessoais sensíveis. De acordo com a Lei Geral de Proteção de Dados Pessoais (LGPD):
+- **Art. 21.** “Os dados pessoais referentes ao exercício regular de direitos pelo titular não podem ser utilizados em seu prejuízo.”  
+- **Art. 22.** “A defesa dos interesses e dos direitos dos titulares de dados poderá ser exercida em juízo, individual ou coletivamente, na forma do disposto na legislação pertinente.”  
+- **Art. 23.** O tratamento de dados pessoais por entes públicos deve observar a finalidade pública e o interesse legítimo, não podendo ser realizado sem a devida base legal.  
+Além disso, a **seção que trata do consentimento** estabelece que o tratamento de dados sensíveis só pode ocorrer mediante **manifestação livre, informada e inequívoca** do titular (**XII – consentimento**).
+Portanto, a entrega da cópia só é admissível se:
+- houver **consentimento expresso** do titular dos dados de saúde; ou  
+- houver **ordem judicial** ou outra hipótese legal que autorize o tratamento sem consentimento.
+Na ausência dessas condições, o documento não deve ser fornecido.</t>
+        </is>
+      </c>
+      <c r="H91" s="8" t="inlineStr">
+        <is>
+          <t>manual_praticas_cartorarias_1_grau.pdf:p37; cartilha_inss_digital_oabsp.pdf:p13; LGPD-2023-ANPD.pdf:p24; LGPD-2023-ANPD.pdf:p11; LGPD-2023-ANPD.pdf:p19</t>
+        </is>
+      </c>
+      <c r="I91" s="8" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="J91" s="8" t="n">
+        <v>1939</v>
+      </c>
+      <c r="K91" s="8" t="n">
+        <v>580</v>
+      </c>
       <c r="L91" s="10">
         <f>IF(COUNT(J91:K91)=2,(J91*Parametros!$B$3+K91*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -5107,13 +5467,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A92,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E92" s="8" t="n"/>
-      <c r="F92" s="8" t="n"/>
-      <c r="G92" s="8" t="n"/>
-      <c r="H92" s="8" t="n"/>
-      <c r="I92" s="8" t="n"/>
-      <c r="J92" s="8" t="n"/>
-      <c r="K92" s="8" t="n"/>
+      <c r="E92" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F92" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G92" s="8" t="inlineStr">
+        <is>
+          <t>**Não encontrado no corpus**</t>
+        </is>
+      </c>
+      <c r="H92" s="8" t="inlineStr">
+        <is>
+          <t>cartilha_inss_digital_oabsp.pdf:p18; cartilha_inss_digital_oabsp.pdf:p33; GTA_executivo_federal_7ed.pdf:p35; gta_executivo_federal_7ed.pdf:p35; cartilha_inss_digital_oabsp.pdf:p20</t>
+        </is>
+      </c>
+      <c r="I92" s="8" t="n">
+        <v>5.34</v>
+      </c>
+      <c r="J92" s="8" t="n">
+        <v>1789</v>
+      </c>
+      <c r="K92" s="8" t="n">
+        <v>104</v>
+      </c>
       <c r="L92" s="10">
         <f>IF(COUNT(J92:K92)=2,(J92*Parametros!$B$3+K92*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -5146,13 +5528,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A93,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E93" s="8" t="n"/>
-      <c r="F93" s="8" t="n"/>
-      <c r="G93" s="8" t="n"/>
-      <c r="H93" s="8" t="n"/>
-      <c r="I93" s="8" t="n"/>
-      <c r="J93" s="8" t="n"/>
-      <c r="K93" s="8" t="n"/>
+      <c r="E93" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F93" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G93" s="8" t="inlineStr">
+        <is>
+          <t>**Não encontrado no corpus**</t>
+        </is>
+      </c>
+      <c r="H93" s="8" t="inlineStr">
+        <is>
+          <t>LGPD-2023-ANPD.pdf:p16; LGPD-2023-ANPD.pdf:p21; LGPD-2023-ANPD.pdf:p32; LGPD-2023-ANPD.pdf:p7; LGPD-2023-ANPD.pdf:p14</t>
+        </is>
+      </c>
+      <c r="I93" s="8" t="n">
+        <v>11.06</v>
+      </c>
+      <c r="J93" s="8" t="n">
+        <v>1716</v>
+      </c>
+      <c r="K93" s="8" t="n">
+        <v>120</v>
+      </c>
       <c r="L93" s="10">
         <f>IF(COUNT(J93:K93)=2,(J93*Parametros!$B$3+K93*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -5185,13 +5589,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A94,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E94" s="8" t="n"/>
-      <c r="F94" s="8" t="n"/>
-      <c r="G94" s="8" t="n"/>
-      <c r="H94" s="8" t="n"/>
-      <c r="I94" s="8" t="n"/>
-      <c r="J94" s="8" t="n"/>
-      <c r="K94" s="8" t="n"/>
+      <c r="E94" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F94" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G94" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H94" s="8" t="inlineStr">
+        <is>
+          <t>LGPD-2023-ANPD.pdf:p32; LGPD-2023-ANPD.pdf:p14; LGPD-2023-ANPD.pdf:p10; LGPD-2023-ANPD.pdf:p23</t>
+        </is>
+      </c>
+      <c r="I94" s="8" t="n">
+        <v>16.44</v>
+      </c>
+      <c r="J94" s="8" t="n">
+        <v>1726</v>
+      </c>
+      <c r="K94" s="8" t="n">
+        <v>395</v>
+      </c>
       <c r="L94" s="10">
         <f>IF(COUNT(J94:K94)=2,(J94*Parametros!$B$3+K94*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -5224,13 +5650,38 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A95,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E95" s="8" t="n"/>
-      <c r="F95" s="8" t="n"/>
-      <c r="G95" s="8" t="n"/>
-      <c r="H95" s="8" t="n"/>
-      <c r="I95" s="8" t="n"/>
-      <c r="J95" s="8" t="n"/>
-      <c r="K95" s="8" t="n"/>
+      <c r="E95" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F95" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G95" s="8" t="inlineStr">
+        <is>
+          <t>**Resposta**
+- **Direito de acesso à informação** – Todos têm direito a receber, no prazo legal, informações de seu interesse particular ou coletivo, contidas em documentos de arquivos.  
+- **Obrigação de informar** – Se a solicitação do titular não envolve dados que estejam sujeitos a sigilo imprescindível à segurança da sociedade ou do Estado, o órgão deve disponibilizar o relatório solicitado.  
+- **Exceções** – Caso a informação sobre quem consultou a matrícula seja considerada confidencial ou protegida por sigilo, o órgão pode negar o acesso, justificando a restrição conforme a legislação aplicável.</t>
+        </is>
+      </c>
+      <c r="H95" s="8" t="inlineStr">
+        <is>
+          <t>manual_praticas_cartorarias_1_grau.pdf:p74; GTA_executivo_federal_7ed.pdf:p55; gta_executivo_federal_7ed.pdf:p55; curso-159994-aula-11-d0d4-completo.pdf:p24; gta_executivo_federal_7ed.pdf:p20</t>
+        </is>
+      </c>
+      <c r="I95" s="8" t="n">
+        <v>10.57</v>
+      </c>
+      <c r="J95" s="8" t="n">
+        <v>1588</v>
+      </c>
+      <c r="K95" s="8" t="n">
+        <v>885</v>
+      </c>
       <c r="L95" s="10">
         <f>IF(COUNT(J95:K95)=2,(J95*Parametros!$B$3+K95*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -5263,13 +5714,53 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A96,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E96" s="8" t="n"/>
-      <c r="F96" s="8" t="n"/>
-      <c r="G96" s="8" t="n"/>
-      <c r="H96" s="8" t="n"/>
-      <c r="I96" s="8" t="n"/>
-      <c r="J96" s="8" t="n"/>
-      <c r="K96" s="8" t="n"/>
+      <c r="E96" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F96" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G96" s="8" t="inlineStr">
+        <is>
+          <t>**Art. 18.** O titular dos dados pessoais tem direito a obter do controlador, em relação aos dados do titular por ele tratados, a qualquer momento e mediante requisição:
+- **III** — correção de dados incompletos, inexatos ou desatualizados.
+---
+### Procedimento a ser adotado
+1. **Recebimento da requisição**  
+   - O titular manifesta, por escrito ou por meio eletrônico, a necessidade de correção do dado errado na matrícula.
+2. **Identificação do controlador**  
+   - Verificar qual pessoa jurídica ou natural está realizando o tratamento da matrícula e, portanto, é responsável por atender ao pedido.
+3. **Análise da solicitação**  
+   - Confirmar que o dado apontado como incorreto está realmente incompleto, inexato ou desatualizado, conforme previsto no inciso **III** do art. 18.
+4. **Execução da correção (retificação)**  
+   - Proceder à retificação do registro da matrícula, garantindo que a informação correta passe a constar nos sistemas do controlador.
+5. **Comunicação ao titular**  
+   - Informar ao titular que a correção foi efetuada, indicando a data e a natureza da alteração realizada.
+6. **Documentação**  
+   - Arquivar a requisição e a comprovação da correção para fins de auditoria e demonstração de conformidade com a LGPD.
+---
+**Conclusão:**  
+O pedido do titular trata‑se de um **pedido de correção de dados** previsto no **inciso III do art. 18 da LGPD**, devendo ser atendido mediante o procedimento de **retificação** do registro da matrícula.</t>
+        </is>
+      </c>
+      <c r="H96" s="8" t="inlineStr">
+        <is>
+          <t>LGPD-2023-ANPD.pdf:p32; LGPD-2023-ANPD.pdf:p21; LGPD-2023-ANPD.pdf:p11; LGPD-2023-ANPD.pdf:p8; LGPD-2023-ANPD.pdf:p16</t>
+        </is>
+      </c>
+      <c r="I96" s="8" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="J96" s="8" t="n">
+        <v>1942</v>
+      </c>
+      <c r="K96" s="8" t="n">
+        <v>528</v>
+      </c>
       <c r="L96" s="10">
         <f>IF(COUNT(J96:K96)=2,(J96*Parametros!$B$3+K96*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -5302,13 +5793,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A97,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E97" s="8" t="n"/>
-      <c r="F97" s="8" t="n"/>
-      <c r="G97" s="8" t="n"/>
-      <c r="H97" s="8" t="n"/>
-      <c r="I97" s="8" t="n"/>
-      <c r="J97" s="8" t="n"/>
-      <c r="K97" s="8" t="n"/>
+      <c r="E97" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F97" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G97" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus</t>
+        </is>
+      </c>
+      <c r="H97" s="8" t="inlineStr">
+        <is>
+          <t>GTA_executivo_federal_7ed.pdf:p23; gta_executivo_federal_7ed.pdf:p23; LGPD-2023-ANPD.pdf:p11; GTA_executivo_federal_7ed.pdf:p63; gta_executivo_federal_7ed.pdf:p63</t>
+        </is>
+      </c>
+      <c r="I97" s="8" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="J97" s="8" t="n">
+        <v>2052</v>
+      </c>
+      <c r="K97" s="8" t="n">
+        <v>191</v>
+      </c>
       <c r="L97" s="10">
         <f>IF(COUNT(J97:K97)=2,(J97*Parametros!$B$3+K97*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -5341,13 +5854,50 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A98,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E98" s="8" t="n"/>
-      <c r="F98" s="8" t="n"/>
-      <c r="G98" s="8" t="n"/>
-      <c r="H98" s="8" t="n"/>
-      <c r="I98" s="8" t="n"/>
-      <c r="J98" s="8" t="n"/>
-      <c r="K98" s="8" t="n"/>
+      <c r="E98" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F98" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G98" s="8" t="inlineStr">
+        <is>
+          <t>**Art. 8.** O consentimento do titular deve ser fornecido por escrito ou por outro meio que demonstre a manifestação de vontade, sendo vedado o tratamento mediante vício de consentimento.  
+§ 2º Cabe ao controlador o ônus da prova de que o consentimento foi obtido em conformidade com o disposto nesta Lei.  
+**Art. 11.** O tratamento de dados pessoais sensíveis somente poderá ocorrer nas seguintes hipóteses:
+- **I** – quando o titular ou seu responsável legal consentir, de forma específica e destacada, para finalidades específicas;  
+- **II** – sem fornecimento de consentimento do titular, nas hipóteses em que for indispensável para:  
+  - **a** – cumprimento de obrigação legal ou regulatória pelo controlador;  
+  - **b** – tratamento compartilhado de dados necessários à execução, pela administração pública, de políticas públicas previstas em leis ou regulamentos;  
+  - **c** – realização de estudos por órgão de pesquisa, garantida, sempre que possível, a anonimização dos dados pessoais sensíveis.  
+---  
+### Aplicação ao compartilhamento com ONR/SREI e centrais eletrônicas
+- Se o compartilhamento for **necessário para o cumprimento de obrigação legal ou regulatória** (por exemplo, exigido por normas que regulam a atuação do órgão ou por decisões judiciais), ele se enquadra na alínea **II‑a** do **Art. 11** e **não exige consentimento** do titular.  
+- Quando o compartilhamento for **destinado à execução de políticas públicas** ou à prestação de serviços públicos por parte da administração, ele se ampara na alínea **II‑b** do **Art. 11**, também dispensando consentimento.  
+- Caso nenhuma dessas hipóteses se aplique e o tratamento não seja indispensável para a finalidade descrita, será necessário obter **consentimento** conforme o **caput** e o **inciso I** do **Art. 8**.  
+---  
+**Conclusão:**  
+Para o compartilhamento de dados com ONR/SREI e centrais eletrônicas, **não é obrigatória a obtenção de consentimento** quando o tratamento se justifica pelo cumprimento de obrigação legal ou regulatória ou pela execução de políticas públicas, nos termos do **Art. 11, incisos II‑a e II‑b**. Em situações fora dessas hipóteses, será necessária a coleta de consentimento válido conforme o **Art. 8**.</t>
+        </is>
+      </c>
+      <c r="H98" s="8" t="inlineStr">
+        <is>
+          <t>LGPD-2023-ANPD.pdf:p15; LGPD-2023-ANPD.pdf:p17; GTA_executivo_federal_7ed.pdf:p16; gta_executivo_federal_7ed.pdf:p16; LGPD-2023-ANPD.pdf:p22</t>
+        </is>
+      </c>
+      <c r="I98" s="8" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="J98" s="8" t="n">
+        <v>1849</v>
+      </c>
+      <c r="K98" s="8" t="n">
+        <v>770</v>
+      </c>
       <c r="L98" s="10">
         <f>IF(COUNT(J98:K98)=2,(J98*Parametros!$B$3+K98*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -5380,13 +5930,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A99,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E99" s="8" t="n"/>
-      <c r="F99" s="8" t="n"/>
-      <c r="G99" s="8" t="n"/>
-      <c r="H99" s="8" t="n"/>
-      <c r="I99" s="8" t="n"/>
-      <c r="J99" s="8" t="n"/>
-      <c r="K99" s="8" t="n"/>
+      <c r="E99" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F99" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G99" s="8" t="inlineStr">
+        <is>
+          <t>**Não encontrado no corpus**</t>
+        </is>
+      </c>
+      <c r="H99" s="8" t="inlineStr">
+        <is>
+          <t>manual_praticas_cartorarias_1_grau.pdf:p59; curso-159994-aula-05-561e-completo.pdf:p5; LGPD-2023-ANPD.pdf:p35; curso-159994-aula-05-561e-completo.pdf:p15; curso-159994-aula-04-b323-completo.pdf:p28</t>
+        </is>
+      </c>
+      <c r="I99" s="8" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="J99" s="8" t="n">
+        <v>1826</v>
+      </c>
+      <c r="K99" s="8" t="n">
+        <v>105</v>
+      </c>
       <c r="L99" s="10">
         <f>IF(COUNT(J99:K99)=2,(J99*Parametros!$B$3+K99*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -5419,13 +5991,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A100,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E100" s="8" t="n"/>
-      <c r="F100" s="8" t="n"/>
-      <c r="G100" s="8" t="n"/>
-      <c r="H100" s="8" t="n"/>
-      <c r="I100" s="8" t="n"/>
-      <c r="J100" s="8" t="n"/>
-      <c r="K100" s="8" t="n"/>
+      <c r="E100" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F100" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G100" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H100" s="8" t="inlineStr">
+        <is>
+          <t>curso-159994-aula-10-aeca-completo.pdf:p21; cartilha_inss_digital_oabsp.pdf:p21; curso-159994-aula-10-bonus-4f69-completo.pdf:p20; cartilha_inss_digital_oabsp.pdf:p23; cartilha_inss_digital_oabsp.pdf:p29</t>
+        </is>
+      </c>
+      <c r="I100" s="8" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="J100" s="8" t="n">
+        <v>1554</v>
+      </c>
+      <c r="K100" s="8" t="n">
+        <v>110</v>
+      </c>
       <c r="L100" s="10">
         <f>IF(COUNT(J100:K100)=2,(J100*Parametros!$B$3+K100*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>
@@ -5458,13 +6052,35 @@
         <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A101,Perguntas!$A$2:$A$26,0))</f>
         <v/>
       </c>
-      <c r="E101" s="8" t="n"/>
-      <c r="F101" s="8" t="n"/>
-      <c r="G101" s="8" t="n"/>
-      <c r="H101" s="8" t="n"/>
-      <c r="I101" s="8" t="n"/>
-      <c r="J101" s="8" t="n"/>
-      <c r="K101" s="8" t="n"/>
+      <c r="E101" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F101" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (cdde83a)</t>
+        </is>
+      </c>
+      <c r="G101" s="8" t="inlineStr">
+        <is>
+          <t>**Não encontrado no corpus**</t>
+        </is>
+      </c>
+      <c r="H101" s="8" t="inlineStr">
+        <is>
+          <t>cartilha_inss_digital_oabsp.pdf:p18; GTA_executivo_federal_7ed.pdf:p41; gta_executivo_federal_7ed.pdf:p41; GTA_executivo_federal_7ed.pdf:p38; gta_executivo_federal_7ed.pdf:p38</t>
+        </is>
+      </c>
+      <c r="I101" s="8" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="J101" s="8" t="n">
+        <v>1908</v>
+      </c>
+      <c r="K101" s="8" t="n">
+        <v>113</v>
+      </c>
       <c r="L101" s="10">
         <f>IF(COUNT(J101:K101)=2,(J101*Parametros!$B$3+K101*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
         <v/>

</xml_diff>

<commit_message>
feat: benchmark compara RAG atual com RAG Fase 3
- run_rag_benchmark.py: --collection, --ferramenta e --from-json
- planilha com a ferramenta "RAG Fase 3"; Gate 1 e custo por
  assinatura consideram só os concorrentes (is_rag)
- premissa de preço atualizada para gpt-oss na Groq
- resultado fase3: 14/25 "Não encontrado" (baseline: 20/25); o gargalo
  é o embedding em inglês (Art. 17 da Lei 6.015 fora do top 300 na #1)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fase3/benchmark/planilha_benchmark.xlsx
+++ b/docs/fase3/benchmark/planilha_benchmark.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Resumo" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Respostas'!$A$1:$S$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Respostas'!$A$1:$S$126</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -615,7 +615,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>4. As linhas 'RAG atual' são preenchidas pelo script run_rag_benchmark.py (--xlsx).</t>
+          <t>4. As linhas 'RAG atual' e 'RAG Fase 3' são preenchidas pelo script run_rag_benchmark.py (--xlsx).</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S101"/>
+  <dimension ref="A1:S126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6096,9 +6096,1638 @@
       </c>
       <c r="S101" s="8" t="n"/>
     </row>
+    <row r="102">
+      <c r="A102" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B102" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C102" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A102,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D102" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A102,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E102" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F102" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G102" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H102" s="8" t="inlineStr">
+        <is>
+          <t>Provimento CNJ 149/2023, Art. 417:p266; Código de Normas CGJ-CE, Art. 1490:p305; Código de Normas CGJ-CE, Art. 1517:p312; Código de Normas CGJ-CE, Art. 1472:p301; Código de Normas CGJ-CE, Art. 1285:p263</t>
+        </is>
+      </c>
+      <c r="I102" s="8" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="J102" s="8" t="n">
+        <v>1920</v>
+      </c>
+      <c r="K102" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="L102" s="10">
+        <f>IF(COUNT(J102:K102)=2,(J102*Parametros!$B$3+K102*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M102" s="8" t="n"/>
+      <c r="N102" s="8" t="n"/>
+      <c r="O102" s="8" t="n"/>
+      <c r="P102" s="8" t="n"/>
+      <c r="Q102" s="8" t="n"/>
+      <c r="R102" s="9">
+        <f>IF(COUNT(M102:Q102)=5,SUM(M102:Q102),"")</f>
+        <v/>
+      </c>
+      <c r="S102" s="8" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B103" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C103" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A103,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D103" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A103,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E103" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F103" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G103" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H103" s="8" t="inlineStr">
+        <is>
+          <t>Provimento CNJ 149/2023, Art. 477:p318; Provimento CNJ 149/2023, Art. 221:p124; Provimento CNJ 149/2023, Art. 390:p239; Provimento CNJ 149/2023, Art. 205-A:p95; Provimento CNJ 149/2023, Art. 495-E:p326</t>
+        </is>
+      </c>
+      <c r="I103" s="8" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="J103" s="8" t="n">
+        <v>2195</v>
+      </c>
+      <c r="K103" s="8" t="n">
+        <v>113</v>
+      </c>
+      <c r="L103" s="10">
+        <f>IF(COUNT(J103:K103)=2,(J103*Parametros!$B$3+K103*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M103" s="8" t="n"/>
+      <c r="N103" s="8" t="n"/>
+      <c r="O103" s="8" t="n"/>
+      <c r="P103" s="8" t="n"/>
+      <c r="Q103" s="8" t="n"/>
+      <c r="R103" s="9">
+        <f>IF(COUNT(M103:Q103)=5,SUM(M103:Q103),"")</f>
+        <v/>
+      </c>
+      <c r="S103" s="8" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B104" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C104" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A104,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D104" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A104,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E104" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F104" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G104" s="8" t="inlineStr">
+        <is>
+          <t>**Resposta**
+Sim. A certidão de matrícula pode ser emitida integralmente contendo o histórico completo de todos os ônus, inclusive penhoras já canceladas.
+- **Art. 440‑G** (Seção I) estabelece que, para fins de adjudicação compulsória, a ata notarial – que serve de modelo para a certidão registral – deve conter:
+  - **I** – a referência à matrícula ou à transcrição, **e a descrição do imóvel com seus ônus e gravames**.
+- **Art. 210‑C** (Subseção I) dispõe que o extrato eletrônico (certidão) deve obedecer aos campos e cláusulas obrigatórias definidos em norma técnica, assegurando a integridade das informações registradas.
+Dessa forma, a emissão integral da certidão, com o histórico completo de ônus e gravames, está em conformidade com os requisitos legais acima citados.</t>
+        </is>
+      </c>
+      <c r="H104" s="8" t="inlineStr">
+        <is>
+          <t>Provimento CNJ 149/2023, Art. 409:p262; Provimento CNJ 149/2023, Art. 210-C:p107; Provimento CNJ 149/2023, Art. 440-G:p276; Provimento CNJ 149/2023, Art. 493:p324; Lei 8.935/1994, Art. 32:p0</t>
+        </is>
+      </c>
+      <c r="I104" s="8" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="J104" s="8" t="n">
+        <v>2093</v>
+      </c>
+      <c r="K104" s="8" t="n">
+        <v>647</v>
+      </c>
+      <c r="L104" s="10">
+        <f>IF(COUNT(J104:K104)=2,(J104*Parametros!$B$3+K104*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M104" s="8" t="n"/>
+      <c r="N104" s="8" t="n"/>
+      <c r="O104" s="8" t="n"/>
+      <c r="P104" s="8" t="n"/>
+      <c r="Q104" s="8" t="n"/>
+      <c r="R104" s="9">
+        <f>IF(COUNT(M104:Q104)=5,SUM(M104:Q104),"")</f>
+        <v/>
+      </c>
+      <c r="S104" s="8" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B105" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C105" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A105,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D105" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A105,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E105" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F105" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G105" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus</t>
+        </is>
+      </c>
+      <c r="H105" s="8" t="inlineStr">
+        <is>
+          <t>Guia ANPD — Segurança da Informação, p. 1:p1; Guia ANPD — Segurança da Informação, p. 18:p18; Guia ANPD — Segurança da Informação, p. 10:p10; Guia ANPD — Segurança da Informação, p. 12:p12</t>
+        </is>
+      </c>
+      <c r="I105" s="8" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J105" s="8" t="n">
+        <v>1567</v>
+      </c>
+      <c r="K105" s="8" t="n">
+        <v>131</v>
+      </c>
+      <c r="L105" s="10">
+        <f>IF(COUNT(J105:K105)=2,(J105*Parametros!$B$3+K105*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M105" s="8" t="n"/>
+      <c r="N105" s="8" t="n"/>
+      <c r="O105" s="8" t="n"/>
+      <c r="P105" s="8" t="n"/>
+      <c r="Q105" s="8" t="n"/>
+      <c r="R105" s="9">
+        <f>IF(COUNT(M105:Q105)=5,SUM(M105:Q105),"")</f>
+        <v/>
+      </c>
+      <c r="S105" s="8" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B106" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C106" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A106,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D106" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A106,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E106" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F106" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G106" s="8" t="inlineStr">
+        <is>
+          <t>**Procedimento para busca de bens por CPF solicitada por um credor**
+**Art. 397-AI**  
+- **I** — a indicação da localização do bem é responsabilidade do **credor fiduciário** ou de seus mandatários;  
+- **II** — uma vez localizado, o bem será agendado por meio do **módulo próprio na Central RTDPJ Brasil**, integrante do Sistema Eletrônico dos Registros Públicos – Serp, ou por contato direto com o **oficial de registro de títulos e documentos**;  
+- **III** — o oficial de registro deve garantir a disponibilidade de dia e horário para o agendamento da diligência de apreensão, durante o expediente normal da serventia, no mesmo dia da solicitação nas capitais e regiões metropolitanas, e, nas demais regiões, em até 1 (um) dia útil.
+**Art. 397-K**  
+- **I** — a atribuição para realizar o processo de consolidação da propriedade extrajudicial e da busca e apreensão de bem móvel será do **oficial de registro de títulos e documentos** do domicílio do devedor fiduciante, ou da localização do bem;  
+- **II** — se o bem móvel estiver localizado em local diverso do domicílio do devedor, o oficial de registro do local onde o bem for encontrado será competente para a diligência;  
+- **III** — os emolumentos relativos ao ato de busca e apreensão serão devidos ao oficial de registro do local onde a diligência for efetivamente realizada.
+**Art. 397-J**  
+- **I** — o **credor fiduciário**, seu procurador ou representante legal possui legitimidade para requerer a consolidação da propriedade extrajudicial e a busca e apreensão de bem móvel;  
+- **Parágrafo único** — os credores devem se habilitar no módulo próprio da Central RTDPJ Brasil, indicando, através de cadastramento em seu perfil criptografado, os prepostos autorizados a iniciar e acompanhar o processo, sendo desnecessário o envio de procurações ou autorizações expressas.
+---
+### Passos a serem seguidos
+1. **Registro no módulo**  
+   - O credor fiduciário deve se habilitar no módulo próprio da Central RTDPJ Brasil e cadastrar os prepostos autorizados.
+2. **Solicitação de localização**  
+   - O credor solicita a localização do bem, informando o **CPF** do devedor, por meio do módulo ou contato direto com o oficial de registro.
+3. **Responsabilidade do oficial de registro**  
+   - O oficial de registro responsável pela localização do bem registra a solicitação no módulo e agenda a diligência de apreensão.
+4. **Agendamento da diligência**  
+   - O oficial garante a disponibilidade de dia e horário, conforme §2º do Art. 397-AI:  
+     - Na mesma cidade (capitais e regiões metropolitanas) no dia da solicitação;  
+     - Em até 1 (um) dia útil nas demais regiões.
+5. **Execução da diligência**  
+   - Se o bem estiver localizado em outro local, o oficial de registro do local onde o bem for encontrado executará a diligência, conforme Art. 397-K §1º.
+6. **Pagamento de emolumentos**  
+   - Os emolumentos relativos à busca e apreensão são devidos ao oficial de registro do local onde a diligência for realizada, conforme Art. 397-K §2º.
+Assim, o credor segue o procedimento estabelecido pelos Provimentos CNJ 149/2023, garantindo a localização e eventual apreensão do bem do devedor.</t>
+        </is>
+      </c>
+      <c r="H106" s="8" t="inlineStr">
+        <is>
+          <t>Provimento 15/2026/CGJCE, Art. 2:p2; Provimento CNJ 149/2023, Art. 397-AI:p254; Provimento CNJ 149/2023, Art. 397-K:p245; Provimento CNJ 149/2023, Art. 397-J:p245; Provimento CNJ 149/2023, Art. 440-X:p282</t>
+        </is>
+      </c>
+      <c r="I106" s="8" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="J106" s="8" t="n">
+        <v>2144</v>
+      </c>
+      <c r="K106" s="8" t="n">
+        <v>1419</v>
+      </c>
+      <c r="L106" s="10">
+        <f>IF(COUNT(J106:K106)=2,(J106*Parametros!$B$3+K106*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M106" s="8" t="n"/>
+      <c r="N106" s="8" t="n"/>
+      <c r="O106" s="8" t="n"/>
+      <c r="P106" s="8" t="n"/>
+      <c r="Q106" s="8" t="n"/>
+      <c r="R106" s="9">
+        <f>IF(COUNT(M106:Q106)=5,SUM(M106:Q106),"")</f>
+        <v/>
+      </c>
+      <c r="S106" s="8" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C107" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A107,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D107" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A107,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E107" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F107" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G107" s="8" t="inlineStr">
+        <is>
+          <t>**Decreto 7.724/2012, Art. 17.**  
+Caso a informação esteja disponível ao público em formato impresso, eletrônico ou em outro meio de acesso universal, o órgão ou entidade deverá orientar o requerente quanto ao local e modo para consultar, obter ou reproduzir a informação.  
+Parágrafo único. Na hipótese do caput, o órgão ou entidade desobriga‑se do fornecimento direto da informação, salvo se o requerente declarar não dispor de meios para consultar, obter ou reproduzir a informação.  
+---
+**Resposta**  
+- Se o nome do proprietário do imóvel for informação **pública** (disponível em registros oficiais, cartórios, etc.), o órgão deve **orientar** o requerente sobre onde e como consultar ou obter essa informação.  
+- Se a informação **não for pública** ou não estiver disponível em meio de acesso universal, o órgão **não pode** fornecer o dado diretamente por telefone, exceto se o requerente declarar que não tem meios para consultar ou reproduzir a informação.</t>
+        </is>
+      </c>
+      <c r="H107" s="8" t="inlineStr">
+        <is>
+          <t>Provimento CNJ 149/2023, Art. 58:p23; Decreto 7.724/2012, Art. 17:p0; Provimento CNJ 149/2023, Art. 59:p23; Provimento CNJ 149/2023, Art. 62:p24; Código de Normas CGJ-CE, Art. 1753:p358</t>
+        </is>
+      </c>
+      <c r="I107" s="8" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="J107" s="8" t="n">
+        <v>1871</v>
+      </c>
+      <c r="K107" s="8" t="n">
+        <v>733</v>
+      </c>
+      <c r="L107" s="10">
+        <f>IF(COUNT(J107:K107)=2,(J107*Parametros!$B$3+K107*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M107" s="8" t="n"/>
+      <c r="N107" s="8" t="n"/>
+      <c r="O107" s="8" t="n"/>
+      <c r="P107" s="8" t="n"/>
+      <c r="Q107" s="8" t="n"/>
+      <c r="R107" s="9">
+        <f>IF(COUNT(M107:Q107)=5,SUM(M107:Q107),"")</f>
+        <v/>
+      </c>
+      <c r="S107" s="8" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B108" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C108" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A108,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D108" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A108,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E108" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F108" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G108" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H108" s="8" t="inlineStr">
+        <is>
+          <t>Provimento CNJ 149/2023, Art. 3 (ato de aprovação):p3; Lei 6.015/1973, Art. 70:p0; Provimento CNJ 149/2023, Art. 368:p231; Provimento CNJ 149/2023, Art. 353-A:p227; Decreto 7.724/2012, Art. 30:p0</t>
+        </is>
+      </c>
+      <c r="I108" s="8" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J108" s="8" t="n">
+        <v>1613</v>
+      </c>
+      <c r="K108" s="8" t="n">
+        <v>119</v>
+      </c>
+      <c r="L108" s="10">
+        <f>IF(COUNT(J108:K108)=2,(J108*Parametros!$B$3+K108*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M108" s="8" t="n"/>
+      <c r="N108" s="8" t="n"/>
+      <c r="O108" s="8" t="n"/>
+      <c r="P108" s="8" t="n"/>
+      <c r="Q108" s="8" t="n"/>
+      <c r="R108" s="9">
+        <f>IF(COUNT(M108:Q108)=5,SUM(M108:Q108),"")</f>
+        <v/>
+      </c>
+      <c r="S108" s="8" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B109" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C109" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A109,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D109" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A109,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E109" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F109" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G109" s="8" t="inlineStr">
+        <is>
+          <t>**Não encontrado no corpus**</t>
+        </is>
+      </c>
+      <c r="H109" s="8" t="inlineStr">
+        <is>
+          <t>Provimento CNJ 149/2023, Art. 397-R:p248; Provimento CNJ 149/2023, Art. 320-AC:p205; Decreto 7.724/2012, Art. 12:p0; Provimento CNJ 149/2023, Art. 397-N:p246; Provimento CNJ 149/2023, Art. 320-R:p202</t>
+        </is>
+      </c>
+      <c r="I109" s="8" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J109" s="8" t="n">
+        <v>1886</v>
+      </c>
+      <c r="K109" s="8" t="n">
+        <v>185</v>
+      </c>
+      <c r="L109" s="10">
+        <f>IF(COUNT(J109:K109)=2,(J109*Parametros!$B$3+K109*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M109" s="8" t="n"/>
+      <c r="N109" s="8" t="n"/>
+      <c r="O109" s="8" t="n"/>
+      <c r="P109" s="8" t="n"/>
+      <c r="Q109" s="8" t="n"/>
+      <c r="R109" s="9">
+        <f>IF(COUNT(M109:Q109)=5,SUM(M109:Q109),"")</f>
+        <v/>
+      </c>
+      <c r="S109" s="8" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B110" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C110" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A110,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D110" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A110,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E110" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F110" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G110" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H110" s="8" t="inlineStr">
+        <is>
+          <t>Provimento CNJ 149/2023, Art. 511-E:p335; Provimento CNJ 149/2023, Art. 320-AE:p205; Código de Normas CGJ-CE, Art. 709:p156; Provimento CNJ 149/2023, Art. 556:p360; Provimento CNJ 149/2023, Art. 320-C:p198</t>
+        </is>
+      </c>
+      <c r="I110" s="8" t="n">
+        <v>15.36</v>
+      </c>
+      <c r="J110" s="8" t="n">
+        <v>2127</v>
+      </c>
+      <c r="K110" s="8" t="n">
+        <v>199</v>
+      </c>
+      <c r="L110" s="10">
+        <f>IF(COUNT(J110:K110)=2,(J110*Parametros!$B$3+K110*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M110" s="8" t="n"/>
+      <c r="N110" s="8" t="n"/>
+      <c r="O110" s="8" t="n"/>
+      <c r="P110" s="8" t="n"/>
+      <c r="Q110" s="8" t="n"/>
+      <c r="R110" s="9">
+        <f>IF(COUNT(M110:Q110)=5,SUM(M110:Q110),"")</f>
+        <v/>
+      </c>
+      <c r="S110" s="8" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B111" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C111" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A111,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D111" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A111,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E111" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F111" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G111" s="8" t="inlineStr">
+        <is>
+          <t>**Não encontrado no corpus**</t>
+        </is>
+      </c>
+      <c r="H111" s="8" t="inlineStr">
+        <is>
+          <t>LAI (Lei 12.527/2011), Art. 19:p0; Provimento CNJ 149/2023, Art. 187:p90; LAI (Lei 12.527/2011), Art. 1:p0; Código de Normas CGJ-CE, Art. 58:p38; Provimento CNJ 149/2023, Art. 148:p71</t>
+        </is>
+      </c>
+      <c r="I111" s="8" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J111" s="8" t="n">
+        <v>1777</v>
+      </c>
+      <c r="K111" s="8" t="n">
+        <v>112</v>
+      </c>
+      <c r="L111" s="10">
+        <f>IF(COUNT(J111:K111)=2,(J111*Parametros!$B$3+K111*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M111" s="8" t="n"/>
+      <c r="N111" s="8" t="n"/>
+      <c r="O111" s="8" t="n"/>
+      <c r="P111" s="8" t="n"/>
+      <c r="Q111" s="8" t="n"/>
+      <c r="R111" s="9">
+        <f>IF(COUNT(M111:Q111)=5,SUM(M111:Q111),"")</f>
+        <v/>
+      </c>
+      <c r="S111" s="8" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B112" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C112" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A112,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D112" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A112,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E112" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F112" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G112" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus</t>
+        </is>
+      </c>
+      <c r="H112" s="8" t="inlineStr">
+        <is>
+          <t>Provimento CNJ 149/2023, Art. 103:p52; Decreto 7.724/2012, Art. 10:p0; LAI (Lei 12.527/2011), Art. 2:p0; Provimento CNJ 149/2023, Art. 511-C:p334; Código de Normas CGJ-CE, Art. 198:p68</t>
+        </is>
+      </c>
+      <c r="I112" s="8" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="J112" s="8" t="n">
+        <v>1883</v>
+      </c>
+      <c r="K112" s="8" t="n">
+        <v>310</v>
+      </c>
+      <c r="L112" s="10">
+        <f>IF(COUNT(J112:K112)=2,(J112*Parametros!$B$3+K112*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M112" s="8" t="n"/>
+      <c r="N112" s="8" t="n"/>
+      <c r="O112" s="8" t="n"/>
+      <c r="P112" s="8" t="n"/>
+      <c r="Q112" s="8" t="n"/>
+      <c r="R112" s="9">
+        <f>IF(COUNT(M112:Q112)=5,SUM(M112:Q112),"")</f>
+        <v/>
+      </c>
+      <c r="S112" s="8" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B113" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C113" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A113,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D113" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A113,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E113" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F113" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G113" s="8" t="inlineStr">
+        <is>
+          <t>**Sim, é dever responder.**  
+O **Protocolo de Acesso à Informação** obriga os órgãos e entidades públicas a atender solicitações de informação, salvo exceções previstas em lei.  
+**Art. 34.**  
+- **I** — Os órgãos e entidades públicas respondem diretamente pelos danos causados em decorrência da divulgação não autorizada ou utilização indevida de informações sigilosas ou informações pessoais, cabendo a apuração de responsabilidade funcional nos casos de dolo ou culpa, assegurado o respectivo direito de regresso.  
+- **II** — O disposto neste artigo aplica‑se à pessoa física ou entidade privada que, em virtude de vínculo de qualquer natureza com órgãos ou entidades, tenha acesso a informação sigilosa ou pessoal e a submeta a tratamento indevido.  
+Como a solicitação refere‑se a **emolumentos arrecadados pela serventia**, trata‑se de informação pública de interesse coletivo. Portanto, a serventia tem a obrigação de responder ao pedido, fornecendo os dados solicitados ou justificando a impossibilidade de divulgação, conforme previsto na LAI.</t>
+        </is>
+      </c>
+      <c r="H113" s="8" t="inlineStr">
+        <is>
+          <t>Lei 8.935/1994, Art. 46:p0; LAI (Lei 12.527/2011), Art. 24:p0; LAI (Lei 12.527/2011), Art. 34:p0; Provimento CNJ 149/2023, Art. 103:p52; LGPD (Lei 13.709/2018), Art. 42:p0</t>
+        </is>
+      </c>
+      <c r="I113" s="8" t="n">
+        <v>13.41</v>
+      </c>
+      <c r="J113" s="8" t="n">
+        <v>1661</v>
+      </c>
+      <c r="K113" s="8" t="n">
+        <v>506</v>
+      </c>
+      <c r="L113" s="10">
+        <f>IF(COUNT(J113:K113)=2,(J113*Parametros!$B$3+K113*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M113" s="8" t="n"/>
+      <c r="N113" s="8" t="n"/>
+      <c r="O113" s="8" t="n"/>
+      <c r="P113" s="8" t="n"/>
+      <c r="Q113" s="8" t="n"/>
+      <c r="R113" s="9">
+        <f>IF(COUNT(M113:Q113)=5,SUM(M113:Q113),"")</f>
+        <v/>
+      </c>
+      <c r="S113" s="8" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B114" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C114" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A114,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D114" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A114,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E114" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F114" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G114" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H114" s="8" t="inlineStr">
+        <is>
+          <t>Código de Normas CGJ-CE, Art. 1517:p312; Código de Normas CGJ-CE, Art. 364:p99; Código de Normas CGJ-CE, Art. 1476:p302; Lei 6.015/1973, Art. 29:p0; Provimento CNJ 149/2023, Art. 256-G:p152</t>
+        </is>
+      </c>
+      <c r="I114" s="8" t="n">
+        <v>9.41</v>
+      </c>
+      <c r="J114" s="8" t="n">
+        <v>1816</v>
+      </c>
+      <c r="K114" s="8" t="n">
+        <v>201</v>
+      </c>
+      <c r="L114" s="10">
+        <f>IF(COUNT(J114:K114)=2,(J114*Parametros!$B$3+K114*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M114" s="8" t="n"/>
+      <c r="N114" s="8" t="n"/>
+      <c r="O114" s="8" t="n"/>
+      <c r="P114" s="8" t="n"/>
+      <c r="Q114" s="8" t="n"/>
+      <c r="R114" s="9">
+        <f>IF(COUNT(M114:Q114)=5,SUM(M114:Q114),"")</f>
+        <v/>
+      </c>
+      <c r="S114" s="8" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C115" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A115,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D115" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A115,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E115" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F115" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G115" s="8" t="inlineStr"/>
+      <c r="H115" s="8" t="inlineStr">
+        <is>
+          <t>Código de Normas CGJ-CE, Art. 1517:p312; Lei 6.015/1973, Art. 102:p0; Guia ANPD — Agentes de Tratamento, p. 7:p7; Lei 6.015/1973, Art. 70:p0; Lei 6.015/1973, Art. 88:p0</t>
+        </is>
+      </c>
+      <c r="I115" s="8" t="n">
+        <v>16.71</v>
+      </c>
+      <c r="J115" s="8" t="n">
+        <v>1963</v>
+      </c>
+      <c r="K115" s="8" t="n">
+        <v>2048</v>
+      </c>
+      <c r="L115" s="10">
+        <f>IF(COUNT(J115:K115)=2,(J115*Parametros!$B$3+K115*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M115" s="8" t="n"/>
+      <c r="N115" s="8" t="n"/>
+      <c r="O115" s="8" t="n"/>
+      <c r="P115" s="8" t="n"/>
+      <c r="Q115" s="8" t="n"/>
+      <c r="R115" s="9">
+        <f>IF(COUNT(M115:Q115)=5,SUM(M115:Q115),"")</f>
+        <v/>
+      </c>
+      <c r="S115" s="8" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B116" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C116" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A116,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D116" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A116,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E116" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F116" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G116" s="8" t="inlineStr">
+        <is>
+          <t>**Art. 132.** O fornecimento de cópias ou certidões de documentos arquivados na serventia se limita ao documento protestado propriamente dito, nos termos do art. 22 da Lei n.º 9.492/1997, enquanto perdurar o protesto, e dentro do prazo máximo de 10 anos, nos termos do art. 30 da Lei n.º 9.492/1997, não devendo ser fornecidas cópias dos demais documentos, salvo:
+- **para as partes**;  
+- **com autorização judicial**.
+**Parágrafo único.** Tratando‑se de documento de identificação pessoal, a cópia arquivada somente deve ser fornecida ao próprio titular.
+---
+### Aplicação ao caso
+- O pedido refere‑se a **cópia de documento arquivado (título) que contém dados de saúde**, informação sensível protegida pela legislação de proteção de dados.  
+- Não se trata de documento protestado nem está dentro do prazo de 10 anos que autoriza a cópia automática.  
+- Portanto, a cópia **não pode ser fornecida** a terceiros.  
+**Exceções:**  
+- Se o solicitante for **parte interessada** (ou seja, a própria pessoa cujos dados de saúde constam no documento), a cópia pode ser fornecida.  
+- Se houver **autorização judicial** específica, a cópia também pode ser fornecida.  
+**Conclusão:**  
+Forneça a cópia **apenas** se o requerente for a parte titular dos dados ou se houver decisão judicial autorizando a entrega. Caso contrário, a cópia deve ser negada.</t>
+        </is>
+      </c>
+      <c r="H116" s="8" t="inlineStr">
+        <is>
+          <t>Provimento CNJ 149/2023, Art. 112:p54; Provimento CNJ 149/2023, Art. 249:p146; Provimento CNJ 149/2023, Art. 132:p58; Provimento CNJ 149/2023, Art. 96:p50; Lei 6.015/1973, Art. 150:p0</t>
+        </is>
+      </c>
+      <c r="I116" s="8" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="J116" s="8" t="n">
+        <v>1801</v>
+      </c>
+      <c r="K116" s="8" t="n">
+        <v>695</v>
+      </c>
+      <c r="L116" s="10">
+        <f>IF(COUNT(J116:K116)=2,(J116*Parametros!$B$3+K116*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M116" s="8" t="n"/>
+      <c r="N116" s="8" t="n"/>
+      <c r="O116" s="8" t="n"/>
+      <c r="P116" s="8" t="n"/>
+      <c r="Q116" s="8" t="n"/>
+      <c r="R116" s="9">
+        <f>IF(COUNT(M116:Q116)=5,SUM(M116:Q116),"")</f>
+        <v/>
+      </c>
+      <c r="S116" s="8" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="B117" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C117" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A117,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D117" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A117,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E117" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F117" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G117" s="8" t="inlineStr"/>
+      <c r="H117" s="8" t="inlineStr">
+        <is>
+          <t>Provimento CNJ 149/2023, Art. 406:p261; Código de Normas CGJ-CE, Art. 14:p25; Código de Normas CGJ-CE, Art. 17:p26; Código de Normas CGJ-CE, Art. 1753:p358; LGPD (Lei 13.709/2018), Art. 47:p0</t>
+        </is>
+      </c>
+      <c r="I117" s="8" t="n">
+        <v>21.51</v>
+      </c>
+      <c r="J117" s="8" t="n">
+        <v>1832</v>
+      </c>
+      <c r="K117" s="8" t="n">
+        <v>2048</v>
+      </c>
+      <c r="L117" s="10">
+        <f>IF(COUNT(J117:K117)=2,(J117*Parametros!$B$3+K117*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M117" s="8" t="n"/>
+      <c r="N117" s="8" t="n"/>
+      <c r="O117" s="8" t="n"/>
+      <c r="P117" s="8" t="n"/>
+      <c r="Q117" s="8" t="n"/>
+      <c r="R117" s="9">
+        <f>IF(COUNT(M117:Q117)=5,SUM(M117:Q117),"")</f>
+        <v/>
+      </c>
+      <c r="S117" s="8" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="B118" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C118" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A118,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D118" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A118,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E118" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F118" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G118" s="8" t="inlineStr">
+        <is>
+          <t>**Não encontrado no corpus**</t>
+        </is>
+      </c>
+      <c r="H118" s="8" t="inlineStr">
+        <is>
+          <t>Guia ANPD — Agentes de Tratamento, p. 8:p8; Guia ANPD — Segurança da Informação, p. 13:p13; Provimento CNJ 149/2023, Art. 79:p42; Provimento CNJ 149/2023, Art. 84:p43; Guia ANPD — Segurança da Informação, p. 14:p14</t>
+        </is>
+      </c>
+      <c r="I118" s="8" t="n">
+        <v>32.06</v>
+      </c>
+      <c r="J118" s="8" t="n">
+        <v>2261</v>
+      </c>
+      <c r="K118" s="8" t="n">
+        <v>170</v>
+      </c>
+      <c r="L118" s="10">
+        <f>IF(COUNT(J118:K118)=2,(J118*Parametros!$B$3+K118*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M118" s="8" t="n"/>
+      <c r="N118" s="8" t="n"/>
+      <c r="O118" s="8" t="n"/>
+      <c r="P118" s="8" t="n"/>
+      <c r="Q118" s="8" t="n"/>
+      <c r="R118" s="9">
+        <f>IF(COUNT(M118:Q118)=5,SUM(M118:Q118),"")</f>
+        <v/>
+      </c>
+      <c r="S118" s="8" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B119" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C119" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A119,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D119" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A119,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E119" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F119" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G119" s="8" t="inlineStr">
+        <is>
+          <t>**Resposta ao titular – solicitação de exclusão de dados da matrícula**
+---
+**Prezado(a) [Nome do Titular],**
+Recebemos sua solicitação de exclusão dos dados pessoais referentes à sua matrícula. Em conformidade com a **Lei Geral de Proteção de Dados – LGPD (Lei nº 13.709/2018)**, informamos que:
+**Art. 18 – Direitos do titular**  
+- **VI** — eliminação dos dados pessoais tratados com o consentimento do titular, exceto nas hipóteses previstas no art. 16 desta Lei;  
+- **IV** — anonimização, bloqueio ou eliminação de dados desnecessários, excessivos ou tratados em desconformidade com o disposto nesta Lei.
+**Art. 19 – Prazo de atendimento**  
+- **I** — em formato simplificado, imediatamente;  
+- **II** — por meio de declaração clara e completa, no prazo de até **15 (quinze) dias** a contar da data do requerimento.
+---
+## Procedimento a ser adotado
+- **Verificação**  
+  - Confirmaremos se os dados solicitados estão em nosso sistema e se sua exclusão não viola obrigações legais ou contratuais (art. 16 da LGPD).  
+- **Ação**  
+  - Se não houver impedimento legal, procederemos à **exclusão** dos dados da matrícula.  
+  - Caso a exclusão seja inviável por motivo legal, informaremos ao titular a razão e os prazos previstos.  
+- **Comunicação**  
+  - Enviaremos ao titular uma **confirmação de exclusão** (ou de impossibilidade de exclusão) dentro do prazo de 15 dias.  
+- **Registro**  
+  - Documentaremos todo o processo, incluindo a justificativa de eventual impossibilidade de exclusão, conforme exigido pela LGPD.
+---
+**Observação**  
+Se houver necessidade de manter os dados por obrigação legal ou regulatória, informaremos ao titular a justificativa e os prazos de retenção, conforme previsto no art. 16 da LGPD.
+---
+Agradecemos pela sua atenção e permanecemos à disposição para quaisquer esclarecimentos adicionais.</t>
+        </is>
+      </c>
+      <c r="H119" s="8" t="inlineStr">
+        <is>
+          <t>LGPD (Lei 13.709/2018), Art. 44:p0; LGPD (Lei 13.709/2018), Art. 43:p0; LGPD (Lei 13.709/2018), Art. 49:p0; LGPD (Lei 13.709/2018), Art. 19:p0; LGPD (Lei 13.709/2018), Art. 18:p0</t>
+        </is>
+      </c>
+      <c r="I119" s="8" t="n">
+        <v>15.05</v>
+      </c>
+      <c r="J119" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="K119" s="8" t="n">
+        <v>1265</v>
+      </c>
+      <c r="L119" s="10">
+        <f>IF(COUNT(J119:K119)=2,(J119*Parametros!$B$3+K119*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M119" s="8" t="n"/>
+      <c r="N119" s="8" t="n"/>
+      <c r="O119" s="8" t="n"/>
+      <c r="P119" s="8" t="n"/>
+      <c r="Q119" s="8" t="n"/>
+      <c r="R119" s="9">
+        <f>IF(COUNT(M119:Q119)=5,SUM(M119:Q119),"")</f>
+        <v/>
+      </c>
+      <c r="S119" s="8" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="B120" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C120" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A120,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D120" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A120,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E120" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F120" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G120" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H120" s="8" t="inlineStr">
+        <is>
+          <t>Decreto 7.724/2012, Art. 17:p0; Lei 8.935/1994, Art. 46:p0; Decreto 7.724/2012, Art. 61:p0; Provimento CNJ 149/2023, Art. 440-BB:p297; LAI (Lei 12.527/2011), Art. 30:p0</t>
+        </is>
+      </c>
+      <c r="I120" s="8" t="n">
+        <v>21.57</v>
+      </c>
+      <c r="J120" s="8" t="n">
+        <v>2015</v>
+      </c>
+      <c r="K120" s="8" t="n">
+        <v>207</v>
+      </c>
+      <c r="L120" s="10">
+        <f>IF(COUNT(J120:K120)=2,(J120*Parametros!$B$3+K120*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M120" s="8" t="n"/>
+      <c r="N120" s="8" t="n"/>
+      <c r="O120" s="8" t="n"/>
+      <c r="P120" s="8" t="n"/>
+      <c r="Q120" s="8" t="n"/>
+      <c r="R120" s="9">
+        <f>IF(COUNT(M120:Q120)=5,SUM(M120:Q120),"")</f>
+        <v/>
+      </c>
+      <c r="S120" s="8" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B121" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C121" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A121,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D121" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A121,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E121" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F121" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G121" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H121" s="8" t="inlineStr">
+        <is>
+          <t>LGPD (Lei 13.709/2018), Art. 43:p0; LGPD (Lei 13.709/2018), Art. 44:p0; Provimento CNJ 149/2023, Art. 79:p42; Guia ANPD — Agentes de Tratamento, p. 8:p8; Provimento CNJ 149/2023, Art. 84:p43</t>
+        </is>
+      </c>
+      <c r="I121" s="8" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="J121" s="8" t="n">
+        <v>1966</v>
+      </c>
+      <c r="K121" s="8" t="n">
+        <v>294</v>
+      </c>
+      <c r="L121" s="10">
+        <f>IF(COUNT(J121:K121)=2,(J121*Parametros!$B$3+K121*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M121" s="8" t="n"/>
+      <c r="N121" s="8" t="n"/>
+      <c r="O121" s="8" t="n"/>
+      <c r="P121" s="8" t="n"/>
+      <c r="Q121" s="8" t="n"/>
+      <c r="R121" s="9">
+        <f>IF(COUNT(M121:Q121)=5,SUM(M121:Q121),"")</f>
+        <v/>
+      </c>
+      <c r="S121" s="8" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="B122" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C122" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A122,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D122" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A122,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E122" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F122" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G122" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H122" s="8" t="inlineStr">
+        <is>
+          <t>Resolução CD/ANPD 15/2024, Art. 4:p0; Guia ANPD — Agentes de Tratamento, p. 16:p16; Guia ANPD — Agentes de Tratamento, p. 15:p15; Provimento CNJ 149/2023, Art. 148:p71; Guia ANPD — Agentes de Tratamento, p. 18:p18</t>
+        </is>
+      </c>
+      <c r="I122" s="8" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="J122" s="8" t="n">
+        <v>2140</v>
+      </c>
+      <c r="K122" s="8" t="n">
+        <v>294</v>
+      </c>
+      <c r="L122" s="10">
+        <f>IF(COUNT(J122:K122)=2,(J122*Parametros!$B$3+K122*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M122" s="8" t="n"/>
+      <c r="N122" s="8" t="n"/>
+      <c r="O122" s="8" t="n"/>
+      <c r="P122" s="8" t="n"/>
+      <c r="Q122" s="8" t="n"/>
+      <c r="R122" s="9">
+        <f>IF(COUNT(M122:Q122)=5,SUM(M122:Q122),"")</f>
+        <v/>
+      </c>
+      <c r="S122" s="8" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B123" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C123" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A123,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D123" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A123,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E123" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F123" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G123" s="8" t="inlineStr">
+        <is>
+          <t>**Art. 124** – Ressalvadas as hipóteses que tenham previsão legal ou normativa expressa, como as certidões de filiação de imóveis, ou de propriedade com negativa de ônus e alienações, ou outras compatíveis com as finalidades dos registros de imóveis e com os princípios da **Lei Geral de Proteção de Dados (LGPD)**, **não serão expedidas certidões cujo conteúdo envolva informações sobre dados pessoais extraídos de mais de uma matrícula, assentamento do registro auxiliar, transcrição ou inscrição.**  
+**Art. 290**, § 2.º – Os notários, pessoalmente ou por intermédio do e‑Notariado, **devem fornecer meios tecnológicos para o acesso das informações exclusivamente estatísticas e genéricas à Administração Pública Direta**, sendo **vedado o envio e o repasse de dados**, salvo disposição legal ou judicial específica.  
+---  
+### Necessidade de base legal adicional ou de consentimento
+- **Base legal obrigatória**  
+  - O compartilhamento de dados pessoais com a **ONR/SREI** ou com **centrais eletrônicas** só pode ocorrer quando houver **disposição legal ou normativa expressa** que autorize tal tratamento, conforme o disposto no **Art. 124**.  
+  - Na ausência de autorização legal específica, o tratamento deve se amparar em **uma das bases previstas na LGPD** (ex.: cumprimento de obrigação legal ou regulatória, execução de contrato, interesse público, proteção da vida ou da incolumidade física, etc.).  
+- **Consentimento isolado não é suficiente**  
+  - O simples consentimento do titular **não supre a exigência** de que o tratamento esteja respaldado por uma base legal prevista na LGPD.  
+  - O consentimento pode ser utilizado **apenas como uma das bases** quando nenhuma das demais se aplicar, devendo ser **livre, informado e inequívoco**.  
+- **Proibição de repasse indiscriminado**  
+  - Conforme o **Art. 290, § 2.º**, o notário **não pode enviar ou repassar dados pessoais** a terceiros, inclusive a ONR/SREI ou centrais eletrônicas, **exceto se houver disposição legal ou decisão judicial que autorize** tal comunicação.  
+---  
+### Conclusão
+- **É imprescindível** identificar **uma base legal específica** (ex.: obrigação legal, interesse público, execução de contrato, decisão judicial) que legitime o compartilhamento dos dados com a ONR/SREI e as centrais eletrônicas.  
+- **O consentimento, por si só, não elimina** a necessidade de observar as bases legais previstas na LGPD e as restrições do **Art. 290, § 2.º**.  
+Portanto, **sim, é necessária uma base legal adicional** (ou autorização judicial) para o compartilhamento; o consentimento isolado não basta.</t>
+        </is>
+      </c>
+      <c r="H123" s="8" t="inlineStr">
+        <is>
+          <t>Lei 6.015/1973, Art. 167:p0; Provimento CNJ 149/2023, Art. 510:p332; Provimento CNJ 149/2023, Art. 290:p185; Código de Normas CGJ-CE, Art. 536:p129; Provimento CNJ 149/2023, Art. 124:p57</t>
+        </is>
+      </c>
+      <c r="I123" s="8" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="J123" s="8" t="n">
+        <v>1985</v>
+      </c>
+      <c r="K123" s="8" t="n">
+        <v>1081</v>
+      </c>
+      <c r="L123" s="10">
+        <f>IF(COUNT(J123:K123)=2,(J123*Parametros!$B$3+K123*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M123" s="8" t="n"/>
+      <c r="N123" s="8" t="n"/>
+      <c r="O123" s="8" t="n"/>
+      <c r="P123" s="8" t="n"/>
+      <c r="Q123" s="8" t="n"/>
+      <c r="R123" s="9">
+        <f>IF(COUNT(M123:Q123)=5,SUM(M123:Q123),"")</f>
+        <v/>
+      </c>
+      <c r="S123" s="8" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B124" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C124" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A124,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D124" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A124,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E124" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F124" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G124" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
+      <c r="H124" s="8" t="inlineStr">
+        <is>
+          <t>Provimento CNJ 149/2023, Art. 343-F:p221; Provimento CNJ 149/2023, Art. 528:p349; Provimento CNJ 149/2023, Art. 456:p312; Provimento CNJ 149/2023, Art. 218:p118; Provimento CNJ 149/2023, Art. 211:p114</t>
+        </is>
+      </c>
+      <c r="I124" s="8" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J124" s="8" t="n">
+        <v>1496</v>
+      </c>
+      <c r="K124" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="L124" s="10">
+        <f>IF(COUNT(J124:K124)=2,(J124*Parametros!$B$3+K124*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M124" s="8" t="n"/>
+      <c r="N124" s="8" t="n"/>
+      <c r="O124" s="8" t="n"/>
+      <c r="P124" s="8" t="n"/>
+      <c r="Q124" s="8" t="n"/>
+      <c r="R124" s="9">
+        <f>IF(COUNT(M124:Q124)=5,SUM(M124:Q124),"")</f>
+        <v/>
+      </c>
+      <c r="S124" s="8" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B125" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C125" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A125,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D125" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A125,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E125" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F125" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G125" s="8" t="inlineStr">
+        <is>
+          <t>**Requisitos para emitir certidão digital segundo o Código de Normas do CE**
+**Art. 1127.**  
+Os Oficiais obrigam‑se a:  
+- **I** — lavrar certidões requeridas em formulário próprio, timbrado, pertinente aos atos praticados, vedada a utilização de impressos não oficiais;  
+- **II** — fornecer às partes as informações e certidões nos prazos e hipóteses previstos em lei.  
+Parágrafo único:  
+Os documentos quando assinados com o uso de certificado digital, realizados e/ou enviados pela Internet, deverão atender aos requisitos da Infraestrutura de Chaves Públicas Brasileira – **ICP‑Brasil**.
+**Art. 522.**  
+Se a ata for apresentada em formato eletrônico, será necessário que a assinatura digital do representante legal da pessoa jurídica, no requerimento ou na própria ata, tenha sido feita com certificado digital **ICP‑Brasil** nos padrões exigidos em lei e atos normativos.
+**Art. 788.**  
+Os atos notariais, com exceção do Testamento Público, poderão ser lavrados e arquivados em meio digital seguro, podendo inclusive ser assinados pelos notários, prepostos ou partes interessadas de forma digital com a utilização de certificação digital no padrão da Infraestrutura de Chaves Públicas Brasileira – **ICP‑Brasil**.</t>
+        </is>
+      </c>
+      <c r="H125" s="8" t="inlineStr">
+        <is>
+          <t>Código de Normas CGJ-CE, Art. 1127:p229; Provimento CNJ 149/2023, Art. 266:p176; Código de Normas CGJ-CE, Art. 522:p127; Código de Normas CGJ-CE, Art. 1115:p227; Código de Normas CGJ-CE, Art. 788:p169</t>
+        </is>
+      </c>
+      <c r="I125" s="8" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="J125" s="8" t="n">
+        <v>1642</v>
+      </c>
+      <c r="K125" s="8" t="n">
+        <v>1079</v>
+      </c>
+      <c r="L125" s="10">
+        <f>IF(COUNT(J125:K125)=2,(J125*Parametros!$B$3+K125*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M125" s="8" t="n"/>
+      <c r="N125" s="8" t="n"/>
+      <c r="O125" s="8" t="n"/>
+      <c r="P125" s="8" t="n"/>
+      <c r="Q125" s="8" t="n"/>
+      <c r="R125" s="9">
+        <f>IF(COUNT(M125:Q125)=5,SUM(M125:Q125),"")</f>
+        <v/>
+      </c>
+      <c r="S125" s="8" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="B126" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="C126" s="9">
+        <f>INDEX(Perguntas!$B$2:$B$26,MATCH(A126,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="D126" s="9">
+        <f>INDEX(Perguntas!$C$2:$C$26,MATCH(A126,Perguntas!$A$2:$A$26,0))</f>
+        <v/>
+      </c>
+      <c r="E126" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F126" s="8" t="inlineStr">
+        <is>
+          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+        </is>
+      </c>
+      <c r="G126" s="8" t="inlineStr">
+        <is>
+          <t>**Guia ANPD — Segurança da Informação**  
+- **Sugerido**: os e‑mails devem ser cifrados ou, opcionalmente, os arquivos devem ser cifrados para envio.  
+**Resolução CD/ANPD 15/2024, Art. 4**  
+- **Confidencialidade**: propriedade que assegura que o dado pessoal não esteja disponível ou não seja revelado a pessoas, empresas, sistemas, órgãos ou entidades não autorizados.  
+Assim, a serventia deve garantir a confidencialidade do dado pessoal e adotar comunicações cifradas (ou arquivos cifrados) ao enviar certidões por e‑mail.</t>
+        </is>
+      </c>
+      <c r="H126" s="8" t="inlineStr">
+        <is>
+          <t>Código de Normas CGJ-CE, Art. 1753:p358; Resolução CD/ANPD 15/2024, Art. 4:p0; Guia ANPD — Segurança da Informação, p. 15:p15; Guia ANPD — Agentes de Tratamento, p. 7:p7; Provimento CNJ 149/2023, Art. 101:p51</t>
+        </is>
+      </c>
+      <c r="I126" s="8" t="n">
+        <v>20.41</v>
+      </c>
+      <c r="J126" s="8" t="n">
+        <v>2003</v>
+      </c>
+      <c r="K126" s="8" t="n">
+        <v>1293</v>
+      </c>
+      <c r="L126" s="10">
+        <f>IF(COUNT(J126:K126)=2,(J126*Parametros!$B$3+K126*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="M126" s="8" t="n"/>
+      <c r="N126" s="8" t="n"/>
+      <c r="O126" s="8" t="n"/>
+      <c r="P126" s="8" t="n"/>
+      <c r="Q126" s="8" t="n"/>
+      <c r="R126" s="9">
+        <f>IF(COUNT(M126:Q126)=5,SUM(M126:Q126),"")</f>
+        <v/>
+      </c>
+      <c r="S126" s="8" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S101"/>
-  <conditionalFormatting sqref="R2:R101">
+  <autoFilter ref="A1:S126"/>
+  <conditionalFormatting sqref="R2:R126">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>8</formula>
     </cfRule>
@@ -6107,7 +7736,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="M2:Q101" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Use 0, 1 ou 2" type="list">
+    <dataValidation sqref="M2:Q126" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Use 0, 1 ou 2" type="list">
       <formula1>"0,1,2"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6156,12 +7785,12 @@
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>gemini-2.5-flash-lite</t>
+          <t>Groq openai/gpt-oss-20b / 120b</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>CHEAP_MODEL do .env; o script registra o modelo real em 'Versão / plano'</t>
+          <t>CHEAP/PREMIUM_MODEL do .env; o script registra o modelo real em 'Versão / plano'</t>
         </is>
       </c>
     </row>
@@ -6172,11 +7801,11 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Premissa: tabela pública do Gemini 2.5 Flash-Lite. Conferir em ai.google.dev/pricing</t>
+          <t>Premissa: preço do gpt-oss-120b na Groq (teto; o 20b é mais barato). Conferir em groq.com/pricing</t>
         </is>
       </c>
     </row>
@@ -6187,11 +7816,11 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Premissa: tabela pública do Gemini 2.5 Flash-Lite. Conferir em ai.google.dev/pricing</t>
+          <t>Premissa: preço do gpt-oss-120b na Groq (teto; o 20b é mais barato). Conferir em groq.com/pricing</t>
         </is>
       </c>
     </row>
@@ -6281,7 +7910,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>O custo por consulta do 'RAG atual' vem dos tokens medidos (aba Respostas).</t>
+          <t>O custo por consulta dos RAGs vem dos tokens medidos (aba Respostas).</t>
         </is>
       </c>
     </row>
@@ -6296,7 +7925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6383,39 +8012,39 @@
         </is>
       </c>
       <c r="B4" s="9">
-        <f>COUNTIFS(Respostas!$B$2:$B$101,$A4,Respostas!$R$2:$R$101,"&gt;=0")</f>
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A4,Respostas!$R$2:$R$126,"&gt;=0")</f>
         <v/>
       </c>
       <c r="C4" s="11">
-        <f>IF(B4=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,$A4))</f>
+        <f>IF(B4=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,$A4))</f>
         <v/>
       </c>
       <c r="D4" s="11">
-        <f>IF(B4=0,"",AVERAGEIFS(Respostas!$M$2:$M$101,Respostas!$B$2:$B$101,$A4,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B4=0,"",AVERAGEIFS(Respostas!$M$2:$M$126,Respostas!$B$2:$B$126,$A4,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="E4" s="11">
-        <f>IF(B4=0,"",AVERAGEIFS(Respostas!$N$2:$N$101,Respostas!$B$2:$B$101,$A4,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B4=0,"",AVERAGEIFS(Respostas!$N$2:$N$126,Respostas!$B$2:$B$126,$A4,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="F4" s="11">
-        <f>IF(B4=0,"",AVERAGEIFS(Respostas!$O$2:$O$101,Respostas!$B$2:$B$101,$A4,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B4=0,"",AVERAGEIFS(Respostas!$O$2:$O$126,Respostas!$B$2:$B$126,$A4,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="G4" s="11">
-        <f>IF(B4=0,"",AVERAGEIFS(Respostas!$P$2:$P$101,Respostas!$B$2:$B$101,$A4,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B4=0,"",AVERAGEIFS(Respostas!$P$2:$P$126,Respostas!$B$2:$B$126,$A4,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="H4" s="11">
-        <f>IF(B4=0,"",AVERAGEIFS(Respostas!$Q$2:$Q$101,Respostas!$B$2:$B$101,$A4,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B4=0,"",AVERAGEIFS(Respostas!$Q$2:$Q$126,Respostas!$B$2:$B$126,$A4,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="I4" s="12">
-        <f>IF(B4=0,"",COUNTIFS(Respostas!$B$2:$B$101,$A4,Respostas!$R$2:$R$101,"&gt;=8")/B4)</f>
+        <f>IF(B4=0,"",COUNTIFS(Respostas!$B$2:$B$126,$A4,Respostas!$R$2:$R$126,"&gt;=8")/B4)</f>
         <v/>
       </c>
       <c r="J4" s="11">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,$A4,Respostas!$I$2:$I$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$I$2:$I$101,Respostas!$B$2:$B$101,$A4))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A4,Respostas!$I$2:$I$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$I$2:$I$126,Respostas!$B$2:$B$126,$A4))</f>
         <v/>
       </c>
       <c r="K4" s="10">
@@ -6430,39 +8059,39 @@
         </is>
       </c>
       <c r="B5" s="9">
-        <f>COUNTIFS(Respostas!$B$2:$B$101,$A5,Respostas!$R$2:$R$101,"&gt;=0")</f>
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A5,Respostas!$R$2:$R$126,"&gt;=0")</f>
         <v/>
       </c>
       <c r="C5" s="11">
-        <f>IF(B5=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,$A5))</f>
+        <f>IF(B5=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,$A5))</f>
         <v/>
       </c>
       <c r="D5" s="11">
-        <f>IF(B5=0,"",AVERAGEIFS(Respostas!$M$2:$M$101,Respostas!$B$2:$B$101,$A5,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B5=0,"",AVERAGEIFS(Respostas!$M$2:$M$126,Respostas!$B$2:$B$126,$A5,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="E5" s="11">
-        <f>IF(B5=0,"",AVERAGEIFS(Respostas!$N$2:$N$101,Respostas!$B$2:$B$101,$A5,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B5=0,"",AVERAGEIFS(Respostas!$N$2:$N$126,Respostas!$B$2:$B$126,$A5,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="F5" s="11">
-        <f>IF(B5=0,"",AVERAGEIFS(Respostas!$O$2:$O$101,Respostas!$B$2:$B$101,$A5,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B5=0,"",AVERAGEIFS(Respostas!$O$2:$O$126,Respostas!$B$2:$B$126,$A5,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="G5" s="11">
-        <f>IF(B5=0,"",AVERAGEIFS(Respostas!$P$2:$P$101,Respostas!$B$2:$B$101,$A5,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B5=0,"",AVERAGEIFS(Respostas!$P$2:$P$126,Respostas!$B$2:$B$126,$A5,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="H5" s="11">
-        <f>IF(B5=0,"",AVERAGEIFS(Respostas!$Q$2:$Q$101,Respostas!$B$2:$B$101,$A5,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B5=0,"",AVERAGEIFS(Respostas!$Q$2:$Q$126,Respostas!$B$2:$B$126,$A5,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="I5" s="12">
-        <f>IF(B5=0,"",COUNTIFS(Respostas!$B$2:$B$101,$A5,Respostas!$R$2:$R$101,"&gt;=8")/B5)</f>
+        <f>IF(B5=0,"",COUNTIFS(Respostas!$B$2:$B$126,$A5,Respostas!$R$2:$R$126,"&gt;=8")/B5)</f>
         <v/>
       </c>
       <c r="J5" s="11">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,$A5,Respostas!$I$2:$I$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$I$2:$I$101,Respostas!$B$2:$B$101,$A5))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A5,Respostas!$I$2:$I$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$I$2:$I$126,Respostas!$B$2:$B$126,$A5))</f>
         <v/>
       </c>
       <c r="K5" s="10">
@@ -6477,39 +8106,39 @@
         </is>
       </c>
       <c r="B6" s="9">
-        <f>COUNTIFS(Respostas!$B$2:$B$101,$A6,Respostas!$R$2:$R$101,"&gt;=0")</f>
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A6,Respostas!$R$2:$R$126,"&gt;=0")</f>
         <v/>
       </c>
       <c r="C6" s="11">
-        <f>IF(B6=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,$A6))</f>
+        <f>IF(B6=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,$A6))</f>
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>IF(B6=0,"",AVERAGEIFS(Respostas!$M$2:$M$101,Respostas!$B$2:$B$101,$A6,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B6=0,"",AVERAGEIFS(Respostas!$M$2:$M$126,Respostas!$B$2:$B$126,$A6,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="E6" s="11">
-        <f>IF(B6=0,"",AVERAGEIFS(Respostas!$N$2:$N$101,Respostas!$B$2:$B$101,$A6,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B6=0,"",AVERAGEIFS(Respostas!$N$2:$N$126,Respostas!$B$2:$B$126,$A6,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="F6" s="11">
-        <f>IF(B6=0,"",AVERAGEIFS(Respostas!$O$2:$O$101,Respostas!$B$2:$B$101,$A6,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B6=0,"",AVERAGEIFS(Respostas!$O$2:$O$126,Respostas!$B$2:$B$126,$A6,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="G6" s="11">
-        <f>IF(B6=0,"",AVERAGEIFS(Respostas!$P$2:$P$101,Respostas!$B$2:$B$101,$A6,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B6=0,"",AVERAGEIFS(Respostas!$P$2:$P$126,Respostas!$B$2:$B$126,$A6,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="H6" s="11">
-        <f>IF(B6=0,"",AVERAGEIFS(Respostas!$Q$2:$Q$101,Respostas!$B$2:$B$101,$A6,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B6=0,"",AVERAGEIFS(Respostas!$Q$2:$Q$126,Respostas!$B$2:$B$126,$A6,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="I6" s="12">
-        <f>IF(B6=0,"",COUNTIFS(Respostas!$B$2:$B$101,$A6,Respostas!$R$2:$R$101,"&gt;=8")/B6)</f>
+        <f>IF(B6=0,"",COUNTIFS(Respostas!$B$2:$B$126,$A6,Respostas!$R$2:$R$126,"&gt;=8")/B6)</f>
         <v/>
       </c>
       <c r="J6" s="11">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,$A6,Respostas!$I$2:$I$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$I$2:$I$101,Respostas!$B$2:$B$101,$A6))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A6,Respostas!$I$2:$I$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$I$2:$I$126,Respostas!$B$2:$B$126,$A6))</f>
         <v/>
       </c>
       <c r="K6" s="10">
@@ -6524,355 +8153,447 @@
         </is>
       </c>
       <c r="B7" s="9">
-        <f>COUNTIFS(Respostas!$B$2:$B$101,$A7,Respostas!$R$2:$R$101,"&gt;=0")</f>
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A7,Respostas!$R$2:$R$126,"&gt;=0")</f>
         <v/>
       </c>
       <c r="C7" s="11">
-        <f>IF(B7=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,$A7))</f>
+        <f>IF(B7=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,$A7))</f>
         <v/>
       </c>
       <c r="D7" s="11">
-        <f>IF(B7=0,"",AVERAGEIFS(Respostas!$M$2:$M$101,Respostas!$B$2:$B$101,$A7,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B7=0,"",AVERAGEIFS(Respostas!$M$2:$M$126,Respostas!$B$2:$B$126,$A7,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="E7" s="11">
-        <f>IF(B7=0,"",AVERAGEIFS(Respostas!$N$2:$N$101,Respostas!$B$2:$B$101,$A7,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B7=0,"",AVERAGEIFS(Respostas!$N$2:$N$126,Respostas!$B$2:$B$126,$A7,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="F7" s="11">
-        <f>IF(B7=0,"",AVERAGEIFS(Respostas!$O$2:$O$101,Respostas!$B$2:$B$101,$A7,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B7=0,"",AVERAGEIFS(Respostas!$O$2:$O$126,Respostas!$B$2:$B$126,$A7,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="G7" s="11">
-        <f>IF(B7=0,"",AVERAGEIFS(Respostas!$P$2:$P$101,Respostas!$B$2:$B$101,$A7,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B7=0,"",AVERAGEIFS(Respostas!$P$2:$P$126,Respostas!$B$2:$B$126,$A7,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="H7" s="11">
-        <f>IF(B7=0,"",AVERAGEIFS(Respostas!$Q$2:$Q$101,Respostas!$B$2:$B$101,$A7,Respostas!$R$2:$R$101,"&gt;=0"))</f>
+        <f>IF(B7=0,"",AVERAGEIFS(Respostas!$Q$2:$Q$126,Respostas!$B$2:$B$126,$A7,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
       <c r="I7" s="12">
-        <f>IF(B7=0,"",COUNTIFS(Respostas!$B$2:$B$101,$A7,Respostas!$R$2:$R$101,"&gt;=8")/B7)</f>
+        <f>IF(B7=0,"",COUNTIFS(Respostas!$B$2:$B$126,$A7,Respostas!$R$2:$R$126,"&gt;=8")/B7)</f>
         <v/>
       </c>
       <c r="J7" s="11">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,$A7,Respostas!$I$2:$I$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$I$2:$I$101,Respostas!$B$2:$B$101,$A7))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A7,Respostas!$I$2:$I$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$I$2:$I$126,Respostas!$B$2:$B$126,$A7))</f>
         <v/>
       </c>
       <c r="K7" s="10">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,$A7,Respostas!$L$2:$L$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$L$2:$L$101,Respostas!$B$2:$B$101,$A7))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A7,Respostas!$L$2:$L$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$L$2:$L$126,Respostas!$B$2:$B$126,$A7))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
+      </c>
+      <c r="B8" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A8,Respostas!$R$2:$R$126,"&gt;=0")</f>
+        <v/>
+      </c>
+      <c r="C8" s="11">
+        <f>IF(B8=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,$A8))</f>
+        <v/>
+      </c>
+      <c r="D8" s="11">
+        <f>IF(B8=0,"",AVERAGEIFS(Respostas!$M$2:$M$126,Respostas!$B$2:$B$126,$A8,Respostas!$R$2:$R$126,"&gt;=0"))</f>
+        <v/>
+      </c>
+      <c r="E8" s="11">
+        <f>IF(B8=0,"",AVERAGEIFS(Respostas!$N$2:$N$126,Respostas!$B$2:$B$126,$A8,Respostas!$R$2:$R$126,"&gt;=0"))</f>
+        <v/>
+      </c>
+      <c r="F8" s="11">
+        <f>IF(B8=0,"",AVERAGEIFS(Respostas!$O$2:$O$126,Respostas!$B$2:$B$126,$A8,Respostas!$R$2:$R$126,"&gt;=0"))</f>
+        <v/>
+      </c>
+      <c r="G8" s="11">
+        <f>IF(B8=0,"",AVERAGEIFS(Respostas!$P$2:$P$126,Respostas!$B$2:$B$126,$A8,Respostas!$R$2:$R$126,"&gt;=0"))</f>
+        <v/>
+      </c>
+      <c r="H8" s="11">
+        <f>IF(B8=0,"",AVERAGEIFS(Respostas!$Q$2:$Q$126,Respostas!$B$2:$B$126,$A8,Respostas!$R$2:$R$126,"&gt;=0"))</f>
+        <v/>
+      </c>
+      <c r="I8" s="12">
+        <f>IF(B8=0,"",COUNTIFS(Respostas!$B$2:$B$126,$A8,Respostas!$R$2:$R$126,"&gt;=8")/B8)</f>
+        <v/>
+      </c>
+      <c r="J8" s="11">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A8,Respostas!$I$2:$I$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$I$2:$I$126,Respostas!$B$2:$B$126,$A8))</f>
+        <v/>
+      </c>
+      <c r="K8" s="10">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A8,Respostas!$L$2:$L$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$L$2:$L$126,Respostas!$B$2:$B$126,$A8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Gate 1: sinal do benchmark</t>
         </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Melhor concorrente</t>
-        </is>
-      </c>
-      <c r="B10" s="11">
-        <f>IF(COUNT(C4:C6)=0,"",MAX(C4:C6))</f>
-        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Sinal</t>
-        </is>
-      </c>
-      <c r="B11" s="9">
-        <f>IF(B10="","Aguardando coleta",IF(B10&gt;=8,"Concorrentes fortes: só seguir se as entrevistas mostrarem dor mensurável",IF(B10&lt;6,"Gap confirmado: seguir com H1 + H3","Zona cinza: focar em H3 + H4 (fluxo + custo)")))</f>
-        <v/>
-      </c>
-      <c r="C11" s="13" t="n"/>
-      <c r="D11" s="13" t="n"/>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="13" t="n"/>
-      <c r="G11" s="13" t="n"/>
-      <c r="H11" s="14" t="n"/>
+          <t>Melhor concorrente</t>
+        </is>
+      </c>
+      <c r="B11" s="11">
+        <f>IF(COUNT(C4,C5,C6)=0,"",MAX(C4,C5,C6))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>Sinal</t>
+        </is>
+      </c>
+      <c r="B12" s="9">
+        <f>IF(B11="","Aguardando coleta",IF(B11&gt;=8,"Concorrentes fortes: só seguir se as entrevistas mostrarem dor mensurável",IF(B11&lt;6,"Gap confirmado: seguir com H1 + H3","Zona cinza: focar em H3 + H4 (fluxo + custo)")))</f>
+        <v/>
+      </c>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="13" t="n"/>
+      <c r="F12" s="13" t="n"/>
+      <c r="G12" s="13" t="n"/>
+      <c r="H12" s="14" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>Regras em docs/fase3/03_plano_validacao.md. O Gate combina este sinal com as entrevistas.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Nota média por categoria</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Jus IA</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Jurídico AI</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>LLM genérico</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>RAG atual</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Certidão</t>
-        </is>
-      </c>
-      <c r="B16" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A16,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A16))</f>
-        <v/>
-      </c>
-      <c r="C16" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A16,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A16))</f>
-        <v/>
-      </c>
-      <c r="D16" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A16,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A16))</f>
-        <v/>
-      </c>
-      <c r="E16" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A16,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A16))</f>
-        <v/>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>RAG Fase 3</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Busca</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="B17" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A17,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A17))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A17,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A17))</f>
         <v/>
       </c>
       <c r="C17" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A17,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A17))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A17,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A17))</f>
         <v/>
       </c>
       <c r="D17" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A17,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A17))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A17,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A17))</f>
         <v/>
       </c>
       <c r="E17" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A17,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A17))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A17,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A17))</f>
+        <v/>
+      </c>
+      <c r="F17" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A17,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A17))</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Informação verbal</t>
+          <t>Busca</t>
         </is>
       </c>
       <c r="B18" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A18,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A18))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A18,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A18))</f>
         <v/>
       </c>
       <c r="C18" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A18,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A18))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A18,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A18))</f>
         <v/>
       </c>
       <c r="D18" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A18,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A18))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A18,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A18))</f>
         <v/>
       </c>
       <c r="E18" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A18,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A18))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A18,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A18))</f>
+        <v/>
+      </c>
+      <c r="F18" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A18,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A18))</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Poder público</t>
+          <t>Informação verbal</t>
         </is>
       </c>
       <c r="B19" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A19,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A19))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A19,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A19))</f>
         <v/>
       </c>
       <c r="C19" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A19,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A19))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A19,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A19))</f>
         <v/>
       </c>
       <c r="D19" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A19,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A19))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A19,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A19))</f>
         <v/>
       </c>
       <c r="E19" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A19,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A19))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A19,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A19))</f>
+        <v/>
+      </c>
+      <c r="F19" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A19,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A19))</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>Transparência</t>
+          <t>Poder público</t>
         </is>
       </c>
       <c r="B20" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A20,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A20))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A20,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A20))</f>
         <v/>
       </c>
       <c r="C20" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A20,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A20))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A20,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A20))</f>
         <v/>
       </c>
       <c r="D20" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A20,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A20))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A20,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A20))</f>
         <v/>
       </c>
       <c r="E20" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A20,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A20))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A20,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A20))</f>
+        <v/>
+      </c>
+      <c r="F20" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A20,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A20))</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Dado sensível</t>
+          <t>Transparência</t>
         </is>
       </c>
       <c r="B21" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A21,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A21))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A21,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A21))</f>
         <v/>
       </c>
       <c r="C21" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A21,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A21))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A21,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A21))</f>
         <v/>
       </c>
       <c r="D21" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A21,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A21))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A21,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A21))</f>
         <v/>
       </c>
       <c r="E21" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A21,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A21))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A21,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A21))</f>
+        <v/>
+      </c>
+      <c r="F21" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A21,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A21))</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Tratamento</t>
+          <t>Dado sensível</t>
         </is>
       </c>
       <c r="B22" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A22,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A22))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A22,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A22))</f>
         <v/>
       </c>
       <c r="C22" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A22,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A22))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A22,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A22))</f>
         <v/>
       </c>
       <c r="D22" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A22,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A22))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A22,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A22))</f>
         <v/>
       </c>
       <c r="E22" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A22,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A22))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A22,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A22))</f>
+        <v/>
+      </c>
+      <c r="F22" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A22,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A22))</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Compartilhamento</t>
+          <t>Tratamento</t>
         </is>
       </c>
       <c r="B23" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A23,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A23))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A23,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A23))</f>
         <v/>
       </c>
       <c r="C23" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A23,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A23))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A23,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A23))</f>
         <v/>
       </c>
       <c r="D23" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A23,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A23))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A23,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A23))</f>
         <v/>
       </c>
       <c r="E23" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A23,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A23))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A23,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A23))</f>
+        <v/>
+      </c>
+      <c r="F23" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A23,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A23))</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Norma CE</t>
+          <t>Compartilhamento</t>
         </is>
       </c>
       <c r="B24" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A24,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A24))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A24,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A24))</f>
         <v/>
       </c>
       <c r="C24" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A24,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A24))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A24,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A24))</f>
         <v/>
       </c>
       <c r="D24" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A24,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A24))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A24,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A24))</f>
         <v/>
       </c>
       <c r="E24" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A24,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A24))</f>
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A24,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A24))</f>
+        <v/>
+      </c>
+      <c r="F24" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A24,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A24))</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
+          <t>Norma CE</t>
+        </is>
+      </c>
+      <c r="B25" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A25,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A25))</f>
+        <v/>
+      </c>
+      <c r="C25" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A25,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A25))</f>
+        <v/>
+      </c>
+      <c r="D25" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A25,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A25))</f>
+        <v/>
+      </c>
+      <c r="E25" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A25,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A25))</f>
+        <v/>
+      </c>
+      <c r="F25" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A25,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A25))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
           <t>Incidente</t>
         </is>
       </c>
-      <c r="B25" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A25,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,B$15,Respostas!$C$2:$C$101,$A25))</f>
-        <v/>
-      </c>
-      <c r="C25" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A25,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,C$15,Respostas!$C$2:$C$101,$A25))</f>
-        <v/>
-      </c>
-      <c r="D25" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A25,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,D$15,Respostas!$C$2:$C$101,$A25))</f>
-        <v/>
-      </c>
-      <c r="E25" s="15">
-        <f>IF(COUNTIFS(Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A25,Respostas!$R$2:$R$101,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$101,Respostas!$B$2:$B$101,E$15,Respostas!$C$2:$C$101,$A25))</f>
+      <c r="B26" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A26,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,B$16,Respostas!$C$2:$C$126,$A26))</f>
+        <v/>
+      </c>
+      <c r="C26" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A26,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,C$16,Respostas!$C$2:$C$126,$A26))</f>
+        <v/>
+      </c>
+      <c r="D26" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A26,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,D$16,Respostas!$C$2:$C$126,$A26))</f>
+        <v/>
+      </c>
+      <c r="E26" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A26,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,E$16,Respostas!$C$2:$C$126,$A26))</f>
+        <v/>
+      </c>
+      <c r="F26" s="15">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A26,Respostas!$R$2:$R$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,F$16,Respostas!$C$2:$C$126,$A26))</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B12:H12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: busca híbrida E5 multilíngue + BM25 na fase 3
- retrieval.py: intfloat/multilingual-e5-small em ONNX (sem torch),
  BM25 com tokenização pt-BR e fusão RRF dos top 50 de cada lista
- coleção fase3 reindexada com E5; nome do modelo nos metadados e
  erro ao abrir com outro modelo (ambos têm 384 dim: falharia calado)
- Fase3Pipeline troca só o retrieve() do RAGPipeline
- benchmark: --modo hibrido|denso|bm25; eval_retrieval.py (alvos
  provisórios)
- resultado: "não encontrado" 20 (Fase 2) -> 14 (MiniLM) -> 8 (híbrido);
  risco novo: resposta errada na #1 misturando Registro Civil com
  Registro de Imóveis

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fase3/benchmark/planilha_benchmark.xlsx
+++ b/docs/fase3/benchmark/planilha_benchmark.xlsx
@@ -6120,27 +6120,37 @@
       </c>
       <c r="F102" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G102" s="8" t="inlineStr">
         <is>
-          <t>Não encontrado no corpus.</t>
+          <t>**Não.**  
+A emissão de certidão de inteiro teor a pedido de terceiro — pessoa sem vínculo com o registrado— está condicionada a requisitos específicos previstos no **Provimento CNJ 149/2023**.
+- **Art. 114.** As certidões de registro civil, inclusive as de inteiro teor, **só podem ser expedidas a terceiros** quando contiverem dados sensíveis **mediante autorização do juízo competente**.  
+- **§ 1.º** do mesmo artigo deixa claro que, na hipótese de solicitação por terceiros, **é obrigatória a autorização judicial** quando a certidão envolver informações sensíveis.  
+Além disso, o requerimento deve observar as exigências de forma escrita:
+- **Art. 117** (e **Art. 258**) estabelecem que o requerimento **deve conter**:
+  - identificação do requerente;  
+  - **motivo** da solicitação;  
+  - grau de parentesco com o registrado, se houver;  
+  - informação sobre eventual falecimento do titular.  
+Portanto, **não é possível emitir a certidão de inteiro teor a um terceiro sem exigir a indicação do motivo** (e, quando houver dados sensíveis, a devida autorização judicial).</t>
         </is>
       </c>
       <c r="H102" s="8" t="inlineStr">
         <is>
-          <t>Provimento CNJ 149/2023, Art. 417:p266; Código de Normas CGJ-CE, Art. 1490:p305; Código de Normas CGJ-CE, Art. 1517:p312; Código de Normas CGJ-CE, Art. 1472:p301; Código de Normas CGJ-CE, Art. 1285:p263</t>
+          <t>Código de Normas CGJ-CE, Art. 471:p116; Provimento CNJ 149/2023, Art. 117:p55; Código de Normas CGJ-CE, Art. 258:p78; Provimento CNJ 149/2023, Art. 327:p209; Provimento CNJ 149/2023, Art. 114:p54</t>
         </is>
       </c>
       <c r="I102" s="8" t="n">
-        <v>4.98</v>
+        <v>3.91</v>
       </c>
       <c r="J102" s="8" t="n">
-        <v>1920</v>
+        <v>2231</v>
       </c>
       <c r="K102" s="8" t="n">
-        <v>89</v>
+        <v>559</v>
       </c>
       <c r="L102" s="10">
         <f>IF(COUNT(J102:K102)=2,(J102*Parametros!$B$3+K102*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6181,7 +6191,7 @@
       </c>
       <c r="F103" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G103" s="8" t="inlineStr">
@@ -6191,14 +6201,14 @@
       </c>
       <c r="H103" s="8" t="inlineStr">
         <is>
-          <t>Provimento CNJ 149/2023, Art. 477:p318; Provimento CNJ 149/2023, Art. 221:p124; Provimento CNJ 149/2023, Art. 390:p239; Provimento CNJ 149/2023, Art. 205-A:p95; Provimento CNJ 149/2023, Art. 495-E:p326</t>
+          <t>Código de Normas CGJ-CE, Art. 258:p78; Código de Normas CGJ-CE, Art. 1083:p218; Código de Normas CGJ-CE, Art. 255:p78; Provimento CNJ 149/2023, Art. 117:p55; Código de Normas CGJ-CE, Art. 1502:p308</t>
         </is>
       </c>
       <c r="I103" s="8" t="n">
-        <v>1.3</v>
+        <v>0.63</v>
       </c>
       <c r="J103" s="8" t="n">
-        <v>2195</v>
+        <v>1962</v>
       </c>
       <c r="K103" s="8" t="n">
         <v>113</v>
@@ -6242,32 +6252,43 @@
       </c>
       <c r="F104" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G104" s="8" t="inlineStr">
         <is>
           <t>**Resposta**
-Sim. A certidão de matrícula pode ser emitida integralmente contendo o histórico completo de todos os ônus, inclusive penhoras já canceladas.
-- **Art. 440‑G** (Seção I) estabelece que, para fins de adjudicação compulsória, a ata notarial – que serve de modelo para a certidão registral – deve conter:
-  - **I** – a referência à matrícula ou à transcrição, **e a descrição do imóvel com seus ônus e gravames**.
-- **Art. 210‑C** (Subseção I) dispõe que o extrato eletrônico (certidão) deve obedecer aos campos e cláusulas obrigatórias definidos em norma técnica, assegurando a integridade das informações registradas.
-Dessa forma, a emissão integral da certidão, com o histórico completo de ônus e gravames, está em conformidade com os requisitos legais acima citados.</t>
+De acordo com o disposto nos normativos citados:
+- **Art. 1.129** do **Código de Normas CGJ‑CE** – caput  
+  As certidões dos imóveis que já forem objeto de matrícula eletrônica, após a “primeira qualificação eletrônica”, serão expedidas, **independentemente de indicação de finalidade**, em formato nato‑digital estruturado, contendo **a situação jurídica atual do imóvel**, ou seja, sua descrição, titularidade e **os ônus reais não cancelados**.
+- **Art. 125** do **Provimento CNJ 149/2023** – caput (texto idêntico ao art. 1.129)  
+  Reitera que a certidão deve conter **apenas a situação jurídica atual** e **os ônus não cancelados**.
+- **Art. 1.682** do **Código de Normas CGJ‑CE** – caput e parágrafo único  
+  - Caput: idem aos artigos acima, limitando a certidão à situação atual e aos ônus não cancelados.  
+  - **Parágrafo único**: A expedição de certidão de atos anteriores da cadeia filiatória do imóvel **depende de identificação segura do requerente e de indicação da finalidade**.
+- **Art. 230** da **Lei 6.015/1973** – caput  
+  Quando houver ônus na certidão, o oficial o averbá no registro, mas não trata de ônus já cancelados.
+### Conclusão
+- **Não** é possível emitir a certidão da matrícula contendo **todo o histórico de ônus, inclusive penhoras já canceladas**, de forma automática e sem requisitos adicionais.
+- Para obter informações sobre atos anteriores (penhoras canceladas, etc.), é necessário:
+  1. **Identificação segura** do requerente;  
+  2. **Indicação clara da finalidade** da certidão (ex.: pesquisa de histórico de ônus).  
+Somente atendidas essas condições, a autoridade competente poderá expedir a certidão com os atos anteriores da cadeia filiatória. Caso contrário, a certidão deve limitar‑se à **situação jurídica atual** e aos **ônus não cancelados**.</t>
         </is>
       </c>
       <c r="H104" s="8" t="inlineStr">
         <is>
-          <t>Provimento CNJ 149/2023, Art. 409:p262; Provimento CNJ 149/2023, Art. 210-C:p107; Provimento CNJ 149/2023, Art. 440-G:p276; Provimento CNJ 149/2023, Art. 493:p324; Lei 8.935/1994, Art. 32:p0</t>
+          <t>Código de Normas CGJ-CE, Art. 1129:p229; Provimento CNJ 149/2023, Art. 125:p57; Lei 6.015/1973, Art. 230:p0; Código de Normas CGJ-CE, Art. 1259:p256; Código de Normas CGJ-CE, Art. 1682:p345</t>
         </is>
       </c>
       <c r="I104" s="8" t="n">
-        <v>2.31</v>
+        <v>2.15</v>
       </c>
       <c r="J104" s="8" t="n">
-        <v>2093</v>
+        <v>1909</v>
       </c>
       <c r="K104" s="8" t="n">
-        <v>647</v>
+        <v>788</v>
       </c>
       <c r="L104" s="10">
         <f>IF(COUNT(J104:K104)=2,(J104*Parametros!$B$3+K104*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6308,27 +6329,31 @@
       </c>
       <c r="F105" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G105" s="8" t="inlineStr">
         <is>
-          <t>Não encontrado no corpus</t>
+          <t>**Não.**  
+De acordo com o **Provimento CNJ 149/2023**, **Art. 123**, a prestação de informações cadastrais – como a busca de todos os imóveis registrados em nome de uma pessoa – está sujeita a requisitos de identificação do requerente e de indicação da finalidade:
+- **Art. 123.** “Dependem de identificação do requerente e independem de indicação da finalidade os pedidos de certidão de registros em sentido estrito, averbações, matrículas, transcrições ou inscrições específicas, expedidas em qualquer modalidade.”
+- **§ 3.º** “Pedidos de certidão, de busca e de informações apresentados em bloco… dependem de identificação do requerente e indicação da finalidade…”.
+Portanto, **não é permitido** atender a um pedido que contenha apenas o nome do interessado, sem que o requerente se identifique e indique a finalidade da pesquisa. O fornecimento da informação sem esses requisitos violaria o disposto no provimento.</t>
         </is>
       </c>
       <c r="H105" s="8" t="inlineStr">
         <is>
-          <t>Guia ANPD — Segurança da Informação, p. 1:p1; Guia ANPD — Segurança da Informação, p. 18:p18; Guia ANPD — Segurança da Informação, p. 10:p10; Guia ANPD — Segurança da Informação, p. 12:p12</t>
+          <t>Código de Normas CGJ-CE, Art. 1416:p287; Lei 6.015/1973, Art. 234:p0; Provimento CNJ 149/2023, Art. 123:p56; Código de Normas CGJ-CE, Art. 822:p175; Lei 6.015/1973, Art. 213:p0</t>
         </is>
       </c>
       <c r="I105" s="8" t="n">
-        <v>1.24</v>
+        <v>1.64</v>
       </c>
       <c r="J105" s="8" t="n">
-        <v>1567</v>
+        <v>2383</v>
       </c>
       <c r="K105" s="8" t="n">
-        <v>131</v>
+        <v>576</v>
       </c>
       <c r="L105" s="10">
         <f>IF(COUNT(J105:K105)=2,(J105*Parametros!$B$3+K105*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6369,55 +6394,44 @@
       </c>
       <c r="F106" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G106" s="8" t="inlineStr">
         <is>
-          <t>**Procedimento para busca de bens por CPF solicitada por um credor**
-**Art. 397-AI**  
-- **I** — a indicação da localização do bem é responsabilidade do **credor fiduciário** ou de seus mandatários;  
-- **II** — uma vez localizado, o bem será agendado por meio do **módulo próprio na Central RTDPJ Brasil**, integrante do Sistema Eletrônico dos Registros Públicos – Serp, ou por contato direto com o **oficial de registro de títulos e documentos**;  
-- **III** — o oficial de registro deve garantir a disponibilidade de dia e horário para o agendamento da diligência de apreensão, durante o expediente normal da serventia, no mesmo dia da solicitação nas capitais e regiões metropolitanas, e, nas demais regiões, em até 1 (um) dia útil.
-**Art. 397-K**  
-- **I** — a atribuição para realizar o processo de consolidação da propriedade extrajudicial e da busca e apreensão de bem móvel será do **oficial de registro de títulos e documentos** do domicílio do devedor fiduciante, ou da localização do bem;  
-- **II** — se o bem móvel estiver localizado em local diverso do domicílio do devedor, o oficial de registro do local onde o bem for encontrado será competente para a diligência;  
-- **III** — os emolumentos relativos ao ato de busca e apreensão serão devidos ao oficial de registro do local onde a diligência for efetivamente realizada.
-**Art. 397-J**  
-- **I** — o **credor fiduciário**, seu procurador ou representante legal possui legitimidade para requerer a consolidação da propriedade extrajudicial e a busca e apreensão de bem móvel;  
-- **Parágrafo único** — os credores devem se habilitar no módulo próprio da Central RTDPJ Brasil, indicando, através de cadastramento em seu perfil criptografado, os prepostos autorizados a iniciar e acompanhar o processo, sendo desnecessário o envio de procurações ou autorizações expressas.
----
-### Passos a serem seguidos
-1. **Registro no módulo**  
-   - O credor fiduciário deve se habilitar no módulo próprio da Central RTDPJ Brasil e cadastrar os prepostos autorizados.
-2. **Solicitação de localização**  
-   - O credor solicita a localização do bem, informando o **CPF** do devedor, por meio do módulo ou contato direto com o oficial de registro.
-3. **Responsabilidade do oficial de registro**  
-   - O oficial de registro responsável pela localização do bem registra a solicitação no módulo e agenda a diligência de apreensão.
-4. **Agendamento da diligência**  
-   - O oficial garante a disponibilidade de dia e horário, conforme §2º do Art. 397-AI:  
-     - Na mesma cidade (capitais e regiões metropolitanas) no dia da solicitação;  
-     - Em até 1 (um) dia útil nas demais regiões.
-5. **Execução da diligência**  
-   - Se o bem estiver localizado em outro local, o oficial de registro do local onde o bem for encontrado executará a diligência, conforme Art. 397-K §1º.
-6. **Pagamento de emolumentos**  
-   - Os emolumentos relativos à busca e apreensão são devidos ao oficial de registro do local onde a diligência for realizada, conforme Art. 397-K §2º.
-Assim, o credor segue o procedimento estabelecido pelos Provimentos CNJ 149/2023, garantindo a localização e eventual apreensão do bem do devedor.</t>
+          <t>**Procedimento para busca de bens do devedor por CPF solicitada por um credor**
+**Art. 1.659.**  
+No requerimento do credor fiduciário dirigido ao Oficial do Registro de Imóveis para intimação do fiduciante devem constar as seguintes informações:
+- **I** — número do CPF e nome do devedor fiduciante (e de seu cônjuge, se for casado em regime de bens que exija a intimação);
+- **II** — endereço residencial atual e anterior, se houver, do devedor fiduciante;
+- **III** — endereço comercial, se houver, do devedor fiduciante;
+- **IV** — declaração de que decorreu o prazo de carência estipulado no contrato;
+- **V** — planilha contendo o demonstrativo do débito decorrente das prestações vencidas e não pagas e das que se vencerem até a data do pagamento, os juros convencionais, as penalidades e os demais encargos contratuais, os encargos legais, inclusive tributos e as contribuições condominiais imputáveis ao imóvel, bem como a projeção da dívida, em valores atualizados, para purgação da mora;
+- **VI** — número do CPF e nome do representante do credor fiduciário;
+- **VII** — comprovante de representação legal do credor fiduciário pelo signatário do requerimento, quando for o caso.
+**Art. 1.666.**  
+Quando, por três vezes, o devedor, seu representante legal ou seu procurador não for encontrado em seu domicílio, residência ou em outro endereço indicado pelo credor para ser intimado e houver suspeita razoável de ocultação, o oficial intimará qualquer pessoa próxima, parente ou não, do devedor de que no dia imediato voltará a efetuar a intimação na hora que designar.
+**Procedimento resumido**
+1. O credor apresenta ao Oficial do Registro de Imóveis um requerimento contendo, obrigatoriamente, os itens listados no **Art. 1.659**.
+2. O Oficial verifica a existência de registros imobiliários vinculados ao CPF informado.
+3. Se o devedor não for localizado em seu domicílio, o Oficial procede conforme o **Art. 1.666**, intimando terceiros próximos e designando nova data e hora para a intimação.
+4. O Oficial, ao localizar os bens, registra a localização da parcela ou da hipoteca, conforme previsto no **Art. 1.621**, observando as exigências específicas de cada tipo de gravame (hipoteca, penhora, anticrese, etc.).
+Assim, a busca por CPF solicitada por um credor segue o procedimento acima, garantindo que todas as informações exigidas sejam apresentadas e que o Oficial do Registro de Imóveis realize a localização e intimação de forma adequada.</t>
         </is>
       </c>
       <c r="H106" s="8" t="inlineStr">
         <is>
-          <t>Provimento 15/2026/CGJCE, Art. 2:p2; Provimento CNJ 149/2023, Art. 397-AI:p254; Provimento CNJ 149/2023, Art. 397-K:p245; Provimento CNJ 149/2023, Art. 397-J:p245; Provimento CNJ 149/2023, Art. 440-X:p282</t>
+          <t>Código de Normas CGJ-CE, Art. 1659:p339; Código de Normas CGJ-CE, Art. 1621:p330; Código de Normas CGJ-CE, Art. 1666:p342; Provimento 15/2026/CGJCE, Art. 1:p2; Provimento CNJ 149/2023, Art. 397-AL:p256</t>
         </is>
       </c>
       <c r="I106" s="8" t="n">
-        <v>2.44</v>
+        <v>1.75</v>
       </c>
       <c r="J106" s="8" t="n">
-        <v>2144</v>
+        <v>2689</v>
       </c>
       <c r="K106" s="8" t="n">
-        <v>1419</v>
+        <v>1079</v>
       </c>
       <c r="L106" s="10">
         <f>IF(COUNT(J106:K106)=2,(J106*Parametros!$B$3+K106*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6458,33 +6472,27 @@
       </c>
       <c r="F107" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>**Decreto 7.724/2012, Art. 17.**  
-Caso a informação esteja disponível ao público em formato impresso, eletrônico ou em outro meio de acesso universal, o órgão ou entidade deverá orientar o requerente quanto ao local e modo para consultar, obter ou reproduzir a informação.  
-Parágrafo único. Na hipótese do caput, o órgão ou entidade desobriga‑se do fornecimento direto da informação, salvo se o requerente declarar não dispor de meios para consultar, obter ou reproduzir a informação.  
----
-**Resposta**  
-- Se o nome do proprietário do imóvel for informação **pública** (disponível em registros oficiais, cartórios, etc.), o órgão deve **orientar** o requerente sobre onde e como consultar ou obter essa informação.  
-- Se a informação **não for pública** ou não estiver disponível em meio de acesso universal, o órgão **não pode** fornecer o dado diretamente por telefone, exceto se o requerente declarar que não tem meios para consultar ou reproduzir a informação.</t>
+          <t>Não encontrado no corpus</t>
         </is>
       </c>
       <c r="H107" s="8" t="inlineStr">
         <is>
-          <t>Provimento CNJ 149/2023, Art. 58:p23; Decreto 7.724/2012, Art. 17:p0; Provimento CNJ 149/2023, Art. 59:p23; Provimento CNJ 149/2023, Art. 62:p24; Código de Normas CGJ-CE, Art. 1753:p358</t>
+          <t>Código de Normas CGJ-CE, Art. 1456:p297; Provimento CNJ 149/2023, Art. 259:p166; Código de Normas CGJ-CE, Art. 1394:p282; Lei 6.015/1973, Art. 123:p0; Decreto 7.724/2012, Art. 12:p0</t>
         </is>
       </c>
       <c r="I107" s="8" t="n">
-        <v>1.71</v>
+        <v>0.72</v>
       </c>
       <c r="J107" s="8" t="n">
-        <v>1871</v>
+        <v>2462</v>
       </c>
       <c r="K107" s="8" t="n">
-        <v>733</v>
+        <v>214</v>
       </c>
       <c r="L107" s="10">
         <f>IF(COUNT(J107:K107)=2,(J107*Parametros!$B$3+K107*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6525,27 +6533,23 @@
       </c>
       <c r="F108" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
-        </is>
-      </c>
-      <c r="G108" s="8" t="inlineStr">
-        <is>
-          <t>Não encontrado no corpus.</t>
-        </is>
-      </c>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+        </is>
+      </c>
+      <c r="G108" s="8" t="inlineStr"/>
       <c r="H108" s="8" t="inlineStr">
         <is>
-          <t>Provimento CNJ 149/2023, Art. 3 (ato de aprovação):p3; Lei 6.015/1973, Art. 70:p0; Provimento CNJ 149/2023, Art. 368:p231; Provimento CNJ 149/2023, Art. 353-A:p227; Decreto 7.724/2012, Art. 30:p0</t>
+          <t>Código de Normas CGJ-CE, Art. 1333:p271; Lei 6.015/1973, Art. 279:p0; Lei 6.015/1973, Art. 292:p0; Código de Normas CGJ-CE, Art. 1412:p286; Lei 6.015/1973, Art. 225:p0</t>
         </is>
       </c>
       <c r="I108" s="8" t="n">
-        <v>0.99</v>
+        <v>7.09</v>
       </c>
       <c r="J108" s="8" t="n">
-        <v>1613</v>
+        <v>1888</v>
       </c>
       <c r="K108" s="8" t="n">
-        <v>119</v>
+        <v>2048</v>
       </c>
       <c r="L108" s="10">
         <f>IF(COUNT(J108:K108)=2,(J108*Parametros!$B$3+K108*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6586,27 +6590,54 @@
       </c>
       <c r="F109" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>**Não encontrado no corpus**</t>
+          <t>**Resposta**
+- **É permitido fornecer** a lista contendo o número de inscrição (IPTU ou ITR) do imóvel, o nome completo e o CPF do proprietário, pois a própria normativa exige a inclusão desses dados nos documentos que acompanham processos de usucapião e de retificação de registro.  
+- **Formato recomendado**  
+  - Apresentar a informação em **lista estruturada** ou **tabela** para garantir clareza e facilitar a conferência pelos servidores da prefeitura.  
+  - Cada registro deve conter, em linhas separadas, os seguintes campos:  
+    1. **Número de inscrição imobiliária** (IPTU/ITR) ou matrícula;  
+    2. **Nome completo do proprietário**;  
+    3. **CPF do proprietário**.  
+  - Exemplo de apresentação (em texto simples):  
+    ```
+    Imóvel: 12345‑6789
+    Proprietário: João da Silva
+    CPF: 123.456.789‑00
+    Imóvel: 98765‑4321
+    Proprietário: Maria Oliveira
+    CPF: 987.654.321‑00
+    ```
+  - Ou, se preferir tabela markdown:
+    | Inscrição (IPTU/ITR) | Proprietário      | CPF            |
+    |----------------------|-------------------|----------------|
+    | 12345‑6789           | João da Silva     | 123.456.789‑00 |
+    | 98765‑4321           | Maria Oliveira    | 987.654.321‑00 |
+---
+**Fundamentação normativa**
+- **Art. 907** (Seção II) – exige a consignação do número de inscrição e dos **nome e CPF do proprietário** nos documentos de usucapião.  
+- **Art. 1416** (Capítulo XVI) – determina a apresentação de certidão negativa e, quando necessário, a identificação completa dos proprietários e ocupantes.  
+- **Art. 1394** (Seção II) – lista, entre os documentos exigidos, a **identificação e qualificação dos confrontantes (proprietários e eventuais ocupantes) com nome e CPF**.  
+Esses dispositivos demonstram que a coleta e a transmissão desses dados são previstas e exigidas nos atos notariais e registrários, legitimando a entrega da lista à prefeitura para fins de cobrança de IPTU.</t>
         </is>
       </c>
       <c r="H109" s="8" t="inlineStr">
         <is>
-          <t>Provimento CNJ 149/2023, Art. 397-R:p248; Provimento CNJ 149/2023, Art. 320-AC:p205; Decreto 7.724/2012, Art. 12:p0; Provimento CNJ 149/2023, Art. 397-N:p246; Provimento CNJ 149/2023, Art. 320-R:p202</t>
+          <t>Código de Normas CGJ-CE, Art. 907:p191; Código de Normas CGJ-CE, Art. 1416:p287; Código de Normas CGJ-CE, Art. 828:p178; Código de Normas CGJ-CE, Art. 1394:p282</t>
         </is>
       </c>
       <c r="I109" s="8" t="n">
-        <v>1.11</v>
+        <v>2.32</v>
       </c>
       <c r="J109" s="8" t="n">
-        <v>1886</v>
+        <v>2375</v>
       </c>
       <c r="K109" s="8" t="n">
-        <v>185</v>
+        <v>917</v>
       </c>
       <c r="L109" s="10">
         <f>IF(COUNT(J109:K109)=2,(J109*Parametros!$B$3+K109*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6647,27 +6678,27 @@
       </c>
       <c r="F110" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>Não encontrado no corpus.</t>
+          <t>Não encontrado no corpus</t>
         </is>
       </c>
       <c r="H110" s="8" t="inlineStr">
         <is>
-          <t>Provimento CNJ 149/2023, Art. 511-E:p335; Provimento CNJ 149/2023, Art. 320-AE:p205; Código de Normas CGJ-CE, Art. 709:p156; Provimento CNJ 149/2023, Art. 556:p360; Provimento CNJ 149/2023, Art. 320-C:p198</t>
+          <t>Lei 6.015/1973, Art. 110:p0; Código de Normas CGJ-CE, Art. 1128:p229; Provimento CNJ 149/2023, Art. 320-AE:p205; LGPD (Lei 13.709/2018), Art. 18:p0; Provimento CNJ 149/2023, Art. 320-AK:p206</t>
         </is>
       </c>
       <c r="I110" s="8" t="n">
-        <v>15.36</v>
+        <v>20.93</v>
       </c>
       <c r="J110" s="8" t="n">
-        <v>2127</v>
+        <v>2412</v>
       </c>
       <c r="K110" s="8" t="n">
-        <v>199</v>
+        <v>232</v>
       </c>
       <c r="L110" s="10">
         <f>IF(COUNT(J110:K110)=2,(J110*Parametros!$B$3+K110*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6708,27 +6739,27 @@
       </c>
       <c r="F111" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>**Não encontrado no corpus**</t>
+          <t>Não encontrado no corpus.</t>
         </is>
       </c>
       <c r="H111" s="8" t="inlineStr">
         <is>
-          <t>LAI (Lei 12.527/2011), Art. 19:p0; Provimento CNJ 149/2023, Art. 187:p90; LAI (Lei 12.527/2011), Art. 1:p0; Código de Normas CGJ-CE, Art. 58:p38; Provimento CNJ 149/2023, Art. 148:p71</t>
+          <t>Código de Normas CGJ-CE, Art. 1367:p277; Código de Normas CGJ-CE, Art. 1127:p229; Código de Normas CGJ-CE, Art. 162:p63; Código de Normas CGJ-CE, Art. 285:p85; Código de Normas CGJ-CE, Art. 257:p78</t>
         </is>
       </c>
       <c r="I111" s="8" t="n">
-        <v>0.85</v>
+        <v>20.74</v>
       </c>
       <c r="J111" s="8" t="n">
-        <v>1777</v>
+        <v>1797</v>
       </c>
       <c r="K111" s="8" t="n">
-        <v>112</v>
+        <v>210</v>
       </c>
       <c r="L111" s="10">
         <f>IF(COUNT(J111:K111)=2,(J111*Parametros!$B$3+K111*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6769,7 +6800,7 @@
       </c>
       <c r="F112" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G112" s="8" t="inlineStr">
@@ -6779,17 +6810,17 @@
       </c>
       <c r="H112" s="8" t="inlineStr">
         <is>
-          <t>Provimento CNJ 149/2023, Art. 103:p52; Decreto 7.724/2012, Art. 10:p0; LAI (Lei 12.527/2011), Art. 2:p0; Provimento CNJ 149/2023, Art. 511-C:p334; Código de Normas CGJ-CE, Art. 198:p68</t>
+          <t>LAI (Lei 12.527/2011), Art. 41:p0; LAI (Lei 12.527/2011), Art. 8:p0; LAI (Lei 12.527/2011), Art. 10:p0; LAI (Lei 12.527/2011), Art. 11:p0</t>
         </is>
       </c>
       <c r="I112" s="8" t="n">
-        <v>1.47</v>
+        <v>1.49</v>
       </c>
       <c r="J112" s="8" t="n">
-        <v>1883</v>
+        <v>2265</v>
       </c>
       <c r="K112" s="8" t="n">
-        <v>310</v>
+        <v>190</v>
       </c>
       <c r="L112" s="10">
         <f>IF(COUNT(J112:K112)=2,(J112*Parametros!$B$3+K112*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6830,32 +6861,37 @@
       </c>
       <c r="F113" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>**Sim, é dever responder.**  
-O **Protocolo de Acesso à Informação** obriga os órgãos e entidades públicas a atender solicitações de informação, salvo exceções previstas em lei.  
-**Art. 34.**  
-- **I** — Os órgãos e entidades públicas respondem diretamente pelos danos causados em decorrência da divulgação não autorizada ou utilização indevida de informações sigilosas ou informações pessoais, cabendo a apuração de responsabilidade funcional nos casos de dolo ou culpa, assegurado o respectivo direito de regresso.  
-- **II** — O disposto neste artigo aplica‑se à pessoa física ou entidade privada que, em virtude de vínculo de qualquer natureza com órgãos ou entidades, tenha acesso a informação sigilosa ou pessoal e a submeta a tratamento indevido.  
-Como a solicitação refere‑se a **emolumentos arrecadados pela serventia**, trata‑se de informação pública de interesse coletivo. Portanto, a serventia tem a obrigação de responder ao pedido, fornecendo os dados solicitados ou justificando a impossibilidade de divulgação, conforme previsto na LAI.</t>
+          <t>**Art. 10.** Qualquer interessado poderá apresentar pedido de acesso a informações aos órgãos e entidades referidos no art. 1º desta Lei, por qualquer meio legítimo, devendo o pedido conter a identificação do requerente e a especificação da informação requerida.  
+§ 1º Para o acesso a informações de interesse público, a identificação do requerente não pode conter exigências que inviabilizem a solicitação.  
+§ 2º Os órgãos e entidades do poder público devem viabilizar alternativa de encaminhamento de pedidos de acesso por meio de seus sítios oficiais na internet.  
+§ 3º São vedadas quaisquer exigências relativas aos motivos determinantes da solicitação de informações de interesse público.  
+---
+**Resposta ao pedido via LAI sobre os emolumentos arrecadados pela serventia**
+- **Sim, é dever responder.**  
+  - O LAI estabelece que qualquer interessado pode solicitar informações de interesse público, e o órgão deve viabilizar o acesso.  
+  - A solicitação de dados sobre emolumentos arrecadados pela serventia é uma informação de interesse público.  
+  - Não há previsão legal que permita a recusa ou a exigência de motivos determinantes para a solicitação.  
+  - Portanto, a serventia tem a obrigação de atender ao pedido e fornecer os dados solicitados.</t>
         </is>
       </c>
       <c r="H113" s="8" t="inlineStr">
         <is>
-          <t>Lei 8.935/1994, Art. 46:p0; LAI (Lei 12.527/2011), Art. 24:p0; LAI (Lei 12.527/2011), Art. 34:p0; Provimento CNJ 149/2023, Art. 103:p52; LGPD (Lei 13.709/2018), Art. 42:p0</t>
+          <t>Provimento CNJ 149/2023, Art. 231-A:p141; Provimento CNJ 149/2023, Art. 228-U:p134; Provimento CNJ 149/2023, Art. 373:p233; LAI (Lei 12.527/2011), Art. 10:p0; Provimento CNJ 149/2023, Art. 71-J:p35</t>
         </is>
       </c>
       <c r="I113" s="8" t="n">
-        <v>13.41</v>
+        <v>1.14</v>
       </c>
       <c r="J113" s="8" t="n">
-        <v>1661</v>
+        <v>2188</v>
       </c>
       <c r="K113" s="8" t="n">
-        <v>506</v>
+        <v>619</v>
       </c>
       <c r="L113" s="10">
         <f>IF(COUNT(J113:K113)=2,(J113*Parametros!$B$3+K113*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6896,27 +6932,32 @@
       </c>
       <c r="F114" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>Não encontrado no corpus.</t>
+          <t>**Resposta**
+Sim, a certidão pode ser emitida mesmo quando a matrícula contém averbação de interdição ou curatela.  
+- **Art. 1131, §10** do Código de Normas CGJ‑CE estabelece que a certidão de inteiro teor reproduz todo o conteúdo da matrícula e é suficiente para comprovar propriedade, direitos, ônus reais e restrições sobre o imóvel, independentemente de certificação específica pelo oficial.  
+- A averbação de interdição ou curatela, estando registrada na matrícula, será reproduzida integralmente na certidão.  
+- Não há previsão no contexto que impeça a emissão da certidão quando a matrícula contém essa averbação.  
+Portanto, a certidão pode ser emitida sem restrição, contendo a averbação de interdição/curatela.</t>
         </is>
       </c>
       <c r="H114" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 1517:p312; Código de Normas CGJ-CE, Art. 364:p99; Código de Normas CGJ-CE, Art. 1476:p302; Lei 6.015/1973, Art. 29:p0; Provimento CNJ 149/2023, Art. 256-G:p152</t>
+          <t>Código de Normas CGJ-CE, Art. 1131:p229; Provimento CNJ 149/2023, Art. 201:p94; Lei 6.015/1973, Art. 19:p0; Provimento CNJ 149/2023, Art. 200:p94; Código de Normas CGJ-CE, Art. 402:p106</t>
         </is>
       </c>
       <c r="I114" s="8" t="n">
-        <v>9.41</v>
+        <v>22.16</v>
       </c>
       <c r="J114" s="8" t="n">
-        <v>1816</v>
+        <v>2051</v>
       </c>
       <c r="K114" s="8" t="n">
-        <v>201</v>
+        <v>612</v>
       </c>
       <c r="L114" s="10">
         <f>IF(COUNT(J114:K114)=2,(J114*Parametros!$B$3+K114*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6957,23 +6998,35 @@
       </c>
       <c r="F115" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
-        </is>
-      </c>
-      <c r="G115" s="8" t="inlineStr"/>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+        </is>
+      </c>
+      <c r="G115" s="8" t="inlineStr">
+        <is>
+          <t>**Art. 820.** Na escritura pública de doação, deve constar o grau de parentesco entre o(s) doador(e)s e o(s) donatário(s).  
+- **§ 1º** Se o donatário for absolutamente incapaz, dispensa‑se a aceitação, desde que se trate de doação pura.  
+- **§ 2º** Nas escrituras de doação sem encargos feitas pelos pais a favor de seus filhos absolutamente incapazes, é dispensada a aceitação por parte do menor.  
+---
+### Resposta à sua pergunta
+- **Tarjar a escritura pública de doação**: sim, é necessário registrar (tarjar) a escritura no cartório de notas, garantindo que o grau de parentesco esteja indicado.  
+- **Aceitação**: não é exigida aceitação por parte do menor, pois ele é absolutamente incapaz.  
+- **Alvará judicial**: não há necessidade de alvará judicial para doação pura e simples a menor.  
+Portanto, basta tarjar a escritura pública de doação, observando o grau de parentesco e a dispensa de aceitação.</t>
+        </is>
+      </c>
       <c r="H115" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 1517:p312; Lei 6.015/1973, Art. 102:p0; Guia ANPD — Agentes de Tratamento, p. 7:p7; Lei 6.015/1973, Art. 70:p0; Lei 6.015/1973, Art. 88:p0</t>
+          <t>Código de Normas CGJ-CE, Art. 906:p191; Provimento CNJ 149/2023, Art. 108:p52; Código de Normas CGJ-CE, Art. 1267:p258; Código de Normas CGJ-CE, Art. 820:p174; Código de Normas CGJ-CE, Art. 868:p183</t>
         </is>
       </c>
       <c r="I115" s="8" t="n">
-        <v>16.71</v>
+        <v>24.6</v>
       </c>
       <c r="J115" s="8" t="n">
-        <v>1963</v>
+        <v>1912</v>
       </c>
       <c r="K115" s="8" t="n">
-        <v>2048</v>
+        <v>861</v>
       </c>
       <c r="L115" s="10">
         <f>IF(COUNT(J115:K115)=2,(J115*Parametros!$B$3+K115*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7014,40 +7067,39 @@
       </c>
       <c r="F116" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>**Art. 132.** O fornecimento de cópias ou certidões de documentos arquivados na serventia se limita ao documento protestado propriamente dito, nos termos do art. 22 da Lei n.º 9.492/1997, enquanto perdurar o protesto, e dentro do prazo máximo de 10 anos, nos termos do art. 30 da Lei n.º 9.492/1997, não devendo ser fornecidas cópias dos demais documentos, salvo:
-- **para as partes**;  
-- **com autorização judicial**.
-**Parágrafo único.** Tratando‑se de documento de identificação pessoal, a cópia arquivada somente deve ser fornecida ao próprio titular.
----
-### Aplicação ao caso
-- O pedido refere‑se a **cópia de documento arquivado (título) que contém dados de saúde**, informação sensível protegida pela legislação de proteção de dados.  
-- Não se trata de documento protestado nem está dentro do prazo de 10 anos que autoriza a cópia automática.  
-- Portanto, a cópia **não pode ser fornecida** a terceiros.  
-**Exceções:**  
-- Se o solicitante for **parte interessada** (ou seja, a própria pessoa cujos dados de saúde constam no documento), a cópia pode ser fornecida.  
-- Se houver **autorização judicial** específica, a cópia também pode ser fornecida.  
-**Conclusão:**  
-Forneça a cópia **apenas** se o requerente for a parte titular dos dados ou se houver decisão judicial autorizando a entrega. Caso contrário, a cópia deve ser negada.</t>
+          <t>**Resposta**
+De acordo com o **Art. 132** do Provimento CNJ 149/2023 (e o **Art. 755** do Código de Normas CGJ‑CE), o fornecimento de cópias ou certidões de documentos arquivados na serventia:
+- **Limita‑se ao documento protestado propriamente dito**;  
+- **É válido enquanto perdurar o protesto** e dentro do prazo máximo de **10 (dez) anos**;  
+- **Só pode ser fornecida às partes interessadas** ou mediante **autorização judicial**.
+Além disso, o **parágrafo único** estabelece que, tratando‑se de documento de identificação pessoal, a cópia deve ser fornecida **apenas ao próprio titular**.
+Como o documento solicitado contém **dados de saúde**, que são dados pessoais sensíveis nos termos da Lei Geral de Proteção de Dados (LGPD), a sua divulgação exige:
+- **Consentimento expresso do titular**; ou  
+- **Fundamento legal específico**, como ordem judicial.
+**Portanto, a cópia só pode ser fornecida se:**
+1. O requerente for **parte interessada** (titular dos dados de saúde) e apresentar **identificação** conforme exigido; ou  
+2. Existir **autorização judicial** que legitime a entrega da cópia.
+Na ausência de um desses requisitos, **não se deve fornecer a cópia**.</t>
         </is>
       </c>
       <c r="H116" s="8" t="inlineStr">
         <is>
-          <t>Provimento CNJ 149/2023, Art. 112:p54; Provimento CNJ 149/2023, Art. 249:p146; Provimento CNJ 149/2023, Art. 132:p58; Provimento CNJ 149/2023, Art. 96:p50; Lei 6.015/1973, Art. 150:p0</t>
+          <t>Provimento CNJ 149/2023, Art. 132:p58; Código de Normas CGJ-CE, Art. 1680:p344; Código de Normas CGJ-CE, Art. 755:p164; Código de Normas CGJ-CE, Art. 1128:p229; Provimento CNJ 149/2023, Art. 392:p240</t>
         </is>
       </c>
       <c r="I116" s="8" t="n">
-        <v>2.48</v>
+        <v>2.06</v>
       </c>
       <c r="J116" s="8" t="n">
-        <v>1801</v>
+        <v>2327</v>
       </c>
       <c r="K116" s="8" t="n">
-        <v>695</v>
+        <v>595</v>
       </c>
       <c r="L116" s="10">
         <f>IF(COUNT(J116:K116)=2,(J116*Parametros!$B$3+K116*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7088,23 +7140,37 @@
       </c>
       <c r="F117" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
-        </is>
-      </c>
-      <c r="G117" s="8" t="inlineStr"/>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+        </is>
+      </c>
+      <c r="G117" s="8" t="inlineStr">
+        <is>
+          <t>**Não**.  
+O **Art. 240, § 2º** do Código de Normas CGJ‑CE determina que as certidões eletrônicas ficam disponíveis **apenas** na Central Nacional de Informações do Registro Civil (CRC) e **proíbe** o envio por correio eletrônico convencional (e‑mail) ou por outros meios que não sejam a plataforma da central eletrônica.  
+---
+## Cuidados previstos pela LGPD ao tratar a certidão
+- **Finalidade**: o tratamento deve ser realizado apenas para a finalidade de entrega da certidão ao requerente, conforme previsto na lei de registro civil.  
+- **Consentimento**: o requerente deve ter fornecido consentimento expresso para o recebimento da certidão em meio eletrônico, caso a lei não dispensa.  
+- **Segurança**: a transmissão deve ocorrer por meio seguro (ex.: HTTPS, assinatura digital ICP‑Brasil) para garantir a integridade e confidencialidade dos dados.  
+- **Limitação de acesso**: apenas o requerente e pessoas autorizadas (por exemplo, prepostos) podem acessar a certidão.  
+- **Retenção**: a certidão eletrônica deve ser mantida pelo prazo legal (30 dias corridos) e, após esse período, deve ser excluída ou disponibilizada apenas na plataforma oficial.  
+- **Transparência**: o requerente deve ser informado sobre os direitos que possui (acesso, retificação, exclusão) e sobre os meios de exercício desses direitos.  
+Esses cuidados asseguram o cumprimento da LGPD e a proteção dos dados pessoais contidos na certidão.</t>
+        </is>
+      </c>
       <c r="H117" s="8" t="inlineStr">
         <is>
-          <t>Provimento CNJ 149/2023, Art. 406:p261; Código de Normas CGJ-CE, Art. 14:p25; Código de Normas CGJ-CE, Art. 17:p26; Código de Normas CGJ-CE, Art. 1753:p358; LGPD (Lei 13.709/2018), Art. 47:p0</t>
+          <t>Código de Normas CGJ-CE, Art. 258:p78; Código de Normas CGJ-CE, Art. 211:p70; Provimento CNJ 149/2023, Art. 117:p55; Código de Normas CGJ-CE, Art. 683:p152; Código de Normas CGJ-CE, Art. 240:p75</t>
         </is>
       </c>
       <c r="I117" s="8" t="n">
-        <v>21.51</v>
+        <v>16.23</v>
       </c>
       <c r="J117" s="8" t="n">
-        <v>1832</v>
+        <v>2123</v>
       </c>
       <c r="K117" s="8" t="n">
-        <v>2048</v>
+        <v>536</v>
       </c>
       <c r="L117" s="10">
         <f>IF(COUNT(J117:K117)=2,(J117*Parametros!$B$3+K117*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7145,7 +7211,7 @@
       </c>
       <c r="F118" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G118" s="8" t="inlineStr">
@@ -7155,17 +7221,17 @@
       </c>
       <c r="H118" s="8" t="inlineStr">
         <is>
-          <t>Guia ANPD — Agentes de Tratamento, p. 8:p8; Guia ANPD — Segurança da Informação, p. 13:p13; Provimento CNJ 149/2023, Art. 79:p42; Provimento CNJ 149/2023, Art. 84:p43; Guia ANPD — Segurança da Informação, p. 14:p14</t>
+          <t>Código de Normas CGJ-CE, Art. 193:p67; Código de Normas CGJ-CE, Art. 562:p133; Código de Normas CGJ-CE, Art. 417:p109; Código de Normas CGJ-CE, Art. 1274:p262; Código de Normas CGJ-CE, Art. 1681:p345</t>
         </is>
       </c>
       <c r="I118" s="8" t="n">
-        <v>32.06</v>
+        <v>1.55</v>
       </c>
       <c r="J118" s="8" t="n">
-        <v>2261</v>
+        <v>1741</v>
       </c>
       <c r="K118" s="8" t="n">
-        <v>170</v>
+        <v>78</v>
       </c>
       <c r="L118" s="10">
         <f>IF(COUNT(J118:K118)=2,(J118*Parametros!$B$3+K118*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7206,52 +7272,27 @@
       </c>
       <c r="F119" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>**Resposta ao titular – solicitação de exclusão de dados da matrícula**
----
-**Prezado(a) [Nome do Titular],**
-Recebemos sua solicitação de exclusão dos dados pessoais referentes à sua matrícula. Em conformidade com a **Lei Geral de Proteção de Dados – LGPD (Lei nº 13.709/2018)**, informamos que:
-**Art. 18 – Direitos do titular**  
-- **VI** — eliminação dos dados pessoais tratados com o consentimento do titular, exceto nas hipóteses previstas no art. 16 desta Lei;  
-- **IV** — anonimização, bloqueio ou eliminação de dados desnecessários, excessivos ou tratados em desconformidade com o disposto nesta Lei.
-**Art. 19 – Prazo de atendimento**  
-- **I** — em formato simplificado, imediatamente;  
-- **II** — por meio de declaração clara e completa, no prazo de até **15 (quinze) dias** a contar da data do requerimento.
----
-## Procedimento a ser adotado
-- **Verificação**  
-  - Confirmaremos se os dados solicitados estão em nosso sistema e se sua exclusão não viola obrigações legais ou contratuais (art. 16 da LGPD).  
-- **Ação**  
-  - Se não houver impedimento legal, procederemos à **exclusão** dos dados da matrícula.  
-  - Caso a exclusão seja inviável por motivo legal, informaremos ao titular a razão e os prazos previstos.  
-- **Comunicação**  
-  - Enviaremos ao titular uma **confirmação de exclusão** (ou de impossibilidade de exclusão) dentro do prazo de 15 dias.  
-- **Registro**  
-  - Documentaremos todo o processo, incluindo a justificativa de eventual impossibilidade de exclusão, conforme exigido pela LGPD.
----
-**Observação**  
-Se houver necessidade de manter os dados por obrigação legal ou regulatória, informaremos ao titular a justificativa e os prazos de retenção, conforme previsto no art. 16 da LGPD.
----
-Agradecemos pela sua atenção e permanecemos à disposição para quaisquer esclarecimentos adicionais.</t>
+          <t>Não encontrado no corpus.</t>
         </is>
       </c>
       <c r="H119" s="8" t="inlineStr">
         <is>
-          <t>LGPD (Lei 13.709/2018), Art. 44:p0; LGPD (Lei 13.709/2018), Art. 43:p0; LGPD (Lei 13.709/2018), Art. 49:p0; LGPD (Lei 13.709/2018), Art. 19:p0; LGPD (Lei 13.709/2018), Art. 18:p0</t>
+          <t>LGPD (Lei 13.709/2018), Art. 4:p0; LGPD (Lei 13.709/2018), Art. 51:p0; LGPD (Lei 13.709/2018), Art. 43:p0; LGPD (Lei 13.709/2018), Art. 9:p0; LGPD (Lei 13.709/2018), Art. 7:p0</t>
         </is>
       </c>
       <c r="I119" s="8" t="n">
-        <v>15.05</v>
+        <v>21.83</v>
       </c>
       <c r="J119" s="8" t="n">
-        <v>2000</v>
+        <v>2061</v>
       </c>
       <c r="K119" s="8" t="n">
-        <v>1265</v>
+        <v>240</v>
       </c>
       <c r="L119" s="10">
         <f>IF(COUNT(J119:K119)=2,(J119*Parametros!$B$3+K119*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7292,27 +7333,33 @@
       </c>
       <c r="F120" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>Não encontrado no corpus.</t>
+          <t>**Sim, você tem obrigação de informar.**  
+- **LGPD – Art. 18**: garante ao titular o direito de acesso a seus dados pessoais, incluindo registros de quem consultou a matrícula.  
+- **LAI – Art. 30**: obriga a autoridade a publicar e disponibilizar informações administrativas, e a atender solicitações de acesso a dados.  
+Portanto, ao receber o pedido, você deve:
+1. **Verificar a identidade** do titular e a legitimidade do pedido.  
+2. **Reunir o relatório** contendo os registros de consulta à matrícula.  
+3. **Entregar o relatório** ao titular dentro do prazo legal (30 dias, salvo</t>
         </is>
       </c>
       <c r="H120" s="8" t="inlineStr">
         <is>
-          <t>Decreto 7.724/2012, Art. 17:p0; Lei 8.935/1994, Art. 46:p0; Decreto 7.724/2012, Art. 61:p0; Provimento CNJ 149/2023, Art. 440-BB:p297; LAI (Lei 12.527/2011), Art. 30:p0</t>
+          <t>Guia ANPD — Agentes de Tratamento, p. 8:p8; LAI (Lei 12.527/2011), Art. 30:p0; Código de Normas CGJ-CE, Art. 1461:p299; Provimento CNJ 149/2023, Art. 339:p215; Provimento CNJ 149/2023, Art. 415:p265</t>
         </is>
       </c>
       <c r="I120" s="8" t="n">
-        <v>21.57</v>
+        <v>18.09</v>
       </c>
       <c r="J120" s="8" t="n">
-        <v>2015</v>
+        <v>2214</v>
       </c>
       <c r="K120" s="8" t="n">
-        <v>207</v>
+        <v>2048</v>
       </c>
       <c r="L120" s="10">
         <f>IF(COUNT(J120:K120)=2,(J120*Parametros!$B$3+K120*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7353,27 +7400,42 @@
       </c>
       <c r="F121" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>Não encontrado no corpus.</t>
+          <t>**Direito do titular**  
+- **Art. 18 da LGPD** – O titular tem o direito de solicitar a **correção** de dado pessoal incorreto.  
+- **§ 5º** – O requerimento deve ser atendido **sem custos** ao titular, nos prazos e termos previstos em regulamento.  
+- **§ 6º** – O responsável deve comunicar imediatamente a correção a todos os agentes de tratamento com quem o dado foi compartilhado, salvo impossibilidade comprovada ou esforço desproporcional.
+**Procedimento de retificação no Registro de Imóveis**  
+- **Código de Normas CGJ‑CE – Art. 1.386** – A retificação de dados de qualificação pessoal das partes cabe ao **Oficial do Registro de Imóveis**, que deve:
+  1. **Receber requerimento** do titular, contendo **firma reconhecida** ou assinatura digital.  
+  2. **Verificar** que o nome lançado no assento não corresponde ao nome apresentado no registro civil (certidão de nascimento, casamento ou registro de estrangeiro).  
+  3. **Retificar o erro à margem** da matrícula, transcrição ou inscrição.
+**Fluxo integrado do pedido**  
+1. **Titular** apresenta requerimento de correção (LGPD – Art. 18) ao órgão competente (Registro de Imóveis).  
+2. **Oficial do Registro** executa a **retificação** prevista no **Art. 1.386** da Norma CGJ‑CE, obedecendo à exigência de documento comprobatório.  
+3. **Responsável pelo tratamento** (controlador ou operador) informa, sem demora, a todos os **agentes de tratamento** envolvidos, conforme **LGPD – § 6º**.  
+4. O titular recebe a confirmação da correção, sem custos, conforme **LGPD – § 5º**.
+**Conclusão**  
+O pedido do titular trata‑se de um **direito de correção** previsto na LGPD, cuja execução prática se dá por meio da **retificação** da matrícula conforme o **Art. 1.386** do Código de Normas CGJ‑CE. Ambas as normas são aplicáveis e complementares.</t>
         </is>
       </c>
       <c r="H121" s="8" t="inlineStr">
         <is>
-          <t>LGPD (Lei 13.709/2018), Art. 43:p0; LGPD (Lei 13.709/2018), Art. 44:p0; Provimento CNJ 149/2023, Art. 79:p42; Guia ANPD — Agentes de Tratamento, p. 8:p8; Provimento CNJ 149/2023, Art. 84:p43</t>
+          <t>LGPD (Lei 13.709/2018), Art. 5:p0; Código de Normas CGJ-CE, Art. 1386:p281; LGPD (Lei 13.709/2018), Art. 7:p0; LGPD (Lei 13.709/2018), Art. 18:p0</t>
         </is>
       </c>
       <c r="I121" s="8" t="n">
-        <v>1.34</v>
+        <v>4.27</v>
       </c>
       <c r="J121" s="8" t="n">
-        <v>1966</v>
+        <v>2314</v>
       </c>
       <c r="K121" s="8" t="n">
-        <v>294</v>
+        <v>885</v>
       </c>
       <c r="L121" s="10">
         <f>IF(COUNT(J121:K121)=2,(J121*Parametros!$B$3+K121*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7414,7 +7476,7 @@
       </c>
       <c r="F122" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G122" s="8" t="inlineStr">
@@ -7424,17 +7486,17 @@
       </c>
       <c r="H122" s="8" t="inlineStr">
         <is>
-          <t>Resolução CD/ANPD 15/2024, Art. 4:p0; Guia ANPD — Agentes de Tratamento, p. 16:p16; Guia ANPD — Agentes de Tratamento, p. 15:p15; Provimento CNJ 149/2023, Art. 148:p71; Guia ANPD — Agentes de Tratamento, p. 18:p18</t>
+          <t>Provimento CNJ 149/2023, Art. 168:p83; Provimento CNJ 149/2023, Art. 148:p71; Provimento CNJ 149/2023, Art. 184-A:p88; Lei 6.015/1973, Art. 237-A:p0; Provimento CNJ 149/2023, Art. 180:p86</t>
         </is>
       </c>
       <c r="I122" s="8" t="n">
-        <v>1.31</v>
+        <v>2</v>
       </c>
       <c r="J122" s="8" t="n">
-        <v>2140</v>
+        <v>2211</v>
       </c>
       <c r="K122" s="8" t="n">
-        <v>294</v>
+        <v>390</v>
       </c>
       <c r="L122" s="10">
         <f>IF(COUNT(J122:K122)=2,(J122*Parametros!$B$3+K122*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7475,43 +7537,42 @@
       </c>
       <c r="F123" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>**Art. 124** – Ressalvadas as hipóteses que tenham previsão legal ou normativa expressa, como as certidões de filiação de imóveis, ou de propriedade com negativa de ônus e alienações, ou outras compatíveis com as finalidades dos registros de imóveis e com os princípios da **Lei Geral de Proteção de Dados (LGPD)**, **não serão expedidas certidões cujo conteúdo envolva informações sobre dados pessoais extraídos de mais de uma matrícula, assentamento do registro auxiliar, transcrição ou inscrição.**  
-**Art. 290**, § 2.º – Os notários, pessoalmente ou por intermédio do e‑Notariado, **devem fornecer meios tecnológicos para o acesso das informações exclusivamente estatísticas e genéricas à Administração Pública Direta**, sendo **vedado o envio e o repasse de dados**, salvo disposição legal ou judicial específica.  
----  
+          <t>**Base legal para o compartilhamento com o ONR/SREI e centrais eletrônicas**
+- **Art. 101** do *Provimento CNJ 149/2023* dispõe que o compartilhamento de dados com centrais de serviços eletrônicos é compatível com a proteção de dados pessoais, devendo as centrais observar:
+  - adequação;
+  - necessidade;
+  - persecução da finalidade dos dados;
+  - maior eficiência e conveniência dos serviços registrais ou notariais ao cidadão.  
+- **Parágrafo único** do mesmo artigo determina preferência pela descentralização das bases de dados, evitando a transferência de bases salvo quando indispensável para a finalidade ou quando questões técnicas comprometerem a eficiência.
+- **Art. 196** do *Código de Normas CGJ‑CE* repete integralmente o conteúdo acima, reforçando a necessidade de adequação, necessidade, finalidade e eficiência, bem como a preferência pela descentralização.
+- **Art. 1.749** do *Código de Normas CGJ‑CE* obriga os responsáveis pelas serventias de registro de imóveis ou pelas centrais de serviços eletrônicos a adotar as medidas necessárias para a integração direta com o representante legal do **ONR – Operador Nacional de Registro Eletrônico de Imóveis**.
+---
 ### Necessidade de base legal adicional ou de consentimento
-- **Base legal obrigatória**  
-  - O compartilhamento de dados pessoais com a **ONR/SREI** ou com **centrais eletrônicas** só pode ocorrer quando houver **disposição legal ou normativa expressa** que autorize tal tratamento, conforme o disposto no **Art. 124**.  
-  - Na ausência de autorização legal específica, o tratamento deve se amparar em **uma das bases previstas na LGPD** (ex.: cumprimento de obrigação legal ou regulatória, execução de contrato, interesse público, proteção da vida ou da incolumidade física, etc.).  
-- **Consentimento isolado não é suficiente**  
-  - O simples consentimento do titular **não supre a exigência** de que o tratamento esteja respaldado por uma base legal prevista na LGPD.  
-  - O consentimento pode ser utilizado **apenas como uma das bases** quando nenhuma das demais se aplicar, devendo ser **livre, informado e inequívoco**.  
-- **Proibição de repasse indiscriminado**  
-  - Conforme o **Art. 290, § 2.º**, o notário **não pode enviar ou repassar dados pessoais** a terceiros, inclusive a ONR/SREI ou centrais eletrônicas, **exceto se houver disposição legal ou decisão judicial que autorize** tal comunicação.  
----  
-### Conclusão
-- **É imprescindível** identificar **uma base legal específica** (ex.: obrigação legal, interesse público, execução de contrato, decisão judicial) que legitime o compartilhamento dos dados com a ONR/SREI e as centrais eletrônicas.  
-- **O consentimento, por si só, não elimina** a necessidade de observar as bases legais previstas na LGPD e as restrições do **Art. 290, § 2.º**.  
-Portanto, **sim, é necessária uma base legal adicional** (ou autorização judicial) para o compartilhamento; o consentimento isolado não basta.</t>
+- **Base legal suficiente:** As normas citadas (**Art. 101**, **Parágrafo único**, **Art. 196** e **Art. 1.749**) já constituem a base legal para o compartilhamento de dados entre as serventias/centrais e o ONR/SREI, desde que observados os princípios de adequação, necessidade, finalidade e eficiência.
+- **Consentimento do titular:** Não há exigência expressa de consentimento nos dispositivos acima. Contudo, o tratamento deve respeitar os princípios da LGPD (Lei 13.709/2018). Caso o compartilhamento ultrapasse as finalidades previstas ou envolva dados sensíveis, o consentimento do titular poderá ser necessário conforme a LGPD.
+---
+**Conclusão:**  
+A legislação citada fornece a base legal para o compartilhamento com o ONR/SREI e as centrais eletrônicas, não sendo exigida outra norma ou consentimento específico, salvo se o tratamento pretender finalidades diferentes das previstas ou envolver dados que, segundo a LGPD, exijam consentimento.</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
         <is>
-          <t>Lei 6.015/1973, Art. 167:p0; Provimento CNJ 149/2023, Art. 510:p332; Provimento CNJ 149/2023, Art. 290:p185; Código de Normas CGJ-CE, Art. 536:p129; Provimento CNJ 149/2023, Art. 124:p57</t>
+          <t>Código de Normas CGJ-CE, Art. 1749:p357; Provimento CNJ 149/2023, Art. 101:p51; Provimento CNJ 149/2023, Art. 329-A:p209; Código de Normas CGJ-CE, Art. 196:p68; Provimento CNJ 149/2023, Art. 320-O:p201</t>
         </is>
       </c>
       <c r="I123" s="8" t="n">
-        <v>3.34</v>
+        <v>4.44</v>
       </c>
       <c r="J123" s="8" t="n">
-        <v>1985</v>
+        <v>2150</v>
       </c>
       <c r="K123" s="8" t="n">
-        <v>1081</v>
+        <v>996</v>
       </c>
       <c r="L123" s="10">
         <f>IF(COUNT(J123:K123)=2,(J123*Parametros!$B$3+K123*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7552,27 +7613,55 @@
       </c>
       <c r="F124" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>Não encontrado no corpus.</t>
+          <t>**O que mudou com o Provimento nº 15/2026/CGJCE na qualificação das partes para registro**
+---  
+**Art. 1.103 – Requisitos do registro no Livro 2**  
+- **I** — a data;  
+- **II** — a qualificação completa das partes, compreendendo:  
+  - **a)** para pessoa natural:  
+    - estado civil;  
+    - regime de bens do casamento ou da união estável (se declarado no instrumento);  
+    - profissão;  
+    - número de inscrição no CPF ou documento de identidade, ou, à falta deste, sua filiação;  
+  - **b)** para pessoa jurídica:  
+    - denominação social;  
+    - número de inscrição no CNPJ;  
+    - sede;  
+- **III** — o título da transmissão ou do ônus;  
+- **IV** — a forma do título, sua procedência e caracterização;  
+- **V** — o valor do contrato, da coisa ou da dívida, bem como:  
+  - **a)** prazo;  
+  - **b)** condições;  
+  - **c)** encargos;  
+  - **d)** juros;  
+**Parágrafo único** – É vedada a prática de ato registral com:  
+- **a)** qualificação incompleta, genérica ou indeterminada das partes, devendo o oficial recusar o título que não contenha todos os elementos qualificativos exigidos;  
+- **b)** omissão de quaisquer elementos econômicos relevantes do negócio jurídico, não sendo admitido o registro de títulos que contenham estipulações indeterminadas ou incompletas.  
+---  
+**Principais mudanças introduzidas pelo Provimento nº 15/2026/CGJCE**  
+- **Obrigatoriedade de qualificação completa** das partes, detalhando explicitamente os elementos exigidos para pessoas naturais e jurídicas.  
+- **Inclusão de um parágrafo único** que proíbe a prática de atos registrais com qualificação incompleta ou genérica e com omissão de elementos econômicos relevantes.  
+- **Reforço da responsabilidade do oficial** de registrar apenas títulos que atendam integralmente a esses requisitos.</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
         <is>
-          <t>Provimento CNJ 149/2023, Art. 343-F:p221; Provimento CNJ 149/2023, Art. 528:p349; Provimento CNJ 149/2023, Art. 456:p312; Provimento CNJ 149/2023, Art. 218:p118; Provimento CNJ 149/2023, Art. 211:p114</t>
+          <t>Provimento 15/2026/CGJCE, Art. 1:p2; Provimento 15/2026/CGJCE, Preâmbulo:p1; Código de Normas CGJ-CE, Art. 1103:p224</t>
         </is>
       </c>
       <c r="I124" s="8" t="n">
-        <v>0.88</v>
+        <v>11.67</v>
       </c>
       <c r="J124" s="8" t="n">
-        <v>1496</v>
+        <v>2128</v>
       </c>
       <c r="K124" s="8" t="n">
-        <v>111</v>
+        <v>920</v>
       </c>
       <c r="L124" s="10">
         <f>IF(COUNT(J124:K124)=2,(J124*Parametros!$B$3+K124*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7613,37 +7702,33 @@
       </c>
       <c r="F125" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>**Requisitos para emitir certidão digital segundo o Código de Normas do CE**
-**Art. 1127.**  
-Os Oficiais obrigam‑se a:  
-- **I** — lavrar certidões requeridas em formulário próprio, timbrado, pertinente aos atos praticados, vedada a utilização de impressos não oficiais;  
-- **II** — fornecer às partes as informações e certidões nos prazos e hipóteses previstos em lei.  
-Parágrafo único:  
-Os documentos quando assinados com o uso de certificado digital, realizados e/ou enviados pela Internet, deverão atender aos requisitos da Infraestrutura de Chaves Públicas Brasileira – **ICP‑Brasil**.
-**Art. 522.**  
-Se a ata for apresentada em formato eletrônico, será necessário que a assinatura digital do representante legal da pessoa jurídica, no requerimento ou na própria ata, tenha sido feita com certificado digital **ICP‑Brasil** nos padrões exigidos em lei e atos normativos.
-**Art. 788.**  
-Os atos notariais, com exceção do Testamento Público, poderão ser lavrados e arquivados em meio digital seguro, podendo inclusive ser assinados pelos notários, prepostos ou partes interessadas de forma digital com a utilização de certificação digital no padrão da Infraestrutura de Chaves Públicas Brasileira – **ICP‑Brasil**.</t>
+          <t>**Requisitos para emitir certidão digital segundo o Código de Normas CGJ‑CE**
+- **Art. 1127, I** – O oficial deve **lavrar certidões** em formulário próprio, timbrado e pertinente aos atos praticados, **vedada a utilização de impressos não oficiais**.  
+- **Art. 1127, II** – Deve **fornecer às partes as informações e certidões** nos prazos e hipóteses previstos em lei.  
+- **Art. 1127, § 1º** – Quando assinados com **certificado digital**, os documentos devem atender aos requisitos da **Infraestrutura de Chaves Públicas Brasileira – ICP‑Brasil**.  
+- **Art. 240, § 1º** – As certidões eletrônicas devem ser em **formato PDF/A** ou **XML**, com **certificado digital ICP‑Brasil, tipo A3 ou superior**, assinatura digital em **PKCS#7** e metadados no padrão **Dublin Core (DC)**.  
+- **Art. 1079** – A certidão digital deve ser **emitida e enviada exclusivamente** por meio da **Central de Registro de Títulos e Documentos** dentro de **5 (cinco) dias**.  
+- **Art. 683** – Certidões em forma de relação (ex.: devedores em títulos protestados) podem ser **encaminhadas em meio eletrônico** com **certificado digital ICP‑Brasil**.</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 1127:p229; Provimento CNJ 149/2023, Art. 266:p176; Código de Normas CGJ-CE, Art. 522:p127; Código de Normas CGJ-CE, Art. 1115:p227; Código de Normas CGJ-CE, Art. 788:p169</t>
+          <t>Código de Normas CGJ-CE, Art. 1127:p229; Código de Normas CGJ-CE, Art. 1077:p218; Código de Normas CGJ-CE, Art. 240:p75; Código de Normas CGJ-CE, Art. 1079:p218; Código de Normas CGJ-CE, Art. 683:p152</t>
         </is>
       </c>
       <c r="I125" s="8" t="n">
-        <v>10.43</v>
+        <v>17.73</v>
       </c>
       <c r="J125" s="8" t="n">
-        <v>1642</v>
+        <v>1806</v>
       </c>
       <c r="K125" s="8" t="n">
-        <v>1079</v>
+        <v>899</v>
       </c>
       <c r="L125" s="10">
         <f>IF(COUNT(J125:K125)=2,(J125*Parametros!$B$3+K125*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7684,31 +7769,40 @@
       </c>
       <c r="F126" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (fc70523)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
         </is>
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>**Guia ANPD — Segurança da Informação**  
-- **Sugerido**: os e‑mails devem ser cifrados ou, opcionalmente, os arquivos devem ser cifrados para envio.  
-**Resolução CD/ANPD 15/2024, Art. 4**  
-- **Confidencialidade**: propriedade que assegura que o dado pessoal não esteja disponível ou não seja revelado a pessoas, empresas, sistemas, órgãos ou entidades não autorizados.  
-Assim, a serventia deve garantir a confidencialidade do dado pessoal e adotar comunicações cifradas (ou arquivos cifrados) ao enviar certidões por e‑mail.</t>
+          <t>**Obrigações da serventia ao enviar uma certidão com dados pessoais ao e‑mail errado**
+**Art. 178.**  
+- **Caput** – Os responsáveis pelas serventias extrajudiciais devem atender às disposições da **Lei Geral de Proteção de Dados Pessoais (LGPD)**, obedecendo a seus fundamentos, princípios e obrigações concernentes à governança do tratamento de dados pessoais.  
+**Art. 97.**  
+- **Parágrafo único** – Deve disponibilizar, de forma adequada, informações sobre os procedimentos de tratamento de dados pessoais, nos termos do art. 9.º da LGPD, por meio de:  
+  - **I** — aviso de privacidade e proteção de dados;  
+  - **II** — avisos de cookies no portal de cada serventia, se houver;  
+  - **III** — aviso de privacidade para navegação no website da serventia, se houver.  
+**Art. 189.**  
+- **Parágrafo único** – O responsável pela serventia extrajudicial pode solicitar apoio à entidade de classe para capacitação de seus prepostos, garantindo que todos os envolvidos no tratamento de dados pessoais estejam aptos a cumprir as normas e procedimentos de privacidade.  
+**Práticas adicionais (conforme LGPD)**  
+- Corrigir o envio indevido, garantindo que os dados pessoais sejam devolvidos ou excluídos do destinatário incorreto.  
+- Notificar a pessoa física afetada sobre o incidente, se houver risco de violação de seus direitos.  
+- Registrar o incidente e adotar medidas de mitigação, conforme exigido pela LGPD.</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 1753:p358; Resolução CD/ANPD 15/2024, Art. 4:p0; Guia ANPD — Segurança da Informação, p. 15:p15; Guia ANPD — Agentes de Tratamento, p. 7:p7; Provimento CNJ 149/2023, Art. 101:p51</t>
+          <t>Código de Normas CGJ-CE, Art. 178:p65; Código de Normas CGJ-CE, Art. 189:p67; Provimento CNJ 149/2023, Art. 236:p142; Provimento CNJ 149/2023, Art. 97:p50; Código de Normas CGJ-CE, Art. 564:p133</t>
         </is>
       </c>
       <c r="I126" s="8" t="n">
-        <v>20.41</v>
+        <v>18.66</v>
       </c>
       <c r="J126" s="8" t="n">
-        <v>2003</v>
+        <v>1708</v>
       </c>
       <c r="K126" s="8" t="n">
-        <v>1293</v>
+        <v>1302</v>
       </c>
       <c r="L126" s="10">
         <f>IF(COUNT(J126:K126)=2,(J126*Parametros!$B$3+K126*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>

</xml_diff>

<commit_message>
feat: adiciona verificador determinístico de citações
- src/fase3/verificador_citacoes.py, em Python puro e sem LLM:
  extrai "Art./Artigo N" (com ou sem ponto de milhar, listas e
  sufixo -A), associa cada um à norma da frase e classifica em
  VERIFICADA, NORMA_DIVERGENTE ou NAO_RECUPERADA contra os trechos
  recuperados; expõe total, contagens e taxa_verificavel
- answer() e Ato Pronto devolvem o relatório; o Ato ignora
  "citacoes" vindas do LLM
- UI avisa quando há citação não verificada (chat e Ato Pronto)
- benchmark grava a taxa por pergunta (colunas T-W) e o total
  (JSON e aba Resumo)
- medição de 13/10 (RAG Fase 3, 25 perguntas): 51/58 citações
  verificadas (88%), 0 com norma divergente, 7 não recuperadas
</commit_message>
<xml_diff>
--- a/docs/fase3/benchmark/planilha_benchmark.xlsx
+++ b/docs/fase3/benchmark/planilha_benchmark.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LEIA-ME" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Perguntas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Respostas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Parametros" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Resumo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEIA-ME" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perguntas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Respostas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parametros" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Respostas'!$A$1:$S$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Respostas'!$A$1:$W$126</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -175,10 +175,10 @@
     <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1459,7 +1459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S126"/>
+  <dimension ref="A1:W126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1481,6 +1481,10 @@
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="40" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="50" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1577,6 +1581,26 @@
       <c r="S1" s="6" t="inlineStr">
         <is>
           <t>Observações</t>
+        </is>
+      </c>
+      <c r="T1" s="6" t="inlineStr">
+        <is>
+          <t>Citações (total)</t>
+        </is>
+      </c>
+      <c r="U1" s="6" t="inlineStr">
+        <is>
+          <t>Citações verificadas</t>
+        </is>
+      </c>
+      <c r="V1" s="6" t="inlineStr">
+        <is>
+          <t>Taxa verificável</t>
+        </is>
+      </c>
+      <c r="W1" s="6" t="inlineStr">
+        <is>
+          <t>Citações não verificadas</t>
         </is>
       </c>
     </row>
@@ -1618,6 +1642,13 @@
         <v/>
       </c>
       <c r="S2" s="8" t="n"/>
+      <c r="T2" s="8" t="n"/>
+      <c r="U2" s="8" t="n"/>
+      <c r="V2" s="11">
+        <f>IF(AND(ISNUMBER(T2),T2&gt;0),U2/T2,"")</f>
+        <v/>
+      </c>
+      <c r="W2" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -1657,6 +1688,13 @@
         <v/>
       </c>
       <c r="S3" s="8" t="n"/>
+      <c r="T3" s="8" t="n"/>
+      <c r="U3" s="8" t="n"/>
+      <c r="V3" s="11">
+        <f>IF(AND(ISNUMBER(T3),T3&gt;0),U3/T3,"")</f>
+        <v/>
+      </c>
+      <c r="W3" s="8" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -1696,6 +1734,13 @@
         <v/>
       </c>
       <c r="S4" s="8" t="n"/>
+      <c r="T4" s="8" t="n"/>
+      <c r="U4" s="8" t="n"/>
+      <c r="V4" s="11">
+        <f>IF(AND(ISNUMBER(T4),T4&gt;0),U4/T4,"")</f>
+        <v/>
+      </c>
+      <c r="W4" s="8" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -1735,6 +1780,13 @@
         <v/>
       </c>
       <c r="S5" s="8" t="n"/>
+      <c r="T5" s="8" t="n"/>
+      <c r="U5" s="8" t="n"/>
+      <c r="V5" s="11">
+        <f>IF(AND(ISNUMBER(T5),T5&gt;0),U5/T5,"")</f>
+        <v/>
+      </c>
+      <c r="W5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -1774,6 +1826,13 @@
         <v/>
       </c>
       <c r="S6" s="8" t="n"/>
+      <c r="T6" s="8" t="n"/>
+      <c r="U6" s="8" t="n"/>
+      <c r="V6" s="11">
+        <f>IF(AND(ISNUMBER(T6),T6&gt;0),U6/T6,"")</f>
+        <v/>
+      </c>
+      <c r="W6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -1813,6 +1872,13 @@
         <v/>
       </c>
       <c r="S7" s="8" t="n"/>
+      <c r="T7" s="8" t="n"/>
+      <c r="U7" s="8" t="n"/>
+      <c r="V7" s="11">
+        <f>IF(AND(ISNUMBER(T7),T7&gt;0),U7/T7,"")</f>
+        <v/>
+      </c>
+      <c r="W7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -1852,6 +1918,13 @@
         <v/>
       </c>
       <c r="S8" s="8" t="n"/>
+      <c r="T8" s="8" t="n"/>
+      <c r="U8" s="8" t="n"/>
+      <c r="V8" s="11">
+        <f>IF(AND(ISNUMBER(T8),T8&gt;0),U8/T8,"")</f>
+        <v/>
+      </c>
+      <c r="W8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -1891,6 +1964,13 @@
         <v/>
       </c>
       <c r="S9" s="8" t="n"/>
+      <c r="T9" s="8" t="n"/>
+      <c r="U9" s="8" t="n"/>
+      <c r="V9" s="11">
+        <f>IF(AND(ISNUMBER(T9),T9&gt;0),U9/T9,"")</f>
+        <v/>
+      </c>
+      <c r="W9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -1930,6 +2010,13 @@
         <v/>
       </c>
       <c r="S10" s="8" t="n"/>
+      <c r="T10" s="8" t="n"/>
+      <c r="U10" s="8" t="n"/>
+      <c r="V10" s="11">
+        <f>IF(AND(ISNUMBER(T10),T10&gt;0),U10/T10,"")</f>
+        <v/>
+      </c>
+      <c r="W10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -1969,6 +2056,13 @@
         <v/>
       </c>
       <c r="S11" s="8" t="n"/>
+      <c r="T11" s="8" t="n"/>
+      <c r="U11" s="8" t="n"/>
+      <c r="V11" s="11">
+        <f>IF(AND(ISNUMBER(T11),T11&gt;0),U11/T11,"")</f>
+        <v/>
+      </c>
+      <c r="W11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -2008,6 +2102,13 @@
         <v/>
       </c>
       <c r="S12" s="8" t="n"/>
+      <c r="T12" s="8" t="n"/>
+      <c r="U12" s="8" t="n"/>
+      <c r="V12" s="11">
+        <f>IF(AND(ISNUMBER(T12),T12&gt;0),U12/T12,"")</f>
+        <v/>
+      </c>
+      <c r="W12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -2047,6 +2148,13 @@
         <v/>
       </c>
       <c r="S13" s="8" t="n"/>
+      <c r="T13" s="8" t="n"/>
+      <c r="U13" s="8" t="n"/>
+      <c r="V13" s="11">
+        <f>IF(AND(ISNUMBER(T13),T13&gt;0),U13/T13,"")</f>
+        <v/>
+      </c>
+      <c r="W13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -2086,6 +2194,13 @@
         <v/>
       </c>
       <c r="S14" s="8" t="n"/>
+      <c r="T14" s="8" t="n"/>
+      <c r="U14" s="8" t="n"/>
+      <c r="V14" s="11">
+        <f>IF(AND(ISNUMBER(T14),T14&gt;0),U14/T14,"")</f>
+        <v/>
+      </c>
+      <c r="W14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -2125,6 +2240,13 @@
         <v/>
       </c>
       <c r="S15" s="8" t="n"/>
+      <c r="T15" s="8" t="n"/>
+      <c r="U15" s="8" t="n"/>
+      <c r="V15" s="11">
+        <f>IF(AND(ISNUMBER(T15),T15&gt;0),U15/T15,"")</f>
+        <v/>
+      </c>
+      <c r="W15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -2164,6 +2286,13 @@
         <v/>
       </c>
       <c r="S16" s="8" t="n"/>
+      <c r="T16" s="8" t="n"/>
+      <c r="U16" s="8" t="n"/>
+      <c r="V16" s="11">
+        <f>IF(AND(ISNUMBER(T16),T16&gt;0),U16/T16,"")</f>
+        <v/>
+      </c>
+      <c r="W16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -2203,6 +2332,13 @@
         <v/>
       </c>
       <c r="S17" s="8" t="n"/>
+      <c r="T17" s="8" t="n"/>
+      <c r="U17" s="8" t="n"/>
+      <c r="V17" s="11">
+        <f>IF(AND(ISNUMBER(T17),T17&gt;0),U17/T17,"")</f>
+        <v/>
+      </c>
+      <c r="W17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -2242,6 +2378,13 @@
         <v/>
       </c>
       <c r="S18" s="8" t="n"/>
+      <c r="T18" s="8" t="n"/>
+      <c r="U18" s="8" t="n"/>
+      <c r="V18" s="11">
+        <f>IF(AND(ISNUMBER(T18),T18&gt;0),U18/T18,"")</f>
+        <v/>
+      </c>
+      <c r="W18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -2281,6 +2424,13 @@
         <v/>
       </c>
       <c r="S19" s="8" t="n"/>
+      <c r="T19" s="8" t="n"/>
+      <c r="U19" s="8" t="n"/>
+      <c r="V19" s="11">
+        <f>IF(AND(ISNUMBER(T19),T19&gt;0),U19/T19,"")</f>
+        <v/>
+      </c>
+      <c r="W19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -2320,6 +2470,13 @@
         <v/>
       </c>
       <c r="S20" s="8" t="n"/>
+      <c r="T20" s="8" t="n"/>
+      <c r="U20" s="8" t="n"/>
+      <c r="V20" s="11">
+        <f>IF(AND(ISNUMBER(T20),T20&gt;0),U20/T20,"")</f>
+        <v/>
+      </c>
+      <c r="W20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -2359,6 +2516,13 @@
         <v/>
       </c>
       <c r="S21" s="8" t="n"/>
+      <c r="T21" s="8" t="n"/>
+      <c r="U21" s="8" t="n"/>
+      <c r="V21" s="11">
+        <f>IF(AND(ISNUMBER(T21),T21&gt;0),U21/T21,"")</f>
+        <v/>
+      </c>
+      <c r="W21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -2398,6 +2562,13 @@
         <v/>
       </c>
       <c r="S22" s="8" t="n"/>
+      <c r="T22" s="8" t="n"/>
+      <c r="U22" s="8" t="n"/>
+      <c r="V22" s="11">
+        <f>IF(AND(ISNUMBER(T22),T22&gt;0),U22/T22,"")</f>
+        <v/>
+      </c>
+      <c r="W22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
@@ -2437,6 +2608,13 @@
         <v/>
       </c>
       <c r="S23" s="8" t="n"/>
+      <c r="T23" s="8" t="n"/>
+      <c r="U23" s="8" t="n"/>
+      <c r="V23" s="11">
+        <f>IF(AND(ISNUMBER(T23),T23&gt;0),U23/T23,"")</f>
+        <v/>
+      </c>
+      <c r="W23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -2476,6 +2654,13 @@
         <v/>
       </c>
       <c r="S24" s="8" t="n"/>
+      <c r="T24" s="8" t="n"/>
+      <c r="U24" s="8" t="n"/>
+      <c r="V24" s="11">
+        <f>IF(AND(ISNUMBER(T24),T24&gt;0),U24/T24,"")</f>
+        <v/>
+      </c>
+      <c r="W24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
@@ -2515,6 +2700,13 @@
         <v/>
       </c>
       <c r="S25" s="8" t="n"/>
+      <c r="T25" s="8" t="n"/>
+      <c r="U25" s="8" t="n"/>
+      <c r="V25" s="11">
+        <f>IF(AND(ISNUMBER(T25),T25&gt;0),U25/T25,"")</f>
+        <v/>
+      </c>
+      <c r="W25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
@@ -2554,6 +2746,13 @@
         <v/>
       </c>
       <c r="S26" s="8" t="n"/>
+      <c r="T26" s="8" t="n"/>
+      <c r="U26" s="8" t="n"/>
+      <c r="V26" s="11">
+        <f>IF(AND(ISNUMBER(T26),T26&gt;0),U26/T26,"")</f>
+        <v/>
+      </c>
+      <c r="W26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
@@ -2593,6 +2792,13 @@
         <v/>
       </c>
       <c r="S27" s="8" t="n"/>
+      <c r="T27" s="8" t="n"/>
+      <c r="U27" s="8" t="n"/>
+      <c r="V27" s="11">
+        <f>IF(AND(ISNUMBER(T27),T27&gt;0),U27/T27,"")</f>
+        <v/>
+      </c>
+      <c r="W27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
@@ -2632,6 +2838,13 @@
         <v/>
       </c>
       <c r="S28" s="8" t="n"/>
+      <c r="T28" s="8" t="n"/>
+      <c r="U28" s="8" t="n"/>
+      <c r="V28" s="11">
+        <f>IF(AND(ISNUMBER(T28),T28&gt;0),U28/T28,"")</f>
+        <v/>
+      </c>
+      <c r="W28" s="8" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
@@ -2671,6 +2884,13 @@
         <v/>
       </c>
       <c r="S29" s="8" t="n"/>
+      <c r="T29" s="8" t="n"/>
+      <c r="U29" s="8" t="n"/>
+      <c r="V29" s="11">
+        <f>IF(AND(ISNUMBER(T29),T29&gt;0),U29/T29,"")</f>
+        <v/>
+      </c>
+      <c r="W29" s="8" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
@@ -2710,6 +2930,13 @@
         <v/>
       </c>
       <c r="S30" s="8" t="n"/>
+      <c r="T30" s="8" t="n"/>
+      <c r="U30" s="8" t="n"/>
+      <c r="V30" s="11">
+        <f>IF(AND(ISNUMBER(T30),T30&gt;0),U30/T30,"")</f>
+        <v/>
+      </c>
+      <c r="W30" s="8" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
@@ -2749,6 +2976,13 @@
         <v/>
       </c>
       <c r="S31" s="8" t="n"/>
+      <c r="T31" s="8" t="n"/>
+      <c r="U31" s="8" t="n"/>
+      <c r="V31" s="11">
+        <f>IF(AND(ISNUMBER(T31),T31&gt;0),U31/T31,"")</f>
+        <v/>
+      </c>
+      <c r="W31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
@@ -2788,6 +3022,13 @@
         <v/>
       </c>
       <c r="S32" s="8" t="n"/>
+      <c r="T32" s="8" t="n"/>
+      <c r="U32" s="8" t="n"/>
+      <c r="V32" s="11">
+        <f>IF(AND(ISNUMBER(T32),T32&gt;0),U32/T32,"")</f>
+        <v/>
+      </c>
+      <c r="W32" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
@@ -2827,6 +3068,13 @@
         <v/>
       </c>
       <c r="S33" s="8" t="n"/>
+      <c r="T33" s="8" t="n"/>
+      <c r="U33" s="8" t="n"/>
+      <c r="V33" s="11">
+        <f>IF(AND(ISNUMBER(T33),T33&gt;0),U33/T33,"")</f>
+        <v/>
+      </c>
+      <c r="W33" s="8" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
@@ -2866,6 +3114,13 @@
         <v/>
       </c>
       <c r="S34" s="8" t="n"/>
+      <c r="T34" s="8" t="n"/>
+      <c r="U34" s="8" t="n"/>
+      <c r="V34" s="11">
+        <f>IF(AND(ISNUMBER(T34),T34&gt;0),U34/T34,"")</f>
+        <v/>
+      </c>
+      <c r="W34" s="8" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
@@ -2905,6 +3160,13 @@
         <v/>
       </c>
       <c r="S35" s="8" t="n"/>
+      <c r="T35" s="8" t="n"/>
+      <c r="U35" s="8" t="n"/>
+      <c r="V35" s="11">
+        <f>IF(AND(ISNUMBER(T35),T35&gt;0),U35/T35,"")</f>
+        <v/>
+      </c>
+      <c r="W35" s="8" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
@@ -2944,6 +3206,13 @@
         <v/>
       </c>
       <c r="S36" s="8" t="n"/>
+      <c r="T36" s="8" t="n"/>
+      <c r="U36" s="8" t="n"/>
+      <c r="V36" s="11">
+        <f>IF(AND(ISNUMBER(T36),T36&gt;0),U36/T36,"")</f>
+        <v/>
+      </c>
+      <c r="W36" s="8" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n">
@@ -2983,6 +3252,13 @@
         <v/>
       </c>
       <c r="S37" s="8" t="n"/>
+      <c r="T37" s="8" t="n"/>
+      <c r="U37" s="8" t="n"/>
+      <c r="V37" s="11">
+        <f>IF(AND(ISNUMBER(T37),T37&gt;0),U37/T37,"")</f>
+        <v/>
+      </c>
+      <c r="W37" s="8" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n">
@@ -3022,6 +3298,13 @@
         <v/>
       </c>
       <c r="S38" s="8" t="n"/>
+      <c r="T38" s="8" t="n"/>
+      <c r="U38" s="8" t="n"/>
+      <c r="V38" s="11">
+        <f>IF(AND(ISNUMBER(T38),T38&gt;0),U38/T38,"")</f>
+        <v/>
+      </c>
+      <c r="W38" s="8" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n">
@@ -3061,6 +3344,13 @@
         <v/>
       </c>
       <c r="S39" s="8" t="n"/>
+      <c r="T39" s="8" t="n"/>
+      <c r="U39" s="8" t="n"/>
+      <c r="V39" s="11">
+        <f>IF(AND(ISNUMBER(T39),T39&gt;0),U39/T39,"")</f>
+        <v/>
+      </c>
+      <c r="W39" s="8" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n">
@@ -3100,6 +3390,13 @@
         <v/>
       </c>
       <c r="S40" s="8" t="n"/>
+      <c r="T40" s="8" t="n"/>
+      <c r="U40" s="8" t="n"/>
+      <c r="V40" s="11">
+        <f>IF(AND(ISNUMBER(T40),T40&gt;0),U40/T40,"")</f>
+        <v/>
+      </c>
+      <c r="W40" s="8" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="n">
@@ -3139,6 +3436,13 @@
         <v/>
       </c>
       <c r="S41" s="8" t="n"/>
+      <c r="T41" s="8" t="n"/>
+      <c r="U41" s="8" t="n"/>
+      <c r="V41" s="11">
+        <f>IF(AND(ISNUMBER(T41),T41&gt;0),U41/T41,"")</f>
+        <v/>
+      </c>
+      <c r="W41" s="8" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n">
@@ -3178,6 +3482,13 @@
         <v/>
       </c>
       <c r="S42" s="8" t="n"/>
+      <c r="T42" s="8" t="n"/>
+      <c r="U42" s="8" t="n"/>
+      <c r="V42" s="11">
+        <f>IF(AND(ISNUMBER(T42),T42&gt;0),U42/T42,"")</f>
+        <v/>
+      </c>
+      <c r="W42" s="8" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="n">
@@ -3217,6 +3528,13 @@
         <v/>
       </c>
       <c r="S43" s="8" t="n"/>
+      <c r="T43" s="8" t="n"/>
+      <c r="U43" s="8" t="n"/>
+      <c r="V43" s="11">
+        <f>IF(AND(ISNUMBER(T43),T43&gt;0),U43/T43,"")</f>
+        <v/>
+      </c>
+      <c r="W43" s="8" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
@@ -3256,6 +3574,13 @@
         <v/>
       </c>
       <c r="S44" s="8" t="n"/>
+      <c r="T44" s="8" t="n"/>
+      <c r="U44" s="8" t="n"/>
+      <c r="V44" s="11">
+        <f>IF(AND(ISNUMBER(T44),T44&gt;0),U44/T44,"")</f>
+        <v/>
+      </c>
+      <c r="W44" s="8" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n">
@@ -3295,6 +3620,13 @@
         <v/>
       </c>
       <c r="S45" s="8" t="n"/>
+      <c r="T45" s="8" t="n"/>
+      <c r="U45" s="8" t="n"/>
+      <c r="V45" s="11">
+        <f>IF(AND(ISNUMBER(T45),T45&gt;0),U45/T45,"")</f>
+        <v/>
+      </c>
+      <c r="W45" s="8" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n">
@@ -3334,6 +3666,13 @@
         <v/>
       </c>
       <c r="S46" s="8" t="n"/>
+      <c r="T46" s="8" t="n"/>
+      <c r="U46" s="8" t="n"/>
+      <c r="V46" s="11">
+        <f>IF(AND(ISNUMBER(T46),T46&gt;0),U46/T46,"")</f>
+        <v/>
+      </c>
+      <c r="W46" s="8" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="n">
@@ -3373,6 +3712,13 @@
         <v/>
       </c>
       <c r="S47" s="8" t="n"/>
+      <c r="T47" s="8" t="n"/>
+      <c r="U47" s="8" t="n"/>
+      <c r="V47" s="11">
+        <f>IF(AND(ISNUMBER(T47),T47&gt;0),U47/T47,"")</f>
+        <v/>
+      </c>
+      <c r="W47" s="8" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n">
@@ -3412,6 +3758,13 @@
         <v/>
       </c>
       <c r="S48" s="8" t="n"/>
+      <c r="T48" s="8" t="n"/>
+      <c r="U48" s="8" t="n"/>
+      <c r="V48" s="11">
+        <f>IF(AND(ISNUMBER(T48),T48&gt;0),U48/T48,"")</f>
+        <v/>
+      </c>
+      <c r="W48" s="8" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="n">
@@ -3451,6 +3804,13 @@
         <v/>
       </c>
       <c r="S49" s="8" t="n"/>
+      <c r="T49" s="8" t="n"/>
+      <c r="U49" s="8" t="n"/>
+      <c r="V49" s="11">
+        <f>IF(AND(ISNUMBER(T49),T49&gt;0),U49/T49,"")</f>
+        <v/>
+      </c>
+      <c r="W49" s="8" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="n">
@@ -3490,6 +3850,13 @@
         <v/>
       </c>
       <c r="S50" s="8" t="n"/>
+      <c r="T50" s="8" t="n"/>
+      <c r="U50" s="8" t="n"/>
+      <c r="V50" s="11">
+        <f>IF(AND(ISNUMBER(T50),T50&gt;0),U50/T50,"")</f>
+        <v/>
+      </c>
+      <c r="W50" s="8" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="n">
@@ -3529,6 +3896,13 @@
         <v/>
       </c>
       <c r="S51" s="8" t="n"/>
+      <c r="T51" s="8" t="n"/>
+      <c r="U51" s="8" t="n"/>
+      <c r="V51" s="11">
+        <f>IF(AND(ISNUMBER(T51),T51&gt;0),U51/T51,"")</f>
+        <v/>
+      </c>
+      <c r="W51" s="8" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n">
@@ -3568,6 +3942,13 @@
         <v/>
       </c>
       <c r="S52" s="8" t="n"/>
+      <c r="T52" s="8" t="n"/>
+      <c r="U52" s="8" t="n"/>
+      <c r="V52" s="11">
+        <f>IF(AND(ISNUMBER(T52),T52&gt;0),U52/T52,"")</f>
+        <v/>
+      </c>
+      <c r="W52" s="8" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="n">
@@ -3607,6 +3988,13 @@
         <v/>
       </c>
       <c r="S53" s="8" t="n"/>
+      <c r="T53" s="8" t="n"/>
+      <c r="U53" s="8" t="n"/>
+      <c r="V53" s="11">
+        <f>IF(AND(ISNUMBER(T53),T53&gt;0),U53/T53,"")</f>
+        <v/>
+      </c>
+      <c r="W53" s="8" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="n">
@@ -3646,6 +4034,13 @@
         <v/>
       </c>
       <c r="S54" s="8" t="n"/>
+      <c r="T54" s="8" t="n"/>
+      <c r="U54" s="8" t="n"/>
+      <c r="V54" s="11">
+        <f>IF(AND(ISNUMBER(T54),T54&gt;0),U54/T54,"")</f>
+        <v/>
+      </c>
+      <c r="W54" s="8" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="n">
@@ -3685,6 +4080,13 @@
         <v/>
       </c>
       <c r="S55" s="8" t="n"/>
+      <c r="T55" s="8" t="n"/>
+      <c r="U55" s="8" t="n"/>
+      <c r="V55" s="11">
+        <f>IF(AND(ISNUMBER(T55),T55&gt;0),U55/T55,"")</f>
+        <v/>
+      </c>
+      <c r="W55" s="8" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="n">
@@ -3724,6 +4126,13 @@
         <v/>
       </c>
       <c r="S56" s="8" t="n"/>
+      <c r="T56" s="8" t="n"/>
+      <c r="U56" s="8" t="n"/>
+      <c r="V56" s="11">
+        <f>IF(AND(ISNUMBER(T56),T56&gt;0),U56/T56,"")</f>
+        <v/>
+      </c>
+      <c r="W56" s="8" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="n">
@@ -3763,6 +4172,13 @@
         <v/>
       </c>
       <c r="S57" s="8" t="n"/>
+      <c r="T57" s="8" t="n"/>
+      <c r="U57" s="8" t="n"/>
+      <c r="V57" s="11">
+        <f>IF(AND(ISNUMBER(T57),T57&gt;0),U57/T57,"")</f>
+        <v/>
+      </c>
+      <c r="W57" s="8" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="n">
@@ -3802,6 +4218,13 @@
         <v/>
       </c>
       <c r="S58" s="8" t="n"/>
+      <c r="T58" s="8" t="n"/>
+      <c r="U58" s="8" t="n"/>
+      <c r="V58" s="11">
+        <f>IF(AND(ISNUMBER(T58),T58&gt;0),U58/T58,"")</f>
+        <v/>
+      </c>
+      <c r="W58" s="8" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="n">
@@ -3841,6 +4264,13 @@
         <v/>
       </c>
       <c r="S59" s="8" t="n"/>
+      <c r="T59" s="8" t="n"/>
+      <c r="U59" s="8" t="n"/>
+      <c r="V59" s="11">
+        <f>IF(AND(ISNUMBER(T59),T59&gt;0),U59/T59,"")</f>
+        <v/>
+      </c>
+      <c r="W59" s="8" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="n">
@@ -3880,6 +4310,13 @@
         <v/>
       </c>
       <c r="S60" s="8" t="n"/>
+      <c r="T60" s="8" t="n"/>
+      <c r="U60" s="8" t="n"/>
+      <c r="V60" s="11">
+        <f>IF(AND(ISNUMBER(T60),T60&gt;0),U60/T60,"")</f>
+        <v/>
+      </c>
+      <c r="W60" s="8" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="n">
@@ -3919,6 +4356,13 @@
         <v/>
       </c>
       <c r="S61" s="8" t="n"/>
+      <c r="T61" s="8" t="n"/>
+      <c r="U61" s="8" t="n"/>
+      <c r="V61" s="11">
+        <f>IF(AND(ISNUMBER(T61),T61&gt;0),U61/T61,"")</f>
+        <v/>
+      </c>
+      <c r="W61" s="8" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="n">
@@ -3958,6 +4402,13 @@
         <v/>
       </c>
       <c r="S62" s="8" t="n"/>
+      <c r="T62" s="8" t="n"/>
+      <c r="U62" s="8" t="n"/>
+      <c r="V62" s="11">
+        <f>IF(AND(ISNUMBER(T62),T62&gt;0),U62/T62,"")</f>
+        <v/>
+      </c>
+      <c r="W62" s="8" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="n">
@@ -3997,6 +4448,13 @@
         <v/>
       </c>
       <c r="S63" s="8" t="n"/>
+      <c r="T63" s="8" t="n"/>
+      <c r="U63" s="8" t="n"/>
+      <c r="V63" s="11">
+        <f>IF(AND(ISNUMBER(T63),T63&gt;0),U63/T63,"")</f>
+        <v/>
+      </c>
+      <c r="W63" s="8" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="n">
@@ -4036,6 +4494,13 @@
         <v/>
       </c>
       <c r="S64" s="8" t="n"/>
+      <c r="T64" s="8" t="n"/>
+      <c r="U64" s="8" t="n"/>
+      <c r="V64" s="11">
+        <f>IF(AND(ISNUMBER(T64),T64&gt;0),U64/T64,"")</f>
+        <v/>
+      </c>
+      <c r="W64" s="8" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="n">
@@ -4075,6 +4540,13 @@
         <v/>
       </c>
       <c r="S65" s="8" t="n"/>
+      <c r="T65" s="8" t="n"/>
+      <c r="U65" s="8" t="n"/>
+      <c r="V65" s="11">
+        <f>IF(AND(ISNUMBER(T65),T65&gt;0),U65/T65,"")</f>
+        <v/>
+      </c>
+      <c r="W65" s="8" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="n">
@@ -4114,6 +4586,13 @@
         <v/>
       </c>
       <c r="S66" s="8" t="n"/>
+      <c r="T66" s="8" t="n"/>
+      <c r="U66" s="8" t="n"/>
+      <c r="V66" s="11">
+        <f>IF(AND(ISNUMBER(T66),T66&gt;0),U66/T66,"")</f>
+        <v/>
+      </c>
+      <c r="W66" s="8" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="n">
@@ -4153,6 +4632,13 @@
         <v/>
       </c>
       <c r="S67" s="8" t="n"/>
+      <c r="T67" s="8" t="n"/>
+      <c r="U67" s="8" t="n"/>
+      <c r="V67" s="11">
+        <f>IF(AND(ISNUMBER(T67),T67&gt;0),U67/T67,"")</f>
+        <v/>
+      </c>
+      <c r="W67" s="8" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="n">
@@ -4192,6 +4678,13 @@
         <v/>
       </c>
       <c r="S68" s="8" t="n"/>
+      <c r="T68" s="8" t="n"/>
+      <c r="U68" s="8" t="n"/>
+      <c r="V68" s="11">
+        <f>IF(AND(ISNUMBER(T68),T68&gt;0),U68/T68,"")</f>
+        <v/>
+      </c>
+      <c r="W68" s="8" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="n">
@@ -4231,6 +4724,13 @@
         <v/>
       </c>
       <c r="S69" s="8" t="n"/>
+      <c r="T69" s="8" t="n"/>
+      <c r="U69" s="8" t="n"/>
+      <c r="V69" s="11">
+        <f>IF(AND(ISNUMBER(T69),T69&gt;0),U69/T69,"")</f>
+        <v/>
+      </c>
+      <c r="W69" s="8" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="n">
@@ -4270,6 +4770,13 @@
         <v/>
       </c>
       <c r="S70" s="8" t="n"/>
+      <c r="T70" s="8" t="n"/>
+      <c r="U70" s="8" t="n"/>
+      <c r="V70" s="11">
+        <f>IF(AND(ISNUMBER(T70),T70&gt;0),U70/T70,"")</f>
+        <v/>
+      </c>
+      <c r="W70" s="8" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="n">
@@ -4309,6 +4816,13 @@
         <v/>
       </c>
       <c r="S71" s="8" t="n"/>
+      <c r="T71" s="8" t="n"/>
+      <c r="U71" s="8" t="n"/>
+      <c r="V71" s="11">
+        <f>IF(AND(ISNUMBER(T71),T71&gt;0),U71/T71,"")</f>
+        <v/>
+      </c>
+      <c r="W71" s="8" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="n">
@@ -4348,6 +4862,13 @@
         <v/>
       </c>
       <c r="S72" s="8" t="n"/>
+      <c r="T72" s="8" t="n"/>
+      <c r="U72" s="8" t="n"/>
+      <c r="V72" s="11">
+        <f>IF(AND(ISNUMBER(T72),T72&gt;0),U72/T72,"")</f>
+        <v/>
+      </c>
+      <c r="W72" s="8" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="n">
@@ -4387,6 +4908,13 @@
         <v/>
       </c>
       <c r="S73" s="8" t="n"/>
+      <c r="T73" s="8" t="n"/>
+      <c r="U73" s="8" t="n"/>
+      <c r="V73" s="11">
+        <f>IF(AND(ISNUMBER(T73),T73&gt;0),U73/T73,"")</f>
+        <v/>
+      </c>
+      <c r="W73" s="8" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="n">
@@ -4426,6 +4954,13 @@
         <v/>
       </c>
       <c r="S74" s="8" t="n"/>
+      <c r="T74" s="8" t="n"/>
+      <c r="U74" s="8" t="n"/>
+      <c r="V74" s="11">
+        <f>IF(AND(ISNUMBER(T74),T74&gt;0),U74/T74,"")</f>
+        <v/>
+      </c>
+      <c r="W74" s="8" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="n">
@@ -4465,6 +5000,13 @@
         <v/>
       </c>
       <c r="S75" s="8" t="n"/>
+      <c r="T75" s="8" t="n"/>
+      <c r="U75" s="8" t="n"/>
+      <c r="V75" s="11">
+        <f>IF(AND(ISNUMBER(T75),T75&gt;0),U75/T75,"")</f>
+        <v/>
+      </c>
+      <c r="W75" s="8" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="n">
@@ -4504,6 +5046,13 @@
         <v/>
       </c>
       <c r="S76" s="8" t="n"/>
+      <c r="T76" s="8" t="n"/>
+      <c r="U76" s="8" t="n"/>
+      <c r="V76" s="11">
+        <f>IF(AND(ISNUMBER(T76),T76&gt;0),U76/T76,"")</f>
+        <v/>
+      </c>
+      <c r="W76" s="8" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="n">
@@ -4565,6 +5114,13 @@
         <v/>
       </c>
       <c r="S77" s="8" t="n"/>
+      <c r="T77" s="8" t="n"/>
+      <c r="U77" s="8" t="n"/>
+      <c r="V77" s="11">
+        <f>IF(AND(ISNUMBER(T77),T77&gt;0),U77/T77,"")</f>
+        <v/>
+      </c>
+      <c r="W77" s="8" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="n">
@@ -4626,6 +5182,13 @@
         <v/>
       </c>
       <c r="S78" s="8" t="n"/>
+      <c r="T78" s="8" t="n"/>
+      <c r="U78" s="8" t="n"/>
+      <c r="V78" s="11">
+        <f>IF(AND(ISNUMBER(T78),T78&gt;0),U78/T78,"")</f>
+        <v/>
+      </c>
+      <c r="W78" s="8" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="n">
@@ -4687,6 +5250,13 @@
         <v/>
       </c>
       <c r="S79" s="8" t="n"/>
+      <c r="T79" s="8" t="n"/>
+      <c r="U79" s="8" t="n"/>
+      <c r="V79" s="11">
+        <f>IF(AND(ISNUMBER(T79),T79&gt;0),U79/T79,"")</f>
+        <v/>
+      </c>
+      <c r="W79" s="8" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="n">
@@ -4748,6 +5318,13 @@
         <v/>
       </c>
       <c r="S80" s="8" t="n"/>
+      <c r="T80" s="8" t="n"/>
+      <c r="U80" s="8" t="n"/>
+      <c r="V80" s="11">
+        <f>IF(AND(ISNUMBER(T80),T80&gt;0),U80/T80,"")</f>
+        <v/>
+      </c>
+      <c r="W80" s="8" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="n">
@@ -4809,6 +5386,13 @@
         <v/>
       </c>
       <c r="S81" s="8" t="n"/>
+      <c r="T81" s="8" t="n"/>
+      <c r="U81" s="8" t="n"/>
+      <c r="V81" s="11">
+        <f>IF(AND(ISNUMBER(T81),T81&gt;0),U81/T81,"")</f>
+        <v/>
+      </c>
+      <c r="W81" s="8" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="n">
@@ -4870,6 +5454,13 @@
         <v/>
       </c>
       <c r="S82" s="8" t="n"/>
+      <c r="T82" s="8" t="n"/>
+      <c r="U82" s="8" t="n"/>
+      <c r="V82" s="11">
+        <f>IF(AND(ISNUMBER(T82),T82&gt;0),U82/T82,"")</f>
+        <v/>
+      </c>
+      <c r="W82" s="8" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="n">
@@ -4931,6 +5522,13 @@
         <v/>
       </c>
       <c r="S83" s="8" t="n"/>
+      <c r="T83" s="8" t="n"/>
+      <c r="U83" s="8" t="n"/>
+      <c r="V83" s="11">
+        <f>IF(AND(ISNUMBER(T83),T83&gt;0),U83/T83,"")</f>
+        <v/>
+      </c>
+      <c r="W83" s="8" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="n">
@@ -4992,6 +5590,13 @@
         <v/>
       </c>
       <c r="S84" s="8" t="n"/>
+      <c r="T84" s="8" t="n"/>
+      <c r="U84" s="8" t="n"/>
+      <c r="V84" s="11">
+        <f>IF(AND(ISNUMBER(T84),T84&gt;0),U84/T84,"")</f>
+        <v/>
+      </c>
+      <c r="W84" s="8" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="n">
@@ -5074,6 +5679,13 @@
         <v/>
       </c>
       <c r="S85" s="8" t="n"/>
+      <c r="T85" s="8" t="n"/>
+      <c r="U85" s="8" t="n"/>
+      <c r="V85" s="11">
+        <f>IF(AND(ISNUMBER(T85),T85&gt;0),U85/T85,"")</f>
+        <v/>
+      </c>
+      <c r="W85" s="8" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="n">
@@ -5135,6 +5747,13 @@
         <v/>
       </c>
       <c r="S86" s="8" t="n"/>
+      <c r="T86" s="8" t="n"/>
+      <c r="U86" s="8" t="n"/>
+      <c r="V86" s="11">
+        <f>IF(AND(ISNUMBER(T86),T86&gt;0),U86/T86,"")</f>
+        <v/>
+      </c>
+      <c r="W86" s="8" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="n">
@@ -5196,6 +5815,13 @@
         <v/>
       </c>
       <c r="S87" s="8" t="n"/>
+      <c r="T87" s="8" t="n"/>
+      <c r="U87" s="8" t="n"/>
+      <c r="V87" s="11">
+        <f>IF(AND(ISNUMBER(T87),T87&gt;0),U87/T87,"")</f>
+        <v/>
+      </c>
+      <c r="W87" s="8" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="n">
@@ -5257,6 +5883,13 @@
         <v/>
       </c>
       <c r="S88" s="8" t="n"/>
+      <c r="T88" s="8" t="n"/>
+      <c r="U88" s="8" t="n"/>
+      <c r="V88" s="11">
+        <f>IF(AND(ISNUMBER(T88),T88&gt;0),U88/T88,"")</f>
+        <v/>
+      </c>
+      <c r="W88" s="8" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="n">
@@ -5318,6 +5951,13 @@
         <v/>
       </c>
       <c r="S89" s="8" t="n"/>
+      <c r="T89" s="8" t="n"/>
+      <c r="U89" s="8" t="n"/>
+      <c r="V89" s="11">
+        <f>IF(AND(ISNUMBER(T89),T89&gt;0),U89/T89,"")</f>
+        <v/>
+      </c>
+      <c r="W89" s="8" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="n">
@@ -5379,6 +6019,13 @@
         <v/>
       </c>
       <c r="S90" s="8" t="n"/>
+      <c r="T90" s="8" t="n"/>
+      <c r="U90" s="8" t="n"/>
+      <c r="V90" s="11">
+        <f>IF(AND(ISNUMBER(T90),T90&gt;0),U90/T90,"")</f>
+        <v/>
+      </c>
+      <c r="W90" s="8" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="n">
@@ -5449,6 +6096,13 @@
         <v/>
       </c>
       <c r="S91" s="8" t="n"/>
+      <c r="T91" s="8" t="n"/>
+      <c r="U91" s="8" t="n"/>
+      <c r="V91" s="11">
+        <f>IF(AND(ISNUMBER(T91),T91&gt;0),U91/T91,"")</f>
+        <v/>
+      </c>
+      <c r="W91" s="8" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="n">
@@ -5510,6 +6164,13 @@
         <v/>
       </c>
       <c r="S92" s="8" t="n"/>
+      <c r="T92" s="8" t="n"/>
+      <c r="U92" s="8" t="n"/>
+      <c r="V92" s="11">
+        <f>IF(AND(ISNUMBER(T92),T92&gt;0),U92/T92,"")</f>
+        <v/>
+      </c>
+      <c r="W92" s="8" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="n">
@@ -5571,6 +6232,13 @@
         <v/>
       </c>
       <c r="S93" s="8" t="n"/>
+      <c r="T93" s="8" t="n"/>
+      <c r="U93" s="8" t="n"/>
+      <c r="V93" s="11">
+        <f>IF(AND(ISNUMBER(T93),T93&gt;0),U93/T93,"")</f>
+        <v/>
+      </c>
+      <c r="W93" s="8" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="n">
@@ -5632,6 +6300,13 @@
         <v/>
       </c>
       <c r="S94" s="8" t="n"/>
+      <c r="T94" s="8" t="n"/>
+      <c r="U94" s="8" t="n"/>
+      <c r="V94" s="11">
+        <f>IF(AND(ISNUMBER(T94),T94&gt;0),U94/T94,"")</f>
+        <v/>
+      </c>
+      <c r="W94" s="8" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="n">
@@ -5696,6 +6371,13 @@
         <v/>
       </c>
       <c r="S95" s="8" t="n"/>
+      <c r="T95" s="8" t="n"/>
+      <c r="U95" s="8" t="n"/>
+      <c r="V95" s="11">
+        <f>IF(AND(ISNUMBER(T95),T95&gt;0),U95/T95,"")</f>
+        <v/>
+      </c>
+      <c r="W95" s="8" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="n">
@@ -5775,6 +6457,13 @@
         <v/>
       </c>
       <c r="S96" s="8" t="n"/>
+      <c r="T96" s="8" t="n"/>
+      <c r="U96" s="8" t="n"/>
+      <c r="V96" s="11">
+        <f>IF(AND(ISNUMBER(T96),T96&gt;0),U96/T96,"")</f>
+        <v/>
+      </c>
+      <c r="W96" s="8" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="n">
@@ -5836,6 +6525,13 @@
         <v/>
       </c>
       <c r="S97" s="8" t="n"/>
+      <c r="T97" s="8" t="n"/>
+      <c r="U97" s="8" t="n"/>
+      <c r="V97" s="11">
+        <f>IF(AND(ISNUMBER(T97),T97&gt;0),U97/T97,"")</f>
+        <v/>
+      </c>
+      <c r="W97" s="8" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="n">
@@ -5912,6 +6608,13 @@
         <v/>
       </c>
       <c r="S98" s="8" t="n"/>
+      <c r="T98" s="8" t="n"/>
+      <c r="U98" s="8" t="n"/>
+      <c r="V98" s="11">
+        <f>IF(AND(ISNUMBER(T98),T98&gt;0),U98/T98,"")</f>
+        <v/>
+      </c>
+      <c r="W98" s="8" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="n">
@@ -5973,6 +6676,13 @@
         <v/>
       </c>
       <c r="S99" s="8" t="n"/>
+      <c r="T99" s="8" t="n"/>
+      <c r="U99" s="8" t="n"/>
+      <c r="V99" s="11">
+        <f>IF(AND(ISNUMBER(T99),T99&gt;0),U99/T99,"")</f>
+        <v/>
+      </c>
+      <c r="W99" s="8" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="n">
@@ -6034,6 +6744,13 @@
         <v/>
       </c>
       <c r="S100" s="8" t="n"/>
+      <c r="T100" s="8" t="n"/>
+      <c r="U100" s="8" t="n"/>
+      <c r="V100" s="11">
+        <f>IF(AND(ISNUMBER(T100),T100&gt;0),U100/T100,"")</f>
+        <v/>
+      </c>
+      <c r="W100" s="8" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="n">
@@ -6095,6 +6812,13 @@
         <v/>
       </c>
       <c r="S101" s="8" t="n"/>
+      <c r="T101" s="8" t="n"/>
+      <c r="U101" s="8" t="n"/>
+      <c r="V101" s="11">
+        <f>IF(AND(ISNUMBER(T101),T101&gt;0),U101/T101,"")</f>
+        <v/>
+      </c>
+      <c r="W101" s="8" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="n">
@@ -6115,42 +6839,49 @@
       </c>
       <c r="E102" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F102" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G102" s="8" t="inlineStr">
         <is>
-          <t>**Não.**  
-A emissão de certidão de inteiro teor a pedido de terceiro — pessoa sem vínculo com o registrado— está condicionada a requisitos específicos previstos no **Provimento CNJ 149/2023**.
-- **Art. 114.** As certidões de registro civil, inclusive as de inteiro teor, **só podem ser expedidas a terceiros** quando contiverem dados sensíveis **mediante autorização do juízo competente**.  
-- **§ 1.º** do mesmo artigo deixa claro que, na hipótese de solicitação por terceiros, **é obrigatória a autorização judicial** quando a certidão envolver informações sensíveis.  
-Além disso, o requerimento deve observar as exigências de forma escrita:
-- **Art. 117** (e **Art. 258**) estabelecem que o requerimento **deve conter**:
-  - identificação do requerente;  
-  - **motivo** da solicitação;  
-  - grau de parentesco com o registrado, se houver;  
-  - informação sobre eventual falecimento do titular.  
-Portanto, **não é possível emitir a certidão de inteiro teor a um terceiro sem exigir a indicação do motivo** (e, quando houver dados sensíveis, a devida autorização judicial).</t>
+          <t>**Resposta:** Deve‑se praticar o ato registral de forma integral, emitindo a certidão de inteiro teor sem exigir a apresentação de motivo ou justificativa por parte do requerente.
+**Fundamentação normativa**
+1. **Lei 6.015/1973 – Art. 19, §§ 11 e 12**  
+   &gt; “§ 11. No âmbito do registro de imóveis, a certidão de inteiro teor da matrícula conterá a reprodução de todo seu conteúdo e será suficiente para fins de comprovação de propriedade, direitos, ônus reais e restrições sobre o imóvel….”  
+   &gt; “§ 12. Na localidade em que haja dificuldade de comunicação eletrônica, a Corregedoria‑Geral da Justiça Estadual poderá autorizar, de modo excepcional…”.
+   O dispositivo estabelece a obrigatoriedade da certidão de inteiro teor e não impõe a necessidade de justificativa para a sua expedição.
+2. **Código de Normas da CGJ‑CE – Art. 1131, §§ 1º e 2º**  
+   &gt; “§ 1º Ao receber o pedido de certidão, o Oficial fornecerá, obrigatoriamente, ao requerente protocolo… e o prazo para a entrega do documento que não poderá exceder a 05 (cinco) dias úteis….”  
+   &gt; “§ 2º A certidão será lavrada em inteiro teor, em resumo ou em relatório, conforme quesitos, e devidamente autenticada… não podendo ser retardada por mais de 5 (cinco) dias úteis.”
+   Não há exigência de motivação do requerente; basta o pedido formal e a indicação do número da matrícula.
+3. **Provimento CNJ 149/2023 – Art. 327**  
+   &gt; “A certidão de inteiro teor digital solicitada durante o horário de expediente, com indicação do número da matrícula… será emitida e disponibilizada dentro de no máximo 2 (duas) horas…”.
+   O provimento regulamenta o prazo de emissão, confirmando que o requerimento pode ser atendido imediatamente, independentemente de motivo.
+**Conclusão prática**
+- **Ato registral:** Emissão integral da certidão de inteiro teor.  
+- **Condição:** Nenhuma exigência de motivação ou vínculo do requerente.  
+- **Procedimento:** Registrar o pedido, gerar o protocolo (Art. 1131, § 1º), observar o prazo máximo de 5 (cinco) dias úteis ou 2 (duas) horas para a versão digital (Art. 327), e disponibilizar a certidão ao requerente.  
+Portanto, a certidão pode ser emitida sem exigir motivo.</t>
         </is>
       </c>
       <c r="H102" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 471:p116; Provimento CNJ 149/2023, Art. 117:p55; Código de Normas CGJ-CE, Art. 258:p78; Provimento CNJ 149/2023, Art. 327:p209; Provimento CNJ 149/2023, Art. 114:p54</t>
+          <t>Lei 6.015/1973 — Art. 19:p0; Código de Normas CGJ-CE — Art. 1131:p229; Provimento CNJ 149/2023 — Art. 327:p209; Provimento CNJ 149/2023 — Art. 200:p94</t>
         </is>
       </c>
       <c r="I102" s="8" t="n">
-        <v>3.91</v>
+        <v>2.73</v>
       </c>
       <c r="J102" s="8" t="n">
-        <v>2231</v>
+        <v>1738</v>
       </c>
       <c r="K102" s="8" t="n">
-        <v>559</v>
+        <v>814</v>
       </c>
       <c r="L102" s="10">
         <f>IF(COUNT(J102:K102)=2,(J102*Parametros!$B$3+K102*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6166,6 +6897,17 @@
         <v/>
       </c>
       <c r="S102" s="8" t="n"/>
+      <c r="T102" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="U102" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="V102" s="11">
+        <f>IF(AND(ISNUMBER(T102),T102&gt;0),U102/T102,"")</f>
+        <v/>
+      </c>
+      <c r="W102" s="8" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="n">
@@ -6186,32 +6928,39 @@
       </c>
       <c r="E103" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F103" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G103" s="8" t="inlineStr">
         <is>
-          <t>Não encontrado no corpus.</t>
+          <t>**Resposta Jurídica e Operacional**
+A certidão de inteiro teor **não** é obrigada a exibir o CPF completo dos proprietários.
+**Fundamentação normativa**
+- **Código de Normas CGJ‑CE – Art. 1131, § 10**  
+  “No âmbito do registro de imóveis, a certidão de inteiro teor da matrícula conterá a reprodução de todo seu conteúdo e será suficiente para fins de comprovação de propriedade, direitos, ônus reais e restrições sobre o imóvel, independentemente de certificação específica pelo Oficial.”
+- **Lei 6.015/1973 – Art. 19, § 11**  
+  “No âmbito do registro de imóveis, a certidão de inteiro teor da matrícula conterá a reprodução de todo seu conteúdo e será suficiente para fins de comprovação de propriedade, direitos, ônus reais e restrições sobre o imóvel, independentemente de certificação específica pelo oficial.”
+Esses dispositivos estabelecem que a certidão reproduz todo o conteúdo da matrícula, mas não impõem a inclusão do CPF completo dos proprietários como requisito obrigatório. Portanto, a prática de registrar o CPF completo não é exigida nem prevista na legislação vigente.</t>
         </is>
       </c>
       <c r="H103" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 258:p78; Código de Normas CGJ-CE, Art. 1083:p218; Código de Normas CGJ-CE, Art. 255:p78; Provimento CNJ 149/2023, Art. 117:p55; Código de Normas CGJ-CE, Art. 1502:p308</t>
+          <t>Código de Normas CGJ-CE — Art. 1502:p308; Código de Normas CGJ-CE — Art. 1131:p229; Lei 6.015/1973 — Art. 19:p0; Código de Normas CGJ-CE — Art. 1633:p333</t>
         </is>
       </c>
       <c r="I103" s="8" t="n">
-        <v>0.63</v>
+        <v>1.3</v>
       </c>
       <c r="J103" s="8" t="n">
-        <v>1962</v>
+        <v>1698</v>
       </c>
       <c r="K103" s="8" t="n">
-        <v>113</v>
+        <v>658</v>
       </c>
       <c r="L103" s="10">
         <f>IF(COUNT(J103:K103)=2,(J103*Parametros!$B$3+K103*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6227,6 +6976,17 @@
         <v/>
       </c>
       <c r="S103" s="8" t="n"/>
+      <c r="T103" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="U103" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="V103" s="11">
+        <f>IF(AND(ISNUMBER(T103),T103&gt;0),U103/T103,"")</f>
+        <v/>
+      </c>
+      <c r="W103" s="8" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="n">
@@ -6247,48 +7007,48 @@
       </c>
       <c r="E104" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F104" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t>**Resposta**
-De acordo com o disposto nos normativos citados:
-- **Art. 1.129** do **Código de Normas CGJ‑CE** – caput  
-  As certidões dos imóveis que já forem objeto de matrícula eletrônica, após a “primeira qualificação eletrônica”, serão expedidas, **independentemente de indicação de finalidade**, em formato nato‑digital estruturado, contendo **a situação jurídica atual do imóvel**, ou seja, sua descrição, titularidade e **os ônus reais não cancelados**.
-- **Art. 125** do **Provimento CNJ 149/2023** – caput (texto idêntico ao art. 1.129)  
-  Reitera que a certidão deve conter **apenas a situação jurídica atual** e **os ônus não cancelados**.
-- **Art. 1.682** do **Código de Normas CGJ‑CE** – caput e parágrafo único  
-  - Caput: idem aos artigos acima, limitando a certidão à situação atual e aos ônus não cancelados.  
-  - **Parágrafo único**: A expedição de certidão de atos anteriores da cadeia filiatória do imóvel **depende de identificação segura do requerente e de indicação da finalidade**.
-- **Art. 230** da **Lei 6.015/1973** – caput  
-  Quando houver ônus na certidão, o oficial o averbá no registro, mas não trata de ônus já cancelados.
-### Conclusão
-- **Não** é possível emitir a certidão da matrícula contendo **todo o histórico de ônus, inclusive penhoras já canceladas**, de forma automática e sem requisitos adicionais.
-- Para obter informações sobre atos anteriores (penhoras canceladas, etc.), é necessário:
-  1. **Identificação segura** do requerente;  
-  2. **Indicação clara da finalidade** da certidão (ex.: pesquisa de histórico de ônus).  
-Somente atendidas essas condições, a autoridade competente poderá expedir a certidão com os atos anteriores da cadeia filiatória. Caso contrário, a certidão deve limitar‑se à **situação jurídica atual** e aos **ônus não cancelados**.</t>
+          <t>**Resposta:** O pedido deve ser **praticado condicionado com tarjamento protetivo**.
+**Fundamentação normativa**
+1. **Certidão padrão – ônus não cancelados**  
+   - **Código de Normas CGJ‑CE, art. 1.129** – “as certidões … serão expedidas … contendo … os ônus reais **não cancelados**.”  
+   - Portanto, a certidão que contém apenas a situação jurídica atual (descrição, titularidade e ônus vigentes) pode ser emitida integralmente, mas **não inclui** ônus já extintos (penhoras canceladas).
+2. **Emissão de certidão com histórico de atos anteriores**  
+   - **Código de Normas CGJ‑CE, art. 1.682, § único** – “a expedição de certidão de atos anteriores da cadeia filiatória do imóvel **depende de identificação segura do requerente e de indicação da finalidade**.”  
+   - Essa exigência caracteriza a necessidade de **tarjamento protetivo** (tratamento de dados pessoais sensíveis) para garantir a proteção dos dados constantes nos registros históricos, em consonância com a LGPD.
+3. **Procedimento recomendado**  
+   - **Passo 1 –** Verificar a identidade do requerente (documentação idônea, assinatura digital ou outro meio que assegure a identificação segura).  
+   - **Passo 2 –** Exigir a indicação clara da finalidade da certidão (ex.: instrução de processo judicial, análise de crédito, pesquisa acadêmica, etc.).  
+   - **Passo 3 –** Aplicar o tarjamento protetivo (mascaramento ou restrição de acesso) aos dados pessoais que constam nos atos extintos, de modo a atender a LGPD (art. 5º, inc. X da LGPD) e o art. 1.682, § único do Código de Normas CGJ‑CE.  
+   - **Passo 4 –** Emitir a certidão contendo **todo o histórico de ônus**, inclusive as penhoras já canceladas, com a devida proteção dos dados.
+**Conclusão prática**
+- **Não** é possível atender ao pedido de forma integral (sem restrições) apenas com base no art. 1.129, pois a certidão padrão exclui ônus cancelados.  
+- **Deve‑se** conceder a certidão histórica **condicionada ao tarjamento protetivo**, atendendo ao requisito de identificação segura e indicação de finalidade previsto no art. 1.682, § único.  
+Assim, o ato registral será praticado **condicionado com tarjamento protetivo**, observando os dispositivos citados.</t>
         </is>
       </c>
       <c r="H104" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 1129:p229; Provimento CNJ 149/2023, Art. 125:p57; Lei 6.015/1973, Art. 230:p0; Código de Normas CGJ-CE, Art. 1259:p256; Código de Normas CGJ-CE, Art. 1682:p345</t>
+          <t>Lei 6.015/1973 — Art. 230:p0; Código de Normas CGJ-CE — Art. 1129:p229; Código de Normas CGJ-CE — Art. 1682:p345; Código de Normas CGJ-CE — Art. 1259:p256</t>
         </is>
       </c>
       <c r="I104" s="8" t="n">
-        <v>2.15</v>
+        <v>2.88</v>
       </c>
       <c r="J104" s="8" t="n">
-        <v>1909</v>
+        <v>1410</v>
       </c>
       <c r="K104" s="8" t="n">
-        <v>788</v>
+        <v>1188</v>
       </c>
       <c r="L104" s="10">
         <f>IF(COUNT(J104:K104)=2,(J104*Parametros!$B$3+K104*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6304,6 +7064,21 @@
         <v/>
       </c>
       <c r="S104" s="8" t="n"/>
+      <c r="T104" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="U104" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="V104" s="11">
+        <f>IF(AND(ISNUMBER(T104),T104&gt;0),U104/T104,"")</f>
+        <v/>
+      </c>
+      <c r="W104" s="8" t="inlineStr">
+        <is>
+          <t>Art. 5 (LGPD (Lei 13.709/2018)) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="n">
@@ -6324,36 +7099,40 @@
       </c>
       <c r="E105" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F105" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G105" s="8" t="inlineStr">
         <is>
-          <t>**Não.**  
-De acordo com o **Provimento CNJ 149/2023**, **Art. 123**, a prestação de informações cadastrais – como a busca de todos os imóveis registrados em nome de uma pessoa – está sujeita a requisitos de identificação do requerente e de indicação da finalidade:
-- **Art. 123.** “Dependem de identificação do requerente e independem de indicação da finalidade os pedidos de certidão de registros em sentido estrito, averbações, matrículas, transcrições ou inscrições específicas, expedidas em qualquer modalidade.”
-- **§ 3.º** “Pedidos de certidão, de busca e de informações apresentados em bloco… dependem de identificação do requerente e indicação da finalidade…”.
-Portanto, **não é permitido** atender a um pedido que contenha apenas o nome do interessado, sem que o requerente se identifique e indique a finalidade da pesquisa. O fornecimento da informação sem esses requisitos violaria o disposto no provimento.</t>
+          <t>**Resposta:** Indeferido via Nota Devolutiva.
+**Fundamentação normativa**
+- **Código de Normas da CGJ‑CE – Art. 1.128, § 2º, inc. V**:  
+  “o fornecimento, pelo registrador, por qualquer meio, de informações sobre o registro não veiculadas por certidão, **exceto nos casos em que o solicitante figure no registro em questão**.”  
+  No pedido apresentado o requerente indica apenas o nome do titular (“fulano”) e não demonstra que ele próprio seja o titular nem apresenta qualquer finalidade legalmente prevista. Assim, a informação solicitada não pode ser fornecida por meio de busca ou comunicação direta, pois não se enquadra na exceção prevista no inciso V.
+- **Lei 6.015/1973 – Art. 222** (obrigatoriedade de referência à matrícula nos atos) reforça que a identificação do imóvel deve ser feita mediante número de matrícula ou registro, não apenas pelo nome do proprietário, o que demonstra a necessidade de dados precisos e vinculados ao registro para qualquer comunicação.
+- **LGPD (Lei Geral de Proteção de Dados Pessoais)** – embora não conste explicitamente no corpus fornecido, o tratamento de dados pessoais (nome e patrimônio imobiliário) só pode ocorrer mediante consentimento do titular ou outra hipótese legal. O simples pedido de “todos os imóveis em nome de fulano” sem consentimento ou legitimidade não atende a esse requisito.
+**Conclusão operativa**
+Diante da ausência de comprovação de que o requerente seja o próprio titular ou que possua autorização legal para acessar tais dados, o ato de busca e a posterior comunicação das informações devem ser **indeferidos**, devendo ser emitida a respectiva **Nota Devolutiva** fundamentada no art. 1.128, § 2º, inc. V, do Código de Normas da CGJ‑CE.</t>
         </is>
       </c>
       <c r="H105" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 1416:p287; Lei 6.015/1973, Art. 234:p0; Provimento CNJ 149/2023, Art. 123:p56; Código de Normas CGJ-CE, Art. 822:p175; Lei 6.015/1973, Art. 213:p0</t>
+          <t>Lei 6.015/1973 — Art. 234:p0; Lei 6.015/1973 — Art. 222:p0; Código de Normas CGJ-CE — Art. 1416:p287; Código de Normas CGJ-CE — Art. 1311:p267; Código de Normas CGJ-CE — Art. 1128:p229</t>
         </is>
       </c>
       <c r="I105" s="8" t="n">
-        <v>1.64</v>
+        <v>2</v>
       </c>
       <c r="J105" s="8" t="n">
-        <v>2383</v>
+        <v>1483</v>
       </c>
       <c r="K105" s="8" t="n">
-        <v>576</v>
+        <v>731</v>
       </c>
       <c r="L105" s="10">
         <f>IF(COUNT(J105:K105)=2,(J105*Parametros!$B$3+K105*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6369,6 +7148,17 @@
         <v/>
       </c>
       <c r="S105" s="8" t="n"/>
+      <c r="T105" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="U105" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="V105" s="11">
+        <f>IF(AND(ISNUMBER(T105),T105&gt;0),U105/T105,"")</f>
+        <v/>
+      </c>
+      <c r="W105" s="8" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="n">
@@ -6389,49 +7179,28 @@
       </c>
       <c r="E106" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F106" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
-        </is>
-      </c>
-      <c r="G106" s="8" t="inlineStr">
-        <is>
-          <t>**Procedimento para busca de bens do devedor por CPF solicitada por um credor**
-**Art. 1.659.**  
-No requerimento do credor fiduciário dirigido ao Oficial do Registro de Imóveis para intimação do fiduciante devem constar as seguintes informações:
-- **I** — número do CPF e nome do devedor fiduciante (e de seu cônjuge, se for casado em regime de bens que exija a intimação);
-- **II** — endereço residencial atual e anterior, se houver, do devedor fiduciante;
-- **III** — endereço comercial, se houver, do devedor fiduciante;
-- **IV** — declaração de que decorreu o prazo de carência estipulado no contrato;
-- **V** — planilha contendo o demonstrativo do débito decorrente das prestações vencidas e não pagas e das que se vencerem até a data do pagamento, os juros convencionais, as penalidades e os demais encargos contratuais, os encargos legais, inclusive tributos e as contribuições condominiais imputáveis ao imóvel, bem como a projeção da dívida, em valores atualizados, para purgação da mora;
-- **VI** — número do CPF e nome do representante do credor fiduciário;
-- **VII** — comprovante de representação legal do credor fiduciário pelo signatário do requerimento, quando for o caso.
-**Art. 1.666.**  
-Quando, por três vezes, o devedor, seu representante legal ou seu procurador não for encontrado em seu domicílio, residência ou em outro endereço indicado pelo credor para ser intimado e houver suspeita razoável de ocultação, o oficial intimará qualquer pessoa próxima, parente ou não, do devedor de que no dia imediato voltará a efetuar a intimação na hora que designar.
-**Procedimento resumido**
-1. O credor apresenta ao Oficial do Registro de Imóveis um requerimento contendo, obrigatoriamente, os itens listados no **Art. 1.659**.
-2. O Oficial verifica a existência de registros imobiliários vinculados ao CPF informado.
-3. Se o devedor não for localizado em seu domicílio, o Oficial procede conforme o **Art. 1.666**, intimando terceiros próximos e designando nova data e hora para a intimação.
-4. O Oficial, ao localizar os bens, registra a localização da parcela ou da hipoteca, conforme previsto no **Art. 1.621**, observando as exigências específicas de cada tipo de gravame (hipoteca, penhora, anticrese, etc.).
-Assim, a busca por CPF solicitada por um credor segue o procedimento acima, garantindo que todas as informações exigidas sejam apresentadas e que o Oficial do Registro de Imóveis realize a localização e intimação de forma adequada.</t>
-        </is>
-      </c>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
+        </is>
+      </c>
+      <c r="G106" s="8" t="inlineStr"/>
       <c r="H106" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 1659:p339; Código de Normas CGJ-CE, Art. 1621:p330; Código de Normas CGJ-CE, Art. 1666:p342; Provimento 15/2026/CGJCE, Art. 1:p2; Provimento CNJ 149/2023, Art. 397-AL:p256</t>
+          <t>Código de Normas CGJ-CE — Art. 1666:p342; Código de Normas CGJ-CE — Art. 1659:p339; Código de Normas CGJ-CE — Art. 1621:p330; Provimento 15/2026/CGJCE — Art. 1:p2</t>
         </is>
       </c>
       <c r="I106" s="8" t="n">
-        <v>1.75</v>
+        <v>2.73</v>
       </c>
       <c r="J106" s="8" t="n">
-        <v>2689</v>
+        <v>2169</v>
       </c>
       <c r="K106" s="8" t="n">
-        <v>1079</v>
+        <v>2048</v>
       </c>
       <c r="L106" s="10">
         <f>IF(COUNT(J106:K106)=2,(J106*Parametros!$B$3+K106*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6447,6 +7216,17 @@
         <v/>
       </c>
       <c r="S106" s="8" t="n"/>
+      <c r="T106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U106" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V106" s="11">
+        <f>IF(AND(ISNUMBER(T106),T106&gt;0),U106/T106,"")</f>
+        <v/>
+      </c>
+      <c r="W106" s="8" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="n">
@@ -6467,32 +7247,32 @@
       </c>
       <c r="E107" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F107" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>Não encontrado no corpus</t>
+          <t>Não encontrado no corpus.</t>
         </is>
       </c>
       <c r="H107" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 1456:p297; Provimento CNJ 149/2023, Art. 259:p166; Código de Normas CGJ-CE, Art. 1394:p282; Lei 6.015/1973, Art. 123:p0; Decreto 7.724/2012, Art. 12:p0</t>
+          <t>Código de Normas CGJ-CE — Art. 1394:p282; Código de Normas CGJ-CE — Art. 1456:p297; Código de Normas CGJ-CE — Art. 1386:p281; Provimento CNJ 149/2023 — Art. 426:p269; Código de Normas CGJ-CE — Art. 1364:p277</t>
         </is>
       </c>
       <c r="I107" s="8" t="n">
-        <v>0.72</v>
+        <v>2.19</v>
       </c>
       <c r="J107" s="8" t="n">
-        <v>2462</v>
+        <v>1783</v>
       </c>
       <c r="K107" s="8" t="n">
-        <v>214</v>
+        <v>782</v>
       </c>
       <c r="L107" s="10">
         <f>IF(COUNT(J107:K107)=2,(J107*Parametros!$B$3+K107*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6508,6 +7288,17 @@
         <v/>
       </c>
       <c r="S107" s="8" t="n"/>
+      <c r="T107" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U107" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V107" s="11">
+        <f>IF(AND(ISNUMBER(T107),T107&gt;0),U107/T107,"")</f>
+        <v/>
+      </c>
+      <c r="W107" s="8" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="n">
@@ -6528,25 +7319,25 @@
       </c>
       <c r="E108" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F108" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G108" s="8" t="inlineStr"/>
       <c r="H108" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 1333:p271; Lei 6.015/1973, Art. 279:p0; Lei 6.015/1973, Art. 292:p0; Código de Normas CGJ-CE, Art. 1412:p286; Lei 6.015/1973, Art. 225:p0</t>
+          <t>Lei 6.015/1973 — Art. 279:p0; Lei 6.015/1973 — Art. 276:p0; Lei 6.015/1973 — Art. 292:p0; Código de Normas CGJ-CE — Art. 1333:p271; Código de Normas CGJ-CE — Art. 1412:p286</t>
         </is>
       </c>
       <c r="I108" s="8" t="n">
-        <v>7.09</v>
+        <v>3</v>
       </c>
       <c r="J108" s="8" t="n">
-        <v>1888</v>
+        <v>1175</v>
       </c>
       <c r="K108" s="8" t="n">
         <v>2048</v>
@@ -6565,6 +7356,17 @@
         <v/>
       </c>
       <c r="S108" s="8" t="n"/>
+      <c r="T108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U108" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V108" s="11">
+        <f>IF(AND(ISNUMBER(T108),T108&gt;0),U108/T108,"")</f>
+        <v/>
+      </c>
+      <c r="W108" s="8" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="n">
@@ -6585,59 +7387,63 @@
       </c>
       <c r="E109" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F109" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>**Resposta**
-- **É permitido fornecer** a lista contendo o número de inscrição (IPTU ou ITR) do imóvel, o nome completo e o CPF do proprietário, pois a própria normativa exige a inclusão desses dados nos documentos que acompanham processos de usucapião e de retificação de registro.  
-- **Formato recomendado**  
-  - Apresentar a informação em **lista estruturada** ou **tabela** para garantir clareza e facilitar a conferência pelos servidores da prefeitura.  
-  - Cada registro deve conter, em linhas separadas, os seguintes campos:  
-    1. **Número de inscrição imobiliária** (IPTU/ITR) ou matrícula;  
-    2. **Nome completo do proprietário**;  
-    3. **CPF do proprietário**.  
-  - Exemplo de apresentação (em texto simples):  
-    ```
-    Imóvel: 12345‑6789
-    Proprietário: João da Silva
-    CPF: 123.456.789‑00
-    Imóvel: 98765‑4321
-    Proprietário: Maria Oliveira
-    CPF: 987.654.321‑00
-    ```
-  - Ou, se preferir tabela markdown:
-    | Inscrição (IPTU/ITR) | Proprietário      | CPF            |
-    |----------------------|-------------------|----------------|
-    | 12345‑6789           | João da Silva     | 123.456.789‑00 |
-    | 98765‑4321           | Maria Oliveira    | 987.654.321‑00 |
+          <t>**Resposta:** A solicitação da Prefeitura deve ser atendida **condicionada com tarjamento protetivo** (proteção de dados), mediante a entrega dos dados no formato eletrônico previsto pelo Provimento CNJ 149/2023.
 ---
-**Fundamentação normativa**
-- **Art. 907** (Seção II) – exige a consignação do número de inscrição e dos **nome e CPF do proprietário** nos documentos de usucapião.  
-- **Art. 1416** (Capítulo XVI) – determina a apresentação de certidão negativa e, quando necessário, a identificação completa dos proprietários e ocupantes.  
-- **Art. 1394** (Seção II) – lista, entre os documentos exigidos, a **identificação e qualificação dos confrontantes (proprietários e eventuais ocupantes) com nome e CPF**.  
-Esses dispositivos demonstram que a coleta e a transmissão desses dados são previstas e exigidas nos atos notariais e registrários, legitimando a entrega da lista à prefeitura para fins de cobrança de IPTU.</t>
+### Fundamentação normativa
+1. **Provimento CNJ 149/2023 – Art. 184‑A, §§ 3 a 6**  
+   - **§ 3º** – “É obrigatória a indicação do fato ou ato jurídico que ensejou a aquisição ou a transmissão do direito real de propriedade (compra e venda, doação, usucapião etc.).”  
+   - **§ 4º** – “O CNB/CF e o ONR disponibilizarão acesso aos municípios, para obtenção das informações, mediante convênio padronizado, para fins de os destinatários das informações atenderem ao disposto nas regras de proteção de dados e de sigilo fiscal.”  
+   - **§ 5º** – “O acesso pode ocorrer mediante plataforma que permita aos municípios obterem, em um mesmo ambiente eletrônico, as informações.”  
+   - **§ 6º** – “Caberão ao CNB/CF e ao ONR a elaboração de manual técnico em que serão estabelecidos o formato dos dados e o padrão dos programas de interface eletrônica (Application Programming Interface – API), a serem utilizados no intercâmbio de dados estruturados entre as serventias extrajudiciais e as municipalidades.”
+2. **LGPD (Lei 13.709/2018) – tratamento de dados pessoais para cumprimento de obrigação legal ou regulatória**  
+   - Embora o texto da LGPD não conste integralmente no corpus, o provimento acima já incorpora a exigência de observância das “regras de proteção de dados”, que decorrem do art. 7º, I da LGPD (tratamento de dados pessoais quando necessário ao cumprimento de obrigação legal ou regulatória).  
+---
+### Como proceder
+| Etapa | Descrição | Base legal |
+|-------|-----------|------------|
+| **1. Convênio padronizado** | Verificar a existência de convênio entre o Cartório de Registro de Imóveis e a Prefeitura, nos termos do **§ 4º** do art. 184‑A. | Provimento CNJ 149/2023, art. 184‑A, § 4º |
+| **2. Utilização da plataforma ONR** | Disponibilizar a lista (imóvel, proprietário, CPF) por meio da plataforma eletrônica do **Operador Nacional do Sistema de Registro Eletrônico de Imóveis (ONR)**, conforme previsto no **§ 5º**. | Provimento CNJ 149/2023, art. 184‑A, § 5º |
+| **3. Formato dos dados** | Seguir o **manual técnico** elaborado pelo CNB/CF e ONR (art. 184‑A, § 6º), que define o padrão de **API/arquivo estruturado (ex.: JSON ou XML) contendo apenas os campos necessários** (número da matrícula, nome completo, CPF, endereço). | Provimento CNJ 149/2023, art. 184‑A, § 6º |
+| **4. Tarjamento protetivo** | Aplicar a classificação de **tarjamento protetivo** aos dados pessoais (CPF) para garantir que o acesso seja restrito ao uso exclusivo da cobrança de IPTU, obedecendo aos princípios da LGPD (necessidade, adequação e minimização). | Provimento CNJ 149/2023, art. 184‑A, §§ 4‑5 (regras de proteção de dados) |
+| **5. Registro da comunicação** | Emitir nota de devolutiva ao requerente (Prefeitura) informando o meio de acesso (API/portal ONR) e as condições de uso dos dados, conforme prática de transparência e rastreabilidade. | Não encontrado no corpus (para formalização de nota de devolutiva) |
+---
+### Conclusão
+- **O ato registral não pode ser indeferido**; a informação é de interesse público para a arrecadação de IPTU, havendo fundamento legal para o seu fornecimento.  
+- **Deve ser fornecida**, porém **condicionada com tarjamento protetivo** e **exclusivamente via plataforma eletrônica (ONR) no formato técnico definido pelo manual de API**, garantindo a observância das normas de proteção de dados previstas no Provimento CNJ 149/2023 e na LGPD.  
+---  
+**Nota de Devolutiva (modelo resumido)**  
+&gt; “Em atendimento ao requerimento da Prefeitura Municipal de ___, informamos que a lista de imóveis com respectivos proprietários e CPFs será disponibilizada por meio da plataforma do Operador Nacional do Sistema de Registro Eletrônico de Imóveis (ONR), conforme o manual técnico de intercâmbio de dados (API). Os dados serão tarifados como protetivos, obedecendo às regras de proteção de dados pessoais previstas no Provimento CNJ 149/2023, art. 184‑A, §§ 4‑6, e na LGPD. O acesso será concedido mediante credenciais específicas e uso exclusivo para fins de cobrança de IPTU.”  
+---  
+**Referências citadas**  
+- Provimento CNJ 149/2023, Art. 184‑A, §§ 3 a 6.  
+- LGPD (Lei 13.709/2018) – tratamento de dados pessoais para cumprimento de obrigação legal (art. 7º, I).  
+---  
+*Esta orientação está baseada **exclusivamente** no corpus normativo apresentado.*</t>
         </is>
       </c>
       <c r="H109" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 907:p191; Código de Normas CGJ-CE, Art. 1416:p287; Código de Normas CGJ-CE, Art. 828:p178; Código de Normas CGJ-CE, Art. 1394:p282</t>
+          <t>Código de Normas CGJ-CE — Art. 1416:p287; Código de Normas CGJ-CE — Art. 1394:p282; Código de Normas CGJ-CE — Art. 1498:p307; Provimento CNJ 149/2023 — Art. 184-A:p88</t>
         </is>
       </c>
       <c r="I109" s="8" t="n">
-        <v>2.32</v>
+        <v>4.29</v>
       </c>
       <c r="J109" s="8" t="n">
-        <v>2375</v>
+        <v>2097</v>
       </c>
       <c r="K109" s="8" t="n">
-        <v>917</v>
+        <v>1754</v>
       </c>
       <c r="L109" s="10">
         <f>IF(COUNT(J109:K109)=2,(J109*Parametros!$B$3+K109*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6653,6 +7459,21 @@
         <v/>
       </c>
       <c r="S109" s="8" t="n"/>
+      <c r="T109" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="U109" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="V109" s="11">
+        <f>IF(AND(ISNUMBER(T109),T109&gt;0),U109/T109,"")</f>
+        <v/>
+      </c>
+      <c r="W109" s="8" t="inlineStr">
+        <is>
+          <t>Art. 7 (LGPD (Lei 13.709/2018)) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="7" t="n">
@@ -6673,32 +7494,37 @@
       </c>
       <c r="E110" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F110" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>Não encontrado no corpus</t>
+          <t>**Indeferir via Nota Devolutiva**  
+O oficial deve recusar o fornecimento dos dados solicitados pela polícia, emitindo uma Nota Devolutiva fundamentada, pois a solicitação não está respaldada por ordem judicial e, portanto, não se enquadra nas finalidades previstas para o tratamento de dados pessoais no Registro de Imóveis.
+**Dispositivo legal aplicável**  
+Art. 1128, § 4º, do Código de Normas CGJ‑CE:  
+&gt; “Caracterizada tentativa de tratamento de dados em desacordo com as finalidades do Registro de Imóveis e com os princípios da Lei Geral de Proteção de Dados Pessoais, poderá o Oficial recusar o fornecimento em nota fundamentada, do que caberá revisão pelo juízo competente.”
+Assim, o ato registral deve ser **indeferido via Nota Devolutiva**.</t>
         </is>
       </c>
       <c r="H110" s="8" t="inlineStr">
         <is>
-          <t>Lei 6.015/1973, Art. 110:p0; Código de Normas CGJ-CE, Art. 1128:p229; Provimento CNJ 149/2023, Art. 320-AE:p205; LGPD (Lei 13.709/2018), Art. 18:p0; Provimento CNJ 149/2023, Art. 320-AK:p206</t>
+          <t>Código de Normas CGJ-CE — Art. 1464:p299; Lei 6.015/1973 — Art. 283:p0; Provimento CNJ 149/2023 — Art. 320-AE:p205; Código de Normas CGJ-CE — Art. 1128:p229; Provimento CNJ 149/2023 — Art. 320-AK:p206</t>
         </is>
       </c>
       <c r="I110" s="8" t="n">
-        <v>20.93</v>
+        <v>20.58</v>
       </c>
       <c r="J110" s="8" t="n">
-        <v>2412</v>
+        <v>1605</v>
       </c>
       <c r="K110" s="8" t="n">
-        <v>232</v>
+        <v>815</v>
       </c>
       <c r="L110" s="10">
         <f>IF(COUNT(J110:K110)=2,(J110*Parametros!$B$3+K110*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6714,6 +7540,17 @@
         <v/>
       </c>
       <c r="S110" s="8" t="n"/>
+      <c r="T110" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="U110" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="V110" s="11">
+        <f>IF(AND(ISNUMBER(T110),T110&gt;0),U110/T110,"")</f>
+        <v/>
+      </c>
+      <c r="W110" s="8" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="n">
@@ -6734,12 +7571,12 @@
       </c>
       <c r="E111" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F111" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G111" s="8" t="inlineStr">
@@ -6749,17 +7586,17 @@
       </c>
       <c r="H111" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 1367:p277; Código de Normas CGJ-CE, Art. 1127:p229; Código de Normas CGJ-CE, Art. 162:p63; Código de Normas CGJ-CE, Art. 285:p85; Código de Normas CGJ-CE, Art. 257:p78</t>
+          <t>Código de Normas CGJ-CE — Art. 1367:p277; Código de Normas CGJ-CE — Art. 1141:p232; Código de Normas CGJ-CE — Art. 1128:p229; Código de Normas CGJ-CE — Art. 1127:p229; Lei 6.015/1973 — Art. 176-O:p0</t>
         </is>
       </c>
       <c r="I111" s="8" t="n">
-        <v>20.74</v>
+        <v>14.49</v>
       </c>
       <c r="J111" s="8" t="n">
-        <v>1797</v>
+        <v>1399</v>
       </c>
       <c r="K111" s="8" t="n">
-        <v>210</v>
+        <v>651</v>
       </c>
       <c r="L111" s="10">
         <f>IF(COUNT(J111:K111)=2,(J111*Parametros!$B$3+K111*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6775,6 +7612,17 @@
         <v/>
       </c>
       <c r="S111" s="8" t="n"/>
+      <c r="T111" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U111" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V111" s="11">
+        <f>IF(AND(ISNUMBER(T111),T111&gt;0),U111/T111,"")</f>
+        <v/>
+      </c>
+      <c r="W111" s="8" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="n">
@@ -6795,32 +7643,32 @@
       </c>
       <c r="E112" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F112" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>Não encontrado no corpus</t>
+          <t>Não encontrado no corpus.</t>
         </is>
       </c>
       <c r="H112" s="8" t="inlineStr">
         <is>
-          <t>LAI (Lei 12.527/2011), Art. 41:p0; LAI (Lei 12.527/2011), Art. 8:p0; LAI (Lei 12.527/2011), Art. 10:p0; LAI (Lei 12.527/2011), Art. 11:p0</t>
+          <t>LAI (Lei 12.527/2011) — Art. 8:p0; LAI (Lei 12.527/2011) — Art. 14:p0; LAI (Lei 12.527/2011) — Art. 11:p0; LAI (Lei 12.527/2011) — Art. 41:p0</t>
         </is>
       </c>
       <c r="I112" s="8" t="n">
-        <v>1.49</v>
+        <v>2.38</v>
       </c>
       <c r="J112" s="8" t="n">
-        <v>2265</v>
+        <v>1578</v>
       </c>
       <c r="K112" s="8" t="n">
-        <v>190</v>
+        <v>431</v>
       </c>
       <c r="L112" s="10">
         <f>IF(COUNT(J112:K112)=2,(J112*Parametros!$B$3+K112*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6836,6 +7684,17 @@
         <v/>
       </c>
       <c r="S112" s="8" t="n"/>
+      <c r="T112" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U112" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V112" s="11">
+        <f>IF(AND(ISNUMBER(T112),T112&gt;0),U112/T112,"")</f>
+        <v/>
+      </c>
+      <c r="W112" s="8" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="n">
@@ -6856,42 +7715,37 @@
       </c>
       <c r="E113" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F113" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>**Art. 10.** Qualquer interessado poderá apresentar pedido de acesso a informações aos órgãos e entidades referidos no art. 1º desta Lei, por qualquer meio legítimo, devendo o pedido conter a identificação do requerente e a especificação da informação requerida.  
-§ 1º Para o acesso a informações de interesse público, a identificação do requerente não pode conter exigências que inviabilizem a solicitação.  
-§ 2º Os órgãos e entidades do poder público devem viabilizar alternativa de encaminhamento de pedidos de acesso por meio de seus sítios oficiais na internet.  
-§ 3º São vedadas quaisquer exigências relativas aos motivos determinantes da solicitação de informações de interesse público.  
----
-**Resposta ao pedido via LAI sobre os emolumentos arrecadados pela serventia**
-- **Sim, é dever responder.**  
-  - O LAI estabelece que qualquer interessado pode solicitar informações de interesse público, e o órgão deve viabilizar o acesso.  
-  - A solicitação de dados sobre emolumentos arrecadados pela serventia é uma informação de interesse público.  
-  - Não há previsão legal que permita a recusa ou a exigência de motivos determinantes para a solicitação.  
-  - Portanto, a serventia tem a obrigação de atender ao pedido e fornecer os dados solicitados.</t>
+          <t>**Resposta Jurídica e Operacional**
+Sim, é dever responder ao pedido de acesso à informação sobre os emolumentos arrecadados pela serventia.
+**Fundamentação normativa**
+- **LAI – Art. 10**: “Qualquer interessado poderá apresentar pedido de acesso a informações aos órgãos e entidades referidos no art. 1º desta Lei…”.  
+- **LAI – Art. 14**: “É direito do requerente obter o inteiro teor de decisão de negativa de acesso, por certidão ou cópia.”  
+O pedido trata de informação de interesse público (emolumentos arrecadados), não se enquadrando em nenhuma exceção prevista na LAI. Portanto, a serventia deve atender ao pedido, fornecendo os dados solicitados ou, se houver impedimento, justificando a negativa conforme previsto no art. 14.</t>
         </is>
       </c>
       <c r="H113" s="8" t="inlineStr">
         <is>
-          <t>Provimento CNJ 149/2023, Art. 231-A:p141; Provimento CNJ 149/2023, Art. 228-U:p134; Provimento CNJ 149/2023, Art. 373:p233; LAI (Lei 12.527/2011), Art. 10:p0; Provimento CNJ 149/2023, Art. 71-J:p35</t>
+          <t>LAI (Lei 12.527/2011) — Art. 14:p0; Provimento CNJ 149/2023 — Art. 228-U:p134; LAI (Lei 12.527/2011) — Art. 10:p0; LAI (Lei 12.527/2011) — Art. 13:p0; Provimento CNJ 149/2023 — Art. 71-J:p35</t>
         </is>
       </c>
       <c r="I113" s="8" t="n">
-        <v>1.14</v>
+        <v>2.4</v>
       </c>
       <c r="J113" s="8" t="n">
-        <v>2188</v>
+        <v>1458</v>
       </c>
       <c r="K113" s="8" t="n">
-        <v>619</v>
+        <v>1540</v>
       </c>
       <c r="L113" s="10">
         <f>IF(COUNT(J113:K113)=2,(J113*Parametros!$B$3+K113*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6907,6 +7761,21 @@
         <v/>
       </c>
       <c r="S113" s="8" t="n"/>
+      <c r="T113" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="U113" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="V113" s="11">
+        <f>IF(AND(ISNUMBER(T113),T113&gt;0),U113/T113,"")</f>
+        <v/>
+      </c>
+      <c r="W113" s="8" t="inlineStr">
+        <is>
+          <t>Art. 1 (LAI (Lei 12.527/2011)) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="7" t="n">
@@ -6927,37 +7796,37 @@
       </c>
       <c r="E114" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F114" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>**Resposta**
-Sim, a certidão pode ser emitida mesmo quando a matrícula contém averbação de interdição ou curatela.  
-- **Art. 1131, §10** do Código de Normas CGJ‑CE estabelece que a certidão de inteiro teor reproduz todo o conteúdo da matrícula e é suficiente para comprovar propriedade, direitos, ônus reais e restrições sobre o imóvel, independentemente de certificação específica pelo oficial.  
-- A averbação de interdição ou curatela, estando registrada na matrícula, será reproduzida integralmente na certidão.  
-- Não há previsão no contexto que impeça a emissão da certidão quando a matrícula contém essa averbação.  
-Portanto, a certidão pode ser emitida sem restrição, contendo a averbação de interdição/curatela.</t>
+          <t>**Resposta**  
+A certidão de inteiro teor **não pode** ser emitida sem incluir a averbação de interdição/curatela que consta na matrícula.  
+**Fundamentação**  
+- **Código de Normas CGJ‑CE, Art. 1131, § 10**: “No âmbito do registro de imóveis, a certidão de inteiro teor da matrícula conterá a reprodução de todo seu conteúdo e será suficiente para fins de comprovação de propriedade, direitos, ônus reais e restrições sobre o imóvel, independentemente de certificação específica pelo Oficial.”  
+- **Lei 6.015/1973, Art. 19, § 11**: “No âmbito do registro de imóveis, a certidão de inteiro teor da matrícula conterá a reprodução de todo seu conteúdo e será suficiente para fins de comprovação de propriedade, direitos, ônus reais e restrições sobre o imóvel, independentemente de certificação específica pelo oficial.”  
+Portanto, a certidão deve ser emitida **completa**, incluindo a averbação de interdição/curatela; não há possibilidade de emissão “sem restrição”.</t>
         </is>
       </c>
       <c r="H114" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 1131:p229; Provimento CNJ 149/2023, Art. 201:p94; Lei 6.015/1973, Art. 19:p0; Provimento CNJ 149/2023, Art. 200:p94; Código de Normas CGJ-CE, Art. 402:p106</t>
+          <t>Código de Normas CGJ-CE — Art. 1131:p229; Lei 6.015/1973 — Art. 19:p0; Lei 6.015/1973 — Art. 230:p0; Código de Normas CGJ-CE — Art. 1416:p287; Provimento CNJ 149/2023 — Art. 201:p94</t>
         </is>
       </c>
       <c r="I114" s="8" t="n">
-        <v>22.16</v>
+        <v>26.74</v>
       </c>
       <c r="J114" s="8" t="n">
-        <v>2051</v>
+        <v>1771</v>
       </c>
       <c r="K114" s="8" t="n">
-        <v>612</v>
+        <v>656</v>
       </c>
       <c r="L114" s="10">
         <f>IF(COUNT(J114:K114)=2,(J114*Parametros!$B$3+K114*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -6973,6 +7842,17 @@
         <v/>
       </c>
       <c r="S114" s="8" t="n"/>
+      <c r="T114" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="U114" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="V114" s="11">
+        <f>IF(AND(ISNUMBER(T114),T114&gt;0),U114/T114,"")</f>
+        <v/>
+      </c>
+      <c r="W114" s="8" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="n">
@@ -6993,40 +7873,41 @@
       </c>
       <c r="E115" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F115" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>**Art. 820.** Na escritura pública de doação, deve constar o grau de parentesco entre o(s) doador(e)s e o(s) donatário(s).  
-- **§ 1º** Se o donatário for absolutamente incapaz, dispensa‑se a aceitação, desde que se trate de doação pura.  
-- **§ 2º** Nas escrituras de doação sem encargos feitas pelos pais a favor de seus filhos absolutamente incapazes, é dispensada a aceitação por parte do menor.  
----
-### Resposta à sua pergunta
-- **Tarjar a escritura pública de doação**: sim, é necessário registrar (tarjar) a escritura no cartório de notas, garantindo que o grau de parentesco esteja indicado.  
-- **Aceitação**: não é exigida aceitação por parte do menor, pois ele é absolutamente incapaz.  
-- **Alvará judicial**: não há necessidade de alvará judicial para doação pura e simples a menor.  
-Portanto, basta tarjar a escritura pública de doação, observando o grau de parentesco e a dispensa de aceitação.</t>
+          <t>**Resposta Jurídica e Operacional**
+Não é necessário tarjar a averbação de doação a menor de idade (incapaz).  
+**Fundamentação normativa**
+- **Art. 1.267, § 1º – Código de Normas CGJ‑CE**  
+  “Os relativamente incapazes poderão aceitar a doação, não constituindo óbice à lavratura do registro a inexistência de representação ou assistência destas pessoas no título apresentado.”  
+- **Art. 1.267, § 3º – Código de Normas CGJ‑CE**  
+  “Não se exigirá alvará judicial para a realização de doação pura e simples para menores, na forma do artigo 543 do Código Civil.”  
+Esses dispositivos dispõem que a doação a menor pode ser registrada sem a necessidade de representação, assistência ou alvará judicial, e não há previsão de tarjar (proteção) nesse caso.  
+**Conclusão**  
+A averbação pode ser praticada integralmente, sem tarjar. Se houver dúvidas sobre a documentação, basta verificar a aceitação do menor e a ausência de impedimentos legais.</t>
         </is>
       </c>
       <c r="H115" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 906:p191; Provimento CNJ 149/2023, Art. 108:p52; Código de Normas CGJ-CE, Art. 1267:p258; Código de Normas CGJ-CE, Art. 820:p174; Código de Normas CGJ-CE, Art. 868:p183</t>
+          <t>Código de Normas CGJ-CE — Art. 1267:p258; Provimento CNJ 149/2023 — Art. 3 (ato de aprovação):p3; Código de Normas CGJ-CE — Art. 157:p62; Lei 6.015/1973 — Art. 247:p0; Lei 6.015/1973 — Art. 232:p0</t>
         </is>
       </c>
       <c r="I115" s="8" t="n">
-        <v>24.6</v>
+        <v>14.04</v>
       </c>
       <c r="J115" s="8" t="n">
-        <v>1912</v>
+        <v>1361</v>
       </c>
       <c r="K115" s="8" t="n">
-        <v>861</v>
+        <v>448</v>
       </c>
       <c r="L115" s="10">
         <f>IF(COUNT(J115:K115)=2,(J115*Parametros!$B$3+K115*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7042,6 +7923,21 @@
         <v/>
       </c>
       <c r="S115" s="8" t="n"/>
+      <c r="T115" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="U115" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="V115" s="11">
+        <f>IF(AND(ISNUMBER(T115),T115&gt;0),U115/T115,"")</f>
+        <v/>
+      </c>
+      <c r="W115" s="8" t="inlineStr">
+        <is>
+          <t>Art. 543 (OUTRA: codigo civil) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="7" t="n">
@@ -7062,44 +7958,45 @@
       </c>
       <c r="E116" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F116" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>**Resposta**
-De acordo com o **Art. 132** do Provimento CNJ 149/2023 (e o **Art. 755** do Código de Normas CGJ‑CE), o fornecimento de cópias ou certidões de documentos arquivados na serventia:
-- **Limita‑se ao documento protestado propriamente dito**;  
-- **É válido enquanto perdurar o protesto** e dentro do prazo máximo de **10 (dez) anos**;  
-- **Só pode ser fornecida às partes interessadas** ou mediante **autorização judicial**.
-Além disso, o **parágrafo único** estabelece que, tratando‑se de documento de identificação pessoal, a cópia deve ser fornecida **apenas ao próprio titular**.
-Como o documento solicitado contém **dados de saúde**, que são dados pessoais sensíveis nos termos da Lei Geral de Proteção de Dados (LGPD), a sua divulgação exige:
-- **Consentimento expresso do titular**; ou  
-- **Fundamento legal específico**, como ordem judicial.
-**Portanto, a cópia só pode ser fornecida se:**
-1. O requerente for **parte interessada** (titular dos dados de saúde) e apresentar **identificação** conforme exigido; ou  
-2. Existir **autorização judicial** que legitime a entrega da cópia.
-Na ausência de um desses requisitos, **não se deve fornecer a cópia**.</t>
+          <t>**Resposta:** Indeferir o pedido via **Nota Devolutiva**.
+**Fundamentação jurídica**
+1. **LGPD – Tratamento de dados pessoais sensíveis**  
+   - **Art. 11, inc. I** – O tratamento de dados sensíveis (como dados de saúde) só pode ocorrer quando houver consentimento específico e destacado do titular para a finalidade pretendida.  
+   - **Art. 11, inc. II, alínea a** – Na ausência de consentimento, o tratamento só é permitido quando for indispensável para o cumprimento de obrigação legal ou regulatória. O simples fornecimento de cópia de documento arquivado a terceiro não se enquadra em nenhuma das hipóteses previstas (não há obrigação legal que imponha a divulgação, nem outra hipótese autorizadora).  
+2. **Procedimentos de certidão e cópia de documentos arquivados**  
+   - **Código de Normas CGJ‑CE, art. 1.128** e **art. 1.680**, §§ 1º e 2º – Os pedidos de certidão ou de documentos arquivados dependem de identificação do requerente e, quando não houver previsão legal específica de expedição, também exigem indicação da finalidade. Contudo, esses dispositivos tratam apenas da **exigência de identificação** e **finalidade**, não autorizam a divulgação de dados sensíveis que estejam protegidos pela LGPD.  
+3. **Conflito de normas**  
+   - A LGPD tem hierarquia superior no que tange à proteção de dados pessoais sensíveis. Assim, ainda que o requerente esteja devidamente identificado (conforme art. 1.128/1.680 da CGJ‑CE), a ausência de consentimento ou de hipótese legal que autorize o tratamento impede a prática do ato registral.  
+4. **Direito de acesso do titular**  
+   - **LGPD, art. 19** – O titular pode requerer acesso aos seus próprios dados, mas o pedido em questão não foi formulado pelo titular nem há comprovação de consentimento. Portanto, o direito de acesso não se aplica ao requerente.  
+**Conclusão operacional**
+- **Deve ser indeferido** o pedido de cópia do documento arquivado que contém dados de saúde, mediante emissão de **Nota Devolutiva** fundamentada nos dispositivos acima citados (LGPD art. 11, inc. I e II; Código de Normas CGJ‑CE art. 1.128 e art. 1.680).  
+*Obs.: Caso o requerente seja o titular dos dados ou apresente consentimento específico e destacado, o pedido poderia ser analisado sob a ótica do art. 11, inc. I, permitindo a entrega da cópia.*</t>
         </is>
       </c>
       <c r="H116" s="8" t="inlineStr">
         <is>
-          <t>Provimento CNJ 149/2023, Art. 132:p58; Código de Normas CGJ-CE, Art. 1680:p344; Código de Normas CGJ-CE, Art. 755:p164; Código de Normas CGJ-CE, Art. 1128:p229; Provimento CNJ 149/2023, Art. 392:p240</t>
+          <t>LGPD (Lei 13.709/2018) — Art. 11:p0; Provimento CNJ 149/2023 — Art. 123:p56; Código de Normas CGJ-CE — Art. 1128:p229; Código de Normas CGJ-CE — Art. 1680:p344; LGPD (Lei 13.709/2018) — Art. 19:p0</t>
         </is>
       </c>
       <c r="I116" s="8" t="n">
-        <v>2.06</v>
+        <v>3.27</v>
       </c>
       <c r="J116" s="8" t="n">
-        <v>2327</v>
+        <v>2082</v>
       </c>
       <c r="K116" s="8" t="n">
-        <v>595</v>
+        <v>1202</v>
       </c>
       <c r="L116" s="10">
         <f>IF(COUNT(J116:K116)=2,(J116*Parametros!$B$3+K116*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7115,6 +8012,17 @@
         <v/>
       </c>
       <c r="S116" s="8" t="n"/>
+      <c r="T116" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="U116" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="V116" s="11">
+        <f>IF(AND(ISNUMBER(T116),T116&gt;0),U116/T116,"")</f>
+        <v/>
+      </c>
+      <c r="W116" s="8" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="n">
@@ -7135,42 +8043,32 @@
       </c>
       <c r="E117" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F117" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>**Não**.  
-O **Art. 240, § 2º** do Código de Normas CGJ‑CE determina que as certidões eletrônicas ficam disponíveis **apenas** na Central Nacional de Informações do Registro Civil (CRC) e **proíbe** o envio por correio eletrônico convencional (e‑mail) ou por outros meios que não sejam a plataforma da central eletrônica.  
----
-## Cuidados previstos pela LGPD ao tratar a certidão
-- **Finalidade**: o tratamento deve ser realizado apenas para a finalidade de entrega da certidão ao requerente, conforme previsto na lei de registro civil.  
-- **Consentimento**: o requerente deve ter fornecido consentimento expresso para o recebimento da certidão em meio eletrônico, caso a lei não dispensa.  
-- **Segurança**: a transmissão deve ocorrer por meio seguro (ex.: HTTPS, assinatura digital ICP‑Brasil) para garantir a integridade e confidencialidade dos dados.  
-- **Limitação de acesso**: apenas o requerente e pessoas autorizadas (por exemplo, prepostos) podem acessar a certidão.  
-- **Retenção**: a certidão eletrônica deve ser mantida pelo prazo legal (30 dias corridos) e, após esse período, deve ser excluída ou disponibilizada apenas na plataforma oficial.  
-- **Transparência**: o requerente deve ser informado sobre os direitos que possui (acesso, retificação, exclusão) e sobre os meios de exercício desses direitos.  
-Esses cuidados asseguram o cumprimento da LGPD e a proteção dos dados pessoais contidos na certidão.</t>
+          <t>Não encontrado no corpus.</t>
         </is>
       </c>
       <c r="H117" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 258:p78; Código de Normas CGJ-CE, Art. 211:p70; Provimento CNJ 149/2023, Art. 117:p55; Código de Normas CGJ-CE, Art. 683:p152; Código de Normas CGJ-CE, Art. 240:p75</t>
+          <t>Provimento CNJ 149/2023 — Art. 124:p57; Provimento CNJ 149/2023 — Art. 105:p52; Provimento CNJ 149/2023 — Art. 100:p51; Código de Normas CGJ-CE — Art. 195:p68; Provimento CNJ 149/2023 — Art. 104:p52</t>
         </is>
       </c>
       <c r="I117" s="8" t="n">
-        <v>16.23</v>
+        <v>0.82</v>
       </c>
       <c r="J117" s="8" t="n">
-        <v>2123</v>
+        <v>1176</v>
       </c>
       <c r="K117" s="8" t="n">
-        <v>536</v>
+        <v>282</v>
       </c>
       <c r="L117" s="10">
         <f>IF(COUNT(J117:K117)=2,(J117*Parametros!$B$3+K117*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7186,6 +8084,17 @@
         <v/>
       </c>
       <c r="S117" s="8" t="n"/>
+      <c r="T117" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U117" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V117" s="11">
+        <f>IF(AND(ISNUMBER(T117),T117&gt;0),U117/T117,"")</f>
+        <v/>
+      </c>
+      <c r="W117" s="8" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="n">
@@ -7206,32 +8115,32 @@
       </c>
       <c r="E118" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F118" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>**Não encontrado no corpus**</t>
+          <t>Não encontrado no corpus.</t>
         </is>
       </c>
       <c r="H118" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 193:p67; Código de Normas CGJ-CE, Art. 562:p133; Código de Normas CGJ-CE, Art. 417:p109; Código de Normas CGJ-CE, Art. 1274:p262; Código de Normas CGJ-CE, Art. 1681:p345</t>
+          <t>Código de Normas CGJ-CE — Art. 193:p67; Provimento CNJ 149/2023 — Art. 105:p52; Provimento CNJ 149/2023 — Art. 124:p57; Provimento CNJ 149/2023 — Art. 104:p52; Provimento CNJ 149/2023 — Art. 128:p57</t>
         </is>
       </c>
       <c r="I118" s="8" t="n">
-        <v>1.55</v>
+        <v>10.11</v>
       </c>
       <c r="J118" s="8" t="n">
-        <v>1741</v>
+        <v>1417</v>
       </c>
       <c r="K118" s="8" t="n">
-        <v>78</v>
+        <v>427</v>
       </c>
       <c r="L118" s="10">
         <f>IF(COUNT(J118:K118)=2,(J118*Parametros!$B$3+K118*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7247,6 +8156,17 @@
         <v/>
       </c>
       <c r="S118" s="8" t="n"/>
+      <c r="T118" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U118" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V118" s="11">
+        <f>IF(AND(ISNUMBER(T118),T118&gt;0),U118/T118,"")</f>
+        <v/>
+      </c>
+      <c r="W118" s="8" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="n">
@@ -7267,32 +8187,28 @@
       </c>
       <c r="E119" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F119" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
-        </is>
-      </c>
-      <c r="G119" s="8" t="inlineStr">
-        <is>
-          <t>Não encontrado no corpus.</t>
-        </is>
-      </c>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
+        </is>
+      </c>
+      <c r="G119" s="8" t="inlineStr"/>
       <c r="H119" s="8" t="inlineStr">
         <is>
-          <t>LGPD (Lei 13.709/2018), Art. 4:p0; LGPD (Lei 13.709/2018), Art. 51:p0; LGPD (Lei 13.709/2018), Art. 43:p0; LGPD (Lei 13.709/2018), Art. 9:p0; LGPD (Lei 13.709/2018), Art. 7:p0</t>
+          <t>LGPD (Lei 13.709/2018) — Art. 9:p0; LGPD (Lei 13.709/2018) — Art. 18:p0; LGPD (Lei 13.709/2018) — Art. 11:p0; LGPD (Lei 13.709/2018) — Art. 4:p0; LGPD (Lei 13.709/2018) — Art. 20:p0</t>
         </is>
       </c>
       <c r="I119" s="8" t="n">
-        <v>21.83</v>
+        <v>18.13</v>
       </c>
       <c r="J119" s="8" t="n">
-        <v>2061</v>
+        <v>1799</v>
       </c>
       <c r="K119" s="8" t="n">
-        <v>240</v>
+        <v>2048</v>
       </c>
       <c r="L119" s="10">
         <f>IF(COUNT(J119:K119)=2,(J119*Parametros!$B$3+K119*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7308,6 +8224,17 @@
         <v/>
       </c>
       <c r="S119" s="8" t="n"/>
+      <c r="T119" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U119" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V119" s="11">
+        <f>IF(AND(ISNUMBER(T119),T119&gt;0),U119/T119,"")</f>
+        <v/>
+      </c>
+      <c r="W119" s="8" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="n">
@@ -7328,35 +8255,25 @@
       </c>
       <c r="E120" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F120" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
-        </is>
-      </c>
-      <c r="G120" s="8" t="inlineStr">
-        <is>
-          <t>**Sim, você tem obrigação de informar.**  
-- **LGPD – Art. 18**: garante ao titular o direito de acesso a seus dados pessoais, incluindo registros de quem consultou a matrícula.  
-- **LAI – Art. 30**: obriga a autoridade a publicar e disponibilizar informações administrativas, e a atender solicitações de acesso a dados.  
-Portanto, ao receber o pedido, você deve:
-1. **Verificar a identidade** do titular e a legitimidade do pedido.  
-2. **Reunir o relatório** contendo os registros de consulta à matrícula.  
-3. **Entregar o relatório** ao titular dentro do prazo legal (30 dias, salvo</t>
-        </is>
-      </c>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
+        </is>
+      </c>
+      <c r="G120" s="8" t="inlineStr"/>
       <c r="H120" s="8" t="inlineStr">
         <is>
-          <t>Guia ANPD — Agentes de Tratamento, p. 8:p8; LAI (Lei 12.527/2011), Art. 30:p0; Código de Normas CGJ-CE, Art. 1461:p299; Provimento CNJ 149/2023, Art. 339:p215; Provimento CNJ 149/2023, Art. 415:p265</t>
+          <t>Guia ANPD — Agentes de Tratamento — p. 8:p8; Código de Normas CGJ-CE — Art. 1461:p299; Provimento CNJ 149/2023 — Art. 415:p265; LAI (Lei 12.527/2011) — Art. 30:p0; Provimento CNJ 149/2023 — Art. 89:p47</t>
         </is>
       </c>
       <c r="I120" s="8" t="n">
-        <v>18.09</v>
+        <v>30.84</v>
       </c>
       <c r="J120" s="8" t="n">
-        <v>2214</v>
+        <v>1851</v>
       </c>
       <c r="K120" s="8" t="n">
         <v>2048</v>
@@ -7375,6 +8292,17 @@
         <v/>
       </c>
       <c r="S120" s="8" t="n"/>
+      <c r="T120" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U120" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V120" s="11">
+        <f>IF(AND(ISNUMBER(T120),T120&gt;0),U120/T120,"")</f>
+        <v/>
+      </c>
+      <c r="W120" s="8" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="n">
@@ -7395,47 +8323,58 @@
       </c>
       <c r="E121" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F121" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>**Direito do titular**  
-- **Art. 18 da LGPD** – O titular tem o direito de solicitar a **correção** de dado pessoal incorreto.  
-- **§ 5º** – O requerimento deve ser atendido **sem custos** ao titular, nos prazos e termos previstos em regulamento.  
-- **§ 6º** – O responsável deve comunicar imediatamente a correção a todos os agentes de tratamento com quem o dado foi compartilhado, salvo impossibilidade comprovada ou esforço desproporcional.
-**Procedimento de retificação no Registro de Imóveis**  
-- **Código de Normas CGJ‑CE – Art. 1.386** – A retificação de dados de qualificação pessoal das partes cabe ao **Oficial do Registro de Imóveis**, que deve:
-  1. **Receber requerimento** do titular, contendo **firma reconhecida** ou assinatura digital.  
-  2. **Verificar** que o nome lançado no assento não corresponde ao nome apresentado no registro civil (certidão de nascimento, casamento ou registro de estrangeiro).  
-  3. **Retificar o erro à margem** da matrícula, transcrição ou inscrição.
-**Fluxo integrado do pedido**  
-1. **Titular** apresenta requerimento de correção (LGPD – Art. 18) ao órgão competente (Registro de Imóveis).  
-2. **Oficial do Registro** executa a **retificação** prevista no **Art. 1.386** da Norma CGJ‑CE, obedecendo à exigência de documento comprobatório.  
-3. **Responsável pelo tratamento** (controlador ou operador) informa, sem demora, a todos os **agentes de tratamento** envolvidos, conforme **LGPD – § 6º**.  
-4. O titular recebe a confirmação da correção, sem custos, conforme **LGPD – § 5º**.
-**Conclusão**  
-O pedido do titular trata‑se de um **direito de correção** previsto na LGPD, cuja execução prática se dá por meio da **retificação** da matrícula conforme o **Art. 1.386** do Código de Normas CGJ‑CE. Ambas as normas são aplicáveis e complementares.</t>
+          <t>**Procedimento a ser adotado:** **Retificação integral da matrícula**, nos termos do **Art. 1.386 do Código de Normas da CGJ‑CE**, mediante requerimento do titular.  
+---
+### Fundamentação normativa
+1. **Código de Normas CGJ‑CE – Art. 1.386**  
+   &gt; “No que diz respeito à **retificação de dados de qualificação pessoal das partes**, caberá ao Oficial do Registro de Imóveis somente **retificar o erro à margem do registro** (matrícula, transcrição ou inscrição) do nome e estado civil do proprietário, que deverá apresentar requerimento com firma reconhecida ou assinado digitalmente, quando comprovado:  
+   &gt; a) que o nome lançado no assento não corresponde ao nome apresentado no registro civil …;  
+   &gt; b) que se trata do titular do domínio.”
+   → O pedido do titular enquadra‑se exatamente nessa hipótese: correção de dado pessoal (nome/estado civil) constante da matrícula.
+2. **LGPD – Art. 5, inc. I (definição de dado pessoal)**  
+   &gt; “**Dado pessoal**: informação relacionada a pessoa natural identificada ou identificável.”  
+   O nome ou estado civil constante da matrícula são dados pessoais, logo a LGPD reconhece o direito à correção.
+3. **LGPD – Art. 7, inc. VI (tratamento para exercício regular de direitos)**  
+   &gt; “Para o **exercício regular de direitos em processo judicial, administrativo ou arbitral**.”  
+   A correção de dados no registro imobiliário é necessária para o exercício de direitos reais sobre o bem.
+4. **LGPD – Art. 18, § 5º**  
+   &gt; “O requerimento referido no § 3º deste artigo será atendido **sem custos para o titular**, nos prazos e nos termos previstos em regulamento.”  
+   Assim, o titular tem direito à correção sem ônus, devendo ser atendido pelo cartório mediante a retificação prevista no art. 1.386.
+---
+### Passos operacionais (conforme Art. 1.386)
+1. **Requerimento do titular** – deverá ser apresentado com **firma reconhecida** ou **assinatura digital**.  
+2. **Documentação comprobatória** – certidão de nascimento, casamento ou registro de estrangeiro, conforme o caso, para demonstrar a divergência entre o dado registrado e o dado constante do registro civil.  
+3. **Análise pelo Oficial** – verificação da autenticidade dos documentos e da pertinência do pedido.  
+4. **Retificação à margem** – inserção da correção na matrícula, transcrição ou inscrição, mantendo a integridade do histórico registral.  
+5. **Comunicação ao titular** – informe de que a retificação foi efetuada, sem custos, nos termos do § 5º do Art. 18 da LGPD.
+---
+### Conclusão
+O pedido de correção de dado pessoal errado na matrícula deve ser **praticado integralmente como retificação registral**, nos termos do **Art. 1.386 do Código de Normas da CGJ‑CE**, atendendo simultaneamente ao direito de correção previsto na LGPD (Art. 5, I; Art. 7, VI; Art. 18, § 5º). Não há necessidade de indeferimento ou de aplicação de “tarjamento protetivo”.</t>
         </is>
       </c>
       <c r="H121" s="8" t="inlineStr">
         <is>
-          <t>LGPD (Lei 13.709/2018), Art. 5:p0; Código de Normas CGJ-CE, Art. 1386:p281; LGPD (Lei 13.709/2018), Art. 7:p0; LGPD (Lei 13.709/2018), Art. 18:p0</t>
+          <t>LGPD (Lei 13.709/2018) — Art. 18:p0; LGPD (Lei 13.709/2018) — Art. 5:p0; Código de Normas CGJ-CE — Art. 1386:p281; LGPD (Lei 13.709/2018) — Art. 7:p0</t>
         </is>
       </c>
       <c r="I121" s="8" t="n">
-        <v>4.27</v>
+        <v>2.83</v>
       </c>
       <c r="J121" s="8" t="n">
-        <v>2314</v>
+        <v>1776</v>
       </c>
       <c r="K121" s="8" t="n">
-        <v>885</v>
+        <v>1081</v>
       </c>
       <c r="L121" s="10">
         <f>IF(COUNT(J121:K121)=2,(J121*Parametros!$B$3+K121*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7451,6 +8390,17 @@
         <v/>
       </c>
       <c r="S121" s="8" t="n"/>
+      <c r="T121" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="U121" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="V121" s="11">
+        <f>IF(AND(ISNUMBER(T121),T121&gt;0),U121/T121,"")</f>
+        <v/>
+      </c>
+      <c r="W121" s="8" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="n">
@@ -7471,32 +8421,46 @@
       </c>
       <c r="E122" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F122" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>Não encontrado no corpus.</t>
+          <t>**Resposta:** Indeferido via Nota Devolutiva.
+**Fundamentação normativa**
+1. **Provimento CNJ 149/2023 – Art. 148**  
+   &gt; “As entidades representativas dos notários e dos registradores poderão firmar convênio com a RFB, as Juntas Comerciais dos estados, o Departamento de Registro Empresarial e Integração (DREI), a Comissão de Valores Mobiliários (CVM) e quaisquer outros órgãos… com o objetivo de manter atualizado o cadastro de que trata esta seção.”  
+   – O dispositivo restringe a celebração de convênios **exclusivamente às entidades representativas dos notários e dos registradores**. Uma empresa privada (imobiliária/fintech) não se enquadra nessa categoria, logo não possui legitimidade para firmar convênio nos termos do art. 148.
+2. **Provimento CNJ 149/2023 – Art. 168**  
+   &gt; “O CNB/CF poderá firmar convênio com a RFB, as Juntas Comerciais dos estados, o Departamento de Registro Empresarial e Integração (DREI), a Comissão de Valores Mobiliários (CVM)… com o objetivo de manter atualizado o cadastro de que trata esta subseção.”  
+   – Também limita a possibilidade de convênio ao **CNB/CF** (Conselho Nacional de Notários e Registradores), não a empresas privadas.
+3. **Provimento CNJ 149/2023 – Art. 334**  
+   &gt; “O acesso dos oficiais de registro de imóveis ao Programa Gerador e Validador será feito mediante certificado digital ICP‑Brasil ou comunicação por Application Programming Interface (API).”  
+   – O acesso ao PGV está **restrito aos oficiais de registro** (ou prepostos designados), mediante certificado digital ou API, não sendo previsto acesso direto a terceiros que não sejam oficiais ou seus prepostos.
+**Conclusão prática**
+- Não há previsão legal que autorize a celebração de convênio entre o Cartório de Registro de Imóveis e uma empresa privada para fornecimento de dados de matrículas em lote ou via API.  
+- O acesso ao Programa Gerador e Validador (PGV) está limitado a oficiais de registro, mediante certificado digital ou API, conforme art. 334.  
+- Portanto, o pedido de convênio deve ser **indeferido** e formalizado mediante **Nota Devolutiva**, indicando a inexistência de amparo normativo para a celebração do referido convênio.</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
         <is>
-          <t>Provimento CNJ 149/2023, Art. 168:p83; Provimento CNJ 149/2023, Art. 148:p71; Provimento CNJ 149/2023, Art. 184-A:p88; Lei 6.015/1973, Art. 237-A:p0; Provimento CNJ 149/2023, Art. 180:p86</t>
+          <t>Provimento CNJ 149/2023 — Art. 168:p83; Provimento CNJ 149/2023 — Art. 148:p71; Provimento CNJ 149/2023 — Art. 334:p212; Lei 6.015/1973 — Art. 237-A:p0; Código de Normas CGJ-CE — Art. 1167:p237</t>
         </is>
       </c>
       <c r="I122" s="8" t="n">
-        <v>2</v>
+        <v>2.48</v>
       </c>
       <c r="J122" s="8" t="n">
-        <v>2211</v>
+        <v>1615</v>
       </c>
       <c r="K122" s="8" t="n">
-        <v>390</v>
+        <v>911</v>
       </c>
       <c r="L122" s="10">
         <f>IF(COUNT(J122:K122)=2,(J122*Parametros!$B$3+K122*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7512,6 +8476,17 @@
         <v/>
       </c>
       <c r="S122" s="8" t="n"/>
+      <c r="T122" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="U122" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="V122" s="11">
+        <f>IF(AND(ISNUMBER(T122),T122&gt;0),U122/T122,"")</f>
+        <v/>
+      </c>
+      <c r="W122" s="8" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="n">
@@ -7532,47 +8507,47 @@
       </c>
       <c r="E123" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F123" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>**Base legal para o compartilhamento com o ONR/SREI e centrais eletrônicas**
-- **Art. 101** do *Provimento CNJ 149/2023* dispõe que o compartilhamento de dados com centrais de serviços eletrônicos é compatível com a proteção de dados pessoais, devendo as centrais observar:
-  - adequação;
-  - necessidade;
-  - persecução da finalidade dos dados;
-  - maior eficiência e conveniência dos serviços registrais ou notariais ao cidadão.  
-- **Parágrafo único** do mesmo artigo determina preferência pela descentralização das bases de dados, evitando a transferência de bases salvo quando indispensável para a finalidade ou quando questões técnicas comprometerem a eficiência.
-- **Art. 196** do *Código de Normas CGJ‑CE* repete integralmente o conteúdo acima, reforçando a necessidade de adequação, necessidade, finalidade e eficiência, bem como a preferência pela descentralização.
-- **Art. 1.749** do *Código de Normas CGJ‑CE* obriga os responsáveis pelas serventias de registro de imóveis ou pelas centrais de serviços eletrônicos a adotar as medidas necessárias para a integração direta com o representante legal do **ONR – Operador Nacional de Registro Eletrônico de Imóveis**.
+          <t>**Resposta:** O compartilhamento de dados com o Operador Nacional de Registro Eletrônico de Imóveis (ONR) / SREI e com as centrais de serviços eletrônicos pode ser realizado **integralmente**, sem a exigência de consentimento adicional ou de base legal suplementar, desde que observados os requisitos já previstos nos dispositivos normativos citados.
 ---
-### Necessidade de base legal adicional ou de consentimento
-- **Base legal suficiente:** As normas citadas (**Art. 101**, **Parágrafo único**, **Art. 196** e **Art. 1.749**) já constituem a base legal para o compartilhamento de dados entre as serventias/centrais e o ONR/SREI, desde que observados os princípios de adequação, necessidade, finalidade e eficiência.
-- **Consentimento do titular:** Não há exigência expressa de consentimento nos dispositivos acima. Contudo, o tratamento deve respeitar os princípios da LGPD (Lei 13.709/2018). Caso o compartilhamento ultrapasse as finalidades previstas ou envolva dados sensíveis, o consentimento do titular poderá ser necessário conforme a LGPD.
+### Fundamentação normativa
+| Norma | Dispositivo | Conteúdo relevante |
+|-------|-------------|--------------------|
+| **Código de Normas CGJ‑CE** | Art. 1749 | “Os responsáveis pelas serventias de registro de imóveis … adotarão as medidas necessárias para a integração, diretamente com o representante legal do ONR – Operador Nacional de Registro Eletrônico de Imóveis.” |
+| **Provimento CNJ 149/2023** | Art. 101 | “O compartilhamento de dados com centrais de serviços eletrônicos compartilhados é compatível com a proteção de dados pessoais, devendo as centrais observar a adequação, necessidade e persecução da finalidade dos dados a serem compartilhados …” |
+| **Provimento CNJ 149/2023** | Art. 101, parágrafo único | “Deverá ser dada preferência … à modalidade de descentralização das bases de dados … evitando a transferência de bases de dados, salvo quando necessária para atingir a finalidade das centrais …” |
+| **Código de Normas CGJ‑CE** | Art. 196 | Reitera o mesmo princípio do art. 101 do Provimento CNJ 149/2023, reforçando a adequação, necessidade e finalidade como requisitos para o compartilhamento. |
+Esses dispositivos já constituem a **base legal** para o tratamento e o compartilhamento de dados pessoais no âmbito do SREI/ONR e das centrais eletrônicas, atendendo aos princípios da LGPD (adequação, necessidade e finalidade) sem necessidade de consentimento específico do titular, quando o tratamento for indispensável ao cumprimento das finalidades previstas na lei de registros (Lei 6.015/1973) e nos regulamentos citados.
 ---
-**Conclusão:**  
-A legislação citada fornece a base legal para o compartilhamento com o ONR/SREI e as centrais eletrônicas, não sendo exigida outra norma ou consentimento específico, salvo se o tratamento pretender finalidades diferentes das previstas ou envolver dados que, segundo a LGPD, exijam consentimento.</t>
+### Conclusão prática
+- **Ato registral:** pode ser praticado **integralmente**.  
+- **Tarjamento protetivo:** não se impõe, pois a normativa já garante a proteção dos dados mediante os requisitos de adequação, necessidade e finalidade.  
+- **Nota Devolutiva:** indeferimento não se justifica, já que não há exigência de consentimento adicional nem de base legal suplementar.
+**Portanto, o compartilhamento com ONR/SREI e com as centrais eletrônicas está plenamente amparado pelos artigos 1749 do Código de Normas CGJ‑CE, 101 (e seu parágrafo único) do Provimento CNJ 149/2023 e 196 do Código de Normas CGJ‑CE, não sendo necessário obter consentimento ou outra base legal adicional.**</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 1749:p357; Provimento CNJ 149/2023, Art. 101:p51; Provimento CNJ 149/2023, Art. 329-A:p209; Código de Normas CGJ-CE, Art. 196:p68; Provimento CNJ 149/2023, Art. 320-O:p201</t>
+          <t>Código de Normas CGJ-CE — Art. 1749:p357; Provimento CNJ 149/2023 — Art. 101:p51; Código de Normas CGJ-CE — Art. 196:p68; Provimento CNJ 149/2023 — Art. 321:p208; Provimento CNJ 149/2023 — Art. 219:p118</t>
         </is>
       </c>
       <c r="I123" s="8" t="n">
-        <v>4.44</v>
+        <v>2.62</v>
       </c>
       <c r="J123" s="8" t="n">
-        <v>2150</v>
+        <v>1529</v>
       </c>
       <c r="K123" s="8" t="n">
-        <v>996</v>
+        <v>969</v>
       </c>
       <c r="L123" s="10">
         <f>IF(COUNT(J123:K123)=2,(J123*Parametros!$B$3+K123*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7588,6 +8563,17 @@
         <v/>
       </c>
       <c r="S123" s="8" t="n"/>
+      <c r="T123" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="U123" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="V123" s="11">
+        <f>IF(AND(ISNUMBER(T123),T123&gt;0),U123/T123,"")</f>
+        <v/>
+      </c>
+      <c r="W123" s="8" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="n">
@@ -7608,60 +8594,58 @@
       </c>
       <c r="E124" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F124" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>**O que mudou com o Provimento nº 15/2026/CGJCE na qualificação das partes para registro**
----  
-**Art. 1.103 – Requisitos do registro no Livro 2**  
-- **I** — a data;  
-- **II** — a qualificação completa das partes, compreendendo:  
-  - **a)** para pessoa natural:  
-    - estado civil;  
-    - regime de bens do casamento ou da união estável (se declarado no instrumento);  
-    - profissão;  
-    - número de inscrição no CPF ou documento de identidade, ou, à falta deste, sua filiação;  
-  - **b)** para pessoa jurídica:  
-    - denominação social;  
-    - número de inscrição no CNPJ;  
-    - sede;  
-- **III** — o título da transmissão ou do ônus;  
-- **IV** — a forma do título, sua procedência e caracterização;  
-- **V** — o valor do contrato, da coisa ou da dívida, bem como:  
-  - **a)** prazo;  
-  - **b)** condições;  
-  - **c)** encargos;  
-  - **d)** juros;  
-**Parágrafo único** – É vedada a prática de ato registral com:  
-- **a)** qualificação incompleta, genérica ou indeterminada das partes, devendo o oficial recusar o título que não contenha todos os elementos qualificativos exigidos;  
-- **b)** omissão de quaisquer elementos econômicos relevantes do negócio jurídico, não sendo admitido o registro de títulos que contenham estipulações indeterminadas ou incompletas.  
----  
-**Principais mudanças introduzidas pelo Provimento nº 15/2026/CGJCE**  
-- **Obrigatoriedade de qualificação completa** das partes, detalhando explicitamente os elementos exigidos para pessoas naturais e jurídicas.  
-- **Inclusão de um parágrafo único** que proíbe a prática de atos registrais com qualificação incompleta ou genérica e com omissão de elementos econômicos relevantes.  
-- **Reforço da responsabilidade do oficial** de registrar apenas títulos que atendam integralmente a esses requisitos.</t>
+          <t>**O que mudou com o Provimento nº 15/2026/CGJCE na qualificação das partes para registro?**
+O provimento alterou a redação dos requisitos de qualificação das partes no registro, conforme disposto no **Art. 1.103** (Código de Normas CGJ‑CE) e no **Art. 817** (Código de Normas CGJ‑CE).  
+1. **Art. 1.103 – Incisos II e V**  
+   - **Inciso II** passou a exigir, para pessoa natural, a **qualificação completa** que inclui:  
+     - nome, domicílio e nacionalidade;  
+     - **estado civil**;  
+     - **regime de bens do casamento ou da união estável** (se declarado no instrumento);  
+     - **profissão**;  
+     - **número de inscrição no CPF ou documento de identidade**; ou, na falta deste, a **filiação**.  
+   - Para pessoa jurídica, a qualificação deve conter:  
+     - **denominação social**;  
+     - **número de inscrição no CNPJ**;  
+     - **sede**.  
+   - **Inciso V** passou a exigir, além do valor do contrato, da coisa ou da dívida, a informação de:  
+     - prazo;  
+     - condições;  
+     - encargos;  
+     - juros.  
+2. **Parágrafo único do Art. 1.103**  
+   - Foi incluído um parágrafo único que **venda a prática de ato registral** com determinados requisitos não atendidos (ex.: ausência de qualificação completa, falta de regime de bens declarado, etc.).  
+3. **Art. 817 – Alínea “a” do Inciso I**  
+   - A redação da alínea “a” do inciso I do art. 817 foi revista para reforçar a obrigatoriedade de incluir, para pessoa física, nacionalidade, estado civil, profissão, número do documento de identidade e repartição expedidora, número de inscrição no CPF, filiação, domicílio e residência, nome do cônjuge ou companheiro (quando for o caso) e regime de bens do casamento ou da união estável (se declarado pelas partes).  
+**Resumo da mudança:**  
+O provimento ampliou e detalhou a qualificação das partes, exigindo a inclusão de estado civil, regime de bens, profissão, CPF ou identidade (ou filiação) para pessoas físicas, e denominação, CNPJ e sede para pessoas jurídicas, além de reforçar a obrigatoriedade de registrar o regime de bens declarado. O parágrafo único agora proíbe a prática de atos registrais que não atendam a esses requisitos.  
+**Dispositivos citados:**  
+- Art. 1.103, incisos II e V, parágrafo único (Código de Normas CGJ‑CE).  
+- Art. 817, alínea “a” do inciso I (Código de Normas CGJ‑CE).</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
         <is>
-          <t>Provimento 15/2026/CGJCE, Art. 1:p2; Provimento 15/2026/CGJCE, Preâmbulo:p1; Código de Normas CGJ-CE, Art. 1103:p224</t>
+          <t>Provimento 15/2026/CGJCE — Art. 1:p2; Provimento 15/2026/CGJCE — Preâmbulo:p1; Código de Normas CGJ-CE — Art. 1103:p224</t>
         </is>
       </c>
       <c r="I124" s="8" t="n">
-        <v>11.67</v>
+        <v>9.35</v>
       </c>
       <c r="J124" s="8" t="n">
-        <v>2128</v>
+        <v>1500</v>
       </c>
       <c r="K124" s="8" t="n">
-        <v>920</v>
+        <v>1475</v>
       </c>
       <c r="L124" s="10">
         <f>IF(COUNT(J124:K124)=2,(J124*Parametros!$B$3+K124*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7677,6 +8661,21 @@
         <v/>
       </c>
       <c r="S124" s="8" t="n"/>
+      <c r="T124" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="U124" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="V124" s="11">
+        <f>IF(AND(ISNUMBER(T124),T124&gt;0),U124/T124,"")</f>
+        <v/>
+      </c>
+      <c r="W124" s="8" t="inlineStr">
+        <is>
+          <t>Art. 817 (Código de Normas CGJ-CE) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]; Art. 817 (norma não informada) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="7" t="n">
@@ -7697,38 +8696,47 @@
       </c>
       <c r="E125" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F125" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>**Requisitos para emitir certidão digital segundo o Código de Normas CGJ‑CE**
-- **Art. 1127, I** – O oficial deve **lavrar certidões** em formulário próprio, timbrado e pertinente aos atos praticados, **vedada a utilização de impressos não oficiais**.  
-- **Art. 1127, II** – Deve **fornecer às partes as informações e certidões** nos prazos e hipóteses previstos em lei.  
-- **Art. 1127, § 1º** – Quando assinados com **certificado digital**, os documentos devem atender aos requisitos da **Infraestrutura de Chaves Públicas Brasileira – ICP‑Brasil**.  
-- **Art. 240, § 1º** – As certidões eletrônicas devem ser em **formato PDF/A** ou **XML**, com **certificado digital ICP‑Brasil, tipo A3 ou superior**, assinatura digital em **PKCS#7** e metadados no padrão **Dublin Core (DC)**.  
-- **Art. 1079** – A certidão digital deve ser **emitida e enviada exclusivamente** por meio da **Central de Registro de Títulos e Documentos** dentro de **5 (cinco) dias**.  
-- **Art. 683** – Certidões em forma de relação (ex.: devedores em títulos protestados) podem ser **encaminhadas em meio eletrônico** com **certificado digital ICP‑Brasil**.</t>
+          <t>**Requisitos para emissão de certidão digital (Código de Normas CGJ‑CE)**  
+| Requisito | Dispositivo legal | Observação |
+|-----------|-------------------|------------|
+| **Uso de formulário próprio, timbrado e oficial** | Art. 1127, § 1º, inciso I | A certidão deve ser lavrada em formulário próprio, timbrado e pertinente ao ato praticado, vedada a utilização de impressos não oficiais. |
+| **Formato digital nativo** | Art. 1129 | Certidões de imóveis já objeto de matrícula eletrônica, após a “primeira qualificação eletrônica”, são expedidas em formato nativo‑digital estruturado, contendo a situação jurídica atual do imóvel (descrição, titularidade e ônus reais não cancelados). |
+| **Assinatura eletrônica com certificado ICP‑Brasil** | Art. 1127, § 1º, Parágrafo único | Documentos assinados com certificado digital, realizados e/ou enviados pela Internet, devem atender aos requisitos da Infraestrutura de Chaves Públicas Brasileira (ICP‑Brasil). |
+| **Carimbo de tempo (timestamp)** | Art. 140, § 3º | A escrituração dos livros em formato digital deve incluir carimbo de tempo, além de assinatura eletrônica com certificado ICP‑Brasil. |
+| **Armazenamento e backup** | Art. 140, § 3º | O arquivo digital deve ser mantido na própria serventia e submetido à cópia de segurança (backup) regular. |
+| **Indicação de finalidade e identificação do solicitante** | Art. 1128, § 3º e § 4º | Fichas físicas ou digitais contendo dados de identificação e indicação de finalidade devem ser formadas; o titular pode requisitar as informações. O oficial pode recusar o fornecimento se houver tentativa de tratamento de dados em desacordo com as finalidades do Registro de Imóveis e os princípios da LGPD. |
+**Resumo**  
+Para emitir uma certidão digital, o oficial deve:  
+1. Utilizar formulário próprio, timbrado e oficial;  
+2. Emitir a certidão em formato nativo‑digital estruturado (para imóveis já eletrônicos, após a primeira qualificação);  
+3. Assinar eletronicamente com certificado ICP‑Brasil e incluir carimbo de tempo;  
+4. Armazenar o arquivo na serventia e manter backup;  
+5. Garantir que a ficha ou prontuário contenha identificação do solicitante e indicação de finalidade, respeitando a LGPD.</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 1127:p229; Código de Normas CGJ-CE, Art. 1077:p218; Código de Normas CGJ-CE, Art. 240:p75; Código de Normas CGJ-CE, Art. 1079:p218; Código de Normas CGJ-CE, Art. 683:p152</t>
+          <t>Código de Normas CGJ-CE — Art. 1127:p229; Código de Normas CGJ-CE — Art. 1128:p229; Código de Normas CGJ-CE — Art. 1685:p345; Código de Normas CGJ-CE — Art. 1129:p229; Código de Normas CGJ-CE — Art. 140:p58</t>
         </is>
       </c>
       <c r="I125" s="8" t="n">
-        <v>17.73</v>
+        <v>14.18</v>
       </c>
       <c r="J125" s="8" t="n">
-        <v>1806</v>
+        <v>1281</v>
       </c>
       <c r="K125" s="8" t="n">
-        <v>899</v>
+        <v>1009</v>
       </c>
       <c r="L125" s="10">
         <f>IF(COUNT(J125:K125)=2,(J125*Parametros!$B$3+K125*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7744,6 +8752,17 @@
         <v/>
       </c>
       <c r="S125" s="8" t="n"/>
+      <c r="T125" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="U125" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="V125" s="11">
+        <f>IF(AND(ISNUMBER(T125),T125&gt;0),U125/T125,"")</f>
+        <v/>
+      </c>
+      <c r="W125" s="8" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="n">
@@ -7764,45 +8783,44 @@
       </c>
       <c r="E126" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F126" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (ea25525)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
         </is>
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>**Obrigações da serventia ao enviar uma certidão com dados pessoais ao e‑mail errado**
-**Art. 178.**  
-- **Caput** – Os responsáveis pelas serventias extrajudiciais devem atender às disposições da **Lei Geral de Proteção de Dados Pessoais (LGPD)**, obedecendo a seus fundamentos, princípios e obrigações concernentes à governança do tratamento de dados pessoais.  
-**Art. 97.**  
-- **Parágrafo único** – Deve disponibilizar, de forma adequada, informações sobre os procedimentos de tratamento de dados pessoais, nos termos do art. 9.º da LGPD, por meio de:  
-  - **I** — aviso de privacidade e proteção de dados;  
-  - **II** — avisos de cookies no portal de cada serventia, se houver;  
-  - **III** — aviso de privacidade para navegação no website da serventia, se houver.  
-**Art. 189.**  
-- **Parágrafo único** – O responsável pela serventia extrajudicial pode solicitar apoio à entidade de classe para capacitação de seus prepostos, garantindo que todos os envolvidos no tratamento de dados pessoais estejam aptos a cumprir as normas e procedimentos de privacidade.  
-**Práticas adicionais (conforme LGPD)**  
-- Corrigir o envio indevido, garantindo que os dados pessoais sejam devolvidos ou excluídos do destinatário incorreto.  
-- Notificar a pessoa física afetada sobre o incidente, se houver risco de violação de seus direitos.  
-- Registrar o incidente e adotar medidas de mitigação, conforme exigido pela LGPD.</t>
+          <t>**Obrigação da serventia**
+O envio indevido de uma certidão contendo dados pessoais exige que a serventia:
+1. **Corrija imediatamente o erro** – remova a certidão do e‑mail errado e envie-a ao destinatário correto.  
+   *Art. 103 do Provimento CNJ 149/2023* – “O responsável pela serventia extrajudicial efetuará, sempre que possível, a criptografia ou a pseudonimização de dados pessoais para o acesso a informações ou transferência dos dados para terceiros.”
+2. **Implemente medidas de proteção** – caso a correção não seja imediata, a serventia deve criptografar ou pseudonimizar os dados antes de reenviá‑los, garantindo que a informação não seja acessível a terceiros não autorizados.  
+   *Art. 103 do Provimento CNJ 149/2023* (mesma referência acima).
+3. **Notifique o destinatário original** – informe ao e‑mail que recebeu a certidão por engano que o documento foi enviado erroneamente e que os dados não devem ser utilizados ou divulgados.  
+   *Art. 178 do Código de Normas CGJ‑CE* – “Os responsáveis pelas serventias extrajudiciais deverão atender às disposições da Lei Geral de Proteção de Dados Pessoais (LGPD) … obedecendo a seus fundamentos, princípios e obrigações concernentes à governança do tratamento de dados pessoais.”
+4. **Forneça transparência** – disponibilize, conforme Art. 97 do Provimento CNJ 149/2023, avisos de privacidade e proteção de dados, explicando o ocorrido e as medidas adotadas.  
+   *Art. 97 do Provimento CNJ 149/2023* – “Deverão ser disponibilizadas pelos responsáveis pelas serventias informações adequadas a respeito dos procedimentos de tratamento de dados pessoais, nos termos do art. 9.º da LGPD, por meio de: I — aviso de privacidade e proteção de dados; …”
+5. **Registre o incidente** – documente a ocorrência e as ações corretivas, para eventual auditoria ou verificação pelo corregedor permanente.  
+   *Art. 105 do Provimento CNJ 149/2023* – “Na correição anual será verificada pelo corregedor permanente a adaptação de suas práticas de tratamento de dados pessoais à LGPD e a este Código de Normas.”
+Em síntese, a serventia deve praticar a correção integral do ato, aplicando criptografia ou pseudonimização quando possível, notificando o destinatário original, garantindo transparência e registrando o incidente, em conformidade com os dispositivos citados.</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
         <is>
-          <t>Código de Normas CGJ-CE, Art. 178:p65; Código de Normas CGJ-CE, Art. 189:p67; Provimento CNJ 149/2023, Art. 236:p142; Provimento CNJ 149/2023, Art. 97:p50; Código de Normas CGJ-CE, Art. 564:p133</t>
+          <t>Provimento CNJ 149/2023 — Art. 103:p52; Provimento CNJ 149/2023 — Art. 105:p52; Provimento CNJ 149/2023 — Art. 100:p51; Código de Normas CGJ-CE — Art. 178:p65; Provimento CNJ 149/2023 — Art. 97:p50</t>
         </is>
       </c>
       <c r="I126" s="8" t="n">
-        <v>18.66</v>
+        <v>18.64</v>
       </c>
       <c r="J126" s="8" t="n">
-        <v>1708</v>
+        <v>1276</v>
       </c>
       <c r="K126" s="8" t="n">
-        <v>1302</v>
+        <v>1363</v>
       </c>
       <c r="L126" s="10">
         <f>IF(COUNT(J126:K126)=2,(J126*Parametros!$B$3+K126*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7818,9 +8836,24 @@
         <v/>
       </c>
       <c r="S126" s="8" t="n"/>
+      <c r="T126" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="U126" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="V126" s="11">
+        <f>IF(AND(ISNUMBER(T126),T126&gt;0),U126/T126,"")</f>
+        <v/>
+      </c>
+      <c r="W126" s="8" t="inlineStr">
+        <is>
+          <t>Art. 9 (LGPD (Lei 13.709/2018)) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S126"/>
+  <autoFilter ref="A1:W126"/>
   <conditionalFormatting sqref="R2:R126">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>8</formula>
@@ -7970,7 +9003,7 @@
       </c>
       <c r="B10" s="8" t="n"/>
       <c r="C10" s="8" t="n"/>
-      <c r="D10" s="11">
+      <c r="D10" s="12">
         <f>IF(AND(ISNUMBER(B10),ISNUMBER(C10),C10&gt;0),B10/C10,"")</f>
         <v/>
       </c>
@@ -7983,7 +9016,7 @@
       </c>
       <c r="B11" s="8" t="n"/>
       <c r="C11" s="8" t="n"/>
-      <c r="D11" s="11">
+      <c r="D11" s="12">
         <f>IF(AND(ISNUMBER(B11),ISNUMBER(C11),C11&gt;0),B11/C11,"")</f>
         <v/>
       </c>
@@ -7996,7 +9029,7 @@
       </c>
       <c r="B12" s="8" t="n"/>
       <c r="C12" s="8" t="n"/>
-      <c r="D12" s="11">
+      <c r="D12" s="12">
         <f>IF(AND(ISNUMBER(B12),ISNUMBER(C12),C12&gt;0),B12/C12,"")</f>
         <v/>
       </c>
@@ -8019,7 +9052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8033,6 +9066,7 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8098,6 +9132,11 @@
           <t>Custo / consulta (R$)</t>
         </is>
       </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Taxa verificável (citações)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -8109,35 +9148,35 @@
         <f>COUNTIFS(Respostas!$B$2:$B$126,$A4,Respostas!$R$2:$R$126,"&gt;=0")</f>
         <v/>
       </c>
-      <c r="C4" s="11">
+      <c r="C4" s="12">
         <f>IF(B4=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,$A4))</f>
         <v/>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="12">
         <f>IF(B4=0,"",AVERAGEIFS(Respostas!$M$2:$M$126,Respostas!$B$2:$B$126,$A4,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="12">
         <f>IF(B4=0,"",AVERAGEIFS(Respostas!$N$2:$N$126,Respostas!$B$2:$B$126,$A4,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="12">
         <f>IF(B4=0,"",AVERAGEIFS(Respostas!$O$2:$O$126,Respostas!$B$2:$B$126,$A4,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="12">
         <f>IF(B4=0,"",AVERAGEIFS(Respostas!$P$2:$P$126,Respostas!$B$2:$B$126,$A4,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="12">
         <f>IF(B4=0,"",AVERAGEIFS(Respostas!$Q$2:$Q$126,Respostas!$B$2:$B$126,$A4,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="I4" s="12">
+      <c r="I4" s="11">
         <f>IF(B4=0,"",COUNTIFS(Respostas!$B$2:$B$126,$A4,Respostas!$R$2:$R$126,"&gt;=8")/B4)</f>
         <v/>
       </c>
-      <c r="J4" s="11">
+      <c r="J4" s="12">
         <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A4,Respostas!$I$2:$I$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$I$2:$I$126,Respostas!$B$2:$B$126,$A4))</f>
         <v/>
       </c>
@@ -8145,6 +9184,10 @@
         <f>IF(ISNUMBER(Parametros!$D$10),Parametros!$D$10,"")</f>
         <v/>
       </c>
+      <c r="L4" s="11">
+        <f>IF(SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A4)=0,"",SUMIFS(Respostas!$U$2:$U$126,Respostas!$B$2:$B$126,$A4)/SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A4))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -8156,35 +9199,35 @@
         <f>COUNTIFS(Respostas!$B$2:$B$126,$A5,Respostas!$R$2:$R$126,"&gt;=0")</f>
         <v/>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="12">
         <f>IF(B5=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,$A5))</f>
         <v/>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="12">
         <f>IF(B5=0,"",AVERAGEIFS(Respostas!$M$2:$M$126,Respostas!$B$2:$B$126,$A5,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="12">
         <f>IF(B5=0,"",AVERAGEIFS(Respostas!$N$2:$N$126,Respostas!$B$2:$B$126,$A5,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="12">
         <f>IF(B5=0,"",AVERAGEIFS(Respostas!$O$2:$O$126,Respostas!$B$2:$B$126,$A5,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="12">
         <f>IF(B5=0,"",AVERAGEIFS(Respostas!$P$2:$P$126,Respostas!$B$2:$B$126,$A5,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="12">
         <f>IF(B5=0,"",AVERAGEIFS(Respostas!$Q$2:$Q$126,Respostas!$B$2:$B$126,$A5,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="I5" s="12">
+      <c r="I5" s="11">
         <f>IF(B5=0,"",COUNTIFS(Respostas!$B$2:$B$126,$A5,Respostas!$R$2:$R$126,"&gt;=8")/B5)</f>
         <v/>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="12">
         <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A5,Respostas!$I$2:$I$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$I$2:$I$126,Respostas!$B$2:$B$126,$A5))</f>
         <v/>
       </c>
@@ -8192,6 +9235,10 @@
         <f>IF(ISNUMBER(Parametros!$D$11),Parametros!$D$11,"")</f>
         <v/>
       </c>
+      <c r="L5" s="11">
+        <f>IF(SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A5)=0,"",SUMIFS(Respostas!$U$2:$U$126,Respostas!$B$2:$B$126,$A5)/SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A5))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -8203,35 +9250,35 @@
         <f>COUNTIFS(Respostas!$B$2:$B$126,$A6,Respostas!$R$2:$R$126,"&gt;=0")</f>
         <v/>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="12">
         <f>IF(B6=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,$A6))</f>
         <v/>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="12">
         <f>IF(B6=0,"",AVERAGEIFS(Respostas!$M$2:$M$126,Respostas!$B$2:$B$126,$A6,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="12">
         <f>IF(B6=0,"",AVERAGEIFS(Respostas!$N$2:$N$126,Respostas!$B$2:$B$126,$A6,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="12">
         <f>IF(B6=0,"",AVERAGEIFS(Respostas!$O$2:$O$126,Respostas!$B$2:$B$126,$A6,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="12">
         <f>IF(B6=0,"",AVERAGEIFS(Respostas!$P$2:$P$126,Respostas!$B$2:$B$126,$A6,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="12">
         <f>IF(B6=0,"",AVERAGEIFS(Respostas!$Q$2:$Q$126,Respostas!$B$2:$B$126,$A6,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="I6" s="12">
+      <c r="I6" s="11">
         <f>IF(B6=0,"",COUNTIFS(Respostas!$B$2:$B$126,$A6,Respostas!$R$2:$R$126,"&gt;=8")/B6)</f>
         <v/>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="12">
         <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A6,Respostas!$I$2:$I$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$I$2:$I$126,Respostas!$B$2:$B$126,$A6))</f>
         <v/>
       </c>
@@ -8239,6 +9286,10 @@
         <f>IF(ISNUMBER(Parametros!$D$12),Parametros!$D$12,"")</f>
         <v/>
       </c>
+      <c r="L6" s="11">
+        <f>IF(SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A6)=0,"",SUMIFS(Respostas!$U$2:$U$126,Respostas!$B$2:$B$126,$A6)/SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A6))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -8250,35 +9301,35 @@
         <f>COUNTIFS(Respostas!$B$2:$B$126,$A7,Respostas!$R$2:$R$126,"&gt;=0")</f>
         <v/>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="12">
         <f>IF(B7=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,$A7))</f>
         <v/>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="12">
         <f>IF(B7=0,"",AVERAGEIFS(Respostas!$M$2:$M$126,Respostas!$B$2:$B$126,$A7,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="12">
         <f>IF(B7=0,"",AVERAGEIFS(Respostas!$N$2:$N$126,Respostas!$B$2:$B$126,$A7,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="12">
         <f>IF(B7=0,"",AVERAGEIFS(Respostas!$O$2:$O$126,Respostas!$B$2:$B$126,$A7,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="12">
         <f>IF(B7=0,"",AVERAGEIFS(Respostas!$P$2:$P$126,Respostas!$B$2:$B$126,$A7,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="12">
         <f>IF(B7=0,"",AVERAGEIFS(Respostas!$Q$2:$Q$126,Respostas!$B$2:$B$126,$A7,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="I7" s="12">
+      <c r="I7" s="11">
         <f>IF(B7=0,"",COUNTIFS(Respostas!$B$2:$B$126,$A7,Respostas!$R$2:$R$126,"&gt;=8")/B7)</f>
         <v/>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="12">
         <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A7,Respostas!$I$2:$I$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$I$2:$I$126,Respostas!$B$2:$B$126,$A7))</f>
         <v/>
       </c>
@@ -8286,6 +9337,10 @@
         <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A7,Respostas!$L$2:$L$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$L$2:$L$126,Respostas!$B$2:$B$126,$A7))</f>
         <v/>
       </c>
+      <c r="L7" s="11">
+        <f>IF(SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A7)=0,"",SUMIFS(Respostas!$U$2:$U$126,Respostas!$B$2:$B$126,$A7)/SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A7))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -8297,35 +9352,35 @@
         <f>COUNTIFS(Respostas!$B$2:$B$126,$A8,Respostas!$R$2:$R$126,"&gt;=0")</f>
         <v/>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="12">
         <f>IF(B8=0,"",AVERAGEIFS(Respostas!$R$2:$R$126,Respostas!$B$2:$B$126,$A8))</f>
         <v/>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="12">
         <f>IF(B8=0,"",AVERAGEIFS(Respostas!$M$2:$M$126,Respostas!$B$2:$B$126,$A8,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="12">
         <f>IF(B8=0,"",AVERAGEIFS(Respostas!$N$2:$N$126,Respostas!$B$2:$B$126,$A8,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="12">
         <f>IF(B8=0,"",AVERAGEIFS(Respostas!$O$2:$O$126,Respostas!$B$2:$B$126,$A8,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="12">
         <f>IF(B8=0,"",AVERAGEIFS(Respostas!$P$2:$P$126,Respostas!$B$2:$B$126,$A8,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="12">
         <f>IF(B8=0,"",AVERAGEIFS(Respostas!$Q$2:$Q$126,Respostas!$B$2:$B$126,$A8,Respostas!$R$2:$R$126,"&gt;=0"))</f>
         <v/>
       </c>
-      <c r="I8" s="12">
+      <c r="I8" s="11">
         <f>IF(B8=0,"",COUNTIFS(Respostas!$B$2:$B$126,$A8,Respostas!$R$2:$R$126,"&gt;=8")/B8)</f>
         <v/>
       </c>
-      <c r="J8" s="11">
+      <c r="J8" s="12">
         <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A8,Respostas!$I$2:$I$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$I$2:$I$126,Respostas!$B$2:$B$126,$A8))</f>
         <v/>
       </c>
@@ -8333,6 +9388,10 @@
         <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A8,Respostas!$L$2:$L$126,"&gt;=0")=0,"",AVERAGEIFS(Respostas!$L$2:$L$126,Respostas!$B$2:$B$126,$A8))</f>
         <v/>
       </c>
+      <c r="L8" s="11">
+        <f>IF(SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A8)=0,"",SUMIFS(Respostas!$U$2:$U$126,Respostas!$B$2:$B$126,$A8)/SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A8))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -8347,7 +9406,7 @@
           <t>Melhor concorrente</t>
         </is>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="12">
         <f>IF(COUNT(C4,C5,C6)=0,"",MAX(C4,C5,C6))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
fix: trata resposta vazia do LLM em vez de contá-la como respondida
- _call_chat_completions detecta finish_reason "length" ou conteúdo
  vazio (exceto tool_calls) e faz UMA nova tentativa com o modelo
  premium (gpt-oss-120b na Groq) e max_tokens=8192
- se falhar de novo, lança RespostaVaziaError; o answer() da Fase 3
  devolve resultado marcado com status RESPOSTA_VAZIA
- benchmark separa RESPONDIDA, NAO_ENCONTRADO, RESPOSTA_VAZIA e ERRO
  (JSON, terminal, coluna X e contagens no Resumo); a contagem de
  tokens inclui a nova tentativa
- reclassificação da execução de 13/10 11h: 4 respostas vazias
  (#5, #7, #18, #19, todas gpt-oss-20b com 2048 tokens) que antes
  contavam como respondidas
</commit_message>
<xml_diff>
--- a/docs/fase3/benchmark/planilha_benchmark.xlsx
+++ b/docs/fase3/benchmark/planilha_benchmark.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Respostas'!$A$1:$W$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Respostas'!$A$1:$X$126</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1459,7 +1459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W126"/>
+  <dimension ref="A1:X126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1485,6 +1485,7 @@
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="11" customWidth="1" min="22" max="22"/>
     <col width="50" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1601,6 +1602,11 @@
       <c r="W1" s="6" t="inlineStr">
         <is>
           <t>Citações não verificadas</t>
+        </is>
+      </c>
+      <c r="X1" s="6" t="inlineStr">
+        <is>
+          <t>Status da resposta</t>
         </is>
       </c>
     </row>
@@ -1649,6 +1655,7 @@
         <v/>
       </c>
       <c r="W2" s="8" t="n"/>
+      <c r="X2" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -1695,6 +1702,7 @@
         <v/>
       </c>
       <c r="W3" s="8" t="n"/>
+      <c r="X3" s="8" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -1741,6 +1749,7 @@
         <v/>
       </c>
       <c r="W4" s="8" t="n"/>
+      <c r="X4" s="8" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -1787,6 +1796,7 @@
         <v/>
       </c>
       <c r="W5" s="8" t="n"/>
+      <c r="X5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -1833,6 +1843,7 @@
         <v/>
       </c>
       <c r="W6" s="8" t="n"/>
+      <c r="X6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -1879,6 +1890,7 @@
         <v/>
       </c>
       <c r="W7" s="8" t="n"/>
+      <c r="X7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -1925,6 +1937,7 @@
         <v/>
       </c>
       <c r="W8" s="8" t="n"/>
+      <c r="X8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -1971,6 +1984,7 @@
         <v/>
       </c>
       <c r="W9" s="8" t="n"/>
+      <c r="X9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -2017,6 +2031,7 @@
         <v/>
       </c>
       <c r="W10" s="8" t="n"/>
+      <c r="X10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -2063,6 +2078,7 @@
         <v/>
       </c>
       <c r="W11" s="8" t="n"/>
+      <c r="X11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -2109,6 +2125,7 @@
         <v/>
       </c>
       <c r="W12" s="8" t="n"/>
+      <c r="X12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -2155,6 +2172,7 @@
         <v/>
       </c>
       <c r="W13" s="8" t="n"/>
+      <c r="X13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -2201,6 +2219,7 @@
         <v/>
       </c>
       <c r="W14" s="8" t="n"/>
+      <c r="X14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -2247,6 +2266,7 @@
         <v/>
       </c>
       <c r="W15" s="8" t="n"/>
+      <c r="X15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -2293,6 +2313,7 @@
         <v/>
       </c>
       <c r="W16" s="8" t="n"/>
+      <c r="X16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -2339,6 +2360,7 @@
         <v/>
       </c>
       <c r="W17" s="8" t="n"/>
+      <c r="X17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -2385,6 +2407,7 @@
         <v/>
       </c>
       <c r="W18" s="8" t="n"/>
+      <c r="X18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -2431,6 +2454,7 @@
         <v/>
       </c>
       <c r="W19" s="8" t="n"/>
+      <c r="X19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -2477,6 +2501,7 @@
         <v/>
       </c>
       <c r="W20" s="8" t="n"/>
+      <c r="X20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -2523,6 +2548,7 @@
         <v/>
       </c>
       <c r="W21" s="8" t="n"/>
+      <c r="X21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -2569,6 +2595,7 @@
         <v/>
       </c>
       <c r="W22" s="8" t="n"/>
+      <c r="X22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
@@ -2615,6 +2642,7 @@
         <v/>
       </c>
       <c r="W23" s="8" t="n"/>
+      <c r="X23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -2661,6 +2689,7 @@
         <v/>
       </c>
       <c r="W24" s="8" t="n"/>
+      <c r="X24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
@@ -2707,6 +2736,7 @@
         <v/>
       </c>
       <c r="W25" s="8" t="n"/>
+      <c r="X25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
@@ -2753,6 +2783,7 @@
         <v/>
       </c>
       <c r="W26" s="8" t="n"/>
+      <c r="X26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
@@ -2799,6 +2830,7 @@
         <v/>
       </c>
       <c r="W27" s="8" t="n"/>
+      <c r="X27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
@@ -2845,6 +2877,7 @@
         <v/>
       </c>
       <c r="W28" s="8" t="n"/>
+      <c r="X28" s="8" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
@@ -2891,6 +2924,7 @@
         <v/>
       </c>
       <c r="W29" s="8" t="n"/>
+      <c r="X29" s="8" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
@@ -2937,6 +2971,7 @@
         <v/>
       </c>
       <c r="W30" s="8" t="n"/>
+      <c r="X30" s="8" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
@@ -2983,6 +3018,7 @@
         <v/>
       </c>
       <c r="W31" s="8" t="n"/>
+      <c r="X31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
@@ -3029,6 +3065,7 @@
         <v/>
       </c>
       <c r="W32" s="8" t="n"/>
+      <c r="X32" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
@@ -3075,6 +3112,7 @@
         <v/>
       </c>
       <c r="W33" s="8" t="n"/>
+      <c r="X33" s="8" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
@@ -3121,6 +3159,7 @@
         <v/>
       </c>
       <c r="W34" s="8" t="n"/>
+      <c r="X34" s="8" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
@@ -3167,6 +3206,7 @@
         <v/>
       </c>
       <c r="W35" s="8" t="n"/>
+      <c r="X35" s="8" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
@@ -3213,6 +3253,7 @@
         <v/>
       </c>
       <c r="W36" s="8" t="n"/>
+      <c r="X36" s="8" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n">
@@ -3259,6 +3300,7 @@
         <v/>
       </c>
       <c r="W37" s="8" t="n"/>
+      <c r="X37" s="8" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n">
@@ -3305,6 +3347,7 @@
         <v/>
       </c>
       <c r="W38" s="8" t="n"/>
+      <c r="X38" s="8" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n">
@@ -3351,6 +3394,7 @@
         <v/>
       </c>
       <c r="W39" s="8" t="n"/>
+      <c r="X39" s="8" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n">
@@ -3397,6 +3441,7 @@
         <v/>
       </c>
       <c r="W40" s="8" t="n"/>
+      <c r="X40" s="8" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="n">
@@ -3443,6 +3488,7 @@
         <v/>
       </c>
       <c r="W41" s="8" t="n"/>
+      <c r="X41" s="8" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n">
@@ -3489,6 +3535,7 @@
         <v/>
       </c>
       <c r="W42" s="8" t="n"/>
+      <c r="X42" s="8" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="n">
@@ -3535,6 +3582,7 @@
         <v/>
       </c>
       <c r="W43" s="8" t="n"/>
+      <c r="X43" s="8" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
@@ -3581,6 +3629,7 @@
         <v/>
       </c>
       <c r="W44" s="8" t="n"/>
+      <c r="X44" s="8" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n">
@@ -3627,6 +3676,7 @@
         <v/>
       </c>
       <c r="W45" s="8" t="n"/>
+      <c r="X45" s="8" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n">
@@ -3673,6 +3723,7 @@
         <v/>
       </c>
       <c r="W46" s="8" t="n"/>
+      <c r="X46" s="8" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="n">
@@ -3719,6 +3770,7 @@
         <v/>
       </c>
       <c r="W47" s="8" t="n"/>
+      <c r="X47" s="8" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n">
@@ -3765,6 +3817,7 @@
         <v/>
       </c>
       <c r="W48" s="8" t="n"/>
+      <c r="X48" s="8" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="n">
@@ -3811,6 +3864,7 @@
         <v/>
       </c>
       <c r="W49" s="8" t="n"/>
+      <c r="X49" s="8" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="n">
@@ -3857,6 +3911,7 @@
         <v/>
       </c>
       <c r="W50" s="8" t="n"/>
+      <c r="X50" s="8" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="n">
@@ -3903,6 +3958,7 @@
         <v/>
       </c>
       <c r="W51" s="8" t="n"/>
+      <c r="X51" s="8" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n">
@@ -3949,6 +4005,7 @@
         <v/>
       </c>
       <c r="W52" s="8" t="n"/>
+      <c r="X52" s="8" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="n">
@@ -3995,6 +4052,7 @@
         <v/>
       </c>
       <c r="W53" s="8" t="n"/>
+      <c r="X53" s="8" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="n">
@@ -4041,6 +4099,7 @@
         <v/>
       </c>
       <c r="W54" s="8" t="n"/>
+      <c r="X54" s="8" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="n">
@@ -4087,6 +4146,7 @@
         <v/>
       </c>
       <c r="W55" s="8" t="n"/>
+      <c r="X55" s="8" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="n">
@@ -4133,6 +4193,7 @@
         <v/>
       </c>
       <c r="W56" s="8" t="n"/>
+      <c r="X56" s="8" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="n">
@@ -4179,6 +4240,7 @@
         <v/>
       </c>
       <c r="W57" s="8" t="n"/>
+      <c r="X57" s="8" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="n">
@@ -4225,6 +4287,7 @@
         <v/>
       </c>
       <c r="W58" s="8" t="n"/>
+      <c r="X58" s="8" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="n">
@@ -4271,6 +4334,7 @@
         <v/>
       </c>
       <c r="W59" s="8" t="n"/>
+      <c r="X59" s="8" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="n">
@@ -4317,6 +4381,7 @@
         <v/>
       </c>
       <c r="W60" s="8" t="n"/>
+      <c r="X60" s="8" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="n">
@@ -4363,6 +4428,7 @@
         <v/>
       </c>
       <c r="W61" s="8" t="n"/>
+      <c r="X61" s="8" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="n">
@@ -4409,6 +4475,7 @@
         <v/>
       </c>
       <c r="W62" s="8" t="n"/>
+      <c r="X62" s="8" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="n">
@@ -4455,6 +4522,7 @@
         <v/>
       </c>
       <c r="W63" s="8" t="n"/>
+      <c r="X63" s="8" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="n">
@@ -4501,6 +4569,7 @@
         <v/>
       </c>
       <c r="W64" s="8" t="n"/>
+      <c r="X64" s="8" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="n">
@@ -4547,6 +4616,7 @@
         <v/>
       </c>
       <c r="W65" s="8" t="n"/>
+      <c r="X65" s="8" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="n">
@@ -4593,6 +4663,7 @@
         <v/>
       </c>
       <c r="W66" s="8" t="n"/>
+      <c r="X66" s="8" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="n">
@@ -4639,6 +4710,7 @@
         <v/>
       </c>
       <c r="W67" s="8" t="n"/>
+      <c r="X67" s="8" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="n">
@@ -4685,6 +4757,7 @@
         <v/>
       </c>
       <c r="W68" s="8" t="n"/>
+      <c r="X68" s="8" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="n">
@@ -4731,6 +4804,7 @@
         <v/>
       </c>
       <c r="W69" s="8" t="n"/>
+      <c r="X69" s="8" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="n">
@@ -4777,6 +4851,7 @@
         <v/>
       </c>
       <c r="W70" s="8" t="n"/>
+      <c r="X70" s="8" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="n">
@@ -4823,6 +4898,7 @@
         <v/>
       </c>
       <c r="W71" s="8" t="n"/>
+      <c r="X71" s="8" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="n">
@@ -4869,6 +4945,7 @@
         <v/>
       </c>
       <c r="W72" s="8" t="n"/>
+      <c r="X72" s="8" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="n">
@@ -4915,6 +4992,7 @@
         <v/>
       </c>
       <c r="W73" s="8" t="n"/>
+      <c r="X73" s="8" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="n">
@@ -4961,6 +5039,7 @@
         <v/>
       </c>
       <c r="W74" s="8" t="n"/>
+      <c r="X74" s="8" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="n">
@@ -5007,6 +5086,7 @@
         <v/>
       </c>
       <c r="W75" s="8" t="n"/>
+      <c r="X75" s="8" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="n">
@@ -5053,6 +5133,7 @@
         <v/>
       </c>
       <c r="W76" s="8" t="n"/>
+      <c r="X76" s="8" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="n">
@@ -5121,6 +5202,11 @@
         <v/>
       </c>
       <c r="W77" s="8" t="n"/>
+      <c r="X77" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="7" t="n">
@@ -5189,6 +5275,11 @@
         <v/>
       </c>
       <c r="W78" s="8" t="n"/>
+      <c r="X78" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="7" t="n">
@@ -5257,6 +5348,11 @@
         <v/>
       </c>
       <c r="W79" s="8" t="n"/>
+      <c r="X79" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="7" t="n">
@@ -5325,6 +5421,11 @@
         <v/>
       </c>
       <c r="W80" s="8" t="n"/>
+      <c r="X80" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="7" t="n">
@@ -5393,6 +5494,11 @@
         <v/>
       </c>
       <c r="W81" s="8" t="n"/>
+      <c r="X81" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="7" t="n">
@@ -5461,6 +5567,11 @@
         <v/>
       </c>
       <c r="W82" s="8" t="n"/>
+      <c r="X82" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="7" t="n">
@@ -5529,6 +5640,11 @@
         <v/>
       </c>
       <c r="W83" s="8" t="n"/>
+      <c r="X83" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="7" t="n">
@@ -5597,6 +5713,11 @@
         <v/>
       </c>
       <c r="W84" s="8" t="n"/>
+      <c r="X84" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="7" t="n">
@@ -5686,6 +5807,11 @@
         <v/>
       </c>
       <c r="W85" s="8" t="n"/>
+      <c r="X85" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="7" t="n">
@@ -5754,6 +5880,11 @@
         <v/>
       </c>
       <c r="W86" s="8" t="n"/>
+      <c r="X86" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="7" t="n">
@@ -5822,6 +5953,11 @@
         <v/>
       </c>
       <c r="W87" s="8" t="n"/>
+      <c r="X87" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="7" t="n">
@@ -5890,6 +6026,11 @@
         <v/>
       </c>
       <c r="W88" s="8" t="n"/>
+      <c r="X88" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="7" t="n">
@@ -5958,6 +6099,11 @@
         <v/>
       </c>
       <c r="W89" s="8" t="n"/>
+      <c r="X89" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="7" t="n">
@@ -6026,6 +6172,11 @@
         <v/>
       </c>
       <c r="W90" s="8" t="n"/>
+      <c r="X90" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="7" t="n">
@@ -6103,6 +6254,11 @@
         <v/>
       </c>
       <c r="W91" s="8" t="n"/>
+      <c r="X91" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="7" t="n">
@@ -6171,6 +6327,11 @@
         <v/>
       </c>
       <c r="W92" s="8" t="n"/>
+      <c r="X92" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="7" t="n">
@@ -6239,6 +6400,11 @@
         <v/>
       </c>
       <c r="W93" s="8" t="n"/>
+      <c r="X93" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="7" t="n">
@@ -6307,6 +6473,11 @@
         <v/>
       </c>
       <c r="W94" s="8" t="n"/>
+      <c r="X94" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="7" t="n">
@@ -6378,6 +6549,11 @@
         <v/>
       </c>
       <c r="W95" s="8" t="n"/>
+      <c r="X95" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="7" t="n">
@@ -6464,6 +6640,11 @@
         <v/>
       </c>
       <c r="W96" s="8" t="n"/>
+      <c r="X96" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="7" t="n">
@@ -6532,6 +6713,11 @@
         <v/>
       </c>
       <c r="W97" s="8" t="n"/>
+      <c r="X97" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="7" t="n">
@@ -6615,6 +6801,11 @@
         <v/>
       </c>
       <c r="W98" s="8" t="n"/>
+      <c r="X98" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="7" t="n">
@@ -6683,6 +6874,11 @@
         <v/>
       </c>
       <c r="W99" s="8" t="n"/>
+      <c r="X99" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="7" t="n">
@@ -6751,6 +6947,11 @@
         <v/>
       </c>
       <c r="W100" s="8" t="n"/>
+      <c r="X100" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="7" t="n">
@@ -6819,6 +7020,11 @@
         <v/>
       </c>
       <c r="W101" s="8" t="n"/>
+      <c r="X101" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="7" t="n">
@@ -6908,6 +7114,11 @@
         <v/>
       </c>
       <c r="W102" s="8" t="inlineStr"/>
+      <c r="X102" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="7" t="n">
@@ -6987,6 +7198,11 @@
         <v/>
       </c>
       <c r="W103" s="8" t="inlineStr"/>
+      <c r="X103" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="7" t="n">
@@ -7079,6 +7295,11 @@
           <t>Art. 5 (LGPD (Lei 13.709/2018)) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
         </is>
       </c>
+      <c r="X104" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="n">
@@ -7159,6 +7380,11 @@
         <v/>
       </c>
       <c r="W105" s="8" t="inlineStr"/>
+      <c r="X105" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="7" t="n">
@@ -7227,6 +7453,11 @@
         <v/>
       </c>
       <c r="W106" s="8" t="inlineStr"/>
+      <c r="X106" s="8" t="inlineStr">
+        <is>
+          <t>RESPOSTA_VAZIA</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="7" t="n">
@@ -7299,6 +7530,11 @@
         <v/>
       </c>
       <c r="W107" s="8" t="inlineStr"/>
+      <c r="X107" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="7" t="n">
@@ -7367,6 +7603,11 @@
         <v/>
       </c>
       <c r="W108" s="8" t="inlineStr"/>
+      <c r="X108" s="8" t="inlineStr">
+        <is>
+          <t>RESPOSTA_VAZIA</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="7" t="n">
@@ -7474,6 +7715,11 @@
           <t>Art. 7 (LGPD (Lei 13.709/2018)) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
         </is>
       </c>
+      <c r="X109" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="7" t="n">
@@ -7551,6 +7797,11 @@
         <v/>
       </c>
       <c r="W110" s="8" t="inlineStr"/>
+      <c r="X110" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="7" t="n">
@@ -7623,6 +7874,11 @@
         <v/>
       </c>
       <c r="W111" s="8" t="inlineStr"/>
+      <c r="X111" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="7" t="n">
@@ -7695,6 +7951,11 @@
         <v/>
       </c>
       <c r="W112" s="8" t="inlineStr"/>
+      <c r="X112" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="7" t="n">
@@ -7776,6 +8037,11 @@
           <t>Art. 1 (LAI (Lei 12.527/2011)) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
         </is>
       </c>
+      <c r="X113" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="7" t="n">
@@ -7853,6 +8119,11 @@
         <v/>
       </c>
       <c r="W114" s="8" t="inlineStr"/>
+      <c r="X114" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="7" t="n">
@@ -7936,6 +8207,11 @@
       <c r="W115" s="8" t="inlineStr">
         <is>
           <t>Art. 543 (OUTRA: codigo civil) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
+        </is>
+      </c>
+      <c r="X115" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
         </is>
       </c>
     </row>
@@ -8023,6 +8299,11 @@
         <v/>
       </c>
       <c r="W116" s="8" t="inlineStr"/>
+      <c r="X116" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="7" t="n">
@@ -8095,6 +8376,11 @@
         <v/>
       </c>
       <c r="W117" s="8" t="inlineStr"/>
+      <c r="X117" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="7" t="n">
@@ -8167,6 +8453,11 @@
         <v/>
       </c>
       <c r="W118" s="8" t="inlineStr"/>
+      <c r="X118" s="8" t="inlineStr">
+        <is>
+          <t>NAO_ENCONTRADO</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="7" t="n">
@@ -8235,6 +8526,11 @@
         <v/>
       </c>
       <c r="W119" s="8" t="inlineStr"/>
+      <c r="X119" s="8" t="inlineStr">
+        <is>
+          <t>RESPOSTA_VAZIA</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="7" t="n">
@@ -8303,6 +8599,11 @@
         <v/>
       </c>
       <c r="W120" s="8" t="inlineStr"/>
+      <c r="X120" s="8" t="inlineStr">
+        <is>
+          <t>RESPOSTA_VAZIA</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="7" t="n">
@@ -8401,6 +8702,11 @@
         <v/>
       </c>
       <c r="W121" s="8" t="inlineStr"/>
+      <c r="X121" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="7" t="n">
@@ -8487,6 +8793,11 @@
         <v/>
       </c>
       <c r="W122" s="8" t="inlineStr"/>
+      <c r="X122" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="7" t="n">
@@ -8574,6 +8885,11 @@
         <v/>
       </c>
       <c r="W123" s="8" t="inlineStr"/>
+      <c r="X123" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="7" t="n">
@@ -8676,6 +8992,11 @@
           <t>Art. 817 (Código de Normas CGJ-CE) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]; Art. 817 (norma não informada) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
         </is>
       </c>
+      <c r="X124" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="7" t="n">
@@ -8763,6 +9084,11 @@
         <v/>
       </c>
       <c r="W125" s="8" t="inlineStr"/>
+      <c r="X125" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="7" t="n">
@@ -8851,9 +9177,14 @@
           <t>Art. 9 (LGPD (Lei 13.709/2018)) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
         </is>
       </c>
+      <c r="X126" s="8" t="inlineStr">
+        <is>
+          <t>RESPONDIDA</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W126"/>
+  <autoFilter ref="A1:X126"/>
   <conditionalFormatting sqref="R2:R126">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>8</formula>
@@ -9052,7 +9383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9067,6 +9398,9 @@
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9137,6 +9471,21 @@
           <t>Taxa verificável (citações)</t>
         </is>
       </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>Respondidas</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>Não encontrado</t>
+        </is>
+      </c>
+      <c r="O3" s="6" t="inlineStr">
+        <is>
+          <t>Resposta vazia</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -9188,6 +9537,18 @@
         <f>IF(SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A4)=0,"",SUMIFS(Respostas!$U$2:$U$126,Respostas!$B$2:$B$126,$A4)/SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A4))</f>
         <v/>
       </c>
+      <c r="M4" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A4,Respostas!$X$2:$X$126,"RESPONDIDA")</f>
+        <v/>
+      </c>
+      <c r="N4" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A4,Respostas!$X$2:$X$126,"NAO_ENCONTRADO")</f>
+        <v/>
+      </c>
+      <c r="O4" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A4,Respostas!$X$2:$X$126,"RESPOSTA_VAZIA")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -9239,6 +9600,18 @@
         <f>IF(SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A5)=0,"",SUMIFS(Respostas!$U$2:$U$126,Respostas!$B$2:$B$126,$A5)/SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A5))</f>
         <v/>
       </c>
+      <c r="M5" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A5,Respostas!$X$2:$X$126,"RESPONDIDA")</f>
+        <v/>
+      </c>
+      <c r="N5" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A5,Respostas!$X$2:$X$126,"NAO_ENCONTRADO")</f>
+        <v/>
+      </c>
+      <c r="O5" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A5,Respostas!$X$2:$X$126,"RESPOSTA_VAZIA")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -9290,6 +9663,18 @@
         <f>IF(SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A6)=0,"",SUMIFS(Respostas!$U$2:$U$126,Respostas!$B$2:$B$126,$A6)/SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A6))</f>
         <v/>
       </c>
+      <c r="M6" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A6,Respostas!$X$2:$X$126,"RESPONDIDA")</f>
+        <v/>
+      </c>
+      <c r="N6" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A6,Respostas!$X$2:$X$126,"NAO_ENCONTRADO")</f>
+        <v/>
+      </c>
+      <c r="O6" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A6,Respostas!$X$2:$X$126,"RESPOSTA_VAZIA")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -9341,6 +9726,18 @@
         <f>IF(SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A7)=0,"",SUMIFS(Respostas!$U$2:$U$126,Respostas!$B$2:$B$126,$A7)/SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A7))</f>
         <v/>
       </c>
+      <c r="M7" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A7,Respostas!$X$2:$X$126,"RESPONDIDA")</f>
+        <v/>
+      </c>
+      <c r="N7" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A7,Respostas!$X$2:$X$126,"NAO_ENCONTRADO")</f>
+        <v/>
+      </c>
+      <c r="O7" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A7,Respostas!$X$2:$X$126,"RESPOSTA_VAZIA")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -9390,6 +9787,18 @@
       </c>
       <c r="L8" s="11">
         <f>IF(SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A8)=0,"",SUMIFS(Respostas!$U$2:$U$126,Respostas!$B$2:$B$126,$A8)/SUMIFS(Respostas!$T$2:$T$126,Respostas!$B$2:$B$126,$A8))</f>
+        <v/>
+      </c>
+      <c r="M8" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A8,Respostas!$X$2:$X$126,"RESPONDIDA")</f>
+        <v/>
+      </c>
+      <c r="N8" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A8,Respostas!$X$2:$X$126,"NAO_ENCONTRADO")</f>
+        <v/>
+      </c>
+      <c r="O8" s="9">
+        <f>COUNTIFS(Respostas!$B$2:$B$126,$A8,Respostas!$X$2:$X$126,"RESPOSTA_VAZIA")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: relatórios da auditoria e resultados pós-correções
- 08: revisão de 13/10 (fundamento invertido do Art. 1.131 e defeitos)
- 09: relatório autossuficiente da auditoria para análise externa
- 10: correções aplicadas, números medidos e itens abertos
- benchmark: execuções de 13/10 (10h10 e 11h35) e a re-pontuação da
  das 11h35 com o verificador corrigido (47/55 citações verificadas,
  19 respondidas, 6 não encontradas, 0 respostas vazias)
- planilha reposta a partir da execução completa re-pontuada
</commit_message>
<xml_diff>
--- a/docs/fase3/benchmark/planilha_benchmark.xlsx
+++ b/docs/fase3/benchmark/planilha_benchmark.xlsx
@@ -7050,29 +7050,28 @@
       </c>
       <c r="F102" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G102" s="8" t="inlineStr">
         <is>
-          <t>**Resposta:** Deve‑se praticar o ato registral de forma integral, emitindo a certidão de inteiro teor sem exigir a apresentação de motivo ou justificativa por parte do requerente.
+          <t>**Resposta:**  
+Sim. A certidão de inteiro teor pode ser emitida ao requerente, ainda que ele seja um terceiro sem vínculo ou sem apresentar justificativa para o pedido.
 **Fundamentação normativa**
-1. **Lei 6.015/1973 – Art. 19, §§ 11 e 12**  
-   &gt; “§ 11. No âmbito do registro de imóveis, a certidão de inteiro teor da matrícula conterá a reprodução de todo seu conteúdo e será suficiente para fins de comprovação de propriedade, direitos, ônus reais e restrições sobre o imóvel….”  
-   &gt; “§ 12. Na localidade em que haja dificuldade de comunicação eletrônica, a Corregedoria‑Geral da Justiça Estadual poderá autorizar, de modo excepcional…”.
-   O dispositivo estabelece a obrigatoriedade da certidão de inteiro teor e não impõe a necessidade de justificativa para a sua expedição.
-2. **Código de Normas da CGJ‑CE – Art. 1131, §§ 1º e 2º**  
-   &gt; “§ 1º Ao receber o pedido de certidão, o Oficial fornecerá, obrigatoriamente, ao requerente protocolo… e o prazo para a entrega do documento que não poderá exceder a 05 (cinco) dias úteis….”  
-   &gt; “§ 2º A certidão será lavrada em inteiro teor, em resumo ou em relatório, conforme quesitos, e devidamente autenticada… não podendo ser retardada por mais de 5 (cinco) dias úteis.”
-   Não há exigência de motivação do requerente; basta o pedido formal e a indicação do número da matrícula.
+1. **Lei nº 6.015/1973 – Art. 19, § 11**  
+   &gt; “No âmbito do registro de imóveis, a certidão de inteiro teor da matrícula conterá a reprodução de todo seu conteúdo e será suficiente para fins de comprovação de propriedade, direitos, ônus reais e restrições sobre o imóvel, independentemente de certificação específica pelo oficial.”  
+   O dispositivo não impõe a exigência de motivação ou vínculo do requerente para a expedição da certidão.
+2. **Código de Normas da CGJ‑CE – Art. 1.131, §§ 1‑2**  
+   &gt; “Ao receber o pedido de certidão, o Oficial fornecerá, obrigatoriamente, ao requerente protocolo… e o prazo para a entrega do documento que não poderá exceder a 05 (cinco) dias úteis… A certidão será lavrada em inteiro teor… não podendo ser retardada por mais de 5 (cinco) dias úteis.”  
+   Não há previsão de necessidade de justificativa ou de vínculo do interessado; o oficial apenas cumpre o prazo e informa os custos.
 3. **Provimento CNJ 149/2023 – Art. 327**  
-   &gt; “A certidão de inteiro teor digital solicitada durante o horário de expediente, com indicação do número da matrícula… será emitida e disponibilizada dentro de no máximo 2 (duas) horas…”.
-   O provimento regulamenta o prazo de emissão, confirmando que o requerimento pode ser atendido imediatamente, independentemente de motivo.
-**Conclusão prática**
-- **Ato registral:** Emissão integral da certidão de inteiro teor.  
-- **Condição:** Nenhuma exigência de motivação ou vínculo do requerente.  
-- **Procedimento:** Registrar o pedido, gerar o protocolo (Art. 1131, § 1º), observar o prazo máximo de 5 (cinco) dias úteis ou 2 (duas) horas para a versão digital (Art. 327), e disponibilizar a certidão ao requerente.  
-Portanto, a certidão pode ser emitida sem exigir motivo.</t>
+   &gt; “A certidão de inteiro teor digital solicitada durante o horário de expediente… será emitida e disponibilizada dentro de no máximo 2 horas… e ficará disponível para download pelo requerente pelo prazo mínimo de 30 dias.”  
+   O provimento regula apenas o prazo e a forma de disponibilização, não condicionando a emissão a motivo ou vínculo.
+4. **Provimento CNJ 149/2023 – Art. 200** (restrição que não se aplica ao caso)  
+   &gt; “É vedada a expedição de nova certidão de inteiro teor… tendo como única fonte de consulta anterior certidão expedida por unidade do serviço extrajudicial.”  
+   Essa vedação refere‑se à origem da informação, não à identidade do requerente.
+**Conclusão prática**  
+O ato registral deve ser praticado integralmente: a serventia pode expedir a certidão de inteiro teor da matrícula ao terceiro, sem necessidade de exigir motivo ou comprovar vínculo. O oficial observará apenas os requisitos de protocolo, pagamento de emolumentos e os prazos estabelecidos nos dispositivos citados.</t>
         </is>
       </c>
       <c r="H102" s="8" t="inlineStr">
@@ -7081,13 +7080,13 @@
         </is>
       </c>
       <c r="I102" s="8" t="n">
-        <v>2.73</v>
+        <v>3</v>
       </c>
       <c r="J102" s="8" t="n">
         <v>1738</v>
       </c>
       <c r="K102" s="8" t="n">
-        <v>814</v>
+        <v>816</v>
       </c>
       <c r="L102" s="10">
         <f>IF(COUNT(J102:K102)=2,(J102*Parametros!$B$3+K102*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7104,10 +7103,10 @@
       </c>
       <c r="S102" s="8" t="n"/>
       <c r="T102" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U102" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V102" s="11">
         <f>IF(AND(ISNUMBER(T102),T102&gt;0),U102/T102,"")</f>
@@ -7144,19 +7143,12 @@
       </c>
       <c r="F103" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G103" s="8" t="inlineStr">
         <is>
-          <t>**Resposta Jurídica e Operacional**
-A certidão de inteiro teor **não** é obrigada a exibir o CPF completo dos proprietários.
-**Fundamentação normativa**
-- **Código de Normas CGJ‑CE – Art. 1131, § 10**  
-  “No âmbito do registro de imóveis, a certidão de inteiro teor da matrícula conterá a reprodução de todo seu conteúdo e será suficiente para fins de comprovação de propriedade, direitos, ônus reais e restrições sobre o imóvel, independentemente de certificação específica pelo Oficial.”
-- **Lei 6.015/1973 – Art. 19, § 11**  
-  “No âmbito do registro de imóveis, a certidão de inteiro teor da matrícula conterá a reprodução de todo seu conteúdo e será suficiente para fins de comprovação de propriedade, direitos, ônus reais e restrições sobre o imóvel, independentemente de certificação específica pelo oficial.”
-Esses dispositivos estabelecem que a certidão reproduz todo o conteúdo da matrícula, mas não impõem a inclusão do CPF completo dos proprietários como requisito obrigatório. Portanto, a prática de registrar o CPF completo não é exigida nem prevista na legislação vigente.</t>
+          <t>Não encontrado no corpus.</t>
         </is>
       </c>
       <c r="H103" s="8" t="inlineStr">
@@ -7165,13 +7157,13 @@
         </is>
       </c>
       <c r="I103" s="8" t="n">
-        <v>1.3</v>
+        <v>0.97</v>
       </c>
       <c r="J103" s="8" t="n">
         <v>1698</v>
       </c>
       <c r="K103" s="8" t="n">
-        <v>658</v>
+        <v>224</v>
       </c>
       <c r="L103" s="10">
         <f>IF(COUNT(J103:K103)=2,(J103*Parametros!$B$3+K103*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7188,10 +7180,10 @@
       </c>
       <c r="S103" s="8" t="n"/>
       <c r="T103" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U103" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V103" s="11">
         <f>IF(AND(ISNUMBER(T103),T103&gt;0),U103/T103,"")</f>
@@ -7200,7 +7192,7 @@
       <c r="W103" s="8" t="inlineStr"/>
       <c r="X103" s="8" t="inlineStr">
         <is>
-          <t>RESPONDIDA</t>
+          <t>NAO_ENCONTRADO</t>
         </is>
       </c>
     </row>
@@ -7228,28 +7220,23 @@
       </c>
       <c r="F104" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t>**Resposta:** O pedido deve ser **praticado condicionado com tarjamento protetivo**.
+          <t>**Decisão:** Indeferir o pedido via **Nota Devolutiva** – a certidão deverá conter apenas os ônus reais **não cancelados**, nos termos da normativa vigente.
 **Fundamentação normativa**
-1. **Certidão padrão – ônus não cancelados**  
-   - **Código de Normas CGJ‑CE, art. 1.129** – “as certidões … serão expedidas … contendo … os ônus reais **não cancelados**.”  
-   - Portanto, a certidão que contém apenas a situação jurídica atual (descrição, titularidade e ônus vigentes) pode ser emitida integralmente, mas **não inclui** ônus já extintos (penhoras canceladas).
-2. **Emissão de certidão com histórico de atos anteriores**  
-   - **Código de Normas CGJ‑CE, art. 1.682, § único** – “a expedição de certidão de atos anteriores da cadeia filiatória do imóvel **depende de identificação segura do requerente e de indicação da finalidade**.”  
-   - Essa exigência caracteriza a necessidade de **tarjamento protetivo** (tratamento de dados pessoais sensíveis) para garantir a proteção dos dados constantes nos registros históricos, em consonância com a LGPD.
-3. **Procedimento recomendado**  
-   - **Passo 1 –** Verificar a identidade do requerente (documentação idônea, assinatura digital ou outro meio que assegure a identificação segura).  
-   - **Passo 2 –** Exigir a indicação clara da finalidade da certidão (ex.: instrução de processo judicial, análise de crédito, pesquisa acadêmica, etc.).  
-   - **Passo 3 –** Aplicar o tarjamento protetivo (mascaramento ou restrição de acesso) aos dados pessoais que constam nos atos extintos, de modo a atender a LGPD (art. 5º, inc. X da LGPD) e o art. 1.682, § único do Código de Normas CGJ‑CE.  
-   - **Passo 4 –** Emitir a certidão contendo **todo o histórico de ônus**, inclusive as penhoras já canceladas, com a devida proteção dos dados.
-**Conclusão prática**
-- **Não** é possível atender ao pedido de forma integral (sem restrições) apenas com base no art. 1.129, pois a certidão padrão exclui ônus cancelados.  
-- **Deve‑se** conceder a certidão histórica **condicionada ao tarjamento protetivo**, atendendo ao requisito de identificação segura e indicação de finalidade previsto no art. 1.682, § único.  
-Assim, o ato registral será praticado **condicionado com tarjamento protetivo**, observando os dispositivos citados.</t>
+1. **Código de Normas da CGJ‑CE – Art. 1.129**  
+   &gt; “As certidões dos imóveis que já forem objeto de matrícula eletrônica, após a ‘primeira qualificação eletrônica’, serão expedidas … contendo a situação jurídica atual do imóvel, ou seja, sua descrição, titularidade e os ônus reais **não cancelados**.”  
+   O dispositivo delimita expressamente o conteúdo da certidão à situação jurídica **atual**, excluindo, portanto, ônus que já tenham sido cancelados.
+2. **Código de Normas da CGJ‑CE – Art. 1.682, parágrafo único**  
+   &gt; “A expedição de certidão de atos anteriores da cadeia filiatória do imóvel depende de identificação segura do requerente e de indicação da finalidade.”  
+   Não há previsão de que a certidão de histórico completo (incluindo ônus cancelados) seja emitida de forma automática; sua expedição exigiria requisitos adicionais que não foram atendidos no pedido.
+**Conclusão operacional**
+- O pedido de certidão contendo **todo o histórico de ônus, inclusive penhoras já canceladas**, ultrapassa o escopo definido pelos artigos acima.  
+- Assim, o ato registral **não deve ser praticado integralmente**.  
+- O cartório deve **indeferir** o pedido mediante **Nota Devolutiva**, orientando o requerente a formular novo pedido específico, com identificação segura e indicação de finalidade, caso deseje acesso a atos anteriores da cadeia filiatória, nos termos do art. 1.682, § único.</t>
         </is>
       </c>
       <c r="H104" s="8" t="inlineStr">
@@ -7258,13 +7245,13 @@
         </is>
       </c>
       <c r="I104" s="8" t="n">
-        <v>2.88</v>
+        <v>2.41</v>
       </c>
       <c r="J104" s="8" t="n">
         <v>1410</v>
       </c>
       <c r="K104" s="8" t="n">
-        <v>1188</v>
+        <v>876</v>
       </c>
       <c r="L104" s="10">
         <f>IF(COUNT(J104:K104)=2,(J104*Parametros!$B$3+K104*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7281,20 +7268,16 @@
       </c>
       <c r="S104" s="8" t="n"/>
       <c r="T104" s="8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U104" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V104" s="11">
         <f>IF(AND(ISNUMBER(T104),T104&gt;0),U104/T104,"")</f>
         <v/>
       </c>
-      <c r="W104" s="8" t="inlineStr">
-        <is>
-          <t>Art. 5 (LGPD (Lei 13.709/2018)) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
-        </is>
-      </c>
+      <c r="W104" s="8" t="inlineStr"/>
       <c r="X104" s="8" t="inlineStr">
         <is>
           <t>RESPONDIDA</t>
@@ -7325,20 +7308,18 @@
       </c>
       <c r="F105" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G105" s="8" t="inlineStr">
         <is>
-          <t>**Resposta:** Indeferido via Nota Devolutiva.
+          <t>**Resposta:** Indeferir o pedido via **Nota Devolutiva**.
 **Fundamentação normativa**
-- **Código de Normas da CGJ‑CE – Art. 1.128, § 2º, inc. V**:  
-  “o fornecimento, pelo registrador, por qualquer meio, de informações sobre o registro não veiculadas por certidão, **exceto nos casos em que o solicitante figure no registro em questão**.”  
-  No pedido apresentado o requerente indica apenas o nome do titular (“fulano”) e não demonstra que ele próprio seja o titular nem apresenta qualquer finalidade legalmente prevista. Assim, a informação solicitada não pode ser fornecida por meio de busca ou comunicação direta, pois não se enquadra na exceção prevista no inciso V.
-- **Lei 6.015/1973 – Art. 222** (obrigatoriedade de referência à matrícula nos atos) reforça que a identificação do imóvel deve ser feita mediante número de matrícula ou registro, não apenas pelo nome do proprietário, o que demonstra a necessidade de dados precisos e vinculados ao registro para qualquer comunicação.
-- **LGPD (Lei Geral de Proteção de Dados Pessoais)** – embora não conste explicitamente no corpus fornecido, o tratamento de dados pessoais (nome e patrimônio imobiliário) só pode ocorrer mediante consentimento do titular ou outra hipótese legal. O simples pedido de “todos os imóveis em nome de fulano” sem consentimento ou legitimidade não atende a esse requisito.
-**Conclusão operativa**
-Diante da ausência de comprovação de que o requerente seja o próprio titular ou que possua autorização legal para acessar tais dados, o ato de busca e a posterior comunicação das informações devem ser **indeferidos**, devendo ser emitida a respectiva **Nota Devolutiva** fundamentada no art. 1.128, § 2º, inc. V, do Código de Normas da CGJ‑CE.</t>
+- **Código de Normas CGJ‑CE – Art. 1.128, § 2º, inc. IV**:  
+  “as requisições de buscas fundadas exclusivamente no indicador pessoal ou real” são vedadas. O pedido “todos os imóveis em nome de fulano”, apresentado apenas com o nome (indicador pessoal), enquadra‑se exatamente nessa hipótese, não havendo a exigência de identificação do requerente nem de finalidade específica.
+- **Lei Geral de Proteção de Dados (LGPD) – Art. 7º** (não explicitado no corpus, mas aplicável por analogia): o tratamento de dados pessoais (lista de imóveis vinculados a pessoa física) só pode ocorrer mediante consentimento ou outra hipótese legal, o que não foi demonstrado no pedido.
+**Conclusão operacional**
+- O registro não deve ser praticado integralmente nem com tarja protetiva; o pedido deve ser **indeferido** mediante emissão de Nota Devolutiva, informando ao solicitante a impossibilidade de atender à busca baseada exclusivamente no nome.</t>
         </is>
       </c>
       <c r="H105" s="8" t="inlineStr">
@@ -7347,13 +7328,13 @@
         </is>
       </c>
       <c r="I105" s="8" t="n">
-        <v>2</v>
+        <v>2.37</v>
       </c>
       <c r="J105" s="8" t="n">
         <v>1483</v>
       </c>
       <c r="K105" s="8" t="n">
-        <v>731</v>
+        <v>775</v>
       </c>
       <c r="L105" s="10">
         <f>IF(COUNT(J105:K105)=2,(J105*Parametros!$B$3+K105*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7370,16 +7351,20 @@
       </c>
       <c r="S105" s="8" t="n"/>
       <c r="T105" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U105" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V105" s="11">
         <f>IF(AND(ISNUMBER(T105),T105&gt;0),U105/T105,"")</f>
         <v/>
       </c>
-      <c r="W105" s="8" t="inlineStr"/>
+      <c r="W105" s="8" t="inlineStr">
+        <is>
+          <t>Art. 7 (LGPD (Lei 13.709/2018)) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
+        </is>
+      </c>
       <c r="X105" s="8" t="inlineStr">
         <is>
           <t>RESPONDIDA</t>
@@ -7410,23 +7395,40 @@
       </c>
       <c r="F106" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
-        </is>
-      </c>
-      <c r="G106" s="8" t="inlineStr"/>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
+        </is>
+      </c>
+      <c r="G106" s="8" t="inlineStr">
+        <is>
+          <t>**Procedimento para busca de bens do devedor por CPF**
+1. **Requerimento ao Oficial do Registro de Imóveis**  
+   O credor deve protocolar um requerimento ao Oficial do Registro de Imóveis, contendo:
+   - CPF e nome do devedor (e, se for casado, do cônjuge) – **Art. 1659, inciso I**;
+   - Endereço residencial atual e anterior, se houver – **Art. 1659, inciso II**;
+   - Endereço comercial, se houver – **Art. 1659, inciso III**;
+   - Qualificação completa das partes (nome, domicílio, nacionalidade, estado civil, regime de bens, profissão, CPF ou documento de identidade) – **Art. 1.103 do Provimento 15/2026/CGJCE**.
+2. **Busca de bens**  
+   O Oficial, com base no CPF informado, realiza a busca no Registro de Imóveis e emite um **certificado de busca de bens** (lista de imóveis registrados em nome do CPF).  
+3. **Intimação do devedor (se necessário)**  
+   Caso o devedor não seja localizado nos endereços indicados, o Oficial procede à intimação conforme **Art. 1666** (intimação por hora certa, com possibilidade de intimar pessoas próximas ou funcionários de portaria, se aplicável).  
+4. **Entrega do resultado**  
+   O certificado de busca, acompanhado de eventuais comprovantes de intimação, é entregue ao credor, permitindo-lhe prosseguir com as medidas de cobrança ou execução.
+&gt; **Resumo**: O credor solicita a busca de bens do devedor por CPF, seguindo os requisitos de Art. 1659 e Art. 1.103, e o Oficial realiza a busca e, se necessário, a intimação conforme Art. 1666.</t>
+        </is>
+      </c>
       <c r="H106" s="8" t="inlineStr">
         <is>
           <t>Código de Normas CGJ-CE — Art. 1666:p342; Código de Normas CGJ-CE — Art. 1659:p339; Código de Normas CGJ-CE — Art. 1621:p330; Provimento 15/2026/CGJCE — Art. 1:p2</t>
         </is>
       </c>
       <c r="I106" s="8" t="n">
-        <v>2.73</v>
+        <v>2.04</v>
       </c>
       <c r="J106" s="8" t="n">
         <v>2169</v>
       </c>
       <c r="K106" s="8" t="n">
-        <v>2048</v>
+        <v>1217</v>
       </c>
       <c r="L106" s="10">
         <f>IF(COUNT(J106:K106)=2,(J106*Parametros!$B$3+K106*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7443,19 +7445,23 @@
       </c>
       <c r="S106" s="8" t="n"/>
       <c r="T106" s="8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="U106" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V106" s="11">
         <f>IF(AND(ISNUMBER(T106),T106&gt;0),U106/T106,"")</f>
         <v/>
       </c>
-      <c r="W106" s="8" t="inlineStr"/>
+      <c r="W106" s="8" t="inlineStr">
+        <is>
+          <t>Art. 1103 (Provimento 15/2026/CGJCE) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]; Art. 1103 (norma não informada) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
+        </is>
+      </c>
       <c r="X106" s="8" t="inlineStr">
         <is>
-          <t>RESPOSTA_VAZIA</t>
+          <t>RESPONDIDA</t>
         </is>
       </c>
     </row>
@@ -7483,7 +7489,7 @@
       </c>
       <c r="F107" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G107" s="8" t="inlineStr">
@@ -7497,13 +7503,13 @@
         </is>
       </c>
       <c r="I107" s="8" t="n">
-        <v>2.19</v>
+        <v>1.83</v>
       </c>
       <c r="J107" s="8" t="n">
         <v>1783</v>
       </c>
       <c r="K107" s="8" t="n">
-        <v>782</v>
+        <v>671</v>
       </c>
       <c r="L107" s="10">
         <f>IF(COUNT(J107:K107)=2,(J107*Parametros!$B$3+K107*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7560,23 +7566,27 @@
       </c>
       <c r="F108" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
-        </is>
-      </c>
-      <c r="G108" s="8" t="inlineStr"/>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
+        </is>
+      </c>
+      <c r="G108" s="8" t="inlineStr">
+        <is>
+          <t>Não encontrado no corpus.</t>
+        </is>
+      </c>
       <c r="H108" s="8" t="inlineStr">
         <is>
-          <t>Lei 6.015/1973 — Art. 279:p0; Lei 6.015/1973 — Art. 276:p0; Lei 6.015/1973 — Art. 292:p0; Código de Normas CGJ-CE — Art. 1333:p271; Código de Normas CGJ-CE — Art. 1412:p286</t>
+          <t>Lei 6.015/1973 — Art. 279:p0; Lei 6.015/1973 — Art. 276:p0; Código de Normas CGJ-CE — Art. 1333:p271; Lei 6.015/1973 — Art. 292:p0; Código de Normas CGJ-CE — Art. 1412:p286</t>
         </is>
       </c>
       <c r="I108" s="8" t="n">
-        <v>3</v>
+        <v>1.03</v>
       </c>
       <c r="J108" s="8" t="n">
         <v>1175</v>
       </c>
       <c r="K108" s="8" t="n">
-        <v>2048</v>
+        <v>571</v>
       </c>
       <c r="L108" s="10">
         <f>IF(COUNT(J108:K108)=2,(J108*Parametros!$B$3+K108*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7605,7 +7615,7 @@
       <c r="W108" s="8" t="inlineStr"/>
       <c r="X108" s="8" t="inlineStr">
         <is>
-          <t>RESPOSTA_VAZIA</t>
+          <t>NAO_ENCONTRADO</t>
         </is>
       </c>
     </row>
@@ -7633,43 +7643,34 @@
       </c>
       <c r="F109" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>**Resposta:** A solicitação da Prefeitura deve ser atendida **condicionada com tarjamento protetivo** (proteção de dados), mediante a entrega dos dados no formato eletrônico previsto pelo Provimento CNJ 149/2023.
----
-### Fundamentação normativa
-1. **Provimento CNJ 149/2023 – Art. 184‑A, §§ 3 a 6**  
-   - **§ 3º** – “É obrigatória a indicação do fato ou ato jurídico que ensejou a aquisição ou a transmissão do direito real de propriedade (compra e venda, doação, usucapião etc.).”  
-   - **§ 4º** – “O CNB/CF e o ONR disponibilizarão acesso aos municípios, para obtenção das informações, mediante convênio padronizado, para fins de os destinatários das informações atenderem ao disposto nas regras de proteção de dados e de sigilo fiscal.”  
-   - **§ 5º** – “O acesso pode ocorrer mediante plataforma que permita aos municípios obterem, em um mesmo ambiente eletrônico, as informações.”  
-   - **§ 6º** – “Caberão ao CNB/CF e ao ONR a elaboração de manual técnico em que serão estabelecidos o formato dos dados e o padrão dos programas de interface eletrônica (Application Programming Interface – API), a serem utilizados no intercâmbio de dados estruturados entre as serventias extrajudiciais e as municipalidades.”
-2. **LGPD (Lei 13.709/2018) – tratamento de dados pessoais para cumprimento de obrigação legal ou regulatória**  
-   - Embora o texto da LGPD não conste integralmente no corpus, o provimento acima já incorpora a exigência de observância das “regras de proteção de dados”, que decorrem do art. 7º, I da LGPD (tratamento de dados pessoais quando necessário ao cumprimento de obrigação legal ou regulatória).  
----
-### Como proceder
+          <t>**Resposta:** Forneça a lista, porém o fornecimento deve ser realizado **integralmente, porém condicionado ao cumprimento das normas de proteção de dados** (LGPD) e ao uso da interface eletrônica prevista no Provimento CNJ 149/2023.
+**Fundamentação normativa**
+1. **Provimento CNJ 149/2023 – Art. 184‑A, §§ 4º, 5º e 6º**  
+   &gt; “§ 4º O CNB/CF e o ONR disponibilizarão acesso aos municípios, para obtenção das informações, mediante convênio padronizado, para fins de os destinatários das informações atenderem ao disposto nas regras de proteção de dados e de sigilo fiscal.”  
+   &gt; “§ 5º O acesso pode ocorrer mediante plataforma que permita aos municípios obterem, em um mesmo ambiente eletrônico, as informações.”  
+   &gt; “§ 6º Caberão ao CNB/CF e ao ONR a elaboração de manual técnico em que serão estabelecidos o formato dos dados e o padrão dos programas de interface eletrônica (API), a serem utilizados no intercâmbio de dados estruturados entre as serventias extrajudiciais e as municipalidades.”
+   Esses dispositivos autorizam o compartilhamento de dados cadastrais (matrícula, proprietário, CPF) com a municipalidade, **desde que obedecidos**:
+   * o **convênio padronizado** entre a serventia e o município;  
+   * o **manual técnico** que define o **formato** (arquivo estruturado – ex.: JSON ou XML) e a **API** a ser utilizada;  
+   * as **regras de proteção de dados e sigilo fiscal** previstas na LGPD (Lei 13.709/2018).
+2. **LGPD (Lei 13.709/2018)** – embora não haja artigo específico citado no corpus, a própria norma impõe que o tratamento de dados pessoais (nome, CPF) seja realizado em conformidade com os princípios de finalidade, adequação, necessidade e segurança, o que reforça a necessidade de uso da interface eletrônica prevista no provimento acima.
+**Procedimento operacional**
 | Etapa | Descrição | Base legal |
-|-------|-----------|------------|
-| **1. Convênio padronizado** | Verificar a existência de convênio entre o Cartório de Registro de Imóveis e a Prefeitura, nos termos do **§ 4º** do art. 184‑A. | Provimento CNJ 149/2023, art. 184‑A, § 4º |
-| **2. Utilização da plataforma ONR** | Disponibilizar a lista (imóvel, proprietário, CPF) por meio da plataforma eletrônica do **Operador Nacional do Sistema de Registro Eletrônico de Imóveis (ONR)**, conforme previsto no **§ 5º**. | Provimento CNJ 149/2023, art. 184‑A, § 5º |
-| **3. Formato dos dados** | Seguir o **manual técnico** elaborado pelo CNB/CF e ONR (art. 184‑A, § 6º), que define o padrão de **API/arquivo estruturado (ex.: JSON ou XML) contendo apenas os campos necessários** (número da matrícula, nome completo, CPF, endereço). | Provimento CNJ 149/2023, art. 184‑A, § 6º |
-| **4. Tarjamento protetivo** | Aplicar a classificação de **tarjamento protetivo** aos dados pessoais (CPF) para garantir que o acesso seja restrito ao uso exclusivo da cobrança de IPTU, obedecendo aos princípios da LGPD (necessidade, adequação e minimização). | Provimento CNJ 149/2023, art. 184‑A, §§ 4‑5 (regras de proteção de dados) |
-| **5. Registro da comunicação** | Emitir nota de devolutiva ao requerente (Prefeitura) informando o meio de acesso (API/portal ONR) e as condições de uso dos dados, conforme prática de transparência e rastreabilidade. | Não encontrado no corpus (para formalização de nota de devolutiva) |
----
-### Conclusão
-- **O ato registral não pode ser indeferido**; a informação é de interesse público para a arrecadação de IPTU, havendo fundamento legal para o seu fornecimento.  
-- **Deve ser fornecida**, porém **condicionada com tarjamento protetivo** e **exclusivamente via plataforma eletrônica (ONR) no formato técnico definido pelo manual de API**, garantindo a observância das normas de proteção de dados previstas no Provimento CNJ 149/2023 e na LGPD.  
----  
-**Nota de Devolutiva (modelo resumido)**  
-&gt; “Em atendimento ao requerimento da Prefeitura Municipal de ___, informamos que a lista de imóveis com respectivos proprietários e CPFs será disponibilizada por meio da plataforma do Operador Nacional do Sistema de Registro Eletrônico de Imóveis (ONR), conforme o manual técnico de intercâmbio de dados (API). Os dados serão tarifados como protetivos, obedecendo às regras de proteção de dados pessoais previstas no Provimento CNJ 149/2023, art. 184‑A, §§ 4‑6, e na LGPD. O acesso será concedido mediante credenciais específicas e uso exclusivo para fins de cobrança de IPTU.”  
----  
-**Referências citadas**  
-- Provimento CNJ 149/2023, Art. 184‑A, §§ 3 a 6.  
-- LGPD (Lei 13.709/2018) – tratamento de dados pessoais para cumprimento de obrigação legal (art. 7º, I).  
----  
-*Esta orientação está baseada **exclusivamente** no corpus normativo apresentado.*</t>
+|------|-----------|------------|
+| **a) Convênio** | Verificar a existência de convênio padronizado entre o cartório e a prefeitura. | Prov. CNJ 149/2023, art. 184‑A, § 4º |
+| **b) Manual técnico** | Utilizar o manual técnico elaborado pelo CNB/CF e ONR para gerar o arquivo no formato definido (ex.: JSON / XML) e disponibilizá‑lo via API. | Prov. CNJ 149/2023, art. 184‑A, § 6º |
+| **c) Proteção de dados** | Garantir que o acesso seja autenticado, que o arquivo contenha apenas os campos necessários (matrícula, nome, CPF) e que seja armazenado e transmitido com criptografia, em observância à LGPD. | LGPD – princípios de necessidade e segurança |
+| **d) Registro da transmissão** | Arquivar a solicitação da prefeitura, o comprovante de envio da API e o relatório de conformidade LGPD. | Não há dispositivo específico no corpus; prática recomendada de controle interno. |
+**Conclusão**
+- O ato de fornecer a lista de imóveis com proprietários e CPFs à prefeitura **deve ser praticado integralmente**, porém **condicionado** ao cumprimento das exigências de **proteção de dados** e ao **uso da interface eletrônica (API) prevista** nos §§ 4º, 5º e 6º do **Art. 184‑A do Provimento CNJ 149/2023**.  
+- Não há necessidade de “tarjamento protetivo” (cobertura de dados) quando o compartilhamento ocorre via canal oficial (API) e dentro do escopo do convênio, pois a proteção será assegurada pelos mecanismos de segurança da própria plataforma.  
+- Caso não exista convênio ou a prefeitura exija o envio em formato físico (planilha impressa), o fornecimento **deve ser indeferido via Nota Devolutiva**, pois violaria a exigência de uso da interface eletrônica e de observância da LGPD.  
+**Portanto:** forneça a lista **integralmente**, mediante a API padronizada estabelecida pelo CNB/CF e ONR, observando integralmente as regras de proteção de dados da LGPD.</t>
         </is>
       </c>
       <c r="H109" s="8" t="inlineStr">
@@ -7678,13 +7679,13 @@
         </is>
       </c>
       <c r="I109" s="8" t="n">
-        <v>4.29</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="J109" s="8" t="n">
         <v>2097</v>
       </c>
       <c r="K109" s="8" t="n">
-        <v>1754</v>
+        <v>1609</v>
       </c>
       <c r="L109" s="10">
         <f>IF(COUNT(J109:K109)=2,(J109*Parametros!$B$3+K109*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7701,7 +7702,7 @@
       </c>
       <c r="S109" s="8" t="n"/>
       <c r="T109" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U109" s="8" t="n">
         <v>1</v>
@@ -7710,11 +7711,7 @@
         <f>IF(AND(ISNUMBER(T109),T109&gt;0),U109/T109,"")</f>
         <v/>
       </c>
-      <c r="W109" s="8" t="inlineStr">
-        <is>
-          <t>Art. 7 (LGPD (Lei 13.709/2018)) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
-        </is>
-      </c>
+      <c r="W109" s="8" t="inlineStr"/>
       <c r="X109" s="8" t="inlineStr">
         <is>
           <t>RESPONDIDA</t>
@@ -7745,17 +7742,16 @@
       </c>
       <c r="F110" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>**Indeferir via Nota Devolutiva**  
-O oficial deve recusar o fornecimento dos dados solicitados pela polícia, emitindo uma Nota Devolutiva fundamentada, pois a solicitação não está respaldada por ordem judicial e, portanto, não se enquadra nas finalidades previstas para o tratamento de dados pessoais no Registro de Imóveis.
-**Dispositivo legal aplicável**  
-Art. 1128, § 4º, do Código de Normas CGJ‑CE:  
-&gt; “Caracterizada tentativa de tratamento de dados em desacordo com as finalidades do Registro de Imóveis e com os princípios da Lei Geral de Proteção de Dados Pessoais, poderá o Oficial recusar o fornecimento em nota fundamentada, do que caberá revisão pelo juízo competente.”
-Assim, o ato registral deve ser **indeferido via Nota Devolutiva**.</t>
+          <t>**Resposta Jurídica e Operacional**
+O ato de fornecer os dados solicitados pela polícia, sem que exista ordem judicial que autorize tal tratamento, deve ser **indeferido por meio de Nota Devolutiva**.
+**Fundamentação:**
+- **Código de Normas CGJ‑CE, Art. 1128, § 4º**: “Caracterizada tentativa de tratamento de dados em desacordo com as finalidades do Registro de Imóveis e com os princípios da Lei Geral de Proteção de Dados Pessoais, poderá o Oficial recusar o fornecimento em nota fundamentada, do que caberá revisão pelo juízo competente.”
+Como não há ordem judicial que autorize a divulgação dos dados pessoais do proprietário, a solicitação viola os princípios da LGPD e as finalidades do Registro de Imóveis. Portanto, o oficial deve recusar o pedido, emitindo uma Nota Devolutiva fundamentada no Art. 1128, § 4º.</t>
         </is>
       </c>
       <c r="H110" s="8" t="inlineStr">
@@ -7764,13 +7760,13 @@
         </is>
       </c>
       <c r="I110" s="8" t="n">
-        <v>20.58</v>
+        <v>1.73</v>
       </c>
       <c r="J110" s="8" t="n">
         <v>1605</v>
       </c>
       <c r="K110" s="8" t="n">
-        <v>815</v>
+        <v>905</v>
       </c>
       <c r="L110" s="10">
         <f>IF(COUNT(J110:K110)=2,(J110*Parametros!$B$3+K110*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7787,10 +7783,10 @@
       </c>
       <c r="S110" s="8" t="n"/>
       <c r="T110" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U110" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V110" s="11">
         <f>IF(AND(ISNUMBER(T110),T110&gt;0),U110/T110,"")</f>
@@ -7827,7 +7823,7 @@
       </c>
       <c r="F111" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G111" s="8" t="inlineStr">
@@ -7841,7 +7837,7 @@
         </is>
       </c>
       <c r="I111" s="8" t="n">
-        <v>14.49</v>
+        <v>11.23</v>
       </c>
       <c r="J111" s="8" t="n">
         <v>1399</v>
@@ -7904,7 +7900,7 @@
       </c>
       <c r="F112" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G112" s="8" t="inlineStr">
@@ -7918,13 +7914,13 @@
         </is>
       </c>
       <c r="I112" s="8" t="n">
-        <v>2.38</v>
+        <v>1.38</v>
       </c>
       <c r="J112" s="8" t="n">
         <v>1578</v>
       </c>
       <c r="K112" s="8" t="n">
-        <v>431</v>
+        <v>396</v>
       </c>
       <c r="L112" s="10">
         <f>IF(COUNT(J112:K112)=2,(J112*Parametros!$B$3+K112*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -7981,7 +7977,7 @@
       </c>
       <c r="F113" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G113" s="8" t="inlineStr">
@@ -7989,9 +7985,15 @@
           <t>**Resposta Jurídica e Operacional**
 Sim, é dever responder ao pedido de acesso à informação sobre os emolumentos arrecadados pela serventia.
 **Fundamentação normativa**
-- **LAI – Art. 10**: “Qualquer interessado poderá apresentar pedido de acesso a informações aos órgãos e entidades referidos no art. 1º desta Lei…”.  
-- **LAI – Art. 14**: “É direito do requerente obter o inteiro teor de decisão de negativa de acesso, por certidão ou cópia.”  
-O pedido trata de informação de interesse público (emolumentos arrecadados), não se enquadrando em nenhuma exceção prevista na LAI. Portanto, a serventia deve atender ao pedido, fornecendo os dados solicitados ou, se houver impedimento, justificando a negativa conforme previsto no art. 14.</t>
+- **LAI – Art. 10**  
+  - § 1º: “Qualquer interessado poderá apresentar pedido de acesso a informações … devendo o pedido conter a identificação do requerente e a especificação da informação requerida.”  
+  - § 2º: “Os órgãos e entidades do poder público devem viabilizar alternativa de encaminhamento de pedidos de acesso por meio de seus sítios oficiais na internet.”  
+  - § 3º: “São vedadas quaisquer exigências relativas aos motivos determinantes da solicitação de informações de interesse público.”  
+- **LAI – Art. 14**  
+  - “É direito do requerente obter o inteiro teor de decisão de negativa de acesso, por certidão ou cópia.”  
+Portanto, a serventia deve atender ao pedido, fornecendo a informação solicitada ou, se houver motivo legítimo para negar, deve apresentar a decisão de negativa com o inteiro teor, conforme Art. 14.  
+**Conclusão**  
+O ato registral de resposta ao pedido via LAI deve ser praticado integralmente, obedecendo aos dispositivos citados.</t>
         </is>
       </c>
       <c r="H113" s="8" t="inlineStr">
@@ -8000,13 +8002,13 @@
         </is>
       </c>
       <c r="I113" s="8" t="n">
-        <v>2.4</v>
+        <v>11.78</v>
       </c>
       <c r="J113" s="8" t="n">
         <v>1458</v>
       </c>
       <c r="K113" s="8" t="n">
-        <v>1540</v>
+        <v>1675</v>
       </c>
       <c r="L113" s="10">
         <f>IF(COUNT(J113:K113)=2,(J113*Parametros!$B$3+K113*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -8026,17 +8028,13 @@
         <v>3</v>
       </c>
       <c r="U113" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V113" s="11">
         <f>IF(AND(ISNUMBER(T113),T113&gt;0),U113/T113,"")</f>
         <v/>
       </c>
-      <c r="W113" s="8" t="inlineStr">
-        <is>
-          <t>Art. 1 (LAI (Lei 12.527/2011)) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
-        </is>
-      </c>
+      <c r="W113" s="8" t="inlineStr"/>
       <c r="X113" s="8" t="inlineStr">
         <is>
           <t>RESPONDIDA</t>
@@ -8067,17 +8065,18 @@
       </c>
       <c r="F114" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
           <t>**Resposta**  
-A certidão de inteiro teor **não pode** ser emitida sem incluir a averbação de interdição/curatela que consta na matrícula.  
-**Fundamentação**  
-- **Código de Normas CGJ‑CE, Art. 1131, § 10**: “No âmbito do registro de imóveis, a certidão de inteiro teor da matrícula conterá a reprodução de todo seu conteúdo e será suficiente para fins de comprovação de propriedade, direitos, ônus reais e restrições sobre o imóvel, independentemente de certificação específica pelo Oficial.”  
-- **Lei 6.015/1973, Art. 19, § 11**: “No âmbito do registro de imóveis, a certidão de inteiro teor da matrícula conterá a reprodução de todo seu conteúdo e será suficiente para fins de comprovação de propriedade, direitos, ônus reais e restrições sobre o imóvel, independentemente de certificação específica pelo oficial.”  
-Portanto, a certidão deve ser emitida **completa**, incluindo a averbação de interdição/curatela; não há possibilidade de emissão “sem restrição”.</t>
+A certidão não pode ser emitida sem incluir a averbação de interdição/curatela que consta na matrícula.  
+**Dispositivo legal**  
+- Lei 6.015/1973, Art. 19, § 11: “No âmbito do registro de imóveis, a certidão de inteiro teor da matrícula conterá a reprodução de todo seu conteúdo e será suficiente para fins de comprovação de propriedade, direitos, ônus reais e restrições sobre o imóvel, independentemente de certificação específica pelo oficial.”  
+- Lei 6.015/1973, Art. 230: “Se na certidão constar ônus, o oficial fará a matrícula, e, logo em seguida ao registro, averbará a existência do ônus, sua natureza e valor, certificando o fato no título que devolverá à parte.”
+**Conclusão**  
+O ato deve ser **indefere via Nota Devolutiva**. A certidão de inteiro teor deve reproduzir integralmente a averbação de interdição/curatela; omiti-la violaria o disposto nos dispositivos citados.</t>
         </is>
       </c>
       <c r="H114" s="8" t="inlineStr">
@@ -8086,13 +8085,13 @@
         </is>
       </c>
       <c r="I114" s="8" t="n">
-        <v>26.74</v>
+        <v>25.55</v>
       </c>
       <c r="J114" s="8" t="n">
         <v>1771</v>
       </c>
       <c r="K114" s="8" t="n">
-        <v>656</v>
+        <v>717</v>
       </c>
       <c r="L114" s="10">
         <f>IF(COUNT(J114:K114)=2,(J114*Parametros!$B$3+K114*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -8149,7 +8148,7 @@
       </c>
       <c r="F115" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G115" s="8" t="inlineStr">
@@ -8172,13 +8171,13 @@
         </is>
       </c>
       <c r="I115" s="8" t="n">
-        <v>14.04</v>
+        <v>9.98</v>
       </c>
       <c r="J115" s="8" t="n">
         <v>1361</v>
       </c>
       <c r="K115" s="8" t="n">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="L115" s="10">
         <f>IF(COUNT(J115:K115)=2,(J115*Parametros!$B$3+K115*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -8239,25 +8238,44 @@
       </c>
       <c r="F116" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>**Resposta:** Indeferir o pedido via **Nota Devolutiva**.
-**Fundamentação jurídica**
-1. **LGPD – Tratamento de dados pessoais sensíveis**  
-   - **Art. 11, inc. I** – O tratamento de dados sensíveis (como dados de saúde) só pode ocorrer quando houver consentimento específico e destacado do titular para a finalidade pretendida.  
-   - **Art. 11, inc. II, alínea a** – Na ausência de consentimento, o tratamento só é permitido quando for indispensável para o cumprimento de obrigação legal ou regulatória. O simples fornecimento de cópia de documento arquivado a terceiro não se enquadra em nenhuma das hipóteses previstas (não há obrigação legal que imponha a divulgação, nem outra hipótese autorizadora).  
-2. **Procedimentos de certidão e cópia de documentos arquivados**  
-   - **Código de Normas CGJ‑CE, art. 1.128** e **art. 1.680**, §§ 1º e 2º – Os pedidos de certidão ou de documentos arquivados dependem de identificação do requerente e, quando não houver previsão legal específica de expedição, também exigem indicação da finalidade. Contudo, esses dispositivos tratam apenas da **exigência de identificação** e **finalidade**, não autorizam a divulgação de dados sensíveis que estejam protegidos pela LGPD.  
-3. **Conflito de normas**  
-   - A LGPD tem hierarquia superior no que tange à proteção de dados pessoais sensíveis. Assim, ainda que o requerente esteja devidamente identificado (conforme art. 1.128/1.680 da CGJ‑CE), a ausência de consentimento ou de hipótese legal que autorize o tratamento impede a prática do ato registral.  
-4. **Direito de acesso do titular**  
-   - **LGPD, art. 19** – O titular pode requerer acesso aos seus próprios dados, mas o pedido em questão não foi formulado pelo titular nem há comprovação de consentimento. Portanto, o direito de acesso não se aplica ao requerente.  
-**Conclusão operacional**
-- **Deve ser indeferido** o pedido de cópia do documento arquivado que contém dados de saúde, mediante emissão de **Nota Devolutiva** fundamentada nos dispositivos acima citados (LGPD art. 11, inc. I e II; Código de Normas CGJ‑CE art. 1.128 e art. 1.680).  
-*Obs.: Caso o requerente seja o titular dos dados ou apresente consentimento específico e destacado, o pedido poderia ser analisado sob a ótica do art. 11, inc. I, permitindo a entrega da cópia.*</t>
+          <t>**Resposta:** O pedido deve ser **praticado condicionado com tarjamento protetivo** (ou, na ausência de consentimento do titular, indeferido mediante Nota Devolutiva).  
+---
+### Fundamentação Legal
+| Norma | Dispositivo | Aplicação ao caso |
+|-------|-------------|-------------------|
+| **LGPD – Lei 13.709/2018** | **Art. 11, inc. I** | O tratamento de dados pessoais sensíveis (dados de saúde) só pode ocorrer com consentimento **específico e destacado** do titular para a finalidade pretendida. Não há indicação de que o titular tenha consentido com a cópia do título. |
+| LGPD | **Art. 11, inc. II‑e‑f** | As hipóteses de tratamento sem consentimento são: cumprimento de obrigação legal, proteção da vida/incolumidade, tutela da saúde etc. O simples fornecimento de cópia a terceiro não se enquadra em nenhuma dessas exceções. |
+| LGPD | **Art. 19** | O direito de acesso (cópia integral) só pode ser exercido **pelo titular** ou por seu representante legal, mediante requisição. Se o requerente não for o titular, o acesso não é permitido. |
+| **Provimento CNJ 149/2023** | **Art. 123, §§ 1‑4** | Pedidos de certidão ou cópia de documentos arquivados dependem de identificação do requerente; quando houver tentativa de tratamento em desacordo com as finalidades do Registro de Imóveis, aplica‑se o § 4º (tratamento inadequado). |
+| **Código de Normas CGJ‑CE** | **Art. 1.680, §§ 1‑4** | Reforça a necessidade de identificação e indica que, na ausência de finalidade compatível, o tratamento (cópia) deve ser vetado ou limitado (tarjamento). |
+| **Código de Normas CGJ‑CE** | **Art. 1.128, § 2** | Exige indicação de finalidade para pedidos de certidão de documentos arquivados sem previsão legal específica – o que se aplica ao título que contém dados de saúde. |
+---
+### Conclusão Operacional
+1. **Verificar a identidade do requerente** – confirmar se ele é o titular dos dados de saúde ou seu representante legal.  
+2. **Se o requerente for o titular** e houver **consentimento explícito** para a cópia, o documento pode ser fornecido integralmente, observando os requisitos de LGPD (art. 19).  
+3. **Se o requerente não for o titular** ou não houver consentimento, o tratamento (cópia integral) viola o art. 11 da LGPD. Nesse caso:  
+   - **Tarjamento protetivo** – disponibilizar a certidão ou cópia contendo apenas as informações necessárias ao ato registral, **ocultando ou anonimizando** os dados de saúde (ex.: rasurar o campo sensível).  
+   - **Nota Devolutiva** – caso o tarjamento inviabilize a finalidade do pedido (ex.: a parte requer a íntegra para comprovar condição de saúde em processo judicial), o pedido deve ser indeferido mediante Nota Devolutiva, indicando a impossibilidade de fornecimento sem violação da LGPD.  
+---
+### Procedimento recomendado
+| Etapa | Ação | Base legal |
+|-------|------|------------|
+| **1. Identificação** | Solicitar documento de identidade e, se necessário, procuração que comprove a qualidade de titular ou representante. | Art. 123, § 1º (CNJ) / Art. 1.680, § 1º (CGJ‑CE) |
+| **2. Verificação de consentimento** | Exigir declaração assinada de consentimento específico para a cópia do título contendo dados de saúde. | LGPD, Art. 11, I |
+| **3. Avaliação da finalidade** | Confirmar se a finalidade do pedido está amparada por alguma exceção do art. 11, II (ex.: tutela da saúde em procedimento médico). | LGPD, Art. 11, II |
+| **4. Decisão** | - **Consentimento válido** → expedir cópia integral.&lt;br&gt;- **Sem consentimento** → aplicar tarjamento protetivo ou indeferir com Nota Devolutiva. | LGPD, Art. 11; CNJ, Art. 123, § 4º; CGJ‑CE, Art. 1.680, § 4º |
+| **5. Registro** | Anotar a decisão (tarjamento ou indeferimento) no livro de notas e arquivar a cópia tarjada, se houver. | Princípio da transparência e prestação de contas (LGPD). |
+---
+**Resumo:**  
+- **Fornecimento integral** → somente se houver **consentimento específico** do titular ou se o requerente for o próprio titular exercendo o direito de acesso (LGPD, art. 19).  
+- **Tarjamento protetivo** → a solução padrão quando o requerente não for titular e não houver consentimento.  
+- **Indeferimento (Nota Devolutiva)** → quando o tarjamento impossibilitar a finalidade do pedido ou quando a solicitação for manifestamente incompatível com as hipóteses de tratamento previstas no art. 11 da LGPD.  
+&gt; **“Não encontrado no corpus.”** (caso a pergunta exigisse norma não presente no contexto fornecido).</t>
         </is>
       </c>
       <c r="H116" s="8" t="inlineStr">
@@ -8266,13 +8284,13 @@
         </is>
       </c>
       <c r="I116" s="8" t="n">
-        <v>3.27</v>
+        <v>4.5</v>
       </c>
       <c r="J116" s="8" t="n">
         <v>2082</v>
       </c>
       <c r="K116" s="8" t="n">
-        <v>1202</v>
+        <v>1795</v>
       </c>
       <c r="L116" s="10">
         <f>IF(COUNT(J116:K116)=2,(J116*Parametros!$B$3+K116*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -8329,12 +8347,22 @@
       </c>
       <c r="F117" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>Não encontrado no corpus.</t>
+          <t>**Ato registral:** praticado integralmente, desde que atendidos os requisitos de LGPD.
+**Fundamentação legal:**
+- **Art. 100 do Provimento CNJ 149/2023** – “Em caso de requerimento de certidões por meio da telemática, havendo necessidade de justificação do interesse na certidão, o solicitante será identificado por meio idôneo, reconhecido pela entidade responsável pela tramitação do serviço eletrônico compartilhado da respectiva especialidade cartorial.”  
+- **Art. 195 do Código de Normas CGJ‑CE** – “Em caso de requerimento de certidões por via telemática, havendo necessidade de justificação do interesse na certidão, o solicitante será identificado por meio idôneo, reconhecido pela entidade responsável pela tramitação do serviço eletrônico compartilhado da respectiva especialidade cartorial.”
+**Cuidados LGPD a observar ao enviar a certidão por e‑mail/WhatsApp:**
+1. **Identificação do solicitante** – confirmar a identidade do requerente por meio idôneo (ex.: assinatura digital, certificado digital, ou outro meio reconhecido pela entidade responsável).  
+2. **Transmissão segura** – utilizar canais criptografados (e‑mail com TLS, WhatsApp com criptografia de ponta a ponta) para evitar interceptação de dados pessoais.  
+3. **Limitação de acesso** – garantir que apenas o destinatário legítimo receba a certidão, evitando divulgação indevida.  
+4. **Registro de tratamento** – documentar o envio, incluindo data, hora, destinatário e meio de transmissão, conforme exigido pela LGPD.  
+5. **Consentimento ou base legal** – assegurar que o envio esteja respaldado por uma base legal adequada (ex.: consentimento do titular ou cumprimento de obrigação legal).  
+**Conclusão:** O envio da certidão por e‑mail ou WhatsApp é permitido, mas deve ser realizado **integralmente** apenas após a verificação da identidade do requerente e adoção de medidas de segurança previstas na LGPD. Se esses requisitos não forem atendidos, o ato deve ser **condicionado com tarjamento protetivo** ou, em caso de descumprimento grave, **indeferido via Nota Devolutiva**.</t>
         </is>
       </c>
       <c r="H117" s="8" t="inlineStr">
@@ -8343,13 +8371,13 @@
         </is>
       </c>
       <c r="I117" s="8" t="n">
-        <v>0.82</v>
+        <v>1.87</v>
       </c>
       <c r="J117" s="8" t="n">
         <v>1176</v>
       </c>
       <c r="K117" s="8" t="n">
-        <v>282</v>
+        <v>910</v>
       </c>
       <c r="L117" s="10">
         <f>IF(COUNT(J117:K117)=2,(J117*Parametros!$B$3+K117*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -8366,10 +8394,10 @@
       </c>
       <c r="S117" s="8" t="n"/>
       <c r="T117" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U117" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V117" s="11">
         <f>IF(AND(ISNUMBER(T117),T117&gt;0),U117/T117,"")</f>
@@ -8378,7 +8406,7 @@
       <c r="W117" s="8" t="inlineStr"/>
       <c r="X117" s="8" t="inlineStr">
         <is>
-          <t>NAO_ENCONTRADO</t>
+          <t>RESPONDIDA</t>
         </is>
       </c>
     </row>
@@ -8406,7 +8434,7 @@
       </c>
       <c r="F118" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G118" s="8" t="inlineStr">
@@ -8420,13 +8448,13 @@
         </is>
       </c>
       <c r="I118" s="8" t="n">
-        <v>10.11</v>
+        <v>20.37</v>
       </c>
       <c r="J118" s="8" t="n">
         <v>1417</v>
       </c>
       <c r="K118" s="8" t="n">
-        <v>427</v>
+        <v>221</v>
       </c>
       <c r="L118" s="10">
         <f>IF(COUNT(J118:K118)=2,(J118*Parametros!$B$3+K118*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -8483,23 +8511,41 @@
       </c>
       <c r="F119" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
-        </is>
-      </c>
-      <c r="G119" s="8" t="inlineStr"/>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
+        </is>
+      </c>
+      <c r="G119" s="8" t="inlineStr">
+        <is>
+          <t>**Decisão:** Praticar o ato registral integralmente – proceder à exclusão dos dados pessoais do titular da matrícula.
+**Fundamentação normativa**
+1. **LGPD – Art. 18, § 5º** – “O requerimento referido no § 3º deste artigo será atendido sem custos para o titular, nos prazos e nos termos previstos em regulamento.”  
+   → O pedido de exclusão constitui requerimento previsto no art. 18 e, portanto, deve ser atendido.
+2. **LGPD – Art. 18, § 6º** – “O responsável deverá informar, de maneira imediata, aos agentes de tratamento com os quais tenha realizado uso compartilhado de dados a correção, a eliminação, a anonimização ou o bloqueio dos dados…”  
+   → Após a exclusão no cartório, o responsável deve comunicar a eliminação aos demais agentes de tratamento que eventualmente tenham recebido esses dados.
+3. **LGPD – Art. 9, incisos I a VII** – Impõe ao controlador a obrigação de disponibilizar ao titular informações claras sobre a finalidade, forma e duração do tratamento, bem como os direitos do titular (art. 9, § 1º).  
+   → O cartório, na qualidade de controlador, deve garantir ao titular a transparência sobre o procedimento de exclusão e confirmar que o tratamento cessará.
+**Procedimento operacional**
+- Receber o requerimento por escrito (ou meio eletrônico que assegure a autenticidade do titular).  
+- Verificar a identidade do titular e a titularidade dos dados constantes na matrícula.  
+- Efetuar a exclusão dos dados pessoais solicitados, observando a necessidade de preservação de informações indispensáveis ao registro público (ex.: dados indispensáveis à validade do ato registral, nos termos da Lei 6.015/1973 – não abordado no corpus, mas que, se necessário, será tratado mediante **tarjamento protetivo**).  
+- Emitir nota de devolutiva confirmando a exclusão e informando a comunicação aos demais agentes de tratamento, nos termos do art. 18, § 6º.  
+- Arquivar o procedimento conforme a política de tratamento de dados pessoais do cartório.  
+**Conclusão:** Conforme o disposto no art. 18, §§ 5º e 6º da LGPD, o pedido de exclusão deve ser atendido integralmente, devendo o cartório proceder à eliminação dos dados pessoais do titular da matrícula e comunicar a eliminação aos demais agentes de tratamento.</t>
+        </is>
+      </c>
       <c r="H119" s="8" t="inlineStr">
         <is>
           <t>LGPD (Lei 13.709/2018) — Art. 9:p0; LGPD (Lei 13.709/2018) — Art. 18:p0; LGPD (Lei 13.709/2018) — Art. 11:p0; LGPD (Lei 13.709/2018) — Art. 4:p0; LGPD (Lei 13.709/2018) — Art. 20:p0</t>
         </is>
       </c>
       <c r="I119" s="8" t="n">
-        <v>18.13</v>
+        <v>12.68</v>
       </c>
       <c r="J119" s="8" t="n">
-        <v>1799</v>
+        <v>3598</v>
       </c>
       <c r="K119" s="8" t="n">
-        <v>2048</v>
+        <v>3057</v>
       </c>
       <c r="L119" s="10">
         <f>IF(COUNT(J119:K119)=2,(J119*Parametros!$B$3+K119*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -8516,10 +8562,10 @@
       </c>
       <c r="S119" s="8" t="n"/>
       <c r="T119" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U119" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="V119" s="11">
         <f>IF(AND(ISNUMBER(T119),T119&gt;0),U119/T119,"")</f>
@@ -8528,7 +8574,7 @@
       <c r="W119" s="8" t="inlineStr"/>
       <c r="X119" s="8" t="inlineStr">
         <is>
-          <t>RESPOSTA_VAZIA</t>
+          <t>RESPONDIDA</t>
         </is>
       </c>
     </row>
@@ -8556,23 +8602,28 @@
       </c>
       <c r="F120" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
-        </is>
-      </c>
-      <c r="G120" s="8" t="inlineStr"/>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
+        </is>
+      </c>
+      <c r="G120" s="8" t="inlineStr">
+        <is>
+          <t>Sim.  
+De acordo com o art. 18 da LGPD, “os direitos dos titulares são, em regra, exercidos em face do controlador, a quem compete, entre outras providências, **fornecer informações relativas ao tratamento**”. Como o registro de imóveis é o controlador dos dados pessoais do titular, você tem obrigação de informar quem consultou a matrícula.</t>
+        </is>
+      </c>
       <c r="H120" s="8" t="inlineStr">
         <is>
           <t>Guia ANPD — Agentes de Tratamento — p. 8:p8; Código de Normas CGJ-CE — Art. 1461:p299; Provimento CNJ 149/2023 — Art. 415:p265; LAI (Lei 12.527/2011) — Art. 30:p0; Provimento CNJ 149/2023 — Art. 89:p47</t>
         </is>
       </c>
       <c r="I120" s="8" t="n">
-        <v>30.84</v>
+        <v>20.78</v>
       </c>
       <c r="J120" s="8" t="n">
         <v>1851</v>
       </c>
       <c r="K120" s="8" t="n">
-        <v>2048</v>
+        <v>746</v>
       </c>
       <c r="L120" s="10">
         <f>IF(COUNT(J120:K120)=2,(J120*Parametros!$B$3+K120*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -8589,7 +8640,7 @@
       </c>
       <c r="S120" s="8" t="n"/>
       <c r="T120" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U120" s="8" t="n">
         <v>0</v>
@@ -8598,10 +8649,14 @@
         <f>IF(AND(ISNUMBER(T120),T120&gt;0),U120/T120,"")</f>
         <v/>
       </c>
-      <c r="W120" s="8" t="inlineStr"/>
+      <c r="W120" s="8" t="inlineStr">
+        <is>
+          <t>Art. 18 (LGPD (Lei 13.709/2018)) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
+        </is>
+      </c>
       <c r="X120" s="8" t="inlineStr">
         <is>
-          <t>RESPOSTA_VAZIA</t>
+          <t>RESPONDIDA</t>
         </is>
       </c>
     </row>
@@ -8629,38 +8684,30 @@
       </c>
       <c r="F121" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>**Procedimento a ser adotado:** **Retificação integral da matrícula**, nos termos do **Art. 1.386 do Código de Normas da CGJ‑CE**, mediante requerimento do titular.  
----
-### Fundamentação normativa
-1. **Código de Normas CGJ‑CE – Art. 1.386**  
-   &gt; “No que diz respeito à **retificação de dados de qualificação pessoal das partes**, caberá ao Oficial do Registro de Imóveis somente **retificar o erro à margem do registro** (matrícula, transcrição ou inscrição) do nome e estado civil do proprietário, que deverá apresentar requerimento com firma reconhecida ou assinado digitalmente, quando comprovado:  
+          <t>**Procedimento a ser adotado:** **Retificação registral praticada integralmente** (sem tarja protetiva e sem indeferimento).
+**Fundamentação normativa**
+1. **Código de Normas da CGJ‑CE – Art. 1.386**  
+   &gt; “No que diz respeito à retificação de dados de qualificação pessoal das partes, caberá ao Oficial do Registro de Imóveis somente retificar o erro à margem do registro (matrícula, transcrição ou inscrição) do nome e estado civil do proprietário, que deverá apresentar requerimento com firma reconhecida ou assinado digitalmente, quando comprovado:  
    &gt; a) que o nome lançado no assento não corresponde ao nome apresentado no registro civil …;  
-   &gt; b) que se trata do titular do domínio.”
-   → O pedido do titular enquadra‑se exatamente nessa hipótese: correção de dado pessoal (nome/estado civil) constante da matrícula.
-2. **LGPD – Art. 5, inc. I (definição de dado pessoal)**  
-   &gt; “**Dado pessoal**: informação relacionada a pessoa natural identificada ou identificável.”  
-   O nome ou estado civil constante da matrícula são dados pessoais, logo a LGPD reconhece o direito à correção.
-3. **LGPD – Art. 7, inc. VI (tratamento para exercício regular de direitos)**  
-   &gt; “Para o **exercício regular de direitos em processo judicial, administrativo ou arbitral**.”  
-   A correção de dados no registro imobiliário é necessária para o exercício de direitos reais sobre o bem.
-4. **LGPD – Art. 18, § 5º**  
-   &gt; “O requerimento referido no § 3º deste artigo será atendido **sem custos para o titular**, nos prazos e nos termos previstos em regulamento.”  
-   Assim, o titular tem direito à correção sem ônus, devendo ser atendido pelo cartório mediante a retificação prevista no art. 1.386.
----
-### Passos operacionais (conforme Art. 1.386)
-1. **Requerimento do titular** – deverá ser apresentado com **firma reconhecida** ou **assinatura digital**.  
-2. **Documentação comprobatória** – certidão de nascimento, casamento ou registro de estrangeiro, conforme o caso, para demonstrar a divergência entre o dado registrado e o dado constante do registro civil.  
-3. **Análise pelo Oficial** – verificação da autenticidade dos documentos e da pertinência do pedido.  
-4. **Retificação à margem** – inserção da correção na matrícula, transcrição ou inscrição, mantendo a integridade do histórico registral.  
-5. **Comunicação ao titular** – informe de que a retificação foi efetuada, sem custos, nos termos do § 5º do Art. 18 da LGPD.
----
-### Conclusão
-O pedido de correção de dado pessoal errado na matrícula deve ser **praticado integralmente como retificação registral**, nos termos do **Art. 1.386 do Código de Normas da CGJ‑CE**, atendendo simultaneamente ao direito de correção previsto na LGPD (Art. 5, I; Art. 7, VI; Art. 18, § 5º). Não há necessidade de indeferimento ou de aplicação de “tarjamento protetivo”.</t>
+   &gt; b) que se trata do titular do domínio.”  
+   – O pedido do titular enquadra‑se exatamente na hipótese (a) e (b) do inciso acima, logo o ato de correção deve ser realizado por **retificação à margem da matrícula**, mediante requerimento formal.
+2. **LGPD – Art. 18, §§ 5º e 6º** (direito à correção de dados pessoais)  
+   &gt; “§ 5º O requerimento referido no § 3º deste artigo será atendido sem custos para o titular…  
+   &gt; § 6º O responsável deverá informar, de maneira imediata, aos agentes de tratamento … a correção, a eliminação, a anonimização ou o bloqueio dos dados…”  
+   – O titular exerce o direito de correção previsto na LGPD; o controlador (no caso, o Cartório de Registro de Imóveis) deve atender ao pedido, o que se operacionaliza mediante a **retificação registral** prevista no art. 1.386 da CGJ‑CE.
+**Conclusão prática**
+- O pedido deve ser **aceito** e **atendido integralmente** por meio de **retificação à margem da matrícula**, nos termos do art. 1.386 da CGJ‑CE.  
+- O requerimento deve conter:  
+  1. Petição assinada digitalmente ou com firma reconhecida;  
+  2. Documentos comprobatórios (certidão de nascimento, casamento ou registro de estrangeiro) que demonstrem o nome correto;  
+  3. Indicação clara do erro a ser corrigido.  
+- Não há necessidade de tarja protetiva, pois o dado a ser corrigido não se trata de informação sensível que exija restrição de acesso.  
+- O cartório deve ainda observar o disposto nos §§ 5º e 6º do art. 18 da LGPD, garantindo que a correção seja efetuada sem custos ao titular e comunicando, se houver outros agentes de tratamento, a atualização dos dados.</t>
         </is>
       </c>
       <c r="H121" s="8" t="inlineStr">
@@ -8669,13 +8716,13 @@
         </is>
       </c>
       <c r="I121" s="8" t="n">
-        <v>2.83</v>
+        <v>2.64</v>
       </c>
       <c r="J121" s="8" t="n">
         <v>1776</v>
       </c>
       <c r="K121" s="8" t="n">
-        <v>1081</v>
+        <v>967</v>
       </c>
       <c r="L121" s="10">
         <f>IF(COUNT(J121:K121)=2,(J121*Parametros!$B$3+K121*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -8692,10 +8739,10 @@
       </c>
       <c r="S121" s="8" t="n"/>
       <c r="T121" s="8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="U121" s="8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="V121" s="11">
         <f>IF(AND(ISNUMBER(T121),T121&gt;0),U121/T121,"")</f>
@@ -8732,26 +8779,19 @@
       </c>
       <c r="F122" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>**Resposta:** Indeferido via Nota Devolutiva.
+          <t>**Resposta:** Sim. O convênio pode ser firmado integralmente.
 **Fundamentação normativa**
-1. **Provimento CNJ 149/2023 – Art. 148**  
-   &gt; “As entidades representativas dos notários e dos registradores poderão firmar convênio com a RFB, as Juntas Comerciais dos estados, o Departamento de Registro Empresarial e Integração (DREI), a Comissão de Valores Mobiliários (CVM) e quaisquer outros órgãos… com o objetivo de manter atualizado o cadastro de que trata esta seção.”  
-   – O dispositivo restringe a celebração de convênios **exclusivamente às entidades representativas dos notários e dos registradores**. Uma empresa privada (imobiliária/fintech) não se enquadra nessa categoria, logo não possui legitimidade para firmar convênio nos termos do art. 148.
-2. **Provimento CNJ 149/2023 – Art. 168**  
-   &gt; “O CNB/CF poderá firmar convênio com a RFB, as Juntas Comerciais dos estados, o Departamento de Registro Empresarial e Integração (DREI), a Comissão de Valores Mobiliários (CVM)… com o objetivo de manter atualizado o cadastro de que trata esta subseção.”  
-   – Também limita a possibilidade de convênio ao **CNB/CF** (Conselho Nacional de Notários e Registradores), não a empresas privadas.
-3. **Provimento CNJ 149/2023 – Art. 334**  
-   &gt; “O acesso dos oficiais de registro de imóveis ao Programa Gerador e Validador será feito mediante certificado digital ICP‑Brasil ou comunicação por Application Programming Interface (API).”  
-   – O acesso ao PGV está **restrito aos oficiais de registro** (ou prepostos designados), mediante certificado digital ou API, não sendo previsto acesso direto a terceiros que não sejam oficiais ou seus prepostos.
-**Conclusão prática**
-- Não há previsão legal que autorize a celebração de convênio entre o Cartório de Registro de Imóveis e uma empresa privada para fornecimento de dados de matrículas em lote ou via API.  
-- O acesso ao Programa Gerador e Validador (PGV) está limitado a oficiais de registro, mediante certificado digital ou API, conforme art. 334.  
-- Portanto, o pedido de convênio deve ser **indeferido** e formalizado mediante **Nota Devolutiva**, indicando a inexistência de amparo normativo para a celebração do referido convênio.</t>
+1. **Provimento CNJ 149/2023 – Art. 148** – “As entidades representativas dos notários e dos registradores poderão firmar convênio com a RFB, as Juntas Comerciais dos estados, o Departamento de Registro Empresarial e Integração (DREI), a Comissão de Valores Mobiliários (CVM) e quaisquer outros órgãos… com o objetivo de manter atualizado o cadastro de que trata esta seção.”  
+2. **Provimento CNJ 149/2023 – Art. 168** – Autoriza o CNB/CF a firmar convênio com a RFB, Juntas Comerciais, DREI, CVM e demais órgãos que detenham dados sobre atos constitutivos, modificativos, extintivos ou participações societárias, visando a atualização do cadastro.  
+3. **Provimento CNJ 149/2023 – Art. 334** – “O acesso dos oficiais de registro de imóveis ao Programa Gerador e Validador será feito mediante certificado digital ICP‑Brasil ou comunicação por Application Programming Interface (API).”  
+**Conclusão operativa:**  
+- É plenamente possível celebrar convênio com a empresa imobiliária/fintech para o acesso em lote ou via API aos dados de matrículas, nos termos dos artigos citados.  
+- Não há necessidade de imposição de tarja protetiva nem de indeferimento; o ato deve ser praticado integralmente.</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
@@ -8760,13 +8800,13 @@
         </is>
       </c>
       <c r="I122" s="8" t="n">
-        <v>2.48</v>
+        <v>3.32</v>
       </c>
       <c r="J122" s="8" t="n">
         <v>1615</v>
       </c>
       <c r="K122" s="8" t="n">
-        <v>911</v>
+        <v>637</v>
       </c>
       <c r="L122" s="10">
         <f>IF(COUNT(J122:K122)=2,(J122*Parametros!$B$3+K122*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -8783,10 +8823,10 @@
       </c>
       <c r="S122" s="8" t="n"/>
       <c r="T122" s="8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U122" s="8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="V122" s="11">
         <f>IF(AND(ISNUMBER(T122),T122&gt;0),U122/T122,"")</f>
@@ -8823,27 +8863,19 @@
       </c>
       <c r="F123" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-120b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-120b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>**Resposta:** O compartilhamento de dados com o Operador Nacional de Registro Eletrônico de Imóveis (ONR) / SREI e com as centrais de serviços eletrônicos pode ser realizado **integralmente**, sem a exigência de consentimento adicional ou de base legal suplementar, desde que observados os requisitos já previstos nos dispositivos normativos citados.
----
-### Fundamentação normativa
-| Norma | Dispositivo | Conteúdo relevante |
-|-------|-------------|--------------------|
-| **Código de Normas CGJ‑CE** | Art. 1749 | “Os responsáveis pelas serventias de registro de imóveis … adotarão as medidas necessárias para a integração, diretamente com o representante legal do ONR – Operador Nacional de Registro Eletrônico de Imóveis.” |
-| **Provimento CNJ 149/2023** | Art. 101 | “O compartilhamento de dados com centrais de serviços eletrônicos compartilhados é compatível com a proteção de dados pessoais, devendo as centrais observar a adequação, necessidade e persecução da finalidade dos dados a serem compartilhados …” |
-| **Provimento CNJ 149/2023** | Art. 101, parágrafo único | “Deverá ser dada preferência … à modalidade de descentralização das bases de dados … evitando a transferência de bases de dados, salvo quando necessária para atingir a finalidade das centrais …” |
-| **Código de Normas CGJ‑CE** | Art. 196 | Reitera o mesmo princípio do art. 101 do Provimento CNJ 149/2023, reforçando a adequação, necessidade e finalidade como requisitos para o compartilhamento. |
-Esses dispositivos já constituem a **base legal** para o tratamento e o compartilhamento de dados pessoais no âmbito do SREI/ONR e das centrais eletrônicas, atendendo aos princípios da LGPD (adequação, necessidade e finalidade) sem necessidade de consentimento específico do titular, quando o tratamento for indispensável ao cumprimento das finalidades previstas na lei de registros (Lei 6.015/1973) e nos regulamentos citados.
----
-### Conclusão prática
-- **Ato registral:** pode ser praticado **integralmente**.  
-- **Tarjamento protetivo:** não se impõe, pois a normativa já garante a proteção dos dados mediante os requisitos de adequação, necessidade e finalidade.  
-- **Nota Devolutiva:** indeferimento não se justifica, já que não há exigência de consentimento adicional nem de base legal suplementar.
-**Portanto, o compartilhamento com ONR/SREI e com as centrais eletrônicas está plenamente amparado pelos artigos 1749 do Código de Normas CGJ‑CE, 101 (e seu parágrafo único) do Provimento CNJ 149/2023 e 196 do Código de Normas CGJ‑CE, não sendo necessário obter consentimento ou outra base legal adicional.**</t>
+          <t>**Resposta:** O ato registral deve ser praticado integralmente.
+**Fundamentação normativa**
+1. **Integração com o ONR** – O Código de Normas da CGJ‑CE, art. 1749, determina que as serventias “adotarão as medidas necessárias para a integração, diretamente com o representante legal do ONR – Operador Nacional de Registro Eletrônico de Imóveis”. Não há exigência de autorização adicional ou de consentimento do titular dos dados para essa integração.
+2. **Compartilhamento de dados com centrais eletrônicas** – O Provimento CNJ 149/2023, art. 101, dispõe que “o compartilhamento de dados com centrais de serviços eletrônicos compartilhados é compatível com a proteção de dados pessoais, devendo as centrais observar a adequação, necessidade e persecução da finalidade dos dados a serem compartilhados…”. O parágrafo único ainda enfatiza a preferência pela **descentralização** das bases, evitando a transferência de bases de dados quando possível. Não há menção à necessidade de consentimento do titular para o compartilhamento nos termos previstos.
+3. **Reforço da mesma regra** – O Código de Normas da CGJ‑CE, art. 196, repete integralmente o conteúdo do art. 101 do Provimento CNJ 149/2023, confirmando que o compartilhamento é permitido desde que observados os princípios de adequação, necessidade e finalidade, sem exigir consentimento adicional.
+**Conclusão prática**
+- Não é necessária **base legal adicional** nem **consentimento explícito** do titular dos dados para o compartilhamento com o ONR/SREI e as centrais eletrônicas, desde que o procedimento observe os requisitos de adequação, necessidade e finalidade previstos nos dispositivos citados.
+- Portanto, o ato registral pode ser **praticado integralmente**, atendendo às exigências dos artigos acima mencionados.</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
@@ -8852,13 +8884,13 @@
         </is>
       </c>
       <c r="I123" s="8" t="n">
-        <v>2.62</v>
+        <v>2.11</v>
       </c>
       <c r="J123" s="8" t="n">
         <v>1529</v>
       </c>
       <c r="K123" s="8" t="n">
-        <v>969</v>
+        <v>669</v>
       </c>
       <c r="L123" s="10">
         <f>IF(COUNT(J123:K123)=2,(J123*Parametros!$B$3+K123*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -8915,53 +8947,34 @@
       </c>
       <c r="F124" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
           <t>**O que mudou com o Provimento nº 15/2026/CGJCE na qualificação das partes para registro?**
-O provimento alterou a redação dos requisitos de qualificação das partes no registro, conforme disposto no **Art. 1.103** (Código de Normas CGJ‑CE) e no **Art. 817** (Código de Normas CGJ‑CE).  
-1. **Art. 1.103 – Incisos II e V**  
-   - **Inciso II** passou a exigir, para pessoa natural, a **qualificação completa** que inclui:  
-     - nome, domicílio e nacionalidade;  
-     - **estado civil**;  
-     - **regime de bens do casamento ou da união estável** (se declarado no instrumento);  
-     - **profissão**;  
-     - **número de inscrição no CPF ou documento de identidade**; ou, na falta deste, a **filiação**.  
-   - Para pessoa jurídica, a qualificação deve conter:  
-     - **denominação social**;  
-     - **número de inscrição no CNPJ**;  
-     - **sede**.  
-   - **Inciso V** passou a exigir, além do valor do contrato, da coisa ou da dívida, a informação de:  
-     - prazo;  
-     - condições;  
-     - encargos;  
-     - juros.  
-2. **Parágrafo único do Art. 1.103**  
-   - Foi incluído um parágrafo único que **venda a prática de ato registral** com determinados requisitos não atendidos (ex.: ausência de qualificação completa, falta de regime de bens declarado, etc.).  
-3. **Art. 817 – Alínea “a” do Inciso I**  
-   - A redação da alínea “a” do inciso I do art. 817 foi revista para reforçar a obrigatoriedade de incluir, para pessoa física, nacionalidade, estado civil, profissão, número do documento de identidade e repartição expedidora, número de inscrição no CPF, filiação, domicílio e residência, nome do cônjuge ou companheiro (quando for o caso) e regime de bens do casamento ou da união estável (se declarado pelas partes).  
-**Resumo da mudança:**  
-O provimento ampliou e detalhou a qualificação das partes, exigindo a inclusão de estado civil, regime de bens, profissão, CPF ou identidade (ou filiação) para pessoas físicas, e denominação, CNPJ e sede para pessoas jurídicas, além de reforçar a obrigatoriedade de registrar o regime de bens declarado. O parágrafo único agora proíbe a prática de atos registrais que não atendam a esses requisitos.  
-**Dispositivos citados:**  
-- Art. 1.103, incisos II e V, parágrafo único (Código de Normas CGJ‑CE).  
-- Art. 817, alínea “a” do inciso I (Código de Normas CGJ‑CE).</t>
+O provimento alterou a redação dos dispositivos que tratam da qualificação das partes nos registros, tornando‑a mais rigorosa e detalhada. As principais mudanças são:
+| Dispositivo | Alteração | Conteúdo exigido |
+|-------------|-----------|------------------|
+| **Art. 817, I a)** | Redação atualizada | Qualificação completa de pessoa física: nacionalidade, estado civil, profissão, número do documento de identidade e repartição expedidora, número de inscrição no CPF, filiação, domicílio e residência, nome do cônjuge ou companheiro (quando houver) e regime de bens do casamento ou da união estável (se declarado). Vedada a utilização das expressões “regime comum” ou “regime legal”. |
+| **Art. 1.103, II a) e b)** | Redação atualizada | 1. **Pessoa natural**: além dos dados já citados, deve constar o número de inscrição no CPF ou documento de identidade, ou, na falta deste, a filiação. &lt;br&gt;2. **Pessoa jurídica**: denominação social, número de inscrição no CNPJ e sede. |
+Essas alterações reforçam a exigência de **qualificação completa e não genérica** das partes, impedindo a prática de atos registrais com qualificação incompleta, genérica ou indeterminada (conforme o § único do Art. 1 do Provimento 15/2026/CGJCE).  
+**Conclusão**: O Provimento nº 15/2026/CGJCE atualizou a qualificação das partes, exigindo que todas as informações obrigatórias estejam presentes e expressas de forma clara, sem o uso de termos genéricos.</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
         <is>
-          <t>Provimento 15/2026/CGJCE — Art. 1:p2; Provimento 15/2026/CGJCE — Preâmbulo:p1; Código de Normas CGJ-CE — Art. 1103:p224</t>
+          <t>Provimento 15/2026/CGJCE — Art. 1:p2; Provimento 15/2026/CGJCE — Preâmbulo:p1</t>
         </is>
       </c>
       <c r="I124" s="8" t="n">
-        <v>9.35</v>
+        <v>1.94</v>
       </c>
       <c r="J124" s="8" t="n">
-        <v>1500</v>
+        <v>1201</v>
       </c>
       <c r="K124" s="8" t="n">
-        <v>1475</v>
+        <v>1331</v>
       </c>
       <c r="L124" s="10">
         <f>IF(COUNT(J124:K124)=2,(J124*Parametros!$B$3+K124*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -8978,10 +8991,10 @@
       </c>
       <c r="S124" s="8" t="n"/>
       <c r="T124" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U124" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V124" s="11">
         <f>IF(AND(ISNUMBER(T124),T124&gt;0),U124/T124,"")</f>
@@ -8989,7 +9002,7 @@
       </c>
       <c r="W124" s="8" t="inlineStr">
         <is>
-          <t>Art. 817 (Código de Normas CGJ-CE) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]; Art. 817 (norma não informada) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
+          <t>Art. 817 (norma não informada) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]; Art. 1103 (norma não informada) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
         </is>
       </c>
       <c r="X124" s="8" t="inlineStr">
@@ -9022,27 +9035,19 @@
       </c>
       <c r="F125" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
           <t>**Requisitos para emissão de certidão digital (Código de Normas CGJ‑CE)**  
-| Requisito | Dispositivo legal | Observação |
-|-----------|-------------------|------------|
-| **Uso de formulário próprio, timbrado e oficial** | Art. 1127, § 1º, inciso I | A certidão deve ser lavrada em formulário próprio, timbrado e pertinente ao ato praticado, vedada a utilização de impressos não oficiais. |
-| **Formato digital nativo** | Art. 1129 | Certidões de imóveis já objeto de matrícula eletrônica, após a “primeira qualificação eletrônica”, são expedidas em formato nativo‑digital estruturado, contendo a situação jurídica atual do imóvel (descrição, titularidade e ônus reais não cancelados). |
-| **Assinatura eletrônica com certificado ICP‑Brasil** | Art. 1127, § 1º, Parágrafo único | Documentos assinados com certificado digital, realizados e/ou enviados pela Internet, devem atender aos requisitos da Infraestrutura de Chaves Públicas Brasileira (ICP‑Brasil). |
-| **Carimbo de tempo (timestamp)** | Art. 140, § 3º | A escrituração dos livros em formato digital deve incluir carimbo de tempo, além de assinatura eletrônica com certificado ICP‑Brasil. |
-| **Armazenamento e backup** | Art. 140, § 3º | O arquivo digital deve ser mantido na própria serventia e submetido à cópia de segurança (backup) regular. |
-| **Indicação de finalidade e identificação do solicitante** | Art. 1128, § 3º e § 4º | Fichas físicas ou digitais contendo dados de identificação e indicação de finalidade devem ser formadas; o titular pode requisitar as informações. O oficial pode recusar o fornecimento se houver tentativa de tratamento de dados em desacordo com as finalidades do Registro de Imóveis e os princípios da LGPD. |
-**Resumo**  
-Para emitir uma certidão digital, o oficial deve:  
-1. Utilizar formulário próprio, timbrado e oficial;  
-2. Emitir a certidão em formato nativo‑digital estruturado (para imóveis já eletrônicos, após a primeira qualificação);  
-3. Assinar eletronicamente com certificado ICP‑Brasil e incluir carimbo de tempo;  
-4. Armazenar o arquivo na serventia e manter backup;  
-5. Garantir que a ficha ou prontuário contenha identificação do solicitante e indicação de finalidade, respeitando a LGPD.</t>
+| Requisito | Dispositivo normativo |
+|-----------|-----------------------|
+| 1. Utilizar formulário próprio, timbrado e oficial, proibida a utilização de impressos não oficiais. | Art. 1127, § 1º, I |
+| 2. Se a certidão for assinada ou enviada pela Internet, deve atender aos requisitos da Infraestrutura de Chaves Públicas Brasileira (ICP‑Brasil). | Art. 1127, § 1º, único |
+| 3. Certidões de imóveis já objeto de matrícula eletrônica, após a “primeira qualificação eletrônica”, devem ser expedidas em formato nato‑digital estruturado, contendo a situação jurídica atual do imóvel (descrição, titularidade e ônus reais não cancelados). | Art. 1129 |
+| 4. Para escrituração de livros em formato digital, o arquivo deve ser assinado eletronicamente com certificado digital padrão ICP‑Brasil, pode incluir carimbo do tempo e deve ser mantido na própria serventia, com cópia de segurança regular. | Art. 140, § 3º |
+Esses são os requisitos expressos no Código de Normas CGJ‑CE para a emissão de certidão digital.</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
@@ -9051,13 +9056,13 @@
         </is>
       </c>
       <c r="I125" s="8" t="n">
-        <v>14.18</v>
+        <v>17.61</v>
       </c>
       <c r="J125" s="8" t="n">
         <v>1281</v>
       </c>
       <c r="K125" s="8" t="n">
-        <v>1009</v>
+        <v>696</v>
       </c>
       <c r="L125" s="10">
         <f>IF(COUNT(J125:K125)=2,(J125*Parametros!$B$3+K125*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -9074,10 +9079,10 @@
       </c>
       <c r="S125" s="8" t="n"/>
       <c r="T125" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U125" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V125" s="11">
         <f>IF(AND(ISNUMBER(T125),T125&gt;0),U125/T125,"")</f>
@@ -9114,24 +9119,26 @@
       </c>
       <c r="F126" s="8" t="inlineStr">
         <is>
-          <t>groq/openai/gpt-oss-20b k=5 (f67f244)</t>
+          <t>groq/openai/gpt-oss-20b k=5 (26168ce)</t>
         </is>
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>**Obrigação da serventia**
-O envio indevido de uma certidão contendo dados pessoais exige que a serventia:
-1. **Corrija imediatamente o erro** – remova a certidão do e‑mail errado e envie-a ao destinatário correto.  
-   *Art. 103 do Provimento CNJ 149/2023* – “O responsável pela serventia extrajudicial efetuará, sempre que possível, a criptografia ou a pseudonimização de dados pessoais para o acesso a informações ou transferência dos dados para terceiros.”
-2. **Implemente medidas de proteção** – caso a correção não seja imediata, a serventia deve criptografar ou pseudonimizar os dados antes de reenviá‑los, garantindo que a informação não seja acessível a terceiros não autorizados.  
-   *Art. 103 do Provimento CNJ 149/2023* (mesma referência acima).
-3. **Notifique o destinatário original** – informe ao e‑mail que recebeu a certidão por engano que o documento foi enviado erroneamente e que os dados não devem ser utilizados ou divulgados.  
-   *Art. 178 do Código de Normas CGJ‑CE* – “Os responsáveis pelas serventias extrajudiciais deverão atender às disposições da Lei Geral de Proteção de Dados Pessoais (LGPD) … obedecendo a seus fundamentos, princípios e obrigações concernentes à governança do tratamento de dados pessoais.”
-4. **Forneça transparência** – disponibilize, conforme Art. 97 do Provimento CNJ 149/2023, avisos de privacidade e proteção de dados, explicando o ocorrido e as medidas adotadas.  
-   *Art. 97 do Provimento CNJ 149/2023* – “Deverão ser disponibilizadas pelos responsáveis pelas serventias informações adequadas a respeito dos procedimentos de tratamento de dados pessoais, nos termos do art. 9.º da LGPD, por meio de: I — aviso de privacidade e proteção de dados; …”
-5. **Registre o incidente** – documente a ocorrência e as ações corretivas, para eventual auditoria ou verificação pelo corregedor permanente.  
-   *Art. 105 do Provimento CNJ 149/2023* – “Na correição anual será verificada pelo corregedor permanente a adaptação de suas práticas de tratamento de dados pessoais à LGPD e a este Código de Normas.”
-Em síntese, a serventia deve praticar a correção integral do ato, aplicando criptografia ou pseudonimização quando possível, notificando o destinatário original, garantindo transparência e registrando o incidente, em conformidade com os dispositivos citados.</t>
+          <t>**Obrigação da serventia**  
+O envio de uma certidão contendo dados pessoais para o e‑mail errado configura, no mínimo, um erro de tratamento de dados que exige correção imediata e medidas de mitigação, nos termos das normas de proteção de dados aplicáveis à serventia.
+| O que deve ser feito | Dispositivo normativo que fundamenta |
+|----------------------|--------------------------------------|
+| **Corrigir o envio** – a serventia deve reenviar a certidão ao destinatário correto e impedir a divulgação indevida. | Art. 103 do Provimento CNJ 149/2023 – “o responsável pela serventia extrajudicial efetuará, sempre que possível, a criptografia ou a pseudonimização de dados pessoais para o acesso a informações ou transferência dos dados para terceiros.” |
+| **Aplicar criptografia ou pseudonimização** – caso a certidão contenha dados sensíveis ou de natureza pessoal, a serventia deve, sempre que possível, proteger esses dados antes de qualquer reenvio ou correção. | Art. 103 do Provimento CNJ 149/2023 |
+| **Garantir a conformidade com a LGPD** – a serventia deve assegurar que o tratamento de dados pessoais, inclusive a correção de erro, esteja em conformidade com os princípios, fundamentos e obrigações da Lei Geral de Proteção de Dados. | Art. 178 do Código de Normas CGJ‑CE |
+| **Fornecer transparência ao titular** – a serventia deve disponibilizar, de forma clara e acessível, informações sobre o tratamento de dados, incluindo a ocorrência do erro e as medidas adotadas para corrigi‑lo. | Art. 97 do Provimento CNJ 149/2023 (aviso de privacidade e proteção de dados) |
+| **Identificar o solicitante** – se a certidão foi solicitada por meio telemático, a serventia deve ter identificado o solicitante de forma idônea, conforme exigido para a tramitação do serviço eletrônico. | Art. 100 do Provimento CNJ 149/2023 |
+Em síntese, a serventia deve:  
+1. **Corrigir imediatamente** o envio incorreto;  
+2. **Aplicar criptografia ou pseudonimização** (se possível) antes de reenviar ou corrigir a certidão;  
+3. **Assegurar a conformidade com a LGPD** (Art. 178);  
+4. **Fornecer transparência** ao titular dos dados (Art. 97); e  
+5. **Confirmar a identificação do solicitante** (Art. 100).</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
@@ -9140,13 +9147,13 @@
         </is>
       </c>
       <c r="I126" s="8" t="n">
-        <v>18.64</v>
+        <v>16.63</v>
       </c>
       <c r="J126" s="8" t="n">
         <v>1276</v>
       </c>
       <c r="K126" s="8" t="n">
-        <v>1363</v>
+        <v>1180</v>
       </c>
       <c r="L126" s="10">
         <f>IF(COUNT(J126:K126)=2,(J126*Parametros!$B$3+K126*Parametros!$B$4)/1000000*Parametros!$B$5,"")</f>
@@ -9163,10 +9170,10 @@
       </c>
       <c r="S126" s="8" t="n"/>
       <c r="T126" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U126" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="V126" s="11">
         <f>IF(AND(ISNUMBER(T126),T126&gt;0),U126/T126,"")</f>
@@ -9174,7 +9181,7 @@
       </c>
       <c r="W126" s="8" t="inlineStr">
         <is>
-          <t>Art. 9 (LGPD (Lei 13.709/2018)) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
+          <t>Art. 178 (LGPD (Lei 13.709/2018)) → NORMA_DIVERGENTE [recuperado em: Código de Normas CGJ-CE]</t>
         </is>
       </c>
       <c r="X126" s="8" t="inlineStr">

</xml_diff>

<commit_message>
feat: versiona o verificador, separa FORA_DO_CORPUS e mede cobertura
- VERIFICADOR_VERSAO = 2 gravada no relatório, no JSON, no terminal e
  na planilha (Parametros!B6 e cabeçalhos das taxas)
- nova categoria FORA_DO_CORPUS: norma citada inexistente no corpus
  (ex.: Código Civil), separada de NAO_RECUPERADA (falha de busca);
  o número de verificadas não muda
- cobertura_fundamentada = perguntas com ao menos uma citação
  verificada / total de perguntas, impressa ao lado da
  taxa_verificavel e na coluna P do Resumo
- verificar(texto, trechos) aceita dicts, tuplas (norma, artigo) e
  rótulos "Norma — Art. N", com nome de norma normalizado, para
  re-pontuar respostas de outros sistemas
- --reverificar: re-pontua um JSON salvo sem LLM
- re-pontuação da execução de 13/10 11h35 (v2): taxa_verificavel
  47/55 = 85%, cobertura_fundamentada 18/25 = 72%, 1 fora do corpus
- relatório 10 com a versão ao lado das taxas
</commit_message>
<xml_diff>
--- a/docs/fase3/benchmark/planilha_benchmark.xlsx
+++ b/docs/fase3/benchmark/planilha_benchmark.xlsx
@@ -1596,7 +1596,7 @@
       </c>
       <c r="V1" s="6" t="inlineStr">
         <is>
-          <t>Taxa verificável</t>
+          <t>Taxa verificável (verificador v2)</t>
         </is>
       </c>
       <c r="W1" s="6" t="inlineStr">
@@ -8205,7 +8205,7 @@
       </c>
       <c r="W115" s="8" t="inlineStr">
         <is>
-          <t>Art. 543 (OUTRA: codigo civil) → NAO_RECUPERADA [recuperado em: nenhum trecho recuperado]</t>
+          <t>Art. 543 (OUTRA: codigo civil) → FORA_DO_CORPUS [recuperado em: nenhum trecho recuperado]</t>
         </is>
       </c>
       <c r="X115" s="8" t="inlineStr">
@@ -9304,6 +9304,21 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Versão do verificador de citações</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Preenchida pelo run_rag_benchmark.py; nenhuma taxa de citações vale sem esta versão</t>
+        </is>
+      </c>
+    </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
@@ -9390,7 +9405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9408,6 +9423,7 @@
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9475,7 +9491,7 @@
       </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>Taxa verificável (citações)</t>
+          <t>Taxa verificável (citações, v2)</t>
         </is>
       </c>
       <c r="M3" s="6" t="inlineStr">
@@ -9491,6 +9507,11 @@
       <c r="O3" s="6" t="inlineStr">
         <is>
           <t>Resposta vazia</t>
+        </is>
+      </c>
+      <c r="P3" s="6" t="inlineStr">
+        <is>
+          <t>Cobertura fundamentada (perguntas, v2)</t>
         </is>
       </c>
     </row>
@@ -9556,6 +9577,10 @@
         <f>COUNTIFS(Respostas!$B$2:$B$126,$A4,Respostas!$X$2:$X$126,"RESPOSTA_VAZIA")</f>
         <v/>
       </c>
+      <c r="P4" s="11">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A4,Respostas!$T$2:$T$126,"&gt;=0")=0,"",COUNTIFS(Respostas!$B$2:$B$126,$A4,Respostas!$U$2:$U$126,"&gt;0")/COUNTIFS(Respostas!$B$2:$B$126,$A4))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -9619,6 +9644,10 @@
         <f>COUNTIFS(Respostas!$B$2:$B$126,$A5,Respostas!$X$2:$X$126,"RESPOSTA_VAZIA")</f>
         <v/>
       </c>
+      <c r="P5" s="11">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A5,Respostas!$T$2:$T$126,"&gt;=0")=0,"",COUNTIFS(Respostas!$B$2:$B$126,$A5,Respostas!$U$2:$U$126,"&gt;0")/COUNTIFS(Respostas!$B$2:$B$126,$A5))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -9682,6 +9711,10 @@
         <f>COUNTIFS(Respostas!$B$2:$B$126,$A6,Respostas!$X$2:$X$126,"RESPOSTA_VAZIA")</f>
         <v/>
       </c>
+      <c r="P6" s="11">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A6,Respostas!$T$2:$T$126,"&gt;=0")=0,"",COUNTIFS(Respostas!$B$2:$B$126,$A6,Respostas!$U$2:$U$126,"&gt;0")/COUNTIFS(Respostas!$B$2:$B$126,$A6))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -9745,6 +9778,10 @@
         <f>COUNTIFS(Respostas!$B$2:$B$126,$A7,Respostas!$X$2:$X$126,"RESPOSTA_VAZIA")</f>
         <v/>
       </c>
+      <c r="P7" s="11">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A7,Respostas!$T$2:$T$126,"&gt;=0")=0,"",COUNTIFS(Respostas!$B$2:$B$126,$A7,Respostas!$U$2:$U$126,"&gt;0")/COUNTIFS(Respostas!$B$2:$B$126,$A7))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -9806,6 +9843,10 @@
       </c>
       <c r="O8" s="9">
         <f>COUNTIFS(Respostas!$B$2:$B$126,$A8,Respostas!$X$2:$X$126,"RESPOSTA_VAZIA")</f>
+        <v/>
+      </c>
+      <c r="P8" s="11">
+        <f>IF(COUNTIFS(Respostas!$B$2:$B$126,$A8,Respostas!$T$2:$T$126,"&gt;=0")=0,"",COUNTIFS(Respostas!$B$2:$B$126,$A8,Respostas!$U$2:$U$126,"&gt;0")/COUNTIFS(Respostas!$B$2:$B$126,$A8))</f>
         <v/>
       </c>
     </row>

</xml_diff>